<commit_message>
Update loco downloads 2026-04-05 11:21:10
</commit_message>
<xml_diff>
--- a/downloads/loco_numbers_only.xlsx
+++ b/downloads/loco_numbers_only.xlsx
@@ -2799,27 +2799,27 @@
       </c>
       <c r="D58" s="1" t="inlineStr">
         <is>
-          <t>MM-796M</t>
+          <t>MM-792M</t>
         </is>
       </c>
       <c r="E58" s="1" t="inlineStr">
         <is>
-          <t>MM-972M</t>
+          <t>MM-970M</t>
         </is>
       </c>
       <c r="F58" s="1" t="inlineStr">
         <is>
-          <t>MRL001</t>
+          <t>MMY032</t>
         </is>
       </c>
       <c r="G58" s="1" t="inlineStr">
         <is>
-          <t>NR75</t>
+          <t>NR72</t>
         </is>
       </c>
       <c r="H58" s="1" t="inlineStr">
         <is>
-          <t>PHC002</t>
+          <t>PHC001</t>
         </is>
       </c>
     </row>
@@ -2841,27 +2841,27 @@
       </c>
       <c r="D59" s="1" t="inlineStr">
         <is>
-          <t>MM-798M</t>
+          <t>MM-796M</t>
         </is>
       </c>
       <c r="E59" s="1" t="inlineStr">
         <is>
-          <t>MM-974M</t>
+          <t>MM-972M</t>
         </is>
       </c>
       <c r="F59" s="1" t="inlineStr">
         <is>
-          <t>MRL004</t>
+          <t>MRL001</t>
         </is>
       </c>
       <c r="G59" s="1" t="inlineStr">
         <is>
-          <t>NR77</t>
+          <t>NR75</t>
         </is>
       </c>
       <c r="H59" s="1" t="inlineStr">
         <is>
-          <t>Q4001</t>
+          <t>PHC002</t>
         </is>
       </c>
     </row>
@@ -2883,27 +2883,27 @@
       </c>
       <c r="D60" s="1" t="inlineStr">
         <is>
-          <t>MM-800M</t>
+          <t>MM-798M</t>
         </is>
       </c>
       <c r="E60" s="1" t="inlineStr">
         <is>
-          <t>MM-976M</t>
+          <t>MM-974M</t>
         </is>
       </c>
       <c r="F60" s="1" t="inlineStr">
         <is>
-          <t>MRL006</t>
+          <t>MRL004</t>
         </is>
       </c>
       <c r="G60" s="1" t="inlineStr">
         <is>
-          <t>NR78</t>
+          <t>NR77</t>
         </is>
       </c>
       <c r="H60" s="1" t="inlineStr">
         <is>
-          <t>Q4003</t>
+          <t>Q4001</t>
         </is>
       </c>
     </row>
@@ -2925,27 +2925,27 @@
       </c>
       <c r="D61" s="1" t="inlineStr">
         <is>
-          <t>MM-802M</t>
+          <t>MM-800M</t>
         </is>
       </c>
       <c r="E61" s="1" t="inlineStr">
         <is>
-          <t>MM-980M</t>
+          <t>MM-976M</t>
         </is>
       </c>
       <c r="F61" s="1" t="inlineStr">
         <is>
-          <t>N452</t>
+          <t>MRL006</t>
         </is>
       </c>
       <c r="G61" s="1" t="inlineStr">
         <is>
-          <t>NR81</t>
+          <t>NR78</t>
         </is>
       </c>
       <c r="H61" s="1" t="inlineStr">
         <is>
-          <t>Q4004</t>
+          <t>Q4003</t>
         </is>
       </c>
     </row>
@@ -2967,27 +2967,27 @@
       </c>
       <c r="D62" s="1" t="inlineStr">
         <is>
-          <t>MM-804M</t>
+          <t>MM-802M</t>
         </is>
       </c>
       <c r="E62" s="1" t="inlineStr">
         <is>
-          <t>MM-982M</t>
+          <t>MM-980M</t>
         </is>
       </c>
       <c r="F62" s="1" t="inlineStr">
         <is>
-          <t>N453</t>
+          <t>N452</t>
         </is>
       </c>
       <c r="G62" s="1" t="inlineStr">
         <is>
-          <t>NR82</t>
+          <t>NR81</t>
         </is>
       </c>
       <c r="H62" s="1" t="inlineStr">
         <is>
-          <t>Q4005</t>
+          <t>Q4004</t>
         </is>
       </c>
     </row>
@@ -3009,27 +3009,27 @@
       </c>
       <c r="D63" s="1" t="inlineStr">
         <is>
-          <t>MM-808M</t>
+          <t>MM-804M</t>
         </is>
       </c>
       <c r="E63" s="1" t="inlineStr">
         <is>
-          <t>MM-984M</t>
+          <t>MM-982M</t>
         </is>
       </c>
       <c r="F63" s="1" t="inlineStr">
         <is>
-          <t>N457</t>
+          <t>N453</t>
         </is>
       </c>
       <c r="G63" s="1" t="inlineStr">
         <is>
-          <t>NR83</t>
+          <t>NR82</t>
         </is>
       </c>
       <c r="H63" s="1" t="inlineStr">
         <is>
-          <t>Q4006</t>
+          <t>Q4005</t>
         </is>
       </c>
     </row>
@@ -3051,27 +3051,27 @@
       </c>
       <c r="D64" s="1" t="inlineStr">
         <is>
-          <t>MM-810M</t>
+          <t>MM-808M</t>
         </is>
       </c>
       <c r="E64" s="1" t="inlineStr">
         <is>
-          <t>MM-986M</t>
+          <t>MM-984M</t>
         </is>
       </c>
       <c r="F64" s="1" t="inlineStr">
         <is>
-          <t>N458</t>
+          <t>N457</t>
         </is>
       </c>
       <c r="G64" s="1" t="inlineStr">
         <is>
-          <t>NR84</t>
+          <t>NR83</t>
         </is>
       </c>
       <c r="H64" s="1" t="inlineStr">
         <is>
-          <t>Q4007</t>
+          <t>Q4006</t>
         </is>
       </c>
     </row>
@@ -3093,27 +3093,27 @@
       </c>
       <c r="D65" s="1" t="inlineStr">
         <is>
-          <t>MM-814M</t>
+          <t>MM-810M</t>
         </is>
       </c>
       <c r="E65" s="1" t="inlineStr">
         <is>
-          <t>MM-9902M</t>
+          <t>MM-986M</t>
         </is>
       </c>
       <c r="F65" s="1" t="inlineStr">
         <is>
-          <t>N465</t>
+          <t>N458</t>
         </is>
       </c>
       <c r="G65" s="1" t="inlineStr">
         <is>
-          <t>NR85</t>
+          <t>NR84</t>
         </is>
       </c>
       <c r="H65" s="1" t="inlineStr">
         <is>
-          <t>Q4009</t>
+          <t>Q4007</t>
         </is>
       </c>
     </row>
@@ -3135,27 +3135,27 @@
       </c>
       <c r="D66" s="1" t="inlineStr">
         <is>
-          <t>MM-816M</t>
+          <t>MM-814M</t>
         </is>
       </c>
       <c r="E66" s="1" t="inlineStr">
         <is>
-          <t>MM-9903M</t>
+          <t>MM-9902M</t>
         </is>
       </c>
       <c r="F66" s="1" t="inlineStr">
         <is>
-          <t>N466</t>
+          <t>N465</t>
         </is>
       </c>
       <c r="G66" s="1" t="inlineStr">
         <is>
-          <t>NR86</t>
+          <t>NR85</t>
         </is>
       </c>
       <c r="H66" s="1" t="inlineStr">
         <is>
-          <t>Q4011</t>
+          <t>Q4009</t>
         </is>
       </c>
     </row>
@@ -3177,27 +3177,27 @@
       </c>
       <c r="D67" s="1" t="inlineStr">
         <is>
-          <t>MM-818M</t>
+          <t>MM-816M</t>
         </is>
       </c>
       <c r="E67" s="1" t="inlineStr">
         <is>
-          <t>MM-9904M</t>
+          <t>MM-9903M</t>
         </is>
       </c>
       <c r="F67" s="1" t="inlineStr">
         <is>
-          <t>N467</t>
+          <t>N466</t>
         </is>
       </c>
       <c r="G67" s="1" t="inlineStr">
         <is>
-          <t>NR87</t>
+          <t>NR86</t>
         </is>
       </c>
       <c r="H67" s="1" t="inlineStr">
         <is>
-          <t>Q4012</t>
+          <t>Q4011</t>
         </is>
       </c>
     </row>
@@ -3219,27 +3219,27 @@
       </c>
       <c r="D68" s="1" t="inlineStr">
         <is>
-          <t>MM-820M</t>
+          <t>MM-818M</t>
         </is>
       </c>
       <c r="E68" s="1" t="inlineStr">
         <is>
-          <t>MM-9906M</t>
+          <t>MM-9904M</t>
         </is>
       </c>
       <c r="F68" s="1" t="inlineStr">
         <is>
-          <t>N469</t>
+          <t>N467</t>
         </is>
       </c>
       <c r="G68" s="1" t="inlineStr">
         <is>
-          <t>NR88</t>
+          <t>NR87</t>
         </is>
       </c>
       <c r="H68" s="1" t="inlineStr">
         <is>
-          <t>Q4013</t>
+          <t>Q4012</t>
         </is>
       </c>
     </row>
@@ -3261,27 +3261,27 @@
       </c>
       <c r="D69" s="1" t="inlineStr">
         <is>
-          <t>MM-824M</t>
+          <t>MM-820M</t>
         </is>
       </c>
       <c r="E69" s="1" t="inlineStr">
         <is>
-          <t>MM-9907M</t>
+          <t>MM-9906M</t>
         </is>
       </c>
       <c r="F69" s="1" t="inlineStr">
         <is>
-          <t>N473</t>
+          <t>N469</t>
         </is>
       </c>
       <c r="G69" s="1" t="inlineStr">
         <is>
-          <t>NR89</t>
+          <t>NR88</t>
         </is>
       </c>
       <c r="H69" s="1" t="inlineStr">
         <is>
-          <t>Q4014</t>
+          <t>Q4013</t>
         </is>
       </c>
     </row>
@@ -3303,27 +3303,27 @@
       </c>
       <c r="D70" s="1" t="inlineStr">
         <is>
-          <t>MM-826M</t>
+          <t>MM-824M</t>
         </is>
       </c>
       <c r="E70" s="1" t="inlineStr">
         <is>
-          <t>MM-9908M</t>
+          <t>MM-9907M</t>
         </is>
       </c>
       <c r="F70" s="1" t="inlineStr">
         <is>
-          <t>NR1</t>
+          <t>N473</t>
         </is>
       </c>
       <c r="G70" s="1" t="inlineStr">
         <is>
-          <t>NR90</t>
+          <t>NR89</t>
         </is>
       </c>
       <c r="H70" s="1" t="inlineStr">
         <is>
-          <t>Q4015</t>
+          <t>Q4014</t>
         </is>
       </c>
     </row>
@@ -3345,27 +3345,27 @@
       </c>
       <c r="D71" s="1" t="inlineStr">
         <is>
-          <t>MM-828M</t>
+          <t>MM-826M</t>
         </is>
       </c>
       <c r="E71" s="1" t="inlineStr">
         <is>
-          <t>MM-9909M</t>
+          <t>MM-9908M</t>
         </is>
       </c>
       <c r="F71" s="1" t="inlineStr">
         <is>
-          <t>NR2</t>
+          <t>NR1</t>
         </is>
       </c>
       <c r="G71" s="1" t="inlineStr">
         <is>
-          <t>NR91</t>
+          <t>NR90</t>
         </is>
       </c>
       <c r="H71" s="1" t="inlineStr">
         <is>
-          <t>Q4016</t>
+          <t>Q4015</t>
         </is>
       </c>
     </row>
@@ -3382,32 +3382,32 @@
       </c>
       <c r="C72" s="1" t="inlineStr">
         <is>
-          <t>MM-588M</t>
+          <t>MM-580M</t>
         </is>
       </c>
       <c r="D72" s="1" t="inlineStr">
         <is>
-          <t>MM-830M</t>
+          <t>MM-828M</t>
         </is>
       </c>
       <c r="E72" s="1" t="inlineStr">
         <is>
-          <t>MM-9912M</t>
+          <t>MM-9909M</t>
         </is>
       </c>
       <c r="F72" s="1" t="inlineStr">
         <is>
-          <t>NR4</t>
+          <t>NR2</t>
         </is>
       </c>
       <c r="G72" s="1" t="inlineStr">
         <is>
-          <t>NR92</t>
+          <t>NR91</t>
         </is>
       </c>
       <c r="H72" s="1" t="inlineStr">
         <is>
-          <t>Q4017</t>
+          <t>Q4016</t>
         </is>
       </c>
     </row>
@@ -3424,32 +3424,32 @@
       </c>
       <c r="C73" s="1" t="inlineStr">
         <is>
-          <t>MM-602M</t>
+          <t>MM-588M</t>
         </is>
       </c>
       <c r="D73" s="1" t="inlineStr">
         <is>
-          <t>MM-832M</t>
+          <t>MM-830M</t>
         </is>
       </c>
       <c r="E73" s="1" t="inlineStr">
         <is>
-          <t>MM-9913M</t>
+          <t>MM-9912M</t>
         </is>
       </c>
       <c r="F73" s="1" t="inlineStr">
         <is>
-          <t>NR5</t>
+          <t>NR4</t>
         </is>
       </c>
       <c r="G73" s="1" t="inlineStr">
         <is>
-          <t>NR93</t>
+          <t>NR92</t>
         </is>
       </c>
       <c r="H73" s="1" t="inlineStr">
         <is>
-          <t>Q4019</t>
+          <t>Q4017</t>
         </is>
       </c>
     </row>
@@ -3466,32 +3466,32 @@
       </c>
       <c r="C74" s="1" t="inlineStr">
         <is>
-          <t>MM-616M</t>
+          <t>MM-602M</t>
         </is>
       </c>
       <c r="D74" s="1" t="inlineStr">
         <is>
-          <t>MM-834M</t>
+          <t>MM-832M</t>
         </is>
       </c>
       <c r="E74" s="1" t="inlineStr">
         <is>
-          <t>MM-9914M</t>
+          <t>MM-9913M</t>
         </is>
       </c>
       <c r="F74" s="1" t="inlineStr">
         <is>
-          <t>NR7</t>
+          <t>NR5</t>
         </is>
       </c>
       <c r="G74" s="1" t="inlineStr">
         <is>
-          <t>NR94</t>
+          <t>NR93</t>
         </is>
       </c>
       <c r="H74" s="1" t="inlineStr">
         <is>
-          <t>QBX003</t>
+          <t>Q4019</t>
         </is>
       </c>
     </row>
@@ -3508,32 +3508,32 @@
       </c>
       <c r="C75" s="1" t="inlineStr">
         <is>
-          <t>MM-624M</t>
+          <t>MM-616M</t>
         </is>
       </c>
       <c r="D75" s="1" t="inlineStr">
         <is>
-          <t>MM-838M</t>
+          <t>MM-834M</t>
         </is>
       </c>
       <c r="E75" s="1" t="inlineStr">
         <is>
-          <t>MM-9915M</t>
+          <t>MM-9914M</t>
         </is>
       </c>
       <c r="F75" s="1" t="inlineStr">
         <is>
-          <t>NR8</t>
+          <t>NR7</t>
         </is>
       </c>
       <c r="G75" s="1" t="inlineStr">
         <is>
-          <t>NR95</t>
+          <t>NR94</t>
         </is>
       </c>
       <c r="H75" s="1" t="inlineStr">
         <is>
-          <t>QBX004</t>
+          <t>QBX003</t>
         </is>
       </c>
     </row>
@@ -3550,32 +3550,32 @@
       </c>
       <c r="C76" s="1" t="inlineStr">
         <is>
-          <t>MM-632M</t>
+          <t>MM-624M</t>
         </is>
       </c>
       <c r="D76" s="1" t="inlineStr">
         <is>
-          <t>MM-842M</t>
+          <t>MM-838M</t>
         </is>
       </c>
       <c r="E76" s="1" t="inlineStr">
         <is>
-          <t>MM-9917M</t>
+          <t>MM-9915M</t>
         </is>
       </c>
       <c r="F76" s="1" t="inlineStr">
         <is>
-          <t>NR9</t>
+          <t>NR8</t>
         </is>
       </c>
       <c r="G76" s="1" t="inlineStr">
         <is>
-          <t>NR96</t>
+          <t>NR95</t>
         </is>
       </c>
       <c r="H76" s="1" t="inlineStr">
         <is>
-          <t>QBX005</t>
+          <t>QBX004</t>
         </is>
       </c>
     </row>
@@ -3592,32 +3592,32 @@
       </c>
       <c r="C77" s="1" t="inlineStr">
         <is>
-          <t>MM-636M</t>
+          <t>MM-632M</t>
         </is>
       </c>
       <c r="D77" s="1" t="inlineStr">
         <is>
-          <t>MM-844M</t>
+          <t>MM-842M</t>
         </is>
       </c>
       <c r="E77" s="1" t="inlineStr">
         <is>
-          <t>MM-9918M</t>
+          <t>MM-9917M</t>
         </is>
       </c>
       <c r="F77" s="1" t="inlineStr">
         <is>
-          <t>NR12</t>
+          <t>NR9</t>
         </is>
       </c>
       <c r="G77" s="1" t="inlineStr">
         <is>
-          <t>NR98</t>
+          <t>NR96</t>
         </is>
       </c>
       <c r="H77" s="1" t="inlineStr">
         <is>
-          <t>QBX006</t>
+          <t>QBX005</t>
         </is>
       </c>
     </row>
@@ -3634,32 +3634,32 @@
       </c>
       <c r="C78" s="1" t="inlineStr">
         <is>
-          <t>MM-640M</t>
+          <t>MM-636M</t>
         </is>
       </c>
       <c r="D78" s="1" t="inlineStr">
         <is>
-          <t>MM-852M</t>
+          <t>MM-844M</t>
         </is>
       </c>
       <c r="E78" s="1" t="inlineStr">
         <is>
-          <t>MM-9919M</t>
+          <t>MM-9918M</t>
         </is>
       </c>
       <c r="F78" s="1" t="inlineStr">
         <is>
-          <t>NR15</t>
+          <t>NR12</t>
         </is>
       </c>
       <c r="G78" s="1" t="inlineStr">
         <is>
-          <t>NR99</t>
+          <t>NR98</t>
         </is>
       </c>
       <c r="H78" s="1" t="inlineStr">
         <is>
-          <t>QE001</t>
+          <t>QBX006</t>
         </is>
       </c>
     </row>
@@ -3676,32 +3676,32 @@
       </c>
       <c r="C79" s="1" t="inlineStr">
         <is>
-          <t>MM-654M</t>
+          <t>MM-640M</t>
         </is>
       </c>
       <c r="D79" s="1" t="inlineStr">
         <is>
-          <t>MM-858M</t>
+          <t>MM-852M</t>
         </is>
       </c>
       <c r="E79" s="1" t="inlineStr">
         <is>
-          <t>MM-9920M</t>
+          <t>MM-9919M</t>
         </is>
       </c>
       <c r="F79" s="1" t="inlineStr">
         <is>
-          <t>NR16</t>
+          <t>NR15</t>
         </is>
       </c>
       <c r="G79" s="1" t="inlineStr">
         <is>
-          <t>NR101</t>
+          <t>NR99</t>
         </is>
       </c>
       <c r="H79" s="1" t="inlineStr">
         <is>
-          <t>QE002</t>
+          <t>QE001</t>
         </is>
       </c>
     </row>
@@ -3718,32 +3718,32 @@
       </c>
       <c r="C80" s="1" t="inlineStr">
         <is>
-          <t>MM-656M</t>
+          <t>MM-654M</t>
         </is>
       </c>
       <c r="D80" s="1" t="inlineStr">
         <is>
-          <t>MM-860M</t>
+          <t>MM-858M</t>
         </is>
       </c>
       <c r="E80" s="1" t="inlineStr">
         <is>
-          <t>MM-9922M</t>
+          <t>MM-9920M</t>
         </is>
       </c>
       <c r="F80" s="1" t="inlineStr">
         <is>
-          <t>NR18</t>
+          <t>NR16</t>
         </is>
       </c>
       <c r="G80" s="1" t="inlineStr">
         <is>
-          <t>NR102</t>
+          <t>NR101</t>
         </is>
       </c>
       <c r="H80" s="1" t="inlineStr">
         <is>
-          <t>QE003</t>
+          <t>QE002</t>
         </is>
       </c>
     </row>
@@ -3760,32 +3760,32 @@
       </c>
       <c r="C81" s="1" t="inlineStr">
         <is>
-          <t>MM-660M</t>
+          <t>MM-656M</t>
         </is>
       </c>
       <c r="D81" s="1" t="inlineStr">
         <is>
-          <t>MM-862M</t>
+          <t>MM-860M</t>
         </is>
       </c>
       <c r="E81" s="1" t="inlineStr">
         <is>
-          <t>MM-9923M</t>
+          <t>MM-9922M</t>
         </is>
       </c>
       <c r="F81" s="1" t="inlineStr">
         <is>
-          <t>NR19</t>
+          <t>NR18</t>
         </is>
       </c>
       <c r="G81" s="1" t="inlineStr">
         <is>
-          <t>NR103</t>
+          <t>NR102</t>
         </is>
       </c>
       <c r="H81" s="1" t="inlineStr">
         <is>
-          <t>QE004</t>
+          <t>QE003</t>
         </is>
       </c>
     </row>
@@ -3802,32 +3802,32 @@
       </c>
       <c r="C82" s="1" t="inlineStr">
         <is>
-          <t>MM-661M</t>
+          <t>MM-660M</t>
         </is>
       </c>
       <c r="D82" s="1" t="inlineStr">
         <is>
-          <t>MM-868M</t>
+          <t>MM-862M</t>
         </is>
       </c>
       <c r="E82" s="1" t="inlineStr">
         <is>
-          <t>MM-9924M</t>
+          <t>MM-9923M</t>
         </is>
       </c>
       <c r="F82" s="1" t="inlineStr">
         <is>
-          <t>NR21</t>
+          <t>NR19</t>
         </is>
       </c>
       <c r="G82" s="1" t="inlineStr">
         <is>
-          <t>NR105</t>
+          <t>NR103</t>
         </is>
       </c>
       <c r="H82" s="1" t="inlineStr">
         <is>
-          <t>QE006</t>
+          <t>QE004</t>
         </is>
       </c>
     </row>
@@ -3844,32 +3844,32 @@
       </c>
       <c r="C83" s="1" t="inlineStr">
         <is>
-          <t>MM-662M</t>
+          <t>MM-661M</t>
         </is>
       </c>
       <c r="D83" s="1" t="inlineStr">
         <is>
-          <t>MM-872M</t>
+          <t>MM-868M</t>
         </is>
       </c>
       <c r="E83" s="1" t="inlineStr">
         <is>
-          <t>MM-9926M</t>
+          <t>MM-9924M</t>
         </is>
       </c>
       <c r="F83" s="1" t="inlineStr">
         <is>
-          <t>NR25</t>
+          <t>NR21</t>
         </is>
       </c>
       <c r="G83" s="1" t="inlineStr">
         <is>
-          <t>NR108</t>
+          <t>NR105</t>
         </is>
       </c>
       <c r="H83" s="1" t="inlineStr">
         <is>
-          <t>QL001</t>
+          <t>QE006</t>
         </is>
       </c>
     </row>
@@ -3886,32 +3886,32 @@
       </c>
       <c r="C84" s="1" t="inlineStr">
         <is>
-          <t>MM-664M</t>
+          <t>MM-662M</t>
         </is>
       </c>
       <c r="D84" s="1" t="inlineStr">
         <is>
-          <t>MM-874M</t>
+          <t>MM-872M</t>
         </is>
       </c>
       <c r="E84" s="1" t="inlineStr">
         <is>
-          <t>MM-9928M</t>
+          <t>MM-9926M</t>
         </is>
       </c>
       <c r="F84" s="1" t="inlineStr">
         <is>
-          <t>NR27</t>
+          <t>NR25</t>
         </is>
       </c>
       <c r="G84" s="1" t="inlineStr">
         <is>
-          <t>NR109</t>
+          <t>NR108</t>
         </is>
       </c>
       <c r="H84" s="1" t="inlineStr">
         <is>
-          <t>QL002</t>
+          <t>QL001</t>
         </is>
       </c>
     </row>
@@ -3928,32 +3928,32 @@
       </c>
       <c r="C85" s="1" t="inlineStr">
         <is>
-          <t>MM-666M</t>
+          <t>MM-664M</t>
         </is>
       </c>
       <c r="D85" s="1" t="inlineStr">
         <is>
-          <t>MM-876M</t>
+          <t>MM-874M</t>
         </is>
       </c>
       <c r="E85" s="1" t="inlineStr">
         <is>
-          <t>MM-9929M</t>
+          <t>MM-9928M</t>
         </is>
       </c>
       <c r="F85" s="1" t="inlineStr">
         <is>
-          <t>NR28</t>
+          <t>NR27</t>
         </is>
       </c>
       <c r="G85" s="1" t="inlineStr">
         <is>
-          <t>NR110</t>
+          <t>NR109</t>
         </is>
       </c>
       <c r="H85" s="1" t="inlineStr">
         <is>
-          <t>QL004</t>
+          <t>QL002</t>
         </is>
       </c>
     </row>
@@ -3970,32 +3970,32 @@
       </c>
       <c r="C86" s="1" t="inlineStr">
         <is>
-          <t>MM-668M</t>
+          <t>MM-666M</t>
         </is>
       </c>
       <c r="D86" s="1" t="inlineStr">
         <is>
-          <t>MM-882M</t>
+          <t>MM-876M</t>
         </is>
       </c>
       <c r="E86" s="1" t="inlineStr">
         <is>
-          <t>MM-9932M</t>
+          <t>MM-9929M</t>
         </is>
       </c>
       <c r="F86" s="1" t="inlineStr">
         <is>
-          <t>NR30</t>
+          <t>NR28</t>
         </is>
       </c>
       <c r="G86" s="1" t="inlineStr">
         <is>
-          <t>NR111</t>
+          <t>NR110</t>
         </is>
       </c>
       <c r="H86" s="1" t="inlineStr">
         <is>
-          <t>QL007</t>
+          <t>QL004</t>
         </is>
       </c>
     </row>
@@ -4012,32 +4012,32 @@
       </c>
       <c r="C87" s="1" t="inlineStr">
         <is>
-          <t>MM-673M</t>
+          <t>MM-668M</t>
         </is>
       </c>
       <c r="D87" s="1" t="inlineStr">
         <is>
-          <t>MM-894M</t>
+          <t>MM-882M</t>
         </is>
       </c>
       <c r="E87" s="1" t="inlineStr">
         <is>
-          <t>MM-9933M</t>
+          <t>MM-9932M</t>
         </is>
       </c>
       <c r="F87" s="1" t="inlineStr">
         <is>
-          <t>NR31</t>
+          <t>NR30</t>
         </is>
       </c>
       <c r="G87" s="1" t="inlineStr">
         <is>
-          <t>NR112</t>
+          <t>NR111</t>
         </is>
       </c>
       <c r="H87" s="1" t="inlineStr">
         <is>
-          <t>QL008</t>
+          <t>QL007</t>
         </is>
       </c>
     </row>
@@ -4054,32 +4054,32 @@
       </c>
       <c r="C88" s="1" t="inlineStr">
         <is>
-          <t>MM-674M</t>
+          <t>MM-673M</t>
         </is>
       </c>
       <c r="D88" s="1" t="inlineStr">
         <is>
-          <t>MM-896M</t>
+          <t>MM-894M</t>
         </is>
       </c>
       <c r="E88" s="1" t="inlineStr">
         <is>
-          <t>MM-9934M</t>
+          <t>MM-9933M</t>
         </is>
       </c>
       <c r="F88" s="1" t="inlineStr">
         <is>
-          <t>NR34</t>
+          <t>NR31</t>
         </is>
       </c>
       <c r="G88" s="1" t="inlineStr">
         <is>
-          <t>NR113</t>
+          <t>NR112</t>
         </is>
       </c>
       <c r="H88" s="1" t="inlineStr">
         <is>
-          <t>QL010</t>
+          <t>QL008</t>
         </is>
       </c>
     </row>
@@ -4096,32 +4096,32 @@
       </c>
       <c r="C89" s="1" t="inlineStr">
         <is>
-          <t>MM-680M</t>
+          <t>MM-674M</t>
         </is>
       </c>
       <c r="D89" s="1" t="inlineStr">
         <is>
-          <t>MM-902M</t>
+          <t>MM-896M</t>
         </is>
       </c>
       <c r="E89" s="1" t="inlineStr">
         <is>
-          <t>MM-9936M</t>
+          <t>MM-9934M</t>
         </is>
       </c>
       <c r="F89" s="1" t="inlineStr">
         <is>
-          <t>NR36</t>
+          <t>NR34</t>
         </is>
       </c>
       <c r="G89" s="1" t="inlineStr">
         <is>
-          <t>NR115</t>
+          <t>NR113</t>
         </is>
       </c>
       <c r="H89" s="1" t="inlineStr">
         <is>
-          <t>QL011</t>
+          <t>QL010</t>
         </is>
       </c>
     </row>
@@ -4138,32 +4138,32 @@
       </c>
       <c r="C90" s="1" t="inlineStr">
         <is>
-          <t>MM-708M</t>
+          <t>MM-680M</t>
         </is>
       </c>
       <c r="D90" s="1" t="inlineStr">
         <is>
-          <t>MM-904M</t>
+          <t>MM-902M</t>
         </is>
       </c>
       <c r="E90" s="1" t="inlineStr">
         <is>
-          <t>MM-9938M</t>
+          <t>MM-9936M</t>
         </is>
       </c>
       <c r="F90" s="1" t="inlineStr">
         <is>
-          <t>NR37</t>
+          <t>NR36</t>
         </is>
       </c>
       <c r="G90" s="1" t="inlineStr">
         <is>
-          <t>NR118</t>
+          <t>NR115</t>
         </is>
       </c>
       <c r="H90" s="1" t="inlineStr">
         <is>
-          <t>QL014</t>
+          <t>QL011</t>
         </is>
       </c>
     </row>
@@ -4180,32 +4180,32 @@
       </c>
       <c r="C91" s="1" t="inlineStr">
         <is>
-          <t>MM-710M</t>
+          <t>MM-708M</t>
         </is>
       </c>
       <c r="D91" s="1" t="inlineStr">
         <is>
-          <t>MM-906M</t>
+          <t>MM-904M</t>
         </is>
       </c>
       <c r="E91" s="1" t="inlineStr">
         <is>
-          <t>MM-9941M</t>
+          <t>MM-9938M</t>
         </is>
       </c>
       <c r="F91" s="1" t="inlineStr">
         <is>
-          <t>NR38</t>
+          <t>NR37</t>
         </is>
       </c>
       <c r="G91" s="1" t="inlineStr">
         <is>
-          <t>NR119</t>
+          <t>NR118</t>
         </is>
       </c>
       <c r="H91" s="1" t="inlineStr">
         <is>
-          <t>QL018</t>
+          <t>QL014</t>
         </is>
       </c>
     </row>
@@ -4222,32 +4222,32 @@
       </c>
       <c r="C92" s="1" t="inlineStr">
         <is>
-          <t>MM-716M</t>
+          <t>MM-710M</t>
         </is>
       </c>
       <c r="D92" s="1" t="inlineStr">
         <is>
-          <t>MM-908M</t>
+          <t>MM-906M</t>
         </is>
       </c>
       <c r="E92" s="1" t="inlineStr">
         <is>
-          <t>MM-9943M</t>
+          <t>MM-9941M</t>
         </is>
       </c>
       <c r="F92" s="1" t="inlineStr">
         <is>
-          <t>NR39</t>
+          <t>NR38</t>
         </is>
       </c>
       <c r="G92" s="1" t="inlineStr">
         <is>
-          <t>NR120</t>
+          <t>NR119</t>
         </is>
       </c>
       <c r="H92" s="1" t="inlineStr">
         <is>
-          <t>QR1744</t>
+          <t>QL018</t>
         </is>
       </c>
     </row>
@@ -4264,32 +4264,32 @@
       </c>
       <c r="C93" s="1" t="inlineStr">
         <is>
-          <t>MM-722M</t>
+          <t>MM-716M</t>
         </is>
       </c>
       <c r="D93" s="1" t="inlineStr">
         <is>
-          <t>MM-910M</t>
+          <t>MM-908M</t>
         </is>
       </c>
       <c r="E93" s="1" t="inlineStr">
         <is>
-          <t>MM-9945M</t>
+          <t>MM-9943M</t>
         </is>
       </c>
       <c r="F93" s="1" t="inlineStr">
         <is>
-          <t>NR40</t>
+          <t>NR39</t>
         </is>
       </c>
       <c r="G93" s="1" t="inlineStr">
         <is>
-          <t>NR122</t>
+          <t>NR120</t>
         </is>
       </c>
       <c r="H93" s="1" t="inlineStr">
         <is>
-          <t>QR1771</t>
+          <t>QR1744</t>
         </is>
       </c>
     </row>
@@ -4306,32 +4306,32 @@
       </c>
       <c r="C94" s="1" t="inlineStr">
         <is>
-          <t>MM-726M</t>
+          <t>MM-722M</t>
         </is>
       </c>
       <c r="D94" s="1" t="inlineStr">
         <is>
-          <t>MM-912M</t>
+          <t>MM-910M</t>
         </is>
       </c>
       <c r="E94" s="1" t="inlineStr">
         <is>
-          <t>MM-9946M</t>
+          <t>MM-9945M</t>
         </is>
       </c>
       <c r="F94" s="1" t="inlineStr">
         <is>
-          <t>NR43</t>
+          <t>NR40</t>
         </is>
       </c>
       <c r="G94" s="1" t="inlineStr">
         <is>
-          <t>P14</t>
+          <t>NR122</t>
         </is>
       </c>
       <c r="H94" s="1" t="inlineStr">
         <is>
-          <t>QR5404</t>
+          <t>QR1771</t>
         </is>
       </c>
     </row>
@@ -4348,32 +4348,32 @@
       </c>
       <c r="C95" s="1" t="inlineStr">
         <is>
-          <t>MM-728M</t>
+          <t>MM-726M</t>
         </is>
       </c>
       <c r="D95" s="1" t="inlineStr">
         <is>
-          <t>MM-914M</t>
+          <t>MM-912M</t>
         </is>
       </c>
       <c r="E95" s="1" t="inlineStr">
         <is>
-          <t>MM-9950M</t>
+          <t>MM-9946M</t>
         </is>
       </c>
       <c r="F95" s="1" t="inlineStr">
         <is>
-          <t>NR44</t>
+          <t>NR43</t>
         </is>
       </c>
       <c r="G95" s="1" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P14</t>
         </is>
       </c>
       <c r="H95" s="1" t="inlineStr">
         <is>
-          <t>R711</t>
+          <t>QR5404</t>
         </is>
       </c>
     </row>
@@ -4390,32 +4390,32 @@
       </c>
       <c r="C96" s="1" t="inlineStr">
         <is>
-          <t>MM-734M</t>
+          <t>MM-728M</t>
         </is>
       </c>
       <c r="D96" s="1" t="inlineStr">
         <is>
-          <t>MM-920M</t>
+          <t>MM-914M</t>
         </is>
       </c>
       <c r="E96" s="1" t="inlineStr">
         <is>
-          <t>MM-9951M</t>
+          <t>MM-9950M</t>
         </is>
       </c>
       <c r="F96" s="1" t="inlineStr">
         <is>
-          <t>NR45</t>
+          <t>NR44</t>
         </is>
       </c>
       <c r="G96" s="1" t="inlineStr">
         <is>
-          <t>P2501</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="H96" s="1" t="inlineStr">
         <is>
-          <t>R766</t>
+          <t>R711</t>
         </is>
       </c>
     </row>
@@ -4432,32 +4432,32 @@
       </c>
       <c r="C97" s="1" t="inlineStr">
         <is>
-          <t>MM-736M</t>
+          <t>MM-734M</t>
         </is>
       </c>
       <c r="D97" s="1" t="inlineStr">
         <is>
-          <t>MM-922M</t>
+          <t>MM-920M</t>
         </is>
       </c>
       <c r="E97" s="1" t="inlineStr">
         <is>
-          <t>MM-9952M</t>
+          <t>MM-9951M</t>
         </is>
       </c>
       <c r="F97" s="1" t="inlineStr">
         <is>
-          <t>NR48</t>
+          <t>NR45</t>
         </is>
       </c>
       <c r="G97" s="1" t="inlineStr">
         <is>
-          <t>P2502</t>
+          <t>P2501</t>
         </is>
       </c>
       <c r="H97" s="1" t="inlineStr">
         <is>
-          <t>RB2353</t>
+          <t>R766</t>
         </is>
       </c>
     </row>
@@ -4474,32 +4474,32 @@
       </c>
       <c r="C98" s="1" t="inlineStr">
         <is>
-          <t>MM-738M</t>
+          <t>MM-736M</t>
         </is>
       </c>
       <c r="D98" s="1" t="inlineStr">
         <is>
-          <t>MM-924M</t>
+          <t>MM-922M</t>
         </is>
       </c>
       <c r="E98" s="1" t="inlineStr">
         <is>
-          <t>MM-9953M</t>
+          <t>MM-9952M</t>
         </is>
       </c>
       <c r="F98" s="1" t="inlineStr">
         <is>
-          <t>NR51</t>
+          <t>NR48</t>
         </is>
       </c>
       <c r="G98" s="1" t="inlineStr">
         <is>
-          <t>P2503</t>
+          <t>P2502</t>
         </is>
       </c>
       <c r="H98" s="1" t="inlineStr">
         <is>
-          <t>RCTST4</t>
+          <t>RB2353</t>
         </is>
       </c>
     </row>
@@ -4516,32 +4516,32 @@
       </c>
       <c r="C99" s="1" t="inlineStr">
         <is>
-          <t>MM-740M</t>
+          <t>MM-738M</t>
         </is>
       </c>
       <c r="D99" s="1" t="inlineStr">
         <is>
-          <t>MM-926M</t>
+          <t>MM-924M</t>
         </is>
       </c>
       <c r="E99" s="1" t="inlineStr">
         <is>
-          <t>MM-9954M</t>
+          <t>MM-9953M</t>
         </is>
       </c>
       <c r="F99" s="1" t="inlineStr">
         <is>
-          <t>NR52</t>
+          <t>NR51</t>
         </is>
       </c>
       <c r="G99" s="1" t="inlineStr">
         <is>
-          <t>P2505</t>
+          <t>P2503</t>
         </is>
       </c>
       <c r="H99" s="1" t="inlineStr">
         <is>
-          <t>RL301</t>
+          <t>RCTST4</t>
         </is>
       </c>
     </row>
@@ -4558,32 +4558,32 @@
       </c>
       <c r="C100" s="1" t="inlineStr">
         <is>
-          <t>MM-742M</t>
+          <t>MM-740M</t>
         </is>
       </c>
       <c r="D100" s="1" t="inlineStr">
         <is>
-          <t>MM-934M</t>
+          <t>MM-926M</t>
         </is>
       </c>
       <c r="E100" s="1" t="inlineStr">
         <is>
-          <t>MM-9955M</t>
+          <t>MM-9954M</t>
         </is>
       </c>
       <c r="F100" s="1" t="inlineStr">
         <is>
-          <t>NR53</t>
+          <t>NR52</t>
         </is>
       </c>
       <c r="G100" s="1" t="inlineStr">
         <is>
-          <t>P2506</t>
+          <t>P2505</t>
         </is>
       </c>
       <c r="H100" s="1" t="inlineStr">
         <is>
-          <t>RL302</t>
+          <t>RL301</t>
         </is>
       </c>
     </row>
@@ -4600,32 +4600,32 @@
       </c>
       <c r="C101" s="1" t="inlineStr">
         <is>
-          <t>MM-744M</t>
+          <t>MM-742M</t>
         </is>
       </c>
       <c r="D101" s="1" t="inlineStr">
         <is>
-          <t>MM-936M</t>
+          <t>MM-934M</t>
         </is>
       </c>
       <c r="E101" s="1" t="inlineStr">
         <is>
-          <t>MM-9957M</t>
+          <t>MM-9955M</t>
         </is>
       </c>
       <c r="F101" s="1" t="inlineStr">
         <is>
-          <t>NR54</t>
+          <t>NR53</t>
         </is>
       </c>
       <c r="G101" s="1" t="inlineStr">
         <is>
-          <t>P2507</t>
+          <t>P2506</t>
         </is>
       </c>
       <c r="H101" s="1" t="inlineStr">
         <is>
-          <t>RL304</t>
+          <t>RL302</t>
         </is>
       </c>
     </row>
@@ -4642,32 +4642,32 @@
       </c>
       <c r="C102" s="1" t="inlineStr">
         <is>
-          <t>MM-752M</t>
+          <t>MM-744M</t>
         </is>
       </c>
       <c r="D102" s="1" t="inlineStr">
         <is>
-          <t>MM-940M</t>
+          <t>MM-936M</t>
         </is>
       </c>
       <c r="E102" s="1" t="inlineStr">
         <is>
-          <t>MM-9959M</t>
+          <t>MM-9957M</t>
         </is>
       </c>
       <c r="F102" s="1" t="inlineStr">
         <is>
-          <t>NR57</t>
+          <t>NR54</t>
         </is>
       </c>
       <c r="G102" s="1" t="inlineStr">
         <is>
-          <t>P2508</t>
+          <t>P2507</t>
         </is>
       </c>
       <c r="H102" s="1" t="inlineStr">
         <is>
-          <t>RL305</t>
+          <t>RL304</t>
         </is>
       </c>
     </row>
@@ -4684,32 +4684,32 @@
       </c>
       <c r="C103" s="1" t="inlineStr">
         <is>
-          <t>MM-756M</t>
+          <t>MM-752M</t>
         </is>
       </c>
       <c r="D103" s="1" t="inlineStr">
         <is>
-          <t>MM-944M</t>
+          <t>MM-940M</t>
         </is>
       </c>
       <c r="E103" s="1" t="inlineStr">
         <is>
-          <t>MM-9960M</t>
+          <t>MM-9959M</t>
         </is>
       </c>
       <c r="F103" s="1" t="inlineStr">
         <is>
-          <t>NR59</t>
+          <t>NR57</t>
         </is>
       </c>
       <c r="G103" s="1" t="inlineStr">
         <is>
-          <t>P2509</t>
+          <t>P2508</t>
         </is>
       </c>
       <c r="H103" s="1" t="inlineStr">
         <is>
-          <t>RL307</t>
+          <t>RL305</t>
         </is>
       </c>
     </row>
@@ -4726,32 +4726,32 @@
       </c>
       <c r="C104" s="1" t="inlineStr">
         <is>
-          <t>MM-760M</t>
+          <t>MM-756M</t>
         </is>
       </c>
       <c r="D104" s="1" t="inlineStr">
         <is>
-          <t>MM-948M</t>
+          <t>MM-944M</t>
         </is>
       </c>
       <c r="E104" s="1" t="inlineStr">
         <is>
-          <t>MM-9961M</t>
+          <t>MM-9960M</t>
         </is>
       </c>
       <c r="F104" s="1" t="inlineStr">
         <is>
-          <t>NR61</t>
+          <t>NR59</t>
         </is>
       </c>
       <c r="G104" s="1" t="inlineStr">
         <is>
-          <t>P2510</t>
+          <t>P2509</t>
         </is>
       </c>
       <c r="H104" s="1" t="inlineStr">
         <is>
-          <t>RL309</t>
+          <t>RL307</t>
         </is>
       </c>
     </row>
@@ -4768,32 +4768,32 @@
       </c>
       <c r="C105" s="1" t="inlineStr">
         <is>
-          <t>MM-764M</t>
+          <t>MM-760M</t>
         </is>
       </c>
       <c r="D105" s="1" t="inlineStr">
         <is>
-          <t>MM-952M</t>
+          <t>MM-948M</t>
         </is>
       </c>
       <c r="E105" s="1" t="inlineStr">
         <is>
-          <t>MM-9962M</t>
+          <t>MM-9961M</t>
         </is>
       </c>
       <c r="F105" s="1" t="inlineStr">
         <is>
-          <t>NR62</t>
+          <t>NR61</t>
         </is>
       </c>
       <c r="G105" s="1" t="inlineStr">
         <is>
-          <t>P2511</t>
+          <t>P2510</t>
         </is>
       </c>
       <c r="H105" s="1" t="inlineStr">
         <is>
-          <t>RL310</t>
+          <t>RL309</t>
         </is>
       </c>
     </row>
@@ -4810,32 +4810,32 @@
       </c>
       <c r="C106" s="1" t="inlineStr">
         <is>
-          <t>MM-768M</t>
+          <t>MM-764M</t>
         </is>
       </c>
       <c r="D106" s="1" t="inlineStr">
         <is>
-          <t>MM-954M</t>
+          <t>MM-952M</t>
         </is>
       </c>
       <c r="E106" s="1" t="inlineStr">
         <is>
-          <t>MM-9963M</t>
+          <t>MM-9962M</t>
         </is>
       </c>
       <c r="F106" s="1" t="inlineStr">
         <is>
-          <t>NR64</t>
+          <t>NR62</t>
         </is>
       </c>
       <c r="G106" s="1" t="inlineStr">
         <is>
-          <t>P2513</t>
+          <t>P2511</t>
         </is>
       </c>
       <c r="H106" s="1" t="inlineStr">
         <is>
-          <t>S312</t>
+          <t>RL310</t>
         </is>
       </c>
     </row>
@@ -4852,32 +4852,32 @@
       </c>
       <c r="C107" s="1" t="inlineStr">
         <is>
-          <t>MM-774M</t>
+          <t>MM-768M</t>
         </is>
       </c>
       <c r="D107" s="1" t="inlineStr">
         <is>
-          <t>MM-956M</t>
+          <t>MM-954M</t>
         </is>
       </c>
       <c r="E107" s="1" t="inlineStr">
         <is>
-          <t>MM-9964M</t>
+          <t>MM-9963M</t>
         </is>
       </c>
       <c r="F107" s="1" t="inlineStr">
         <is>
-          <t>NR65</t>
+          <t>NR64</t>
         </is>
       </c>
       <c r="G107" s="1" t="inlineStr">
         <is>
-          <t>P2514</t>
+          <t>P2513</t>
         </is>
       </c>
       <c r="H107" s="1" t="inlineStr">
         <is>
-          <t>S317</t>
+          <t>S312</t>
         </is>
       </c>
     </row>
@@ -4894,32 +4894,32 @@
       </c>
       <c r="C108" s="1" t="inlineStr">
         <is>
-          <t>MM-776M</t>
+          <t>MM-774M</t>
         </is>
       </c>
       <c r="D108" s="1" t="inlineStr">
         <is>
-          <t>MM-958M</t>
+          <t>MM-956M</t>
         </is>
       </c>
       <c r="E108" s="1" t="inlineStr">
         <is>
-          <t>MM-9965M</t>
+          <t>MM-9964M</t>
         </is>
       </c>
       <c r="F108" s="1" t="inlineStr">
         <is>
-          <t>NR66</t>
+          <t>NR65</t>
         </is>
       </c>
       <c r="G108" s="1" t="inlineStr">
         <is>
-          <t>P2515</t>
+          <t>P2514</t>
         </is>
       </c>
       <c r="H108" s="1" t="inlineStr">
         <is>
-          <t>S3301</t>
+          <t>S317</t>
         </is>
       </c>
     </row>
@@ -4936,32 +4936,32 @@
       </c>
       <c r="C109" s="1" t="inlineStr">
         <is>
-          <t>MM-778M</t>
+          <t>MM-776M</t>
         </is>
       </c>
       <c r="D109" s="1" t="inlineStr">
         <is>
-          <t>MM-962M</t>
+          <t>MM-958M</t>
         </is>
       </c>
       <c r="E109" s="1" t="inlineStr">
         <is>
-          <t>MM-9966M</t>
+          <t>MM-9965M</t>
         </is>
       </c>
       <c r="F109" s="1" t="inlineStr">
         <is>
-          <t>NR67</t>
+          <t>NR66</t>
         </is>
       </c>
       <c r="G109" s="1" t="inlineStr">
         <is>
-          <t>P2516</t>
+          <t>P2515</t>
         </is>
       </c>
       <c r="H109" s="1" t="inlineStr">
         <is>
-          <t>S3302</t>
+          <t>S3301</t>
         </is>
       </c>
     </row>
@@ -4978,32 +4978,32 @@
       </c>
       <c r="C110" s="1" t="inlineStr">
         <is>
-          <t>MM-780M</t>
+          <t>MM-778M</t>
         </is>
       </c>
       <c r="D110" s="1" t="inlineStr">
         <is>
-          <t>MM-964M</t>
+          <t>MM-962M</t>
         </is>
       </c>
       <c r="E110" s="1" t="inlineStr">
         <is>
-          <t>MM-9967M</t>
+          <t>MM-9966M</t>
         </is>
       </c>
       <c r="F110" s="1" t="inlineStr">
         <is>
-          <t>NR68</t>
+          <t>NR67</t>
         </is>
       </c>
       <c r="G110" s="1" t="inlineStr">
         <is>
-          <t>PB1</t>
+          <t>P2516</t>
         </is>
       </c>
       <c r="H110" s="1" t="inlineStr">
         <is>
-          <t>S3304</t>
+          <t>S3302</t>
         </is>
       </c>
     </row>
@@ -5020,32 +5020,32 @@
       </c>
       <c r="C111" s="1" t="inlineStr">
         <is>
-          <t>MM-784M</t>
+          <t>MM-780M</t>
         </is>
       </c>
       <c r="D111" s="1" t="inlineStr">
         <is>
-          <t>MM-966M</t>
+          <t>MM-964M</t>
         </is>
       </c>
       <c r="E111" s="1" t="inlineStr">
         <is>
-          <t>MM-9969M</t>
+          <t>MM-9967M</t>
         </is>
       </c>
       <c r="F111" s="1" t="inlineStr">
         <is>
-          <t>NR69</t>
+          <t>NR68</t>
         </is>
       </c>
       <c r="G111" s="1" t="inlineStr">
         <is>
-          <t>PB2</t>
+          <t>PB1</t>
         </is>
       </c>
       <c r="H111" s="1" t="inlineStr">
         <is>
-          <t>S3305</t>
+          <t>S3304</t>
         </is>
       </c>
     </row>
@@ -5062,32 +5062,32 @@
       </c>
       <c r="C112" s="1" t="inlineStr">
         <is>
-          <t>MM-790M</t>
+          <t>MM-784M</t>
         </is>
       </c>
       <c r="D112" s="1" t="inlineStr">
         <is>
-          <t>MM-968M</t>
+          <t>MM-966M</t>
         </is>
       </c>
       <c r="E112" s="1" t="inlineStr">
         <is>
-          <t>MM-9970M</t>
+          <t>MM-9969M</t>
         </is>
       </c>
       <c r="F112" s="1" t="inlineStr">
         <is>
-          <t>NR71</t>
+          <t>NR69</t>
         </is>
       </c>
       <c r="G112" s="1" t="inlineStr">
         <is>
-          <t>PB4</t>
+          <t>PB2</t>
         </is>
       </c>
       <c r="H112" s="1" t="inlineStr">
         <is>
-          <t>S3306</t>
+          <t>S3305</t>
         </is>
       </c>
     </row>
@@ -5104,2079 +5104,2084 @@
       </c>
       <c r="C113" s="1" t="inlineStr">
         <is>
-          <t>MM-792M</t>
+          <t>MM-790M</t>
         </is>
       </c>
       <c r="D113" s="1" t="inlineStr">
         <is>
-          <t>MM-970M</t>
+          <t>MM-968M</t>
         </is>
       </c>
       <c r="E113" s="1" t="inlineStr">
         <is>
-          <t>MMY032</t>
+          <t>MM-9970M</t>
         </is>
       </c>
       <c r="F113" s="1" t="inlineStr">
         <is>
-          <t>NR72</t>
+          <t>NR71</t>
         </is>
       </c>
       <c r="G113" s="1" t="inlineStr">
         <is>
-          <t>PHC001</t>
+          <t>PB4</t>
         </is>
       </c>
       <c r="H113" s="1" t="inlineStr">
         <is>
-          <t>S3307</t>
+          <t>S3306</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
         <is>
-          <t>S3309</t>
+          <t>S3307</t>
         </is>
       </c>
       <c r="B115" s="1" t="inlineStr">
         <is>
-          <t>TT108</t>
+          <t>TT107</t>
         </is>
       </c>
       <c r="C115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8110</t>
+          <t>VLINE-8107</t>
         </is>
       </c>
       <c r="D115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8311</t>
+          <t>VLINE-8306</t>
         </is>
       </c>
       <c r="E115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8449</t>
+          <t>VLINE-8447</t>
         </is>
       </c>
       <c r="F115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8754</t>
+          <t>VLINE-8753</t>
         </is>
       </c>
       <c r="G115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8819</t>
+          <t>VLINE-8818</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
         <is>
-          <t>S3310</t>
+          <t>S3309</t>
         </is>
       </c>
       <c r="B116" s="1" t="inlineStr">
         <is>
-          <t>TT110</t>
+          <t>TT108</t>
         </is>
       </c>
       <c r="C116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8111</t>
+          <t>VLINE-8110</t>
         </is>
       </c>
       <c r="D116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8313</t>
+          <t>VLINE-8311</t>
         </is>
       </c>
       <c r="E116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8450</t>
+          <t>VLINE-8449</t>
         </is>
       </c>
       <c r="F116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8755</t>
+          <t>VLINE-8754</t>
         </is>
       </c>
       <c r="G116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8822</t>
+          <t>VLINE-8819</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="1" t="inlineStr">
         <is>
-          <t>S7001</t>
+          <t>S3310</t>
         </is>
       </c>
       <c r="B117" s="1" t="inlineStr">
         <is>
-          <t>TT113</t>
+          <t>TT110</t>
         </is>
       </c>
       <c r="C117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8113</t>
+          <t>VLINE-8111</t>
         </is>
       </c>
       <c r="D117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8314</t>
+          <t>VLINE-8313</t>
         </is>
       </c>
       <c r="E117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8451</t>
+          <t>VLINE-8450</t>
         </is>
       </c>
       <c r="F117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8756</t>
+          <t>VLINE-8755</t>
         </is>
       </c>
       <c r="G117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8860</t>
+          <t>VLINE-8822</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
         <is>
-          <t>S7002</t>
+          <t>S7001</t>
         </is>
       </c>
       <c r="B118" s="1" t="inlineStr">
         <is>
-          <t>TT114</t>
+          <t>TT113</t>
         </is>
       </c>
       <c r="C118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8114</t>
+          <t>VLINE-8113</t>
         </is>
       </c>
       <c r="D118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8316</t>
+          <t>VLINE-8314</t>
         </is>
       </c>
       <c r="E118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8452</t>
+          <t>VLINE-8451</t>
         </is>
       </c>
       <c r="F118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8757</t>
+          <t>VLINE-8756</t>
         </is>
       </c>
       <c r="G118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8861</t>
+          <t>VLINE-8860</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
         <is>
-          <t>S7003</t>
+          <t>S7002</t>
         </is>
       </c>
       <c r="B119" s="1" t="inlineStr">
         <is>
-          <t>TT115</t>
+          <t>TT114</t>
         </is>
       </c>
       <c r="C119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8115</t>
+          <t>VLINE-8114</t>
         </is>
       </c>
       <c r="D119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8318</t>
+          <t>VLINE-8316</t>
         </is>
       </c>
       <c r="E119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8453</t>
+          <t>VLINE-8452</t>
         </is>
       </c>
       <c r="F119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8758</t>
+          <t>VLINE-8757</t>
         </is>
       </c>
       <c r="G119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8862</t>
+          <t>VLINE-8861</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="1" t="inlineStr">
         <is>
-          <t>S7005</t>
+          <t>S7003</t>
         </is>
       </c>
       <c r="B120" s="1" t="inlineStr">
         <is>
-          <t>TT116</t>
+          <t>TT115</t>
         </is>
       </c>
       <c r="C120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8119</t>
+          <t>VLINE-8115</t>
         </is>
       </c>
       <c r="D120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8321</t>
+          <t>VLINE-8318</t>
         </is>
       </c>
       <c r="E120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8454</t>
+          <t>VLINE-8453</t>
         </is>
       </c>
       <c r="F120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8759</t>
+          <t>VLINE-8758</t>
         </is>
       </c>
       <c r="G120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8863</t>
+          <t>VLINE-8862</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="1" t="inlineStr">
         <is>
-          <t>S7006</t>
+          <t>S7005</t>
         </is>
       </c>
       <c r="B121" s="1" t="inlineStr">
         <is>
-          <t>TT117</t>
+          <t>TT116</t>
         </is>
       </c>
       <c r="C121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8120</t>
+          <t>VLINE-8119</t>
         </is>
       </c>
       <c r="D121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8323</t>
+          <t>VLINE-8321</t>
         </is>
       </c>
       <c r="E121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8455</t>
+          <t>VLINE-8454</t>
         </is>
       </c>
       <c r="F121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8760</t>
+          <t>VLINE-8759</t>
         </is>
       </c>
       <c r="G121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8864</t>
+          <t>VLINE-8863</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="1" t="inlineStr">
         <is>
-          <t>S7007</t>
+          <t>S7006</t>
         </is>
       </c>
       <c r="B122" s="1" t="inlineStr">
         <is>
-          <t>TT122</t>
+          <t>TT117</t>
         </is>
       </c>
       <c r="C122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8121</t>
+          <t>VLINE-8120</t>
         </is>
       </c>
       <c r="D122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8324</t>
+          <t>VLINE-8323</t>
         </is>
       </c>
       <c r="E122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8456</t>
+          <t>VLINE-8455</t>
         </is>
       </c>
       <c r="F122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8761</t>
+          <t>VLINE-8760</t>
         </is>
       </c>
       <c r="G122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8865</t>
+          <t>VLINE-8864</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="1" t="inlineStr">
         <is>
-          <t>S7008</t>
+          <t>S7007</t>
         </is>
       </c>
       <c r="B123" s="1" t="inlineStr">
         <is>
-          <t>TT127</t>
+          <t>TT122</t>
         </is>
       </c>
       <c r="C123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8123</t>
+          <t>VLINE-8121</t>
         </is>
       </c>
       <c r="D123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8325</t>
+          <t>VLINE-8324</t>
         </is>
       </c>
       <c r="E123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8457</t>
+          <t>VLINE-8456</t>
         </is>
       </c>
       <c r="F123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8762</t>
+          <t>VLINE-8761</t>
         </is>
       </c>
       <c r="G123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8866</t>
+          <t>VLINE-8865</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="1" t="inlineStr">
         <is>
-          <t>S7012</t>
+          <t>S7008</t>
         </is>
       </c>
       <c r="B124" s="1" t="inlineStr">
         <is>
-          <t>TT128</t>
+          <t>TT127</t>
         </is>
       </c>
       <c r="C124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8124</t>
+          <t>VLINE-8123</t>
         </is>
       </c>
       <c r="D124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8328</t>
+          <t>VLINE-8325</t>
         </is>
       </c>
       <c r="E124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8460</t>
+          <t>VLINE-8457</t>
         </is>
       </c>
       <c r="F124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8763</t>
+          <t>VLINE-8762</t>
         </is>
       </c>
       <c r="G124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8867</t>
+          <t>VLINE-8866</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="1" t="inlineStr">
         <is>
-          <t>S7014</t>
+          <t>S7012</t>
         </is>
       </c>
       <c r="B125" s="1" t="inlineStr">
         <is>
-          <t>TT130</t>
+          <t>TT128</t>
         </is>
       </c>
       <c r="C125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8126</t>
+          <t>VLINE-8124</t>
         </is>
       </c>
       <c r="D125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8329</t>
+          <t>VLINE-8328</t>
         </is>
       </c>
       <c r="E125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8461</t>
+          <t>VLINE-8460</t>
         </is>
       </c>
       <c r="F125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8765</t>
+          <t>VLINE-8763</t>
         </is>
       </c>
       <c r="G125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8868</t>
+          <t>VLINE-8867</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="1" t="inlineStr">
         <is>
-          <t>S7015</t>
+          <t>S7014</t>
         </is>
       </c>
       <c r="B126" s="1" t="inlineStr">
         <is>
-          <t>TT131</t>
+          <t>TT130</t>
         </is>
       </c>
       <c r="C126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8127</t>
+          <t>VLINE-8126</t>
         </is>
       </c>
       <c r="D126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8332</t>
+          <t>VLINE-8329</t>
         </is>
       </c>
       <c r="E126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8464</t>
+          <t>VLINE-8461</t>
         </is>
       </c>
       <c r="F126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8766</t>
+          <t>VLINE-8765</t>
         </is>
       </c>
       <c r="G126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8869</t>
+          <t>VLINE-8868</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
         <is>
-          <t>S7017</t>
+          <t>S7015</t>
         </is>
       </c>
       <c r="B127" s="1" t="inlineStr">
         <is>
-          <t>TT202</t>
+          <t>TT131</t>
         </is>
       </c>
       <c r="C127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8128</t>
+          <t>VLINE-8127</t>
         </is>
       </c>
       <c r="D127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8336</t>
+          <t>VLINE-8332</t>
         </is>
       </c>
       <c r="E127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8465</t>
+          <t>VLINE-8464</t>
         </is>
       </c>
       <c r="F127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8767</t>
+          <t>VLINE-8766</t>
         </is>
       </c>
       <c r="G127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8890</t>
+          <t>VLINE-8869</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
         <is>
-          <t>S7018</t>
+          <t>S7017</t>
         </is>
       </c>
       <c r="B128" s="1" t="inlineStr">
         <is>
-          <t>TT206</t>
+          <t>TT202</t>
         </is>
       </c>
       <c r="C128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8129</t>
+          <t>VLINE-8128</t>
         </is>
       </c>
       <c r="D128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8337</t>
+          <t>VLINE-8336</t>
         </is>
       </c>
       <c r="E128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8468</t>
+          <t>VLINE-8465</t>
         </is>
       </c>
       <c r="F128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8768</t>
+          <t>VLINE-8767</t>
         </is>
       </c>
       <c r="G128" s="1" t="inlineStr">
         <is>
-          <t>WH001</t>
+          <t>VLINE-8890</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
         <is>
-          <t>S7020</t>
+          <t>S7018</t>
         </is>
       </c>
       <c r="B129" s="1" t="inlineStr">
         <is>
-          <t>VL352</t>
+          <t>TT206</t>
         </is>
       </c>
       <c r="C129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8131</t>
+          <t>VLINE-8129</t>
         </is>
       </c>
       <c r="D129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8338</t>
+          <t>VLINE-8337</t>
         </is>
       </c>
       <c r="E129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8469</t>
+          <t>VLINE-8468</t>
         </is>
       </c>
       <c r="F129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8769</t>
+          <t>VLINE-8768</t>
         </is>
       </c>
       <c r="G129" s="1" t="inlineStr">
         <is>
-          <t>WH003</t>
+          <t>WH001</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="1" t="inlineStr">
         <is>
-          <t>S7022</t>
+          <t>S7020</t>
         </is>
       </c>
       <c r="B130" s="1" t="inlineStr">
         <is>
-          <t>VL353</t>
+          <t>VL352</t>
         </is>
       </c>
       <c r="C130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8132</t>
+          <t>VLINE-8131</t>
         </is>
       </c>
       <c r="D130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8339</t>
+          <t>VLINE-8338</t>
         </is>
       </c>
       <c r="E130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8605</t>
+          <t>VLINE-8469</t>
         </is>
       </c>
       <c r="F130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8770</t>
+          <t>VLINE-8769</t>
         </is>
       </c>
       <c r="G130" s="1" t="inlineStr">
         <is>
-          <t>WL02</t>
+          <t>WH003</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="1" t="inlineStr">
         <is>
-          <t>SCT001</t>
+          <t>S7022</t>
         </is>
       </c>
       <c r="B131" s="1" t="inlineStr">
         <is>
-          <t>VL357</t>
+          <t>VL353</t>
         </is>
       </c>
       <c r="C131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8133</t>
+          <t>VLINE-8132</t>
         </is>
       </c>
       <c r="D131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8362</t>
+          <t>VLINE-8339</t>
         </is>
       </c>
       <c r="E131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8610</t>
+          <t>VLINE-8605</t>
         </is>
       </c>
       <c r="F131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8772</t>
+          <t>VLINE-8770</t>
         </is>
       </c>
       <c r="G131" s="1" t="inlineStr">
         <is>
-          <t>X12-X14</t>
+          <t>WL02</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="1" t="inlineStr">
         <is>
-          <t>SCT002</t>
+          <t>SCT001</t>
         </is>
       </c>
       <c r="B132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8004</t>
+          <t>VL357</t>
         </is>
       </c>
       <c r="C132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8134</t>
+          <t>VLINE-8133</t>
         </is>
       </c>
       <c r="D132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8363</t>
+          <t>VLINE-8362</t>
         </is>
       </c>
       <c r="E132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8612</t>
+          <t>VLINE-8610</t>
         </is>
       </c>
       <c r="F132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8773</t>
+          <t>VLINE-8772</t>
         </is>
       </c>
       <c r="G132" s="1" t="inlineStr">
         <is>
-          <t>X31</t>
+          <t>X12-X14</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="1" t="inlineStr">
         <is>
-          <t>SCT006</t>
+          <t>SCT002</t>
         </is>
       </c>
       <c r="B133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8007</t>
+          <t>VLINE-8004</t>
         </is>
       </c>
       <c r="C133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8136</t>
+          <t>VLINE-8134</t>
         </is>
       </c>
       <c r="D133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8365</t>
+          <t>VLINE-8363</t>
         </is>
       </c>
       <c r="E133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8615</t>
+          <t>VLINE-8612</t>
         </is>
       </c>
       <c r="F133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8774</t>
+          <t>VLINE-8773</t>
         </is>
       </c>
       <c r="G133" s="1" t="inlineStr">
         <is>
-          <t>XP2000</t>
+          <t>X31</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="1" t="inlineStr">
         <is>
-          <t>SCT007</t>
+          <t>SCT006</t>
         </is>
       </c>
       <c r="B134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8011</t>
+          <t>VLINE-8007</t>
         </is>
       </c>
       <c r="C134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8137</t>
+          <t>VLINE-8136</t>
         </is>
       </c>
       <c r="D134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8366</t>
+          <t>VLINE-8365</t>
         </is>
       </c>
       <c r="E134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8617</t>
+          <t>VLINE-8615</t>
         </is>
       </c>
       <c r="F134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8776</t>
+          <t>VLINE-8774</t>
         </is>
       </c>
       <c r="G134" s="1" t="inlineStr">
         <is>
-          <t>XP2003</t>
+          <t>XP2000</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="1" t="inlineStr">
         <is>
-          <t>SCT009</t>
+          <t>SCT007</t>
         </is>
       </c>
       <c r="B135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8013</t>
+          <t>VLINE-8011</t>
         </is>
       </c>
       <c r="C135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8140</t>
+          <t>VLINE-8137</t>
         </is>
       </c>
       <c r="D135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8368</t>
+          <t>VLINE-8366</t>
         </is>
       </c>
       <c r="E135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8620</t>
+          <t>VLINE-8617</t>
         </is>
       </c>
       <c r="F135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8778</t>
+          <t>VLINE-8776</t>
         </is>
       </c>
       <c r="G135" s="1" t="inlineStr">
         <is>
-          <t>XP2004</t>
+          <t>XP2003</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="1" t="inlineStr">
         <is>
-          <t>SCT011</t>
+          <t>SCT009</t>
         </is>
       </c>
       <c r="B136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8019</t>
+          <t>VLINE-8013</t>
         </is>
       </c>
       <c r="C136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8141</t>
+          <t>VLINE-8140</t>
         </is>
       </c>
       <c r="D136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8369</t>
+          <t>VLINE-8368</t>
         </is>
       </c>
       <c r="E136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8625</t>
+          <t>VLINE-8620</t>
         </is>
       </c>
       <c r="F136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8779</t>
+          <t>VLINE-8778</t>
         </is>
       </c>
       <c r="G136" s="1" t="inlineStr">
         <is>
-          <t>XP2005</t>
+          <t>XP2004</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="1" t="inlineStr">
         <is>
-          <t>SCT013</t>
+          <t>SCT011</t>
         </is>
       </c>
       <c r="B137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8020</t>
+          <t>VLINE-8019</t>
         </is>
       </c>
       <c r="C137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8142</t>
+          <t>VLINE-8141</t>
         </is>
       </c>
       <c r="D137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8403</t>
+          <t>VLINE-8369</t>
         </is>
       </c>
       <c r="E137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8630</t>
+          <t>VLINE-8625</t>
         </is>
       </c>
       <c r="F137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8780</t>
+          <t>VLINE-8779</t>
         </is>
       </c>
       <c r="G137" s="1" t="inlineStr">
         <is>
-          <t>XP2007</t>
+          <t>XP2005</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="1" t="inlineStr">
         <is>
-          <t>SCT014</t>
+          <t>SCT013</t>
         </is>
       </c>
       <c r="B138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8023</t>
+          <t>VLINE-8020</t>
         </is>
       </c>
       <c r="C138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8144</t>
+          <t>VLINE-8142</t>
         </is>
       </c>
       <c r="D138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8404</t>
+          <t>VLINE-8403</t>
         </is>
       </c>
       <c r="E138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8671</t>
+          <t>VLINE-8630</t>
         </is>
       </c>
       <c r="F138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8781</t>
+          <t>VLINE-8780</t>
         </is>
       </c>
       <c r="G138" s="1" t="inlineStr">
         <is>
-          <t>XP2008</t>
+          <t>XP2007</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="1" t="inlineStr">
         <is>
-          <t>SCT015</t>
+          <t>SCT014</t>
         </is>
       </c>
       <c r="B139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8025</t>
+          <t>VLINE-8023</t>
         </is>
       </c>
       <c r="C139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8145</t>
+          <t>VLINE-8144</t>
         </is>
       </c>
       <c r="D139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8406</t>
+          <t>VLINE-8404</t>
         </is>
       </c>
       <c r="E139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8706</t>
+          <t>VLINE-8671</t>
         </is>
       </c>
       <c r="F139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8782</t>
+          <t>VLINE-8781</t>
         </is>
       </c>
       <c r="G139" s="1" t="inlineStr">
         <is>
-          <t>XP2010</t>
+          <t>XP2008</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="1" t="inlineStr">
         <is>
-          <t>SO2</t>
+          <t>SCT015</t>
         </is>
       </c>
       <c r="B140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8026</t>
+          <t>VLINE-8025</t>
         </is>
       </c>
       <c r="C140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8148</t>
+          <t>VLINE-8145</t>
         </is>
       </c>
       <c r="D140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8408</t>
+          <t>VLINE-8406</t>
         </is>
       </c>
       <c r="E140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8711</t>
+          <t>VLINE-8706</t>
         </is>
       </c>
       <c r="F140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8783</t>
+          <t>VLINE-8782</t>
         </is>
       </c>
       <c r="G140" s="1" t="inlineStr">
         <is>
-          <t>XP2011</t>
+          <t>XP2010</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="1" t="inlineStr">
         <is>
-          <t>SSR101</t>
+          <t>SO2</t>
         </is>
       </c>
       <c r="B141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8027</t>
+          <t>VLINE-8026</t>
         </is>
       </c>
       <c r="C141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8150</t>
+          <t>VLINE-8148</t>
         </is>
       </c>
       <c r="D141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8410</t>
+          <t>VLINE-8408</t>
         </is>
       </c>
       <c r="E141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8714</t>
+          <t>VLINE-8711</t>
         </is>
       </c>
       <c r="F141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8784</t>
+          <t>VLINE-8783</t>
         </is>
       </c>
       <c r="G141" s="1" t="inlineStr">
         <is>
-          <t>XP2012</t>
+          <t>XP2011</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="1" t="inlineStr">
         <is>
-          <t>SSR102</t>
+          <t>SSR101</t>
         </is>
       </c>
       <c r="B142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8028</t>
+          <t>VLINE-8027</t>
         </is>
       </c>
       <c r="C142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8151</t>
+          <t>VLINE-8150</t>
         </is>
       </c>
       <c r="D142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8411</t>
+          <t>VLINE-8410</t>
         </is>
       </c>
       <c r="E142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8717</t>
+          <t>VLINE-8714</t>
         </is>
       </c>
       <c r="F142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8786</t>
+          <t>VLINE-8784</t>
         </is>
       </c>
       <c r="G142" s="1" t="inlineStr">
         <is>
-          <t>XP2013</t>
+          <t>XP2012</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="1" t="inlineStr">
         <is>
-          <t>SSR103</t>
+          <t>SSR102</t>
         </is>
       </c>
       <c r="B143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8029</t>
+          <t>VLINE-8028</t>
         </is>
       </c>
       <c r="C143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8152</t>
+          <t>VLINE-8151</t>
         </is>
       </c>
       <c r="D143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8413</t>
+          <t>VLINE-8411</t>
         </is>
       </c>
       <c r="E143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8720</t>
+          <t>VLINE-8717</t>
         </is>
       </c>
       <c r="F143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8787</t>
+          <t>VLINE-8786</t>
         </is>
       </c>
       <c r="G143" s="1" t="inlineStr">
         <is>
-          <t>XP2014</t>
+          <t>XP2013</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="1" t="inlineStr">
         <is>
-          <t>SSR104</t>
+          <t>SSR103</t>
         </is>
       </c>
       <c r="B144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8030</t>
+          <t>VLINE-8029</t>
         </is>
       </c>
       <c r="C144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8153</t>
+          <t>VLINE-8152</t>
         </is>
       </c>
       <c r="D144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8415</t>
+          <t>VLINE-8413</t>
         </is>
       </c>
       <c r="E144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8721</t>
+          <t>VLINE-8720</t>
         </is>
       </c>
       <c r="F144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8788</t>
+          <t>VLINE-8787</t>
         </is>
       </c>
       <c r="G144" s="1" t="inlineStr">
         <is>
-          <t>XP2015</t>
+          <t>XP2014</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="1" t="inlineStr">
         <is>
-          <t>T363</t>
+          <t>SSR104</t>
         </is>
       </c>
       <c r="B145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8031</t>
+          <t>VLINE-8030</t>
         </is>
       </c>
       <c r="C145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8154</t>
+          <t>VLINE-8153</t>
         </is>
       </c>
       <c r="D145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8417</t>
+          <t>VLINE-8415</t>
         </is>
       </c>
       <c r="E145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8723</t>
+          <t>VLINE-8721</t>
         </is>
       </c>
       <c r="F145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8790</t>
+          <t>VLINE-8788</t>
         </is>
       </c>
       <c r="G145" s="1" t="inlineStr">
         <is>
-          <t>XP2016</t>
+          <t>XP2015</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="1" t="inlineStr">
         <is>
-          <t>T386</t>
+          <t>T363</t>
         </is>
       </c>
       <c r="B146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8032</t>
+          <t>VLINE-8031</t>
         </is>
       </c>
       <c r="C146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8155</t>
+          <t>VLINE-8154</t>
         </is>
       </c>
       <c r="D146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8418</t>
+          <t>VLINE-8417</t>
         </is>
       </c>
       <c r="E146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8725</t>
+          <t>VLINE-8723</t>
         </is>
       </c>
       <c r="F146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8792</t>
+          <t>VLINE-8790</t>
         </is>
       </c>
       <c r="G146" s="1" t="inlineStr">
         <is>
-          <t>XP2017</t>
+          <t>XP2016</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="1" t="inlineStr">
         <is>
-          <t>TDX101</t>
+          <t>T386</t>
         </is>
       </c>
       <c r="B147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8036</t>
+          <t>VLINE-8032</t>
         </is>
       </c>
       <c r="C147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8157</t>
+          <t>VLINE-8155</t>
         </is>
       </c>
       <c r="D147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8419</t>
+          <t>VLINE-8418</t>
         </is>
       </c>
       <c r="E147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8726</t>
+          <t>VLINE-8725</t>
         </is>
       </c>
       <c r="F147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8793</t>
+          <t>VLINE-8792</t>
         </is>
       </c>
       <c r="G147" s="1" t="inlineStr">
         <is>
-          <t>XP2019</t>
+          <t>XP2017</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="1" t="inlineStr">
         <is>
-          <t>TE2801</t>
+          <t>TDX101</t>
         </is>
       </c>
       <c r="B148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8038</t>
+          <t>VLINE-8036</t>
         </is>
       </c>
       <c r="C148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8158</t>
+          <t>VLINE-8157</t>
         </is>
       </c>
       <c r="D148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8420</t>
+          <t>VLINE-8419</t>
         </is>
       </c>
       <c r="E148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8727</t>
+          <t>VLINE-8726</t>
         </is>
       </c>
       <c r="F148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8794</t>
+          <t>VLINE-8793</t>
         </is>
       </c>
       <c r="G148" s="1" t="inlineStr">
         <is>
-          <t>XR552</t>
+          <t>XP2019</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="1" t="inlineStr">
         <is>
-          <t>TE2802</t>
+          <t>TE2801</t>
         </is>
       </c>
       <c r="B149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8042</t>
+          <t>VLINE-8038</t>
         </is>
       </c>
       <c r="C149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8159</t>
+          <t>VLINE-8158</t>
         </is>
       </c>
       <c r="D149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8421</t>
+          <t>VLINE-8420</t>
         </is>
       </c>
       <c r="E149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8729</t>
+          <t>VLINE-8727</t>
         </is>
       </c>
       <c r="F149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8795</t>
+          <t>VLINE-8794</t>
         </is>
       </c>
       <c r="G149" s="1" t="inlineStr">
         <is>
-          <t>XRN001</t>
+          <t>XR552</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="1" t="inlineStr">
         <is>
-          <t>TE2803</t>
+          <t>TE2802</t>
         </is>
       </c>
       <c r="B150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8051</t>
+          <t>VLINE-8042</t>
         </is>
       </c>
       <c r="C150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8160</t>
+          <t>VLINE-8159</t>
         </is>
       </c>
       <c r="D150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8422</t>
+          <t>VLINE-8421</t>
         </is>
       </c>
       <c r="E150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8730</t>
+          <t>VLINE-8729</t>
         </is>
       </c>
       <c r="F150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8796</t>
+          <t>VLINE-8795</t>
         </is>
       </c>
       <c r="G150" s="1" t="inlineStr">
         <is>
-          <t>XRN004</t>
+          <t>XRN001</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="1" t="inlineStr">
         <is>
-          <t>TE2804</t>
+          <t>TE2803</t>
         </is>
       </c>
       <c r="B151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8052</t>
+          <t>VLINE-8051</t>
         </is>
       </c>
       <c r="C151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8161</t>
+          <t>VLINE-8160</t>
         </is>
       </c>
       <c r="D151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8424</t>
+          <t>VLINE-8422</t>
         </is>
       </c>
       <c r="E151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8731</t>
+          <t>VLINE-8730</t>
         </is>
       </c>
       <c r="F151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8797</t>
+          <t>VLINE-8796</t>
         </is>
       </c>
       <c r="G151" s="1" t="inlineStr">
         <is>
-          <t>XRN005</t>
+          <t>XRN004</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="1" t="inlineStr">
         <is>
-          <t>TE2805</t>
+          <t>TE2804</t>
         </is>
       </c>
       <c r="B152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8053</t>
+          <t>VLINE-8052</t>
         </is>
       </c>
       <c r="C152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8162</t>
+          <t>VLINE-8161</t>
         </is>
       </c>
       <c r="D152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8425</t>
+          <t>VLINE-8424</t>
         </is>
       </c>
       <c r="E152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8733</t>
+          <t>VLINE-8731</t>
         </is>
       </c>
       <c r="F152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8799</t>
+          <t>VLINE-8797</t>
         </is>
       </c>
       <c r="G152" s="1" t="inlineStr">
         <is>
-          <t>XRN006</t>
+          <t>XRN005</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="1" t="inlineStr">
         <is>
-          <t>TE2806</t>
+          <t>TE2805</t>
         </is>
       </c>
       <c r="B153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8055</t>
+          <t>VLINE-8053</t>
         </is>
       </c>
       <c r="C153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8171</t>
+          <t>VLINE-8162</t>
         </is>
       </c>
       <c r="D153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8426</t>
+          <t>VLINE-8425</t>
         </is>
       </c>
       <c r="E153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8735</t>
+          <t>VLINE-8733</t>
         </is>
       </c>
       <c r="F153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8800</t>
+          <t>VLINE-8799</t>
         </is>
       </c>
       <c r="G153" s="1" t="inlineStr">
         <is>
-          <t>XRN007</t>
+          <t>XRN006</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="1" t="inlineStr">
         <is>
-          <t>TE2807</t>
+          <t>TE2806</t>
         </is>
       </c>
       <c r="B154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8056</t>
+          <t>VLINE-8055</t>
         </is>
       </c>
       <c r="C154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8172</t>
+          <t>VLINE-8171</t>
         </is>
       </c>
       <c r="D154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8427</t>
+          <t>VLINE-8426</t>
         </is>
       </c>
       <c r="E154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8736</t>
+          <t>VLINE-8735</t>
         </is>
       </c>
       <c r="F154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8801</t>
+          <t>VLINE-8800</t>
         </is>
       </c>
       <c r="G154" s="1" t="inlineStr">
         <is>
-          <t>XRN009</t>
+          <t>XRN007</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="1" t="inlineStr">
         <is>
-          <t>TE2808</t>
+          <t>TE2807</t>
         </is>
       </c>
       <c r="B155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8057</t>
+          <t>VLINE-8056</t>
         </is>
       </c>
       <c r="C155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8176</t>
+          <t>VLINE-8172</t>
         </is>
       </c>
       <c r="D155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8428</t>
+          <t>VLINE-8427</t>
         </is>
       </c>
       <c r="E155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8737</t>
+          <t>VLINE-8736</t>
         </is>
       </c>
       <c r="F155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8802</t>
+          <t>VLINE-8801</t>
         </is>
       </c>
       <c r="G155" s="1" t="inlineStr">
         <is>
-          <t>XRN011</t>
+          <t>XRN009</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="1" t="inlineStr">
         <is>
-          <t>TE2809</t>
+          <t>TE2808</t>
         </is>
       </c>
       <c r="B156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8058</t>
+          <t>VLINE-8057</t>
         </is>
       </c>
       <c r="C156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8179</t>
+          <t>VLINE-8176</t>
         </is>
       </c>
       <c r="D156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8429</t>
+          <t>VLINE-8428</t>
         </is>
       </c>
       <c r="E156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8739</t>
+          <t>VLINE-8737</t>
         </is>
       </c>
       <c r="F156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8803</t>
+          <t>VLINE-8802</t>
         </is>
       </c>
       <c r="G156" s="1" t="inlineStr">
         <is>
-          <t>XRN014</t>
+          <t>XRN011</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="1" t="inlineStr">
         <is>
-          <t>TE2810</t>
+          <t>TE2809</t>
         </is>
       </c>
       <c r="B157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8059</t>
+          <t>VLINE-8058</t>
         </is>
       </c>
       <c r="C157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8180</t>
+          <t>VLINE-8179</t>
         </is>
       </c>
       <c r="D157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8430</t>
+          <t>VLINE-8429</t>
         </is>
       </c>
       <c r="E157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8740</t>
+          <t>VLINE-8739</t>
         </is>
       </c>
       <c r="F157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8804</t>
+          <t>VLINE-8803</t>
         </is>
       </c>
       <c r="G157" s="1" t="inlineStr">
         <is>
-          <t>XRN017</t>
+          <t>XRN014</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="1" t="inlineStr">
         <is>
-          <t>TE2812</t>
+          <t>TE2810</t>
         </is>
       </c>
       <c r="B158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8061</t>
+          <t>VLINE-8059</t>
         </is>
       </c>
       <c r="C158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8181</t>
+          <t>VLINE-8180</t>
         </is>
       </c>
       <c r="D158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8431</t>
+          <t>VLINE-8430</t>
         </is>
       </c>
       <c r="E158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8741</t>
+          <t>VLINE-8740</t>
         </is>
       </c>
       <c r="F158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8805</t>
+          <t>VLINE-8804</t>
         </is>
       </c>
       <c r="G158" s="1" t="inlineStr">
         <is>
-          <t>XRN018</t>
+          <t>XRN017</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="1" t="inlineStr">
         <is>
-          <t>TE2813</t>
+          <t>TE2812</t>
         </is>
       </c>
       <c r="B159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8072</t>
+          <t>VLINE-8061</t>
         </is>
       </c>
       <c r="C159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8182</t>
+          <t>VLINE-8181</t>
         </is>
       </c>
       <c r="D159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8432</t>
+          <t>VLINE-8431</t>
         </is>
       </c>
       <c r="E159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8742</t>
+          <t>VLINE-8741</t>
         </is>
       </c>
       <c r="F159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8806</t>
+          <t>VLINE-8805</t>
         </is>
       </c>
       <c r="G159" s="1" t="inlineStr">
         <is>
-          <t>XRN020</t>
+          <t>XRN018</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="1" t="inlineStr">
         <is>
-          <t>TE2814</t>
+          <t>TE2813</t>
         </is>
       </c>
       <c r="B160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8074</t>
+          <t>VLINE-8072</t>
         </is>
       </c>
       <c r="C160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8183</t>
+          <t>VLINE-8182</t>
         </is>
       </c>
       <c r="D160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8433</t>
+          <t>VLINE-8432</t>
         </is>
       </c>
       <c r="E160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8743</t>
+          <t>VLINE-8742</t>
         </is>
       </c>
       <c r="F160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8807</t>
+          <t>VLINE-8806</t>
         </is>
       </c>
       <c r="G160" s="1" t="inlineStr">
         <is>
-          <t>XRN021</t>
+          <t>XRN020</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="1" t="inlineStr">
         <is>
-          <t>TJ096</t>
+          <t>TE2814</t>
         </is>
       </c>
       <c r="B161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8075</t>
+          <t>VLINE-8074</t>
         </is>
       </c>
       <c r="C161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8184</t>
+          <t>VLINE-8183</t>
         </is>
       </c>
       <c r="D161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8434</t>
+          <t>VLINE-8433</t>
         </is>
       </c>
       <c r="E161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8744</t>
+          <t>VLINE-8743</t>
         </is>
       </c>
       <c r="F161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8808</t>
+          <t>VLINE-8807</t>
         </is>
       </c>
       <c r="G161" s="1" t="inlineStr">
         <is>
-          <t>XRN023</t>
+          <t>XRN021</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="1" t="inlineStr">
         <is>
-          <t>TJ107</t>
+          <t>TJ096</t>
         </is>
       </c>
       <c r="B162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8076</t>
+          <t>VLINE-8075</t>
         </is>
       </c>
       <c r="C162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8185</t>
+          <t>VLINE-8184</t>
         </is>
       </c>
       <c r="D162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8435</t>
+          <t>VLINE-8434</t>
         </is>
       </c>
       <c r="E162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8745</t>
+          <t>VLINE-8744</t>
         </is>
       </c>
       <c r="F162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8809</t>
+          <t>VLINE-8808</t>
         </is>
       </c>
       <c r="G162" s="1" t="inlineStr">
         <is>
-          <t>XRN025</t>
+          <t>XRN023</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="1" t="inlineStr">
         <is>
-          <t>TT03</t>
+          <t>TJ107</t>
         </is>
       </c>
       <c r="B163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8077</t>
+          <t>VLINE-8076</t>
         </is>
       </c>
       <c r="C163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8186</t>
+          <t>VLINE-8185</t>
         </is>
       </c>
       <c r="D163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8438</t>
+          <t>VLINE-8435</t>
         </is>
       </c>
       <c r="E163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8746</t>
+          <t>VLINE-8745</t>
         </is>
       </c>
       <c r="F163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8810</t>
+          <t>VLINE-8809</t>
         </is>
       </c>
       <c r="G163" s="1" t="inlineStr">
         <is>
-          <t>XRN026</t>
+          <t>XRN025</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="1" t="inlineStr">
         <is>
-          <t>TT04</t>
+          <t>TT03</t>
         </is>
       </c>
       <c r="B164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8080</t>
+          <t>VLINE-8077</t>
         </is>
       </c>
       <c r="C164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8187</t>
+          <t>VLINE-8186</t>
         </is>
       </c>
       <c r="D164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8440</t>
+          <t>VLINE-8438</t>
         </is>
       </c>
       <c r="E164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8747</t>
+          <t>VLINE-8746</t>
         </is>
       </c>
       <c r="F164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8811</t>
+          <t>VLINE-8810</t>
         </is>
       </c>
       <c r="G164" s="1" t="inlineStr">
         <is>
-          <t>XRN027</t>
+          <t>XRN026</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="1" t="inlineStr">
         <is>
-          <t>TT05</t>
+          <t>TT04</t>
         </is>
       </c>
       <c r="B165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8081</t>
+          <t>VLINE-8080</t>
         </is>
       </c>
       <c r="C165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8188</t>
+          <t>VLINE-8187</t>
         </is>
       </c>
       <c r="D165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8441</t>
+          <t>VLINE-8440</t>
         </is>
       </c>
       <c r="E165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8748</t>
+          <t>VLINE-8747</t>
         </is>
       </c>
       <c r="F165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8812</t>
+          <t>VLINE-8811</t>
         </is>
       </c>
       <c r="G165" s="1" t="inlineStr">
         <is>
-          <t>Y163</t>
+          <t>XRN027</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="1" t="inlineStr">
         <is>
-          <t>TT07</t>
+          <t>TT05</t>
         </is>
       </c>
       <c r="B166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8084</t>
+          <t>VLINE-8081</t>
         </is>
       </c>
       <c r="C166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8189</t>
+          <t>VLINE-8188</t>
         </is>
       </c>
       <c r="D166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8442</t>
+          <t>VLINE-8441</t>
         </is>
       </c>
       <c r="E166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8749</t>
+          <t>VLINE-8748</t>
         </is>
       </c>
       <c r="F166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8813</t>
+          <t>VLINE-8812</t>
+        </is>
+      </c>
+      <c r="G166" s="1" t="inlineStr">
+        <is>
+          <t>Y163</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="1" t="inlineStr">
         <is>
-          <t>TT08</t>
+          <t>TT07</t>
         </is>
       </c>
       <c r="B167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8088</t>
+          <t>VLINE-8084</t>
         </is>
       </c>
       <c r="C167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8293</t>
+          <t>VLINE-8189</t>
         </is>
       </c>
       <c r="D167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8443</t>
+          <t>VLINE-8442</t>
         </is>
       </c>
       <c r="E167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8750</t>
+          <t>VLINE-8749</t>
         </is>
       </c>
       <c r="F167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8814</t>
+          <t>VLINE-8813</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="1" t="inlineStr">
         <is>
-          <t>TT103</t>
+          <t>TT08</t>
         </is>
       </c>
       <c r="B168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8089</t>
+          <t>VLINE-8088</t>
         </is>
       </c>
       <c r="C168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8303</t>
+          <t>VLINE-8293</t>
         </is>
       </c>
       <c r="D168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8444</t>
+          <t>VLINE-8443</t>
         </is>
       </c>
       <c r="E168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8751</t>
+          <t>VLINE-8750</t>
         </is>
       </c>
       <c r="F168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8816</t>
+          <t>VLINE-8814</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="1" t="inlineStr">
         <is>
-          <t>TT106</t>
+          <t>TT103</t>
         </is>
       </c>
       <c r="B169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8104</t>
+          <t>VLINE-8089</t>
         </is>
       </c>
       <c r="C169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8304</t>
+          <t>VLINE-8303</t>
         </is>
       </c>
       <c r="D169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8446</t>
+          <t>VLINE-8444</t>
         </is>
       </c>
       <c r="E169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8752</t>
+          <t>VLINE-8751</t>
         </is>
       </c>
       <c r="F169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8817</t>
+          <t>VLINE-8816</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="1" t="inlineStr">
         <is>
-          <t>TT107</t>
+          <t>TT106</t>
         </is>
       </c>
       <c r="B170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8107</t>
+          <t>VLINE-8104</t>
         </is>
       </c>
       <c r="C170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8306</t>
+          <t>VLINE-8304</t>
         </is>
       </c>
       <c r="D170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8447</t>
+          <t>VLINE-8446</t>
         </is>
       </c>
       <c r="E170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8753</t>
+          <t>VLINE-8752</t>
         </is>
       </c>
       <c r="F170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8818</t>
+          <t>VLINE-8817</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update loco downloads 2026-04-05 11:50:37
</commit_message>
<xml_diff>
--- a/downloads/loco_numbers_only.xlsx
+++ b/downloads/loco_numbers_only.xlsx
@@ -2799,27 +2799,27 @@
       </c>
       <c r="D58" s="1" t="inlineStr">
         <is>
-          <t>MM-792M</t>
+          <t>MM-790M</t>
         </is>
       </c>
       <c r="E58" s="1" t="inlineStr">
         <is>
-          <t>MM-970M</t>
+          <t>MM-968M</t>
         </is>
       </c>
       <c r="F58" s="1" t="inlineStr">
         <is>
-          <t>MMY032</t>
+          <t>MM-9970M</t>
         </is>
       </c>
       <c r="G58" s="1" t="inlineStr">
         <is>
-          <t>NR72</t>
+          <t>NR71</t>
         </is>
       </c>
       <c r="H58" s="1" t="inlineStr">
         <is>
-          <t>PHC001</t>
+          <t>PB4</t>
         </is>
       </c>
     </row>
@@ -2841,27 +2841,27 @@
       </c>
       <c r="D59" s="1" t="inlineStr">
         <is>
-          <t>MM-796M</t>
+          <t>MM-792M</t>
         </is>
       </c>
       <c r="E59" s="1" t="inlineStr">
         <is>
-          <t>MM-972M</t>
+          <t>MM-970M</t>
         </is>
       </c>
       <c r="F59" s="1" t="inlineStr">
         <is>
-          <t>MRL001</t>
+          <t>MMY032</t>
         </is>
       </c>
       <c r="G59" s="1" t="inlineStr">
         <is>
-          <t>NR75</t>
+          <t>NR72</t>
         </is>
       </c>
       <c r="H59" s="1" t="inlineStr">
         <is>
-          <t>PHC002</t>
+          <t>PHC001</t>
         </is>
       </c>
     </row>
@@ -2883,27 +2883,27 @@
       </c>
       <c r="D60" s="1" t="inlineStr">
         <is>
-          <t>MM-798M</t>
+          <t>MM-796M</t>
         </is>
       </c>
       <c r="E60" s="1" t="inlineStr">
         <is>
-          <t>MM-974M</t>
+          <t>MM-972M</t>
         </is>
       </c>
       <c r="F60" s="1" t="inlineStr">
         <is>
-          <t>MRL004</t>
+          <t>MRL001</t>
         </is>
       </c>
       <c r="G60" s="1" t="inlineStr">
         <is>
-          <t>NR77</t>
+          <t>NR75</t>
         </is>
       </c>
       <c r="H60" s="1" t="inlineStr">
         <is>
-          <t>Q4001</t>
+          <t>PHC002</t>
         </is>
       </c>
     </row>
@@ -2925,27 +2925,27 @@
       </c>
       <c r="D61" s="1" t="inlineStr">
         <is>
-          <t>MM-800M</t>
+          <t>MM-798M</t>
         </is>
       </c>
       <c r="E61" s="1" t="inlineStr">
         <is>
-          <t>MM-976M</t>
+          <t>MM-974M</t>
         </is>
       </c>
       <c r="F61" s="1" t="inlineStr">
         <is>
-          <t>MRL006</t>
+          <t>MRL004</t>
         </is>
       </c>
       <c r="G61" s="1" t="inlineStr">
         <is>
-          <t>NR78</t>
+          <t>NR77</t>
         </is>
       </c>
       <c r="H61" s="1" t="inlineStr">
         <is>
-          <t>Q4003</t>
+          <t>Q4001</t>
         </is>
       </c>
     </row>
@@ -2967,27 +2967,27 @@
       </c>
       <c r="D62" s="1" t="inlineStr">
         <is>
-          <t>MM-802M</t>
+          <t>MM-800M</t>
         </is>
       </c>
       <c r="E62" s="1" t="inlineStr">
         <is>
-          <t>MM-980M</t>
+          <t>MM-976M</t>
         </is>
       </c>
       <c r="F62" s="1" t="inlineStr">
         <is>
-          <t>N452</t>
+          <t>MRL006</t>
         </is>
       </c>
       <c r="G62" s="1" t="inlineStr">
         <is>
-          <t>NR81</t>
+          <t>NR78</t>
         </is>
       </c>
       <c r="H62" s="1" t="inlineStr">
         <is>
-          <t>Q4004</t>
+          <t>Q4003</t>
         </is>
       </c>
     </row>
@@ -3009,27 +3009,27 @@
       </c>
       <c r="D63" s="1" t="inlineStr">
         <is>
-          <t>MM-804M</t>
+          <t>MM-802M</t>
         </is>
       </c>
       <c r="E63" s="1" t="inlineStr">
         <is>
-          <t>MM-982M</t>
+          <t>MM-980M</t>
         </is>
       </c>
       <c r="F63" s="1" t="inlineStr">
         <is>
-          <t>N453</t>
+          <t>N452</t>
         </is>
       </c>
       <c r="G63" s="1" t="inlineStr">
         <is>
-          <t>NR82</t>
+          <t>NR81</t>
         </is>
       </c>
       <c r="H63" s="1" t="inlineStr">
         <is>
-          <t>Q4005</t>
+          <t>Q4004</t>
         </is>
       </c>
     </row>
@@ -3051,27 +3051,27 @@
       </c>
       <c r="D64" s="1" t="inlineStr">
         <is>
-          <t>MM-808M</t>
+          <t>MM-804M</t>
         </is>
       </c>
       <c r="E64" s="1" t="inlineStr">
         <is>
-          <t>MM-984M</t>
+          <t>MM-982M</t>
         </is>
       </c>
       <c r="F64" s="1" t="inlineStr">
         <is>
-          <t>N457</t>
+          <t>N453</t>
         </is>
       </c>
       <c r="G64" s="1" t="inlineStr">
         <is>
-          <t>NR83</t>
+          <t>NR82</t>
         </is>
       </c>
       <c r="H64" s="1" t="inlineStr">
         <is>
-          <t>Q4006</t>
+          <t>Q4005</t>
         </is>
       </c>
     </row>
@@ -3093,27 +3093,27 @@
       </c>
       <c r="D65" s="1" t="inlineStr">
         <is>
-          <t>MM-810M</t>
+          <t>MM-808M</t>
         </is>
       </c>
       <c r="E65" s="1" t="inlineStr">
         <is>
-          <t>MM-986M</t>
+          <t>MM-984M</t>
         </is>
       </c>
       <c r="F65" s="1" t="inlineStr">
         <is>
-          <t>N458</t>
+          <t>N457</t>
         </is>
       </c>
       <c r="G65" s="1" t="inlineStr">
         <is>
-          <t>NR84</t>
+          <t>NR83</t>
         </is>
       </c>
       <c r="H65" s="1" t="inlineStr">
         <is>
-          <t>Q4007</t>
+          <t>Q4006</t>
         </is>
       </c>
     </row>
@@ -3135,27 +3135,27 @@
       </c>
       <c r="D66" s="1" t="inlineStr">
         <is>
-          <t>MM-814M</t>
+          <t>MM-810M</t>
         </is>
       </c>
       <c r="E66" s="1" t="inlineStr">
         <is>
-          <t>MM-9902M</t>
+          <t>MM-986M</t>
         </is>
       </c>
       <c r="F66" s="1" t="inlineStr">
         <is>
-          <t>N465</t>
+          <t>N458</t>
         </is>
       </c>
       <c r="G66" s="1" t="inlineStr">
         <is>
-          <t>NR85</t>
+          <t>NR84</t>
         </is>
       </c>
       <c r="H66" s="1" t="inlineStr">
         <is>
-          <t>Q4009</t>
+          <t>Q4007</t>
         </is>
       </c>
     </row>
@@ -3177,27 +3177,27 @@
       </c>
       <c r="D67" s="1" t="inlineStr">
         <is>
-          <t>MM-816M</t>
+          <t>MM-814M</t>
         </is>
       </c>
       <c r="E67" s="1" t="inlineStr">
         <is>
-          <t>MM-9903M</t>
+          <t>MM-9902M</t>
         </is>
       </c>
       <c r="F67" s="1" t="inlineStr">
         <is>
-          <t>N466</t>
+          <t>N465</t>
         </is>
       </c>
       <c r="G67" s="1" t="inlineStr">
         <is>
-          <t>NR86</t>
+          <t>NR85</t>
         </is>
       </c>
       <c r="H67" s="1" t="inlineStr">
         <is>
-          <t>Q4011</t>
+          <t>Q4009</t>
         </is>
       </c>
     </row>
@@ -3219,27 +3219,27 @@
       </c>
       <c r="D68" s="1" t="inlineStr">
         <is>
-          <t>MM-818M</t>
+          <t>MM-816M</t>
         </is>
       </c>
       <c r="E68" s="1" t="inlineStr">
         <is>
-          <t>MM-9904M</t>
+          <t>MM-9903M</t>
         </is>
       </c>
       <c r="F68" s="1" t="inlineStr">
         <is>
-          <t>N467</t>
+          <t>N466</t>
         </is>
       </c>
       <c r="G68" s="1" t="inlineStr">
         <is>
-          <t>NR87</t>
+          <t>NR86</t>
         </is>
       </c>
       <c r="H68" s="1" t="inlineStr">
         <is>
-          <t>Q4012</t>
+          <t>Q4011</t>
         </is>
       </c>
     </row>
@@ -3261,27 +3261,27 @@
       </c>
       <c r="D69" s="1" t="inlineStr">
         <is>
-          <t>MM-820M</t>
+          <t>MM-818M</t>
         </is>
       </c>
       <c r="E69" s="1" t="inlineStr">
         <is>
-          <t>MM-9906M</t>
+          <t>MM-9904M</t>
         </is>
       </c>
       <c r="F69" s="1" t="inlineStr">
         <is>
-          <t>N469</t>
+          <t>N467</t>
         </is>
       </c>
       <c r="G69" s="1" t="inlineStr">
         <is>
-          <t>NR88</t>
+          <t>NR87</t>
         </is>
       </c>
       <c r="H69" s="1" t="inlineStr">
         <is>
-          <t>Q4013</t>
+          <t>Q4012</t>
         </is>
       </c>
     </row>
@@ -3303,27 +3303,27 @@
       </c>
       <c r="D70" s="1" t="inlineStr">
         <is>
-          <t>MM-824M</t>
+          <t>MM-820M</t>
         </is>
       </c>
       <c r="E70" s="1" t="inlineStr">
         <is>
-          <t>MM-9907M</t>
+          <t>MM-9906M</t>
         </is>
       </c>
       <c r="F70" s="1" t="inlineStr">
         <is>
-          <t>N473</t>
+          <t>N469</t>
         </is>
       </c>
       <c r="G70" s="1" t="inlineStr">
         <is>
-          <t>NR89</t>
+          <t>NR88</t>
         </is>
       </c>
       <c r="H70" s="1" t="inlineStr">
         <is>
-          <t>Q4014</t>
+          <t>Q4013</t>
         </is>
       </c>
     </row>
@@ -3345,27 +3345,27 @@
       </c>
       <c r="D71" s="1" t="inlineStr">
         <is>
-          <t>MM-826M</t>
+          <t>MM-824M</t>
         </is>
       </c>
       <c r="E71" s="1" t="inlineStr">
         <is>
-          <t>MM-9908M</t>
+          <t>MM-9907M</t>
         </is>
       </c>
       <c r="F71" s="1" t="inlineStr">
         <is>
-          <t>NR1</t>
+          <t>N473</t>
         </is>
       </c>
       <c r="G71" s="1" t="inlineStr">
         <is>
-          <t>NR90</t>
+          <t>NR89</t>
         </is>
       </c>
       <c r="H71" s="1" t="inlineStr">
         <is>
-          <t>Q4015</t>
+          <t>Q4014</t>
         </is>
       </c>
     </row>
@@ -3387,27 +3387,27 @@
       </c>
       <c r="D72" s="1" t="inlineStr">
         <is>
-          <t>MM-828M</t>
+          <t>MM-826M</t>
         </is>
       </c>
       <c r="E72" s="1" t="inlineStr">
         <is>
-          <t>MM-9909M</t>
+          <t>MM-9908M</t>
         </is>
       </c>
       <c r="F72" s="1" t="inlineStr">
         <is>
-          <t>NR2</t>
+          <t>NR1</t>
         </is>
       </c>
       <c r="G72" s="1" t="inlineStr">
         <is>
-          <t>NR91</t>
+          <t>NR90</t>
         </is>
       </c>
       <c r="H72" s="1" t="inlineStr">
         <is>
-          <t>Q4016</t>
+          <t>Q4015</t>
         </is>
       </c>
     </row>
@@ -3429,27 +3429,27 @@
       </c>
       <c r="D73" s="1" t="inlineStr">
         <is>
-          <t>MM-830M</t>
+          <t>MM-828M</t>
         </is>
       </c>
       <c r="E73" s="1" t="inlineStr">
         <is>
-          <t>MM-9912M</t>
+          <t>MM-9909M</t>
         </is>
       </c>
       <c r="F73" s="1" t="inlineStr">
         <is>
-          <t>NR4</t>
+          <t>NR2</t>
         </is>
       </c>
       <c r="G73" s="1" t="inlineStr">
         <is>
-          <t>NR92</t>
+          <t>NR91</t>
         </is>
       </c>
       <c r="H73" s="1" t="inlineStr">
         <is>
-          <t>Q4017</t>
+          <t>Q4016</t>
         </is>
       </c>
     </row>
@@ -3471,27 +3471,27 @@
       </c>
       <c r="D74" s="1" t="inlineStr">
         <is>
-          <t>MM-832M</t>
+          <t>MM-830M</t>
         </is>
       </c>
       <c r="E74" s="1" t="inlineStr">
         <is>
-          <t>MM-9913M</t>
+          <t>MM-9912M</t>
         </is>
       </c>
       <c r="F74" s="1" t="inlineStr">
         <is>
-          <t>NR5</t>
+          <t>NR4</t>
         </is>
       </c>
       <c r="G74" s="1" t="inlineStr">
         <is>
-          <t>NR93</t>
+          <t>NR92</t>
         </is>
       </c>
       <c r="H74" s="1" t="inlineStr">
         <is>
-          <t>Q4019</t>
+          <t>Q4017</t>
         </is>
       </c>
     </row>
@@ -3508,32 +3508,32 @@
       </c>
       <c r="C75" s="1" t="inlineStr">
         <is>
-          <t>MM-616M</t>
+          <t>MM-608M</t>
         </is>
       </c>
       <c r="D75" s="1" t="inlineStr">
         <is>
-          <t>MM-834M</t>
+          <t>MM-832M</t>
         </is>
       </c>
       <c r="E75" s="1" t="inlineStr">
         <is>
-          <t>MM-9914M</t>
+          <t>MM-9913M</t>
         </is>
       </c>
       <c r="F75" s="1" t="inlineStr">
         <is>
-          <t>NR7</t>
+          <t>NR5</t>
         </is>
       </c>
       <c r="G75" s="1" t="inlineStr">
         <is>
-          <t>NR94</t>
+          <t>NR93</t>
         </is>
       </c>
       <c r="H75" s="1" t="inlineStr">
         <is>
-          <t>QBX003</t>
+          <t>Q4019</t>
         </is>
       </c>
     </row>
@@ -3550,32 +3550,32 @@
       </c>
       <c r="C76" s="1" t="inlineStr">
         <is>
-          <t>MM-624M</t>
+          <t>MM-616M</t>
         </is>
       </c>
       <c r="D76" s="1" t="inlineStr">
         <is>
-          <t>MM-838M</t>
+          <t>MM-834M</t>
         </is>
       </c>
       <c r="E76" s="1" t="inlineStr">
         <is>
-          <t>MM-9915M</t>
+          <t>MM-9914M</t>
         </is>
       </c>
       <c r="F76" s="1" t="inlineStr">
         <is>
-          <t>NR8</t>
+          <t>NR7</t>
         </is>
       </c>
       <c r="G76" s="1" t="inlineStr">
         <is>
-          <t>NR95</t>
+          <t>NR94</t>
         </is>
       </c>
       <c r="H76" s="1" t="inlineStr">
         <is>
-          <t>QBX004</t>
+          <t>QBX003</t>
         </is>
       </c>
     </row>
@@ -3592,32 +3592,32 @@
       </c>
       <c r="C77" s="1" t="inlineStr">
         <is>
-          <t>MM-632M</t>
+          <t>MM-624M</t>
         </is>
       </c>
       <c r="D77" s="1" t="inlineStr">
         <is>
-          <t>MM-842M</t>
+          <t>MM-838M</t>
         </is>
       </c>
       <c r="E77" s="1" t="inlineStr">
         <is>
-          <t>MM-9917M</t>
+          <t>MM-9915M</t>
         </is>
       </c>
       <c r="F77" s="1" t="inlineStr">
         <is>
-          <t>NR9</t>
+          <t>NR8</t>
         </is>
       </c>
       <c r="G77" s="1" t="inlineStr">
         <is>
-          <t>NR96</t>
+          <t>NR95</t>
         </is>
       </c>
       <c r="H77" s="1" t="inlineStr">
         <is>
-          <t>QBX005</t>
+          <t>QBX004</t>
         </is>
       </c>
     </row>
@@ -3634,32 +3634,32 @@
       </c>
       <c r="C78" s="1" t="inlineStr">
         <is>
-          <t>MM-636M</t>
+          <t>MM-632M</t>
         </is>
       </c>
       <c r="D78" s="1" t="inlineStr">
         <is>
-          <t>MM-844M</t>
+          <t>MM-842M</t>
         </is>
       </c>
       <c r="E78" s="1" t="inlineStr">
         <is>
-          <t>MM-9918M</t>
+          <t>MM-9917M</t>
         </is>
       </c>
       <c r="F78" s="1" t="inlineStr">
         <is>
-          <t>NR12</t>
+          <t>NR9</t>
         </is>
       </c>
       <c r="G78" s="1" t="inlineStr">
         <is>
-          <t>NR98</t>
+          <t>NR96</t>
         </is>
       </c>
       <c r="H78" s="1" t="inlineStr">
         <is>
-          <t>QBX006</t>
+          <t>QBX005</t>
         </is>
       </c>
     </row>
@@ -3676,32 +3676,32 @@
       </c>
       <c r="C79" s="1" t="inlineStr">
         <is>
-          <t>MM-640M</t>
+          <t>MM-636M</t>
         </is>
       </c>
       <c r="D79" s="1" t="inlineStr">
         <is>
-          <t>MM-852M</t>
+          <t>MM-844M</t>
         </is>
       </c>
       <c r="E79" s="1" t="inlineStr">
         <is>
-          <t>MM-9919M</t>
+          <t>MM-9918M</t>
         </is>
       </c>
       <c r="F79" s="1" t="inlineStr">
         <is>
-          <t>NR15</t>
+          <t>NR12</t>
         </is>
       </c>
       <c r="G79" s="1" t="inlineStr">
         <is>
-          <t>NR99</t>
+          <t>NR98</t>
         </is>
       </c>
       <c r="H79" s="1" t="inlineStr">
         <is>
-          <t>QE001</t>
+          <t>QBX006</t>
         </is>
       </c>
     </row>
@@ -3718,32 +3718,32 @@
       </c>
       <c r="C80" s="1" t="inlineStr">
         <is>
-          <t>MM-654M</t>
+          <t>MM-640M</t>
         </is>
       </c>
       <c r="D80" s="1" t="inlineStr">
         <is>
-          <t>MM-858M</t>
+          <t>MM-852M</t>
         </is>
       </c>
       <c r="E80" s="1" t="inlineStr">
         <is>
-          <t>MM-9920M</t>
+          <t>MM-9919M</t>
         </is>
       </c>
       <c r="F80" s="1" t="inlineStr">
         <is>
-          <t>NR16</t>
+          <t>NR15</t>
         </is>
       </c>
       <c r="G80" s="1" t="inlineStr">
         <is>
-          <t>NR101</t>
+          <t>NR99</t>
         </is>
       </c>
       <c r="H80" s="1" t="inlineStr">
         <is>
-          <t>QE002</t>
+          <t>QE001</t>
         </is>
       </c>
     </row>
@@ -3760,32 +3760,32 @@
       </c>
       <c r="C81" s="1" t="inlineStr">
         <is>
-          <t>MM-656M</t>
+          <t>MM-654M</t>
         </is>
       </c>
       <c r="D81" s="1" t="inlineStr">
         <is>
-          <t>MM-860M</t>
+          <t>MM-858M</t>
         </is>
       </c>
       <c r="E81" s="1" t="inlineStr">
         <is>
-          <t>MM-9922M</t>
+          <t>MM-9920M</t>
         </is>
       </c>
       <c r="F81" s="1" t="inlineStr">
         <is>
-          <t>NR18</t>
+          <t>NR16</t>
         </is>
       </c>
       <c r="G81" s="1" t="inlineStr">
         <is>
-          <t>NR102</t>
+          <t>NR101</t>
         </is>
       </c>
       <c r="H81" s="1" t="inlineStr">
         <is>
-          <t>QE003</t>
+          <t>QE002</t>
         </is>
       </c>
     </row>
@@ -3802,32 +3802,32 @@
       </c>
       <c r="C82" s="1" t="inlineStr">
         <is>
-          <t>MM-660M</t>
+          <t>MM-656M</t>
         </is>
       </c>
       <c r="D82" s="1" t="inlineStr">
         <is>
-          <t>MM-862M</t>
+          <t>MM-860M</t>
         </is>
       </c>
       <c r="E82" s="1" t="inlineStr">
         <is>
-          <t>MM-9923M</t>
+          <t>MM-9922M</t>
         </is>
       </c>
       <c r="F82" s="1" t="inlineStr">
         <is>
-          <t>NR19</t>
+          <t>NR18</t>
         </is>
       </c>
       <c r="G82" s="1" t="inlineStr">
         <is>
-          <t>NR103</t>
+          <t>NR102</t>
         </is>
       </c>
       <c r="H82" s="1" t="inlineStr">
         <is>
-          <t>QE004</t>
+          <t>QE003</t>
         </is>
       </c>
     </row>
@@ -3844,32 +3844,32 @@
       </c>
       <c r="C83" s="1" t="inlineStr">
         <is>
-          <t>MM-661M</t>
+          <t>MM-660M</t>
         </is>
       </c>
       <c r="D83" s="1" t="inlineStr">
         <is>
-          <t>MM-868M</t>
+          <t>MM-862M</t>
         </is>
       </c>
       <c r="E83" s="1" t="inlineStr">
         <is>
-          <t>MM-9924M</t>
+          <t>MM-9923M</t>
         </is>
       </c>
       <c r="F83" s="1" t="inlineStr">
         <is>
-          <t>NR21</t>
+          <t>NR19</t>
         </is>
       </c>
       <c r="G83" s="1" t="inlineStr">
         <is>
-          <t>NR105</t>
+          <t>NR103</t>
         </is>
       </c>
       <c r="H83" s="1" t="inlineStr">
         <is>
-          <t>QE006</t>
+          <t>QE004</t>
         </is>
       </c>
     </row>
@@ -3886,32 +3886,32 @@
       </c>
       <c r="C84" s="1" t="inlineStr">
         <is>
-          <t>MM-662M</t>
+          <t>MM-661M</t>
         </is>
       </c>
       <c r="D84" s="1" t="inlineStr">
         <is>
-          <t>MM-872M</t>
+          <t>MM-868M</t>
         </is>
       </c>
       <c r="E84" s="1" t="inlineStr">
         <is>
-          <t>MM-9926M</t>
+          <t>MM-9924M</t>
         </is>
       </c>
       <c r="F84" s="1" t="inlineStr">
         <is>
-          <t>NR25</t>
+          <t>NR21</t>
         </is>
       </c>
       <c r="G84" s="1" t="inlineStr">
         <is>
-          <t>NR108</t>
+          <t>NR105</t>
         </is>
       </c>
       <c r="H84" s="1" t="inlineStr">
         <is>
-          <t>QL001</t>
+          <t>QE006</t>
         </is>
       </c>
     </row>
@@ -3928,32 +3928,32 @@
       </c>
       <c r="C85" s="1" t="inlineStr">
         <is>
-          <t>MM-664M</t>
+          <t>MM-662M</t>
         </is>
       </c>
       <c r="D85" s="1" t="inlineStr">
         <is>
-          <t>MM-874M</t>
+          <t>MM-872M</t>
         </is>
       </c>
       <c r="E85" s="1" t="inlineStr">
         <is>
-          <t>MM-9928M</t>
+          <t>MM-9926M</t>
         </is>
       </c>
       <c r="F85" s="1" t="inlineStr">
         <is>
-          <t>NR27</t>
+          <t>NR25</t>
         </is>
       </c>
       <c r="G85" s="1" t="inlineStr">
         <is>
-          <t>NR109</t>
+          <t>NR108</t>
         </is>
       </c>
       <c r="H85" s="1" t="inlineStr">
         <is>
-          <t>QL002</t>
+          <t>QL001</t>
         </is>
       </c>
     </row>
@@ -3970,32 +3970,32 @@
       </c>
       <c r="C86" s="1" t="inlineStr">
         <is>
-          <t>MM-666M</t>
+          <t>MM-664M</t>
         </is>
       </c>
       <c r="D86" s="1" t="inlineStr">
         <is>
-          <t>MM-876M</t>
+          <t>MM-874M</t>
         </is>
       </c>
       <c r="E86" s="1" t="inlineStr">
         <is>
-          <t>MM-9929M</t>
+          <t>MM-9928M</t>
         </is>
       </c>
       <c r="F86" s="1" t="inlineStr">
         <is>
-          <t>NR28</t>
+          <t>NR27</t>
         </is>
       </c>
       <c r="G86" s="1" t="inlineStr">
         <is>
-          <t>NR110</t>
+          <t>NR109</t>
         </is>
       </c>
       <c r="H86" s="1" t="inlineStr">
         <is>
-          <t>QL004</t>
+          <t>QL002</t>
         </is>
       </c>
     </row>
@@ -4012,32 +4012,32 @@
       </c>
       <c r="C87" s="1" t="inlineStr">
         <is>
-          <t>MM-668M</t>
+          <t>MM-666M</t>
         </is>
       </c>
       <c r="D87" s="1" t="inlineStr">
         <is>
-          <t>MM-882M</t>
+          <t>MM-876M</t>
         </is>
       </c>
       <c r="E87" s="1" t="inlineStr">
         <is>
-          <t>MM-9932M</t>
+          <t>MM-9929M</t>
         </is>
       </c>
       <c r="F87" s="1" t="inlineStr">
         <is>
-          <t>NR30</t>
+          <t>NR28</t>
         </is>
       </c>
       <c r="G87" s="1" t="inlineStr">
         <is>
-          <t>NR111</t>
+          <t>NR110</t>
         </is>
       </c>
       <c r="H87" s="1" t="inlineStr">
         <is>
-          <t>QL007</t>
+          <t>QL004</t>
         </is>
       </c>
     </row>
@@ -4054,32 +4054,32 @@
       </c>
       <c r="C88" s="1" t="inlineStr">
         <is>
-          <t>MM-673M</t>
+          <t>MM-668M</t>
         </is>
       </c>
       <c r="D88" s="1" t="inlineStr">
         <is>
-          <t>MM-894M</t>
+          <t>MM-882M</t>
         </is>
       </c>
       <c r="E88" s="1" t="inlineStr">
         <is>
-          <t>MM-9933M</t>
+          <t>MM-9932M</t>
         </is>
       </c>
       <c r="F88" s="1" t="inlineStr">
         <is>
-          <t>NR31</t>
+          <t>NR30</t>
         </is>
       </c>
       <c r="G88" s="1" t="inlineStr">
         <is>
-          <t>NR112</t>
+          <t>NR111</t>
         </is>
       </c>
       <c r="H88" s="1" t="inlineStr">
         <is>
-          <t>QL008</t>
+          <t>QL007</t>
         </is>
       </c>
     </row>
@@ -4096,32 +4096,32 @@
       </c>
       <c r="C89" s="1" t="inlineStr">
         <is>
-          <t>MM-674M</t>
+          <t>MM-673M</t>
         </is>
       </c>
       <c r="D89" s="1" t="inlineStr">
         <is>
-          <t>MM-896M</t>
+          <t>MM-894M</t>
         </is>
       </c>
       <c r="E89" s="1" t="inlineStr">
         <is>
-          <t>MM-9934M</t>
+          <t>MM-9933M</t>
         </is>
       </c>
       <c r="F89" s="1" t="inlineStr">
         <is>
-          <t>NR34</t>
+          <t>NR31</t>
         </is>
       </c>
       <c r="G89" s="1" t="inlineStr">
         <is>
-          <t>NR113</t>
+          <t>NR112</t>
         </is>
       </c>
       <c r="H89" s="1" t="inlineStr">
         <is>
-          <t>QL010</t>
+          <t>QL008</t>
         </is>
       </c>
     </row>
@@ -4138,32 +4138,32 @@
       </c>
       <c r="C90" s="1" t="inlineStr">
         <is>
-          <t>MM-680M</t>
+          <t>MM-674M</t>
         </is>
       </c>
       <c r="D90" s="1" t="inlineStr">
         <is>
-          <t>MM-902M</t>
+          <t>MM-896M</t>
         </is>
       </c>
       <c r="E90" s="1" t="inlineStr">
         <is>
-          <t>MM-9936M</t>
+          <t>MM-9934M</t>
         </is>
       </c>
       <c r="F90" s="1" t="inlineStr">
         <is>
-          <t>NR36</t>
+          <t>NR34</t>
         </is>
       </c>
       <c r="G90" s="1" t="inlineStr">
         <is>
-          <t>NR115</t>
+          <t>NR113</t>
         </is>
       </c>
       <c r="H90" s="1" t="inlineStr">
         <is>
-          <t>QL011</t>
+          <t>QL010</t>
         </is>
       </c>
     </row>
@@ -4180,32 +4180,32 @@
       </c>
       <c r="C91" s="1" t="inlineStr">
         <is>
-          <t>MM-708M</t>
+          <t>MM-680M</t>
         </is>
       </c>
       <c r="D91" s="1" t="inlineStr">
         <is>
-          <t>MM-904M</t>
+          <t>MM-902M</t>
         </is>
       </c>
       <c r="E91" s="1" t="inlineStr">
         <is>
-          <t>MM-9938M</t>
+          <t>MM-9936M</t>
         </is>
       </c>
       <c r="F91" s="1" t="inlineStr">
         <is>
-          <t>NR37</t>
+          <t>NR36</t>
         </is>
       </c>
       <c r="G91" s="1" t="inlineStr">
         <is>
-          <t>NR118</t>
+          <t>NR115</t>
         </is>
       </c>
       <c r="H91" s="1" t="inlineStr">
         <is>
-          <t>QL014</t>
+          <t>QL011</t>
         </is>
       </c>
     </row>
@@ -4222,32 +4222,32 @@
       </c>
       <c r="C92" s="1" t="inlineStr">
         <is>
-          <t>MM-710M</t>
+          <t>MM-708M</t>
         </is>
       </c>
       <c r="D92" s="1" t="inlineStr">
         <is>
-          <t>MM-906M</t>
+          <t>MM-904M</t>
         </is>
       </c>
       <c r="E92" s="1" t="inlineStr">
         <is>
-          <t>MM-9941M</t>
+          <t>MM-9938M</t>
         </is>
       </c>
       <c r="F92" s="1" t="inlineStr">
         <is>
-          <t>NR38</t>
+          <t>NR37</t>
         </is>
       </c>
       <c r="G92" s="1" t="inlineStr">
         <is>
-          <t>NR119</t>
+          <t>NR118</t>
         </is>
       </c>
       <c r="H92" s="1" t="inlineStr">
         <is>
-          <t>QL018</t>
+          <t>QL014</t>
         </is>
       </c>
     </row>
@@ -4264,32 +4264,32 @@
       </c>
       <c r="C93" s="1" t="inlineStr">
         <is>
-          <t>MM-716M</t>
+          <t>MM-710M</t>
         </is>
       </c>
       <c r="D93" s="1" t="inlineStr">
         <is>
-          <t>MM-908M</t>
+          <t>MM-906M</t>
         </is>
       </c>
       <c r="E93" s="1" t="inlineStr">
         <is>
-          <t>MM-9943M</t>
+          <t>MM-9941M</t>
         </is>
       </c>
       <c r="F93" s="1" t="inlineStr">
         <is>
-          <t>NR39</t>
+          <t>NR38</t>
         </is>
       </c>
       <c r="G93" s="1" t="inlineStr">
         <is>
-          <t>NR120</t>
+          <t>NR119</t>
         </is>
       </c>
       <c r="H93" s="1" t="inlineStr">
         <is>
-          <t>QR1744</t>
+          <t>QL018</t>
         </is>
       </c>
     </row>
@@ -4306,32 +4306,32 @@
       </c>
       <c r="C94" s="1" t="inlineStr">
         <is>
-          <t>MM-722M</t>
+          <t>MM-716M</t>
         </is>
       </c>
       <c r="D94" s="1" t="inlineStr">
         <is>
-          <t>MM-910M</t>
+          <t>MM-908M</t>
         </is>
       </c>
       <c r="E94" s="1" t="inlineStr">
         <is>
-          <t>MM-9945M</t>
+          <t>MM-9943M</t>
         </is>
       </c>
       <c r="F94" s="1" t="inlineStr">
         <is>
-          <t>NR40</t>
+          <t>NR39</t>
         </is>
       </c>
       <c r="G94" s="1" t="inlineStr">
         <is>
-          <t>NR122</t>
+          <t>NR120</t>
         </is>
       </c>
       <c r="H94" s="1" t="inlineStr">
         <is>
-          <t>QR1771</t>
+          <t>QR1744</t>
         </is>
       </c>
     </row>
@@ -4348,32 +4348,32 @@
       </c>
       <c r="C95" s="1" t="inlineStr">
         <is>
-          <t>MM-726M</t>
+          <t>MM-722M</t>
         </is>
       </c>
       <c r="D95" s="1" t="inlineStr">
         <is>
-          <t>MM-912M</t>
+          <t>MM-910M</t>
         </is>
       </c>
       <c r="E95" s="1" t="inlineStr">
         <is>
-          <t>MM-9946M</t>
+          <t>MM-9945M</t>
         </is>
       </c>
       <c r="F95" s="1" t="inlineStr">
         <is>
-          <t>NR43</t>
+          <t>NR40</t>
         </is>
       </c>
       <c r="G95" s="1" t="inlineStr">
         <is>
-          <t>P14</t>
+          <t>NR122</t>
         </is>
       </c>
       <c r="H95" s="1" t="inlineStr">
         <is>
-          <t>QR5404</t>
+          <t>QR1771</t>
         </is>
       </c>
     </row>
@@ -4390,32 +4390,32 @@
       </c>
       <c r="C96" s="1" t="inlineStr">
         <is>
-          <t>MM-728M</t>
+          <t>MM-726M</t>
         </is>
       </c>
       <c r="D96" s="1" t="inlineStr">
         <is>
-          <t>MM-914M</t>
+          <t>MM-912M</t>
         </is>
       </c>
       <c r="E96" s="1" t="inlineStr">
         <is>
-          <t>MM-9950M</t>
+          <t>MM-9946M</t>
         </is>
       </c>
       <c r="F96" s="1" t="inlineStr">
         <is>
-          <t>NR44</t>
+          <t>NR43</t>
         </is>
       </c>
       <c r="G96" s="1" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P14</t>
         </is>
       </c>
       <c r="H96" s="1" t="inlineStr">
         <is>
-          <t>R711</t>
+          <t>QR5404</t>
         </is>
       </c>
     </row>
@@ -4432,32 +4432,32 @@
       </c>
       <c r="C97" s="1" t="inlineStr">
         <is>
-          <t>MM-734M</t>
+          <t>MM-728M</t>
         </is>
       </c>
       <c r="D97" s="1" t="inlineStr">
         <is>
-          <t>MM-920M</t>
+          <t>MM-914M</t>
         </is>
       </c>
       <c r="E97" s="1" t="inlineStr">
         <is>
-          <t>MM-9951M</t>
+          <t>MM-9950M</t>
         </is>
       </c>
       <c r="F97" s="1" t="inlineStr">
         <is>
-          <t>NR45</t>
+          <t>NR44</t>
         </is>
       </c>
       <c r="G97" s="1" t="inlineStr">
         <is>
-          <t>P2501</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="H97" s="1" t="inlineStr">
         <is>
-          <t>R766</t>
+          <t>R711</t>
         </is>
       </c>
     </row>
@@ -4474,32 +4474,32 @@
       </c>
       <c r="C98" s="1" t="inlineStr">
         <is>
-          <t>MM-736M</t>
+          <t>MM-734M</t>
         </is>
       </c>
       <c r="D98" s="1" t="inlineStr">
         <is>
-          <t>MM-922M</t>
+          <t>MM-920M</t>
         </is>
       </c>
       <c r="E98" s="1" t="inlineStr">
         <is>
-          <t>MM-9952M</t>
+          <t>MM-9951M</t>
         </is>
       </c>
       <c r="F98" s="1" t="inlineStr">
         <is>
-          <t>NR48</t>
+          <t>NR45</t>
         </is>
       </c>
       <c r="G98" s="1" t="inlineStr">
         <is>
-          <t>P2502</t>
+          <t>P2501</t>
         </is>
       </c>
       <c r="H98" s="1" t="inlineStr">
         <is>
-          <t>RB2353</t>
+          <t>R766</t>
         </is>
       </c>
     </row>
@@ -4516,32 +4516,32 @@
       </c>
       <c r="C99" s="1" t="inlineStr">
         <is>
-          <t>MM-738M</t>
+          <t>MM-736M</t>
         </is>
       </c>
       <c r="D99" s="1" t="inlineStr">
         <is>
-          <t>MM-924M</t>
+          <t>MM-922M</t>
         </is>
       </c>
       <c r="E99" s="1" t="inlineStr">
         <is>
-          <t>MM-9953M</t>
+          <t>MM-9952M</t>
         </is>
       </c>
       <c r="F99" s="1" t="inlineStr">
         <is>
-          <t>NR51</t>
+          <t>NR48</t>
         </is>
       </c>
       <c r="G99" s="1" t="inlineStr">
         <is>
-          <t>P2503</t>
+          <t>P2502</t>
         </is>
       </c>
       <c r="H99" s="1" t="inlineStr">
         <is>
-          <t>RCTST4</t>
+          <t>RB2353</t>
         </is>
       </c>
     </row>
@@ -4558,32 +4558,32 @@
       </c>
       <c r="C100" s="1" t="inlineStr">
         <is>
-          <t>MM-740M</t>
+          <t>MM-738M</t>
         </is>
       </c>
       <c r="D100" s="1" t="inlineStr">
         <is>
-          <t>MM-926M</t>
+          <t>MM-924M</t>
         </is>
       </c>
       <c r="E100" s="1" t="inlineStr">
         <is>
-          <t>MM-9954M</t>
+          <t>MM-9953M</t>
         </is>
       </c>
       <c r="F100" s="1" t="inlineStr">
         <is>
-          <t>NR52</t>
+          <t>NR51</t>
         </is>
       </c>
       <c r="G100" s="1" t="inlineStr">
         <is>
-          <t>P2505</t>
+          <t>P2503</t>
         </is>
       </c>
       <c r="H100" s="1" t="inlineStr">
         <is>
-          <t>RL301</t>
+          <t>RCTST4</t>
         </is>
       </c>
     </row>
@@ -4600,32 +4600,32 @@
       </c>
       <c r="C101" s="1" t="inlineStr">
         <is>
-          <t>MM-742M</t>
+          <t>MM-740M</t>
         </is>
       </c>
       <c r="D101" s="1" t="inlineStr">
         <is>
-          <t>MM-934M</t>
+          <t>MM-926M</t>
         </is>
       </c>
       <c r="E101" s="1" t="inlineStr">
         <is>
-          <t>MM-9955M</t>
+          <t>MM-9954M</t>
         </is>
       </c>
       <c r="F101" s="1" t="inlineStr">
         <is>
-          <t>NR53</t>
+          <t>NR52</t>
         </is>
       </c>
       <c r="G101" s="1" t="inlineStr">
         <is>
-          <t>P2506</t>
+          <t>P2505</t>
         </is>
       </c>
       <c r="H101" s="1" t="inlineStr">
         <is>
-          <t>RL302</t>
+          <t>RL301</t>
         </is>
       </c>
     </row>
@@ -4642,32 +4642,32 @@
       </c>
       <c r="C102" s="1" t="inlineStr">
         <is>
-          <t>MM-744M</t>
+          <t>MM-742M</t>
         </is>
       </c>
       <c r="D102" s="1" t="inlineStr">
         <is>
-          <t>MM-936M</t>
+          <t>MM-934M</t>
         </is>
       </c>
       <c r="E102" s="1" t="inlineStr">
         <is>
-          <t>MM-9957M</t>
+          <t>MM-9955M</t>
         </is>
       </c>
       <c r="F102" s="1" t="inlineStr">
         <is>
-          <t>NR54</t>
+          <t>NR53</t>
         </is>
       </c>
       <c r="G102" s="1" t="inlineStr">
         <is>
-          <t>P2507</t>
+          <t>P2506</t>
         </is>
       </c>
       <c r="H102" s="1" t="inlineStr">
         <is>
-          <t>RL304</t>
+          <t>RL302</t>
         </is>
       </c>
     </row>
@@ -4684,32 +4684,32 @@
       </c>
       <c r="C103" s="1" t="inlineStr">
         <is>
-          <t>MM-752M</t>
+          <t>MM-744M</t>
         </is>
       </c>
       <c r="D103" s="1" t="inlineStr">
         <is>
-          <t>MM-940M</t>
+          <t>MM-936M</t>
         </is>
       </c>
       <c r="E103" s="1" t="inlineStr">
         <is>
-          <t>MM-9959M</t>
+          <t>MM-9957M</t>
         </is>
       </c>
       <c r="F103" s="1" t="inlineStr">
         <is>
-          <t>NR57</t>
+          <t>NR54</t>
         </is>
       </c>
       <c r="G103" s="1" t="inlineStr">
         <is>
-          <t>P2508</t>
+          <t>P2507</t>
         </is>
       </c>
       <c r="H103" s="1" t="inlineStr">
         <is>
-          <t>RL305</t>
+          <t>RL304</t>
         </is>
       </c>
     </row>
@@ -4726,32 +4726,32 @@
       </c>
       <c r="C104" s="1" t="inlineStr">
         <is>
-          <t>MM-756M</t>
+          <t>MM-752M</t>
         </is>
       </c>
       <c r="D104" s="1" t="inlineStr">
         <is>
-          <t>MM-944M</t>
+          <t>MM-940M</t>
         </is>
       </c>
       <c r="E104" s="1" t="inlineStr">
         <is>
-          <t>MM-9960M</t>
+          <t>MM-9959M</t>
         </is>
       </c>
       <c r="F104" s="1" t="inlineStr">
         <is>
-          <t>NR59</t>
+          <t>NR57</t>
         </is>
       </c>
       <c r="G104" s="1" t="inlineStr">
         <is>
-          <t>P2509</t>
+          <t>P2508</t>
         </is>
       </c>
       <c r="H104" s="1" t="inlineStr">
         <is>
-          <t>RL307</t>
+          <t>RL305</t>
         </is>
       </c>
     </row>
@@ -4768,32 +4768,32 @@
       </c>
       <c r="C105" s="1" t="inlineStr">
         <is>
-          <t>MM-760M</t>
+          <t>MM-756M</t>
         </is>
       </c>
       <c r="D105" s="1" t="inlineStr">
         <is>
-          <t>MM-948M</t>
+          <t>MM-944M</t>
         </is>
       </c>
       <c r="E105" s="1" t="inlineStr">
         <is>
-          <t>MM-9961M</t>
+          <t>MM-9960M</t>
         </is>
       </c>
       <c r="F105" s="1" t="inlineStr">
         <is>
-          <t>NR61</t>
+          <t>NR59</t>
         </is>
       </c>
       <c r="G105" s="1" t="inlineStr">
         <is>
-          <t>P2510</t>
+          <t>P2509</t>
         </is>
       </c>
       <c r="H105" s="1" t="inlineStr">
         <is>
-          <t>RL309</t>
+          <t>RL307</t>
         </is>
       </c>
     </row>
@@ -4810,32 +4810,32 @@
       </c>
       <c r="C106" s="1" t="inlineStr">
         <is>
-          <t>MM-764M</t>
+          <t>MM-760M</t>
         </is>
       </c>
       <c r="D106" s="1" t="inlineStr">
         <is>
-          <t>MM-952M</t>
+          <t>MM-948M</t>
         </is>
       </c>
       <c r="E106" s="1" t="inlineStr">
         <is>
-          <t>MM-9962M</t>
+          <t>MM-9961M</t>
         </is>
       </c>
       <c r="F106" s="1" t="inlineStr">
         <is>
-          <t>NR62</t>
+          <t>NR61</t>
         </is>
       </c>
       <c r="G106" s="1" t="inlineStr">
         <is>
-          <t>P2511</t>
+          <t>P2510</t>
         </is>
       </c>
       <c r="H106" s="1" t="inlineStr">
         <is>
-          <t>RL310</t>
+          <t>RL309</t>
         </is>
       </c>
     </row>
@@ -4852,32 +4852,32 @@
       </c>
       <c r="C107" s="1" t="inlineStr">
         <is>
-          <t>MM-768M</t>
+          <t>MM-764M</t>
         </is>
       </c>
       <c r="D107" s="1" t="inlineStr">
         <is>
-          <t>MM-954M</t>
+          <t>MM-952M</t>
         </is>
       </c>
       <c r="E107" s="1" t="inlineStr">
         <is>
-          <t>MM-9963M</t>
+          <t>MM-9962M</t>
         </is>
       </c>
       <c r="F107" s="1" t="inlineStr">
         <is>
-          <t>NR64</t>
+          <t>NR62</t>
         </is>
       </c>
       <c r="G107" s="1" t="inlineStr">
         <is>
-          <t>P2513</t>
+          <t>P2511</t>
         </is>
       </c>
       <c r="H107" s="1" t="inlineStr">
         <is>
-          <t>S312</t>
+          <t>RL310</t>
         </is>
       </c>
     </row>
@@ -4894,32 +4894,32 @@
       </c>
       <c r="C108" s="1" t="inlineStr">
         <is>
-          <t>MM-774M</t>
+          <t>MM-768M</t>
         </is>
       </c>
       <c r="D108" s="1" t="inlineStr">
         <is>
-          <t>MM-956M</t>
+          <t>MM-954M</t>
         </is>
       </c>
       <c r="E108" s="1" t="inlineStr">
         <is>
-          <t>MM-9964M</t>
+          <t>MM-9963M</t>
         </is>
       </c>
       <c r="F108" s="1" t="inlineStr">
         <is>
-          <t>NR65</t>
+          <t>NR64</t>
         </is>
       </c>
       <c r="G108" s="1" t="inlineStr">
         <is>
-          <t>P2514</t>
+          <t>P2513</t>
         </is>
       </c>
       <c r="H108" s="1" t="inlineStr">
         <is>
-          <t>S317</t>
+          <t>S312</t>
         </is>
       </c>
     </row>
@@ -4936,32 +4936,32 @@
       </c>
       <c r="C109" s="1" t="inlineStr">
         <is>
-          <t>MM-776M</t>
+          <t>MM-774M</t>
         </is>
       </c>
       <c r="D109" s="1" t="inlineStr">
         <is>
-          <t>MM-958M</t>
+          <t>MM-956M</t>
         </is>
       </c>
       <c r="E109" s="1" t="inlineStr">
         <is>
-          <t>MM-9965M</t>
+          <t>MM-9964M</t>
         </is>
       </c>
       <c r="F109" s="1" t="inlineStr">
         <is>
-          <t>NR66</t>
+          <t>NR65</t>
         </is>
       </c>
       <c r="G109" s="1" t="inlineStr">
         <is>
-          <t>P2515</t>
+          <t>P2514</t>
         </is>
       </c>
       <c r="H109" s="1" t="inlineStr">
         <is>
-          <t>S3301</t>
+          <t>S317</t>
         </is>
       </c>
     </row>
@@ -4978,32 +4978,32 @@
       </c>
       <c r="C110" s="1" t="inlineStr">
         <is>
-          <t>MM-778M</t>
+          <t>MM-776M</t>
         </is>
       </c>
       <c r="D110" s="1" t="inlineStr">
         <is>
-          <t>MM-962M</t>
+          <t>MM-958M</t>
         </is>
       </c>
       <c r="E110" s="1" t="inlineStr">
         <is>
-          <t>MM-9966M</t>
+          <t>MM-9965M</t>
         </is>
       </c>
       <c r="F110" s="1" t="inlineStr">
         <is>
-          <t>NR67</t>
+          <t>NR66</t>
         </is>
       </c>
       <c r="G110" s="1" t="inlineStr">
         <is>
-          <t>P2516</t>
+          <t>P2515</t>
         </is>
       </c>
       <c r="H110" s="1" t="inlineStr">
         <is>
-          <t>S3302</t>
+          <t>S3301</t>
         </is>
       </c>
     </row>
@@ -5020,32 +5020,32 @@
       </c>
       <c r="C111" s="1" t="inlineStr">
         <is>
-          <t>MM-780M</t>
+          <t>MM-778M</t>
         </is>
       </c>
       <c r="D111" s="1" t="inlineStr">
         <is>
-          <t>MM-964M</t>
+          <t>MM-962M</t>
         </is>
       </c>
       <c r="E111" s="1" t="inlineStr">
         <is>
-          <t>MM-9967M</t>
+          <t>MM-9966M</t>
         </is>
       </c>
       <c r="F111" s="1" t="inlineStr">
         <is>
-          <t>NR68</t>
+          <t>NR67</t>
         </is>
       </c>
       <c r="G111" s="1" t="inlineStr">
         <is>
-          <t>PB1</t>
+          <t>P2516</t>
         </is>
       </c>
       <c r="H111" s="1" t="inlineStr">
         <is>
-          <t>S3304</t>
+          <t>S3302</t>
         </is>
       </c>
     </row>
@@ -5062,32 +5062,32 @@
       </c>
       <c r="C112" s="1" t="inlineStr">
         <is>
-          <t>MM-784M</t>
+          <t>MM-780M</t>
         </is>
       </c>
       <c r="D112" s="1" t="inlineStr">
         <is>
-          <t>MM-966M</t>
+          <t>MM-964M</t>
         </is>
       </c>
       <c r="E112" s="1" t="inlineStr">
         <is>
-          <t>MM-9969M</t>
+          <t>MM-9967M</t>
         </is>
       </c>
       <c r="F112" s="1" t="inlineStr">
         <is>
-          <t>NR69</t>
+          <t>NR68</t>
         </is>
       </c>
       <c r="G112" s="1" t="inlineStr">
         <is>
-          <t>PB2</t>
+          <t>PB1</t>
         </is>
       </c>
       <c r="H112" s="1" t="inlineStr">
         <is>
-          <t>S3305</t>
+          <t>S3304</t>
         </is>
       </c>
     </row>
@@ -5104,2084 +5104,2089 @@
       </c>
       <c r="C113" s="1" t="inlineStr">
         <is>
-          <t>MM-790M</t>
+          <t>MM-784M</t>
         </is>
       </c>
       <c r="D113" s="1" t="inlineStr">
         <is>
-          <t>MM-968M</t>
+          <t>MM-966M</t>
         </is>
       </c>
       <c r="E113" s="1" t="inlineStr">
         <is>
-          <t>MM-9970M</t>
+          <t>MM-9969M</t>
         </is>
       </c>
       <c r="F113" s="1" t="inlineStr">
         <is>
-          <t>NR71</t>
+          <t>NR69</t>
         </is>
       </c>
       <c r="G113" s="1" t="inlineStr">
         <is>
-          <t>PB4</t>
+          <t>PB2</t>
         </is>
       </c>
       <c r="H113" s="1" t="inlineStr">
         <is>
-          <t>S3306</t>
+          <t>S3305</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
         <is>
-          <t>S3307</t>
+          <t>S3306</t>
         </is>
       </c>
       <c r="B115" s="1" t="inlineStr">
         <is>
-          <t>TT107</t>
+          <t>TT106</t>
         </is>
       </c>
       <c r="C115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8107</t>
+          <t>VLINE-8104</t>
         </is>
       </c>
       <c r="D115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8306</t>
+          <t>VLINE-8304</t>
         </is>
       </c>
       <c r="E115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8447</t>
+          <t>VLINE-8446</t>
         </is>
       </c>
       <c r="F115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8753</t>
+          <t>VLINE-8752</t>
         </is>
       </c>
       <c r="G115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8818</t>
+          <t>VLINE-8817</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
         <is>
-          <t>S3309</t>
+          <t>S3307</t>
         </is>
       </c>
       <c r="B116" s="1" t="inlineStr">
         <is>
-          <t>TT108</t>
+          <t>TT107</t>
         </is>
       </c>
       <c r="C116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8110</t>
+          <t>VLINE-8107</t>
         </is>
       </c>
       <c r="D116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8311</t>
+          <t>VLINE-8306</t>
         </is>
       </c>
       <c r="E116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8449</t>
+          <t>VLINE-8447</t>
         </is>
       </c>
       <c r="F116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8754</t>
+          <t>VLINE-8753</t>
         </is>
       </c>
       <c r="G116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8819</t>
+          <t>VLINE-8818</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="1" t="inlineStr">
         <is>
-          <t>S3310</t>
+          <t>S3309</t>
         </is>
       </c>
       <c r="B117" s="1" t="inlineStr">
         <is>
-          <t>TT110</t>
+          <t>TT108</t>
         </is>
       </c>
       <c r="C117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8111</t>
+          <t>VLINE-8110</t>
         </is>
       </c>
       <c r="D117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8313</t>
+          <t>VLINE-8311</t>
         </is>
       </c>
       <c r="E117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8450</t>
+          <t>VLINE-8449</t>
         </is>
       </c>
       <c r="F117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8755</t>
+          <t>VLINE-8754</t>
         </is>
       </c>
       <c r="G117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8822</t>
+          <t>VLINE-8819</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
         <is>
-          <t>S7001</t>
+          <t>S3310</t>
         </is>
       </c>
       <c r="B118" s="1" t="inlineStr">
         <is>
-          <t>TT113</t>
+          <t>TT110</t>
         </is>
       </c>
       <c r="C118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8113</t>
+          <t>VLINE-8111</t>
         </is>
       </c>
       <c r="D118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8314</t>
+          <t>VLINE-8313</t>
         </is>
       </c>
       <c r="E118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8451</t>
+          <t>VLINE-8450</t>
         </is>
       </c>
       <c r="F118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8756</t>
+          <t>VLINE-8755</t>
         </is>
       </c>
       <c r="G118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8860</t>
+          <t>VLINE-8822</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
         <is>
-          <t>S7002</t>
+          <t>S7001</t>
         </is>
       </c>
       <c r="B119" s="1" t="inlineStr">
         <is>
-          <t>TT114</t>
+          <t>TT113</t>
         </is>
       </c>
       <c r="C119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8114</t>
+          <t>VLINE-8113</t>
         </is>
       </c>
       <c r="D119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8316</t>
+          <t>VLINE-8314</t>
         </is>
       </c>
       <c r="E119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8452</t>
+          <t>VLINE-8451</t>
         </is>
       </c>
       <c r="F119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8757</t>
+          <t>VLINE-8756</t>
         </is>
       </c>
       <c r="G119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8861</t>
+          <t>VLINE-8860</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="1" t="inlineStr">
         <is>
-          <t>S7003</t>
+          <t>S7002</t>
         </is>
       </c>
       <c r="B120" s="1" t="inlineStr">
         <is>
-          <t>TT115</t>
+          <t>TT114</t>
         </is>
       </c>
       <c r="C120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8115</t>
+          <t>VLINE-8114</t>
         </is>
       </c>
       <c r="D120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8318</t>
+          <t>VLINE-8316</t>
         </is>
       </c>
       <c r="E120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8453</t>
+          <t>VLINE-8452</t>
         </is>
       </c>
       <c r="F120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8758</t>
+          <t>VLINE-8757</t>
         </is>
       </c>
       <c r="G120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8862</t>
+          <t>VLINE-8861</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="1" t="inlineStr">
         <is>
-          <t>S7005</t>
+          <t>S7003</t>
         </is>
       </c>
       <c r="B121" s="1" t="inlineStr">
         <is>
-          <t>TT116</t>
+          <t>TT115</t>
         </is>
       </c>
       <c r="C121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8119</t>
+          <t>VLINE-8115</t>
         </is>
       </c>
       <c r="D121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8321</t>
+          <t>VLINE-8318</t>
         </is>
       </c>
       <c r="E121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8454</t>
+          <t>VLINE-8453</t>
         </is>
       </c>
       <c r="F121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8759</t>
+          <t>VLINE-8758</t>
         </is>
       </c>
       <c r="G121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8863</t>
+          <t>VLINE-8862</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="1" t="inlineStr">
         <is>
-          <t>S7006</t>
+          <t>S7005</t>
         </is>
       </c>
       <c r="B122" s="1" t="inlineStr">
         <is>
-          <t>TT117</t>
+          <t>TT116</t>
         </is>
       </c>
       <c r="C122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8120</t>
+          <t>VLINE-8119</t>
         </is>
       </c>
       <c r="D122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8323</t>
+          <t>VLINE-8321</t>
         </is>
       </c>
       <c r="E122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8455</t>
+          <t>VLINE-8454</t>
         </is>
       </c>
       <c r="F122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8760</t>
+          <t>VLINE-8759</t>
         </is>
       </c>
       <c r="G122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8864</t>
+          <t>VLINE-8863</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="1" t="inlineStr">
         <is>
-          <t>S7007</t>
+          <t>S7006</t>
         </is>
       </c>
       <c r="B123" s="1" t="inlineStr">
         <is>
-          <t>TT122</t>
+          <t>TT117</t>
         </is>
       </c>
       <c r="C123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8121</t>
+          <t>VLINE-8120</t>
         </is>
       </c>
       <c r="D123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8324</t>
+          <t>VLINE-8323</t>
         </is>
       </c>
       <c r="E123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8456</t>
+          <t>VLINE-8455</t>
         </is>
       </c>
       <c r="F123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8761</t>
+          <t>VLINE-8760</t>
         </is>
       </c>
       <c r="G123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8865</t>
+          <t>VLINE-8864</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="1" t="inlineStr">
         <is>
-          <t>S7008</t>
+          <t>S7007</t>
         </is>
       </c>
       <c r="B124" s="1" t="inlineStr">
         <is>
-          <t>TT127</t>
+          <t>TT122</t>
         </is>
       </c>
       <c r="C124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8123</t>
+          <t>VLINE-8121</t>
         </is>
       </c>
       <c r="D124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8325</t>
+          <t>VLINE-8324</t>
         </is>
       </c>
       <c r="E124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8457</t>
+          <t>VLINE-8456</t>
         </is>
       </c>
       <c r="F124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8762</t>
+          <t>VLINE-8761</t>
         </is>
       </c>
       <c r="G124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8866</t>
+          <t>VLINE-8865</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="1" t="inlineStr">
         <is>
-          <t>S7012</t>
+          <t>S7008</t>
         </is>
       </c>
       <c r="B125" s="1" t="inlineStr">
         <is>
-          <t>TT128</t>
+          <t>TT127</t>
         </is>
       </c>
       <c r="C125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8124</t>
+          <t>VLINE-8123</t>
         </is>
       </c>
       <c r="D125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8328</t>
+          <t>VLINE-8325</t>
         </is>
       </c>
       <c r="E125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8460</t>
+          <t>VLINE-8457</t>
         </is>
       </c>
       <c r="F125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8763</t>
+          <t>VLINE-8762</t>
         </is>
       </c>
       <c r="G125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8867</t>
+          <t>VLINE-8866</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="1" t="inlineStr">
         <is>
-          <t>S7014</t>
+          <t>S7012</t>
         </is>
       </c>
       <c r="B126" s="1" t="inlineStr">
         <is>
-          <t>TT130</t>
+          <t>TT128</t>
         </is>
       </c>
       <c r="C126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8126</t>
+          <t>VLINE-8124</t>
         </is>
       </c>
       <c r="D126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8329</t>
+          <t>VLINE-8328</t>
         </is>
       </c>
       <c r="E126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8461</t>
+          <t>VLINE-8460</t>
         </is>
       </c>
       <c r="F126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8765</t>
+          <t>VLINE-8763</t>
         </is>
       </c>
       <c r="G126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8868</t>
+          <t>VLINE-8867</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
         <is>
-          <t>S7015</t>
+          <t>S7014</t>
         </is>
       </c>
       <c r="B127" s="1" t="inlineStr">
         <is>
-          <t>TT131</t>
+          <t>TT130</t>
         </is>
       </c>
       <c r="C127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8127</t>
+          <t>VLINE-8126</t>
         </is>
       </c>
       <c r="D127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8332</t>
+          <t>VLINE-8329</t>
         </is>
       </c>
       <c r="E127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8464</t>
+          <t>VLINE-8461</t>
         </is>
       </c>
       <c r="F127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8766</t>
+          <t>VLINE-8765</t>
         </is>
       </c>
       <c r="G127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8869</t>
+          <t>VLINE-8868</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
         <is>
-          <t>S7017</t>
+          <t>S7015</t>
         </is>
       </c>
       <c r="B128" s="1" t="inlineStr">
         <is>
-          <t>TT202</t>
+          <t>TT131</t>
         </is>
       </c>
       <c r="C128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8128</t>
+          <t>VLINE-8127</t>
         </is>
       </c>
       <c r="D128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8336</t>
+          <t>VLINE-8332</t>
         </is>
       </c>
       <c r="E128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8465</t>
+          <t>VLINE-8464</t>
         </is>
       </c>
       <c r="F128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8767</t>
+          <t>VLINE-8766</t>
         </is>
       </c>
       <c r="G128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8890</t>
+          <t>VLINE-8869</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
         <is>
-          <t>S7018</t>
+          <t>S7017</t>
         </is>
       </c>
       <c r="B129" s="1" t="inlineStr">
         <is>
-          <t>TT206</t>
+          <t>TT202</t>
         </is>
       </c>
       <c r="C129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8129</t>
+          <t>VLINE-8128</t>
         </is>
       </c>
       <c r="D129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8337</t>
+          <t>VLINE-8336</t>
         </is>
       </c>
       <c r="E129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8468</t>
+          <t>VLINE-8465</t>
         </is>
       </c>
       <c r="F129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8768</t>
+          <t>VLINE-8767</t>
         </is>
       </c>
       <c r="G129" s="1" t="inlineStr">
         <is>
-          <t>WH001</t>
+          <t>VLINE-8890</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="1" t="inlineStr">
         <is>
-          <t>S7020</t>
+          <t>S7018</t>
         </is>
       </c>
       <c r="B130" s="1" t="inlineStr">
         <is>
-          <t>VL352</t>
+          <t>TT206</t>
         </is>
       </c>
       <c r="C130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8131</t>
+          <t>VLINE-8129</t>
         </is>
       </c>
       <c r="D130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8338</t>
+          <t>VLINE-8337</t>
         </is>
       </c>
       <c r="E130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8469</t>
+          <t>VLINE-8468</t>
         </is>
       </c>
       <c r="F130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8769</t>
+          <t>VLINE-8768</t>
         </is>
       </c>
       <c r="G130" s="1" t="inlineStr">
         <is>
-          <t>WH003</t>
+          <t>WH001</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="1" t="inlineStr">
         <is>
-          <t>S7022</t>
+          <t>S7020</t>
         </is>
       </c>
       <c r="B131" s="1" t="inlineStr">
         <is>
-          <t>VL353</t>
+          <t>VL352</t>
         </is>
       </c>
       <c r="C131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8132</t>
+          <t>VLINE-8131</t>
         </is>
       </c>
       <c r="D131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8339</t>
+          <t>VLINE-8338</t>
         </is>
       </c>
       <c r="E131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8605</t>
+          <t>VLINE-8469</t>
         </is>
       </c>
       <c r="F131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8770</t>
+          <t>VLINE-8769</t>
         </is>
       </c>
       <c r="G131" s="1" t="inlineStr">
         <is>
-          <t>WL02</t>
+          <t>WH003</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="1" t="inlineStr">
         <is>
-          <t>SCT001</t>
+          <t>S7022</t>
         </is>
       </c>
       <c r="B132" s="1" t="inlineStr">
         <is>
-          <t>VL357</t>
+          <t>VL353</t>
         </is>
       </c>
       <c r="C132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8133</t>
+          <t>VLINE-8132</t>
         </is>
       </c>
       <c r="D132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8362</t>
+          <t>VLINE-8339</t>
         </is>
       </c>
       <c r="E132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8610</t>
+          <t>VLINE-8605</t>
         </is>
       </c>
       <c r="F132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8772</t>
+          <t>VLINE-8770</t>
         </is>
       </c>
       <c r="G132" s="1" t="inlineStr">
         <is>
-          <t>X12-X14</t>
+          <t>WL02</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="1" t="inlineStr">
         <is>
-          <t>SCT002</t>
+          <t>SCT001</t>
         </is>
       </c>
       <c r="B133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8004</t>
+          <t>VL357</t>
         </is>
       </c>
       <c r="C133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8134</t>
+          <t>VLINE-8133</t>
         </is>
       </c>
       <c r="D133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8363</t>
+          <t>VLINE-8362</t>
         </is>
       </c>
       <c r="E133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8612</t>
+          <t>VLINE-8610</t>
         </is>
       </c>
       <c r="F133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8773</t>
+          <t>VLINE-8772</t>
         </is>
       </c>
       <c r="G133" s="1" t="inlineStr">
         <is>
-          <t>X31</t>
+          <t>X12-X14</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="1" t="inlineStr">
         <is>
-          <t>SCT006</t>
+          <t>SCT002</t>
         </is>
       </c>
       <c r="B134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8007</t>
+          <t>VLINE-8004</t>
         </is>
       </c>
       <c r="C134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8136</t>
+          <t>VLINE-8134</t>
         </is>
       </c>
       <c r="D134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8365</t>
+          <t>VLINE-8363</t>
         </is>
       </c>
       <c r="E134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8615</t>
+          <t>VLINE-8612</t>
         </is>
       </c>
       <c r="F134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8774</t>
+          <t>VLINE-8773</t>
         </is>
       </c>
       <c r="G134" s="1" t="inlineStr">
         <is>
-          <t>XP2000</t>
+          <t>X31</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="1" t="inlineStr">
         <is>
-          <t>SCT007</t>
+          <t>SCT006</t>
         </is>
       </c>
       <c r="B135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8011</t>
+          <t>VLINE-8007</t>
         </is>
       </c>
       <c r="C135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8137</t>
+          <t>VLINE-8136</t>
         </is>
       </c>
       <c r="D135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8366</t>
+          <t>VLINE-8365</t>
         </is>
       </c>
       <c r="E135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8617</t>
+          <t>VLINE-8615</t>
         </is>
       </c>
       <c r="F135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8776</t>
+          <t>VLINE-8774</t>
         </is>
       </c>
       <c r="G135" s="1" t="inlineStr">
         <is>
-          <t>XP2003</t>
+          <t>XP2000</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="1" t="inlineStr">
         <is>
-          <t>SCT009</t>
+          <t>SCT007</t>
         </is>
       </c>
       <c r="B136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8013</t>
+          <t>VLINE-8011</t>
         </is>
       </c>
       <c r="C136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8140</t>
+          <t>VLINE-8137</t>
         </is>
       </c>
       <c r="D136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8368</t>
+          <t>VLINE-8366</t>
         </is>
       </c>
       <c r="E136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8620</t>
+          <t>VLINE-8617</t>
         </is>
       </c>
       <c r="F136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8778</t>
+          <t>VLINE-8776</t>
         </is>
       </c>
       <c r="G136" s="1" t="inlineStr">
         <is>
-          <t>XP2004</t>
+          <t>XP2003</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="1" t="inlineStr">
         <is>
-          <t>SCT011</t>
+          <t>SCT009</t>
         </is>
       </c>
       <c r="B137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8019</t>
+          <t>VLINE-8013</t>
         </is>
       </c>
       <c r="C137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8141</t>
+          <t>VLINE-8140</t>
         </is>
       </c>
       <c r="D137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8369</t>
+          <t>VLINE-8368</t>
         </is>
       </c>
       <c r="E137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8625</t>
+          <t>VLINE-8620</t>
         </is>
       </c>
       <c r="F137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8779</t>
+          <t>VLINE-8778</t>
         </is>
       </c>
       <c r="G137" s="1" t="inlineStr">
         <is>
-          <t>XP2005</t>
+          <t>XP2004</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="1" t="inlineStr">
         <is>
-          <t>SCT013</t>
+          <t>SCT011</t>
         </is>
       </c>
       <c r="B138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8020</t>
+          <t>VLINE-8019</t>
         </is>
       </c>
       <c r="C138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8142</t>
+          <t>VLINE-8141</t>
         </is>
       </c>
       <c r="D138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8403</t>
+          <t>VLINE-8369</t>
         </is>
       </c>
       <c r="E138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8630</t>
+          <t>VLINE-8625</t>
         </is>
       </c>
       <c r="F138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8780</t>
+          <t>VLINE-8779</t>
         </is>
       </c>
       <c r="G138" s="1" t="inlineStr">
         <is>
-          <t>XP2007</t>
+          <t>XP2005</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="1" t="inlineStr">
         <is>
-          <t>SCT014</t>
+          <t>SCT013</t>
         </is>
       </c>
       <c r="B139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8023</t>
+          <t>VLINE-8020</t>
         </is>
       </c>
       <c r="C139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8144</t>
+          <t>VLINE-8142</t>
         </is>
       </c>
       <c r="D139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8404</t>
+          <t>VLINE-8403</t>
         </is>
       </c>
       <c r="E139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8671</t>
+          <t>VLINE-8630</t>
         </is>
       </c>
       <c r="F139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8781</t>
+          <t>VLINE-8780</t>
         </is>
       </c>
       <c r="G139" s="1" t="inlineStr">
         <is>
-          <t>XP2008</t>
+          <t>XP2007</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="1" t="inlineStr">
         <is>
-          <t>SCT015</t>
+          <t>SCT014</t>
         </is>
       </c>
       <c r="B140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8025</t>
+          <t>VLINE-8023</t>
         </is>
       </c>
       <c r="C140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8145</t>
+          <t>VLINE-8144</t>
         </is>
       </c>
       <c r="D140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8406</t>
+          <t>VLINE-8404</t>
         </is>
       </c>
       <c r="E140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8706</t>
+          <t>VLINE-8671</t>
         </is>
       </c>
       <c r="F140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8782</t>
+          <t>VLINE-8781</t>
         </is>
       </c>
       <c r="G140" s="1" t="inlineStr">
         <is>
-          <t>XP2010</t>
+          <t>XP2008</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="1" t="inlineStr">
         <is>
-          <t>SO2</t>
+          <t>SCT015</t>
         </is>
       </c>
       <c r="B141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8026</t>
+          <t>VLINE-8025</t>
         </is>
       </c>
       <c r="C141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8148</t>
+          <t>VLINE-8145</t>
         </is>
       </c>
       <c r="D141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8408</t>
+          <t>VLINE-8406</t>
         </is>
       </c>
       <c r="E141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8711</t>
+          <t>VLINE-8706</t>
         </is>
       </c>
       <c r="F141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8783</t>
+          <t>VLINE-8782</t>
         </is>
       </c>
       <c r="G141" s="1" t="inlineStr">
         <is>
-          <t>XP2011</t>
+          <t>XP2010</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="1" t="inlineStr">
         <is>
-          <t>SSR101</t>
+          <t>SO2</t>
         </is>
       </c>
       <c r="B142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8027</t>
+          <t>VLINE-8026</t>
         </is>
       </c>
       <c r="C142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8150</t>
+          <t>VLINE-8148</t>
         </is>
       </c>
       <c r="D142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8410</t>
+          <t>VLINE-8408</t>
         </is>
       </c>
       <c r="E142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8714</t>
+          <t>VLINE-8711</t>
         </is>
       </c>
       <c r="F142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8784</t>
+          <t>VLINE-8783</t>
         </is>
       </c>
       <c r="G142" s="1" t="inlineStr">
         <is>
-          <t>XP2012</t>
+          <t>XP2011</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="1" t="inlineStr">
         <is>
-          <t>SSR102</t>
+          <t>SSR101</t>
         </is>
       </c>
       <c r="B143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8028</t>
+          <t>VLINE-8027</t>
         </is>
       </c>
       <c r="C143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8151</t>
+          <t>VLINE-8150</t>
         </is>
       </c>
       <c r="D143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8411</t>
+          <t>VLINE-8410</t>
         </is>
       </c>
       <c r="E143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8717</t>
+          <t>VLINE-8714</t>
         </is>
       </c>
       <c r="F143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8786</t>
+          <t>VLINE-8784</t>
         </is>
       </c>
       <c r="G143" s="1" t="inlineStr">
         <is>
-          <t>XP2013</t>
+          <t>XP2012</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="1" t="inlineStr">
         <is>
-          <t>SSR103</t>
+          <t>SSR102</t>
         </is>
       </c>
       <c r="B144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8029</t>
+          <t>VLINE-8028</t>
         </is>
       </c>
       <c r="C144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8152</t>
+          <t>VLINE-8151</t>
         </is>
       </c>
       <c r="D144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8413</t>
+          <t>VLINE-8411</t>
         </is>
       </c>
       <c r="E144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8720</t>
+          <t>VLINE-8717</t>
         </is>
       </c>
       <c r="F144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8787</t>
+          <t>VLINE-8786</t>
         </is>
       </c>
       <c r="G144" s="1" t="inlineStr">
         <is>
-          <t>XP2014</t>
+          <t>XP2013</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="1" t="inlineStr">
         <is>
-          <t>SSR104</t>
+          <t>SSR103</t>
         </is>
       </c>
       <c r="B145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8030</t>
+          <t>VLINE-8029</t>
         </is>
       </c>
       <c r="C145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8153</t>
+          <t>VLINE-8152</t>
         </is>
       </c>
       <c r="D145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8415</t>
+          <t>VLINE-8413</t>
         </is>
       </c>
       <c r="E145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8721</t>
+          <t>VLINE-8720</t>
         </is>
       </c>
       <c r="F145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8788</t>
+          <t>VLINE-8787</t>
         </is>
       </c>
       <c r="G145" s="1" t="inlineStr">
         <is>
-          <t>XP2015</t>
+          <t>XP2014</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="1" t="inlineStr">
         <is>
-          <t>T363</t>
+          <t>SSR104</t>
         </is>
       </c>
       <c r="B146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8031</t>
+          <t>VLINE-8030</t>
         </is>
       </c>
       <c r="C146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8154</t>
+          <t>VLINE-8153</t>
         </is>
       </c>
       <c r="D146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8417</t>
+          <t>VLINE-8415</t>
         </is>
       </c>
       <c r="E146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8723</t>
+          <t>VLINE-8721</t>
         </is>
       </c>
       <c r="F146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8790</t>
+          <t>VLINE-8788</t>
         </is>
       </c>
       <c r="G146" s="1" t="inlineStr">
         <is>
-          <t>XP2016</t>
+          <t>XP2015</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="1" t="inlineStr">
         <is>
-          <t>T386</t>
+          <t>T363</t>
         </is>
       </c>
       <c r="B147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8032</t>
+          <t>VLINE-8031</t>
         </is>
       </c>
       <c r="C147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8155</t>
+          <t>VLINE-8154</t>
         </is>
       </c>
       <c r="D147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8418</t>
+          <t>VLINE-8417</t>
         </is>
       </c>
       <c r="E147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8725</t>
+          <t>VLINE-8723</t>
         </is>
       </c>
       <c r="F147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8792</t>
+          <t>VLINE-8790</t>
         </is>
       </c>
       <c r="G147" s="1" t="inlineStr">
         <is>
-          <t>XP2017</t>
+          <t>XP2016</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="1" t="inlineStr">
         <is>
-          <t>TDX101</t>
+          <t>T386</t>
         </is>
       </c>
       <c r="B148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8036</t>
+          <t>VLINE-8032</t>
         </is>
       </c>
       <c r="C148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8157</t>
+          <t>VLINE-8155</t>
         </is>
       </c>
       <c r="D148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8419</t>
+          <t>VLINE-8418</t>
         </is>
       </c>
       <c r="E148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8726</t>
+          <t>VLINE-8725</t>
         </is>
       </c>
       <c r="F148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8793</t>
+          <t>VLINE-8792</t>
         </is>
       </c>
       <c r="G148" s="1" t="inlineStr">
         <is>
-          <t>XP2019</t>
+          <t>XP2017</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="1" t="inlineStr">
         <is>
-          <t>TE2801</t>
+          <t>TDX101</t>
         </is>
       </c>
       <c r="B149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8038</t>
+          <t>VLINE-8036</t>
         </is>
       </c>
       <c r="C149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8158</t>
+          <t>VLINE-8157</t>
         </is>
       </c>
       <c r="D149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8420</t>
+          <t>VLINE-8419</t>
         </is>
       </c>
       <c r="E149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8727</t>
+          <t>VLINE-8726</t>
         </is>
       </c>
       <c r="F149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8794</t>
+          <t>VLINE-8793</t>
         </is>
       </c>
       <c r="G149" s="1" t="inlineStr">
         <is>
-          <t>XR552</t>
+          <t>XP2019</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="1" t="inlineStr">
         <is>
-          <t>TE2802</t>
+          <t>TE2801</t>
         </is>
       </c>
       <c r="B150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8042</t>
+          <t>VLINE-8038</t>
         </is>
       </c>
       <c r="C150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8159</t>
+          <t>VLINE-8158</t>
         </is>
       </c>
       <c r="D150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8421</t>
+          <t>VLINE-8420</t>
         </is>
       </c>
       <c r="E150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8729</t>
+          <t>VLINE-8727</t>
         </is>
       </c>
       <c r="F150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8795</t>
+          <t>VLINE-8794</t>
         </is>
       </c>
       <c r="G150" s="1" t="inlineStr">
         <is>
-          <t>XRN001</t>
+          <t>XR552</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="1" t="inlineStr">
         <is>
-          <t>TE2803</t>
+          <t>TE2802</t>
         </is>
       </c>
       <c r="B151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8051</t>
+          <t>VLINE-8042</t>
         </is>
       </c>
       <c r="C151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8160</t>
+          <t>VLINE-8159</t>
         </is>
       </c>
       <c r="D151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8422</t>
+          <t>VLINE-8421</t>
         </is>
       </c>
       <c r="E151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8730</t>
+          <t>VLINE-8729</t>
         </is>
       </c>
       <c r="F151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8796</t>
+          <t>VLINE-8795</t>
         </is>
       </c>
       <c r="G151" s="1" t="inlineStr">
         <is>
-          <t>XRN004</t>
+          <t>XRN001</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="1" t="inlineStr">
         <is>
-          <t>TE2804</t>
+          <t>TE2803</t>
         </is>
       </c>
       <c r="B152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8052</t>
+          <t>VLINE-8051</t>
         </is>
       </c>
       <c r="C152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8161</t>
+          <t>VLINE-8160</t>
         </is>
       </c>
       <c r="D152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8424</t>
+          <t>VLINE-8422</t>
         </is>
       </c>
       <c r="E152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8731</t>
+          <t>VLINE-8730</t>
         </is>
       </c>
       <c r="F152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8797</t>
+          <t>VLINE-8796</t>
         </is>
       </c>
       <c r="G152" s="1" t="inlineStr">
         <is>
-          <t>XRN005</t>
+          <t>XRN004</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="1" t="inlineStr">
         <is>
-          <t>TE2805</t>
+          <t>TE2804</t>
         </is>
       </c>
       <c r="B153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8053</t>
+          <t>VLINE-8052</t>
         </is>
       </c>
       <c r="C153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8162</t>
+          <t>VLINE-8161</t>
         </is>
       </c>
       <c r="D153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8425</t>
+          <t>VLINE-8424</t>
         </is>
       </c>
       <c r="E153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8733</t>
+          <t>VLINE-8731</t>
         </is>
       </c>
       <c r="F153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8799</t>
+          <t>VLINE-8797</t>
         </is>
       </c>
       <c r="G153" s="1" t="inlineStr">
         <is>
-          <t>XRN006</t>
+          <t>XRN005</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="1" t="inlineStr">
         <is>
-          <t>TE2806</t>
+          <t>TE2805</t>
         </is>
       </c>
       <c r="B154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8055</t>
+          <t>VLINE-8053</t>
         </is>
       </c>
       <c r="C154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8171</t>
+          <t>VLINE-8162</t>
         </is>
       </c>
       <c r="D154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8426</t>
+          <t>VLINE-8425</t>
         </is>
       </c>
       <c r="E154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8735</t>
+          <t>VLINE-8733</t>
         </is>
       </c>
       <c r="F154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8800</t>
+          <t>VLINE-8799</t>
         </is>
       </c>
       <c r="G154" s="1" t="inlineStr">
         <is>
-          <t>XRN007</t>
+          <t>XRN006</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="1" t="inlineStr">
         <is>
-          <t>TE2807</t>
+          <t>TE2806</t>
         </is>
       </c>
       <c r="B155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8056</t>
+          <t>VLINE-8055</t>
         </is>
       </c>
       <c r="C155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8172</t>
+          <t>VLINE-8171</t>
         </is>
       </c>
       <c r="D155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8427</t>
+          <t>VLINE-8426</t>
         </is>
       </c>
       <c r="E155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8736</t>
+          <t>VLINE-8735</t>
         </is>
       </c>
       <c r="F155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8801</t>
+          <t>VLINE-8800</t>
         </is>
       </c>
       <c r="G155" s="1" t="inlineStr">
         <is>
-          <t>XRN009</t>
+          <t>XRN007</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="1" t="inlineStr">
         <is>
-          <t>TE2808</t>
+          <t>TE2807</t>
         </is>
       </c>
       <c r="B156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8057</t>
+          <t>VLINE-8056</t>
         </is>
       </c>
       <c r="C156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8176</t>
+          <t>VLINE-8172</t>
         </is>
       </c>
       <c r="D156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8428</t>
+          <t>VLINE-8427</t>
         </is>
       </c>
       <c r="E156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8737</t>
+          <t>VLINE-8736</t>
         </is>
       </c>
       <c r="F156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8802</t>
+          <t>VLINE-8801</t>
         </is>
       </c>
       <c r="G156" s="1" t="inlineStr">
         <is>
-          <t>XRN011</t>
+          <t>XRN009</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="1" t="inlineStr">
         <is>
-          <t>TE2809</t>
+          <t>TE2808</t>
         </is>
       </c>
       <c r="B157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8058</t>
+          <t>VLINE-8057</t>
         </is>
       </c>
       <c r="C157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8179</t>
+          <t>VLINE-8176</t>
         </is>
       </c>
       <c r="D157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8429</t>
+          <t>VLINE-8428</t>
         </is>
       </c>
       <c r="E157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8739</t>
+          <t>VLINE-8737</t>
         </is>
       </c>
       <c r="F157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8803</t>
+          <t>VLINE-8802</t>
         </is>
       </c>
       <c r="G157" s="1" t="inlineStr">
         <is>
-          <t>XRN014</t>
+          <t>XRN011</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="1" t="inlineStr">
         <is>
-          <t>TE2810</t>
+          <t>TE2809</t>
         </is>
       </c>
       <c r="B158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8059</t>
+          <t>VLINE-8058</t>
         </is>
       </c>
       <c r="C158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8180</t>
+          <t>VLINE-8179</t>
         </is>
       </c>
       <c r="D158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8430</t>
+          <t>VLINE-8429</t>
         </is>
       </c>
       <c r="E158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8740</t>
+          <t>VLINE-8739</t>
         </is>
       </c>
       <c r="F158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8804</t>
+          <t>VLINE-8803</t>
         </is>
       </c>
       <c r="G158" s="1" t="inlineStr">
         <is>
-          <t>XRN017</t>
+          <t>XRN014</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="1" t="inlineStr">
         <is>
-          <t>TE2812</t>
+          <t>TE2810</t>
         </is>
       </c>
       <c r="B159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8061</t>
+          <t>VLINE-8059</t>
         </is>
       </c>
       <c r="C159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8181</t>
+          <t>VLINE-8180</t>
         </is>
       </c>
       <c r="D159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8431</t>
+          <t>VLINE-8430</t>
         </is>
       </c>
       <c r="E159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8741</t>
+          <t>VLINE-8740</t>
         </is>
       </c>
       <c r="F159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8805</t>
+          <t>VLINE-8804</t>
         </is>
       </c>
       <c r="G159" s="1" t="inlineStr">
         <is>
-          <t>XRN018</t>
+          <t>XRN017</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="1" t="inlineStr">
         <is>
-          <t>TE2813</t>
+          <t>TE2812</t>
         </is>
       </c>
       <c r="B160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8072</t>
+          <t>VLINE-8061</t>
         </is>
       </c>
       <c r="C160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8182</t>
+          <t>VLINE-8181</t>
         </is>
       </c>
       <c r="D160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8432</t>
+          <t>VLINE-8431</t>
         </is>
       </c>
       <c r="E160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8742</t>
+          <t>VLINE-8741</t>
         </is>
       </c>
       <c r="F160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8806</t>
+          <t>VLINE-8805</t>
         </is>
       </c>
       <c r="G160" s="1" t="inlineStr">
         <is>
-          <t>XRN020</t>
+          <t>XRN018</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="1" t="inlineStr">
         <is>
-          <t>TE2814</t>
+          <t>TE2813</t>
         </is>
       </c>
       <c r="B161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8074</t>
+          <t>VLINE-8072</t>
         </is>
       </c>
       <c r="C161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8183</t>
+          <t>VLINE-8182</t>
         </is>
       </c>
       <c r="D161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8433</t>
+          <t>VLINE-8432</t>
         </is>
       </c>
       <c r="E161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8743</t>
+          <t>VLINE-8742</t>
         </is>
       </c>
       <c r="F161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8807</t>
+          <t>VLINE-8806</t>
         </is>
       </c>
       <c r="G161" s="1" t="inlineStr">
         <is>
-          <t>XRN021</t>
+          <t>XRN020</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="1" t="inlineStr">
         <is>
-          <t>TJ096</t>
+          <t>TE2814</t>
         </is>
       </c>
       <c r="B162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8075</t>
+          <t>VLINE-8074</t>
         </is>
       </c>
       <c r="C162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8184</t>
+          <t>VLINE-8183</t>
         </is>
       </c>
       <c r="D162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8434</t>
+          <t>VLINE-8433</t>
         </is>
       </c>
       <c r="E162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8744</t>
+          <t>VLINE-8743</t>
         </is>
       </c>
       <c r="F162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8808</t>
+          <t>VLINE-8807</t>
         </is>
       </c>
       <c r="G162" s="1" t="inlineStr">
         <is>
-          <t>XRN023</t>
+          <t>XRN021</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="1" t="inlineStr">
         <is>
-          <t>TJ107</t>
+          <t>TJ096</t>
         </is>
       </c>
       <c r="B163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8076</t>
+          <t>VLINE-8075</t>
         </is>
       </c>
       <c r="C163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8185</t>
+          <t>VLINE-8184</t>
         </is>
       </c>
       <c r="D163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8435</t>
+          <t>VLINE-8434</t>
         </is>
       </c>
       <c r="E163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8745</t>
+          <t>VLINE-8744</t>
         </is>
       </c>
       <c r="F163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8809</t>
+          <t>VLINE-8808</t>
         </is>
       </c>
       <c r="G163" s="1" t="inlineStr">
         <is>
-          <t>XRN025</t>
+          <t>XRN023</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="1" t="inlineStr">
         <is>
-          <t>TT03</t>
+          <t>TJ107</t>
         </is>
       </c>
       <c r="B164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8077</t>
+          <t>VLINE-8076</t>
         </is>
       </c>
       <c r="C164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8186</t>
+          <t>VLINE-8185</t>
         </is>
       </c>
       <c r="D164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8438</t>
+          <t>VLINE-8435</t>
         </is>
       </c>
       <c r="E164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8746</t>
+          <t>VLINE-8745</t>
         </is>
       </c>
       <c r="F164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8810</t>
+          <t>VLINE-8809</t>
         </is>
       </c>
       <c r="G164" s="1" t="inlineStr">
         <is>
-          <t>XRN026</t>
+          <t>XRN025</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="1" t="inlineStr">
         <is>
-          <t>TT04</t>
+          <t>TT03</t>
         </is>
       </c>
       <c r="B165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8080</t>
+          <t>VLINE-8077</t>
         </is>
       </c>
       <c r="C165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8187</t>
+          <t>VLINE-8186</t>
         </is>
       </c>
       <c r="D165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8440</t>
+          <t>VLINE-8438</t>
         </is>
       </c>
       <c r="E165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8747</t>
+          <t>VLINE-8746</t>
         </is>
       </c>
       <c r="F165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8811</t>
+          <t>VLINE-8810</t>
         </is>
       </c>
       <c r="G165" s="1" t="inlineStr">
         <is>
-          <t>XRN027</t>
+          <t>XRN026</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="1" t="inlineStr">
         <is>
-          <t>TT05</t>
+          <t>TT04</t>
         </is>
       </c>
       <c r="B166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8081</t>
+          <t>VLINE-8080</t>
         </is>
       </c>
       <c r="C166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8188</t>
+          <t>VLINE-8187</t>
         </is>
       </c>
       <c r="D166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8441</t>
+          <t>VLINE-8440</t>
         </is>
       </c>
       <c r="E166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8748</t>
+          <t>VLINE-8747</t>
         </is>
       </c>
       <c r="F166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8812</t>
+          <t>VLINE-8811</t>
         </is>
       </c>
       <c r="G166" s="1" t="inlineStr">
         <is>
-          <t>Y163</t>
+          <t>XRN027</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="1" t="inlineStr">
         <is>
-          <t>TT07</t>
+          <t>TT05</t>
         </is>
       </c>
       <c r="B167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8084</t>
+          <t>VLINE-8081</t>
         </is>
       </c>
       <c r="C167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8189</t>
+          <t>VLINE-8188</t>
         </is>
       </c>
       <c r="D167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8442</t>
+          <t>VLINE-8441</t>
         </is>
       </c>
       <c r="E167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8749</t>
+          <t>VLINE-8748</t>
         </is>
       </c>
       <c r="F167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8813</t>
+          <t>VLINE-8812</t>
+        </is>
+      </c>
+      <c r="G167" s="1" t="inlineStr">
+        <is>
+          <t>Y163</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="1" t="inlineStr">
         <is>
-          <t>TT08</t>
+          <t>TT07</t>
         </is>
       </c>
       <c r="B168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8088</t>
+          <t>VLINE-8084</t>
         </is>
       </c>
       <c r="C168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8293</t>
+          <t>VLINE-8189</t>
         </is>
       </c>
       <c r="D168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8443</t>
+          <t>VLINE-8442</t>
         </is>
       </c>
       <c r="E168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8750</t>
+          <t>VLINE-8749</t>
         </is>
       </c>
       <c r="F168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8814</t>
+          <t>VLINE-8813</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="1" t="inlineStr">
         <is>
-          <t>TT103</t>
+          <t>TT08</t>
         </is>
       </c>
       <c r="B169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8089</t>
+          <t>VLINE-8088</t>
         </is>
       </c>
       <c r="C169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8303</t>
+          <t>VLINE-8293</t>
         </is>
       </c>
       <c r="D169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8444</t>
+          <t>VLINE-8443</t>
         </is>
       </c>
       <c r="E169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8751</t>
+          <t>VLINE-8750</t>
         </is>
       </c>
       <c r="F169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8816</t>
+          <t>VLINE-8814</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="1" t="inlineStr">
         <is>
-          <t>TT106</t>
+          <t>TT103</t>
         </is>
       </c>
       <c r="B170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8104</t>
+          <t>VLINE-8089</t>
         </is>
       </c>
       <c r="C170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8304</t>
+          <t>VLINE-8303</t>
         </is>
       </c>
       <c r="D170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8446</t>
+          <t>VLINE-8444</t>
         </is>
       </c>
       <c r="E170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8752</t>
+          <t>VLINE-8751</t>
         </is>
       </c>
       <c r="F170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8817</t>
+          <t>VLINE-8816</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update loco downloads 2026-04-05 16:33:21
</commit_message>
<xml_diff>
--- a/downloads/loco_numbers_only.xlsx
+++ b/downloads/loco_numbers_only.xlsx
@@ -2819,7 +2819,7 @@
       </c>
       <c r="H58" s="1" t="inlineStr">
         <is>
-          <t>P2505</t>
+          <t>P2504</t>
         </is>
       </c>
     </row>
@@ -2861,7 +2861,7 @@
       </c>
       <c r="H59" s="1" t="inlineStr">
         <is>
-          <t>P2506</t>
+          <t>P2505</t>
         </is>
       </c>
     </row>
@@ -2903,7 +2903,7 @@
       </c>
       <c r="H60" s="1" t="inlineStr">
         <is>
-          <t>P2507</t>
+          <t>P2506</t>
         </is>
       </c>
     </row>
@@ -2945,7 +2945,7 @@
       </c>
       <c r="H61" s="1" t="inlineStr">
         <is>
-          <t>P2508</t>
+          <t>P2507</t>
         </is>
       </c>
     </row>
@@ -2987,7 +2987,7 @@
       </c>
       <c r="H62" s="1" t="inlineStr">
         <is>
-          <t>P2509</t>
+          <t>P2508</t>
         </is>
       </c>
     </row>
@@ -3029,7 +3029,7 @@
       </c>
       <c r="H63" s="1" t="inlineStr">
         <is>
-          <t>P2510</t>
+          <t>P2509</t>
         </is>
       </c>
     </row>
@@ -3071,7 +3071,7 @@
       </c>
       <c r="H64" s="1" t="inlineStr">
         <is>
-          <t>P2511</t>
+          <t>P2510</t>
         </is>
       </c>
     </row>
@@ -3113,7 +3113,7 @@
       </c>
       <c r="H65" s="1" t="inlineStr">
         <is>
-          <t>P2513</t>
+          <t>P2511</t>
         </is>
       </c>
     </row>
@@ -3155,7 +3155,7 @@
       </c>
       <c r="H66" s="1" t="inlineStr">
         <is>
-          <t>P2514</t>
+          <t>P2513</t>
         </is>
       </c>
     </row>
@@ -3197,7 +3197,7 @@
       </c>
       <c r="H67" s="1" t="inlineStr">
         <is>
-          <t>P2515</t>
+          <t>P2514</t>
         </is>
       </c>
     </row>
@@ -3239,7 +3239,7 @@
       </c>
       <c r="H68" s="1" t="inlineStr">
         <is>
-          <t>P2516</t>
+          <t>P2515</t>
         </is>
       </c>
     </row>
@@ -3281,7 +3281,7 @@
       </c>
       <c r="H69" s="1" t="inlineStr">
         <is>
-          <t>PB1</t>
+          <t>P2516</t>
         </is>
       </c>
     </row>
@@ -3323,7 +3323,7 @@
       </c>
       <c r="H70" s="1" t="inlineStr">
         <is>
-          <t>PB2</t>
+          <t>PB1</t>
         </is>
       </c>
     </row>
@@ -3365,7 +3365,7 @@
       </c>
       <c r="H71" s="1" t="inlineStr">
         <is>
-          <t>PB4</t>
+          <t>PB2</t>
         </is>
       </c>
     </row>
@@ -3407,7 +3407,7 @@
       </c>
       <c r="H72" s="1" t="inlineStr">
         <is>
-          <t>PHC001</t>
+          <t>PB4</t>
         </is>
       </c>
     </row>
@@ -3449,7 +3449,7 @@
       </c>
       <c r="H73" s="1" t="inlineStr">
         <is>
-          <t>PHC002</t>
+          <t>PHC001</t>
         </is>
       </c>
     </row>
@@ -3491,7 +3491,7 @@
       </c>
       <c r="H74" s="1" t="inlineStr">
         <is>
-          <t>Q4001</t>
+          <t>PHC002</t>
         </is>
       </c>
     </row>
@@ -3533,7 +3533,7 @@
       </c>
       <c r="H75" s="1" t="inlineStr">
         <is>
-          <t>Q4003</t>
+          <t>Q4001</t>
         </is>
       </c>
     </row>
@@ -3575,7 +3575,7 @@
       </c>
       <c r="H76" s="1" t="inlineStr">
         <is>
-          <t>Q4004</t>
+          <t>Q4003</t>
         </is>
       </c>
     </row>
@@ -3617,7 +3617,7 @@
       </c>
       <c r="H77" s="1" t="inlineStr">
         <is>
-          <t>Q4005</t>
+          <t>Q4004</t>
         </is>
       </c>
     </row>
@@ -3659,7 +3659,7 @@
       </c>
       <c r="H78" s="1" t="inlineStr">
         <is>
-          <t>Q4006</t>
+          <t>Q4005</t>
         </is>
       </c>
     </row>
@@ -3701,7 +3701,7 @@
       </c>
       <c r="H79" s="1" t="inlineStr">
         <is>
-          <t>Q4007</t>
+          <t>Q4006</t>
         </is>
       </c>
     </row>
@@ -3743,7 +3743,7 @@
       </c>
       <c r="H80" s="1" t="inlineStr">
         <is>
-          <t>Q4009</t>
+          <t>Q4007</t>
         </is>
       </c>
     </row>
@@ -3785,7 +3785,7 @@
       </c>
       <c r="H81" s="1" t="inlineStr">
         <is>
-          <t>Q4011</t>
+          <t>Q4009</t>
         </is>
       </c>
     </row>
@@ -3827,7 +3827,7 @@
       </c>
       <c r="H82" s="1" t="inlineStr">
         <is>
-          <t>Q4012</t>
+          <t>Q4011</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
       </c>
       <c r="H83" s="1" t="inlineStr">
         <is>
-          <t>Q4013</t>
+          <t>Q4012</t>
         </is>
       </c>
     </row>
@@ -3911,7 +3911,7 @@
       </c>
       <c r="H84" s="1" t="inlineStr">
         <is>
-          <t>Q4014</t>
+          <t>Q4013</t>
         </is>
       </c>
     </row>
@@ -3953,7 +3953,7 @@
       </c>
       <c r="H85" s="1" t="inlineStr">
         <is>
-          <t>Q4015</t>
+          <t>Q4014</t>
         </is>
       </c>
     </row>
@@ -3995,7 +3995,7 @@
       </c>
       <c r="H86" s="1" t="inlineStr">
         <is>
-          <t>Q4016</t>
+          <t>Q4015</t>
         </is>
       </c>
     </row>
@@ -4037,7 +4037,7 @@
       </c>
       <c r="H87" s="1" t="inlineStr">
         <is>
-          <t>Q4017</t>
+          <t>Q4016</t>
         </is>
       </c>
     </row>
@@ -4079,7 +4079,7 @@
       </c>
       <c r="H88" s="1" t="inlineStr">
         <is>
-          <t>Q4019</t>
+          <t>Q4017</t>
         </is>
       </c>
     </row>
@@ -4121,7 +4121,7 @@
       </c>
       <c r="H89" s="1" t="inlineStr">
         <is>
-          <t>QBX003</t>
+          <t>Q4019</t>
         </is>
       </c>
     </row>
@@ -4163,7 +4163,7 @@
       </c>
       <c r="H90" s="1" t="inlineStr">
         <is>
-          <t>QBX004</t>
+          <t>QBX003</t>
         </is>
       </c>
     </row>
@@ -4205,7 +4205,7 @@
       </c>
       <c r="H91" s="1" t="inlineStr">
         <is>
-          <t>QBX005</t>
+          <t>QBX004</t>
         </is>
       </c>
     </row>
@@ -4247,7 +4247,7 @@
       </c>
       <c r="H92" s="1" t="inlineStr">
         <is>
-          <t>QBX006</t>
+          <t>QBX005</t>
         </is>
       </c>
     </row>
@@ -4289,7 +4289,7 @@
       </c>
       <c r="H93" s="1" t="inlineStr">
         <is>
-          <t>QE001</t>
+          <t>QBX006</t>
         </is>
       </c>
     </row>
@@ -4331,7 +4331,7 @@
       </c>
       <c r="H94" s="1" t="inlineStr">
         <is>
-          <t>QE002</t>
+          <t>QE001</t>
         </is>
       </c>
     </row>
@@ -4373,7 +4373,7 @@
       </c>
       <c r="H95" s="1" t="inlineStr">
         <is>
-          <t>QE003</t>
+          <t>QE002</t>
         </is>
       </c>
     </row>
@@ -4415,7 +4415,7 @@
       </c>
       <c r="H96" s="1" t="inlineStr">
         <is>
-          <t>QE004</t>
+          <t>QE003</t>
         </is>
       </c>
     </row>
@@ -4457,7 +4457,7 @@
       </c>
       <c r="H97" s="1" t="inlineStr">
         <is>
-          <t>QE006</t>
+          <t>QE004</t>
         </is>
       </c>
     </row>
@@ -4499,7 +4499,7 @@
       </c>
       <c r="H98" s="1" t="inlineStr">
         <is>
-          <t>QL001</t>
+          <t>QE006</t>
         </is>
       </c>
     </row>
@@ -4541,7 +4541,7 @@
       </c>
       <c r="H99" s="1" t="inlineStr">
         <is>
-          <t>QL002</t>
+          <t>QL001</t>
         </is>
       </c>
     </row>
@@ -4583,7 +4583,7 @@
       </c>
       <c r="H100" s="1" t="inlineStr">
         <is>
-          <t>QL004</t>
+          <t>QL002</t>
         </is>
       </c>
     </row>
@@ -4625,7 +4625,7 @@
       </c>
       <c r="H101" s="1" t="inlineStr">
         <is>
-          <t>QL007</t>
+          <t>QL004</t>
         </is>
       </c>
     </row>
@@ -4667,7 +4667,7 @@
       </c>
       <c r="H102" s="1" t="inlineStr">
         <is>
-          <t>QL008</t>
+          <t>QL007</t>
         </is>
       </c>
     </row>
@@ -4709,7 +4709,7 @@
       </c>
       <c r="H103" s="1" t="inlineStr">
         <is>
-          <t>QL010</t>
+          <t>QL008</t>
         </is>
       </c>
     </row>
@@ -4751,7 +4751,7 @@
       </c>
       <c r="H104" s="1" t="inlineStr">
         <is>
-          <t>QL011</t>
+          <t>QL010</t>
         </is>
       </c>
     </row>
@@ -4793,7 +4793,7 @@
       </c>
       <c r="H105" s="1" t="inlineStr">
         <is>
-          <t>QL014</t>
+          <t>QL011</t>
         </is>
       </c>
     </row>
@@ -4835,7 +4835,7 @@
       </c>
       <c r="H106" s="1" t="inlineStr">
         <is>
-          <t>QL018</t>
+          <t>QL014</t>
         </is>
       </c>
     </row>
@@ -4877,7 +4877,7 @@
       </c>
       <c r="H107" s="1" t="inlineStr">
         <is>
-          <t>QR1744</t>
+          <t>QL018</t>
         </is>
       </c>
     </row>
@@ -4919,7 +4919,7 @@
       </c>
       <c r="H108" s="1" t="inlineStr">
         <is>
-          <t>QR1771</t>
+          <t>QR1744</t>
         </is>
       </c>
     </row>
@@ -4961,7 +4961,7 @@
       </c>
       <c r="H109" s="1" t="inlineStr">
         <is>
-          <t>QR5404</t>
+          <t>QR1771</t>
         </is>
       </c>
     </row>
@@ -5003,7 +5003,7 @@
       </c>
       <c r="H110" s="1" t="inlineStr">
         <is>
-          <t>R711</t>
+          <t>QR5404</t>
         </is>
       </c>
     </row>
@@ -5045,7 +5045,7 @@
       </c>
       <c r="H111" s="1" t="inlineStr">
         <is>
-          <t>R766</t>
+          <t>R711</t>
         </is>
       </c>
     </row>
@@ -5087,7 +5087,7 @@
       </c>
       <c r="H112" s="1" t="inlineStr">
         <is>
-          <t>RB2353</t>
+          <t>R766</t>
         </is>
       </c>
     </row>
@@ -5129,2149 +5129,2154 @@
       </c>
       <c r="H113" s="1" t="inlineStr">
         <is>
-          <t>RCTST4</t>
+          <t>RB2353</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
         <is>
-          <t>RL301</t>
+          <t>RCTST4</t>
         </is>
       </c>
       <c r="B115" s="1" t="inlineStr">
         <is>
-          <t>TE2807</t>
+          <t>TE2806</t>
         </is>
       </c>
       <c r="C115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8056</t>
+          <t>VLINE-8055</t>
         </is>
       </c>
       <c r="D115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8172</t>
+          <t>VLINE-8171</t>
         </is>
       </c>
       <c r="E115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8426</t>
+          <t>VLINE-8425</t>
         </is>
       </c>
       <c r="F115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8735</t>
+          <t>VLINE-8733</t>
         </is>
       </c>
       <c r="G115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8800</t>
+          <t>VLINE-8799</t>
         </is>
       </c>
       <c r="H115" s="1" t="inlineStr">
         <is>
-          <t>XRN006</t>
+          <t>XRN005</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
         <is>
-          <t>RL302</t>
+          <t>RL301</t>
         </is>
       </c>
       <c r="B116" s="1" t="inlineStr">
         <is>
-          <t>TE2808</t>
+          <t>TE2807</t>
         </is>
       </c>
       <c r="C116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8057</t>
+          <t>VLINE-8056</t>
         </is>
       </c>
       <c r="D116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8176</t>
+          <t>VLINE-8172</t>
         </is>
       </c>
       <c r="E116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8427</t>
+          <t>VLINE-8426</t>
         </is>
       </c>
       <c r="F116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8736</t>
+          <t>VLINE-8735</t>
         </is>
       </c>
       <c r="G116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8801</t>
+          <t>VLINE-8800</t>
         </is>
       </c>
       <c r="H116" s="1" t="inlineStr">
         <is>
-          <t>XRN007</t>
+          <t>XRN006</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="1" t="inlineStr">
         <is>
-          <t>RL304</t>
+          <t>RL302</t>
         </is>
       </c>
       <c r="B117" s="1" t="inlineStr">
         <is>
-          <t>TE2809</t>
+          <t>TE2808</t>
         </is>
       </c>
       <c r="C117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8058</t>
+          <t>VLINE-8057</t>
         </is>
       </c>
       <c r="D117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8179</t>
+          <t>VLINE-8176</t>
         </is>
       </c>
       <c r="E117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8428</t>
+          <t>VLINE-8427</t>
         </is>
       </c>
       <c r="F117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8737</t>
+          <t>VLINE-8736</t>
         </is>
       </c>
       <c r="G117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8802</t>
+          <t>VLINE-8801</t>
         </is>
       </c>
       <c r="H117" s="1" t="inlineStr">
         <is>
-          <t>XRN009</t>
+          <t>XRN007</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
         <is>
-          <t>RL305</t>
+          <t>RL304</t>
         </is>
       </c>
       <c r="B118" s="1" t="inlineStr">
         <is>
-          <t>TE2810</t>
+          <t>TE2809</t>
         </is>
       </c>
       <c r="C118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8059</t>
+          <t>VLINE-8058</t>
         </is>
       </c>
       <c r="D118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8180</t>
+          <t>VLINE-8179</t>
         </is>
       </c>
       <c r="E118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8429</t>
+          <t>VLINE-8428</t>
         </is>
       </c>
       <c r="F118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8739</t>
+          <t>VLINE-8737</t>
         </is>
       </c>
       <c r="G118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8803</t>
+          <t>VLINE-8802</t>
         </is>
       </c>
       <c r="H118" s="1" t="inlineStr">
         <is>
-          <t>XRN011</t>
+          <t>XRN009</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
         <is>
-          <t>RL307</t>
+          <t>RL305</t>
         </is>
       </c>
       <c r="B119" s="1" t="inlineStr">
         <is>
-          <t>TE2812</t>
+          <t>TE2810</t>
         </is>
       </c>
       <c r="C119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8061</t>
+          <t>VLINE-8059</t>
         </is>
       </c>
       <c r="D119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8181</t>
+          <t>VLINE-8180</t>
         </is>
       </c>
       <c r="E119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8430</t>
+          <t>VLINE-8429</t>
         </is>
       </c>
       <c r="F119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8740</t>
+          <t>VLINE-8739</t>
         </is>
       </c>
       <c r="G119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8804</t>
+          <t>VLINE-8803</t>
         </is>
       </c>
       <c r="H119" s="1" t="inlineStr">
         <is>
-          <t>XRN014</t>
+          <t>XRN011</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="1" t="inlineStr">
         <is>
-          <t>RL309</t>
+          <t>RL307</t>
         </is>
       </c>
       <c r="B120" s="1" t="inlineStr">
         <is>
-          <t>TE2813</t>
+          <t>TE2812</t>
         </is>
       </c>
       <c r="C120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8072</t>
+          <t>VLINE-8061</t>
         </is>
       </c>
       <c r="D120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8182</t>
+          <t>VLINE-8181</t>
         </is>
       </c>
       <c r="E120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8431</t>
+          <t>VLINE-8430</t>
         </is>
       </c>
       <c r="F120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8741</t>
+          <t>VLINE-8740</t>
         </is>
       </c>
       <c r="G120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8805</t>
+          <t>VLINE-8804</t>
         </is>
       </c>
       <c r="H120" s="1" t="inlineStr">
         <is>
-          <t>XRN017</t>
+          <t>XRN014</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="1" t="inlineStr">
         <is>
-          <t>RL310</t>
+          <t>RL309</t>
         </is>
       </c>
       <c r="B121" s="1" t="inlineStr">
         <is>
-          <t>TE2814</t>
+          <t>TE2813</t>
         </is>
       </c>
       <c r="C121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8074</t>
+          <t>VLINE-8072</t>
         </is>
       </c>
       <c r="D121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8183</t>
+          <t>VLINE-8182</t>
         </is>
       </c>
       <c r="E121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8432</t>
+          <t>VLINE-8431</t>
         </is>
       </c>
       <c r="F121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8742</t>
+          <t>VLINE-8741</t>
         </is>
       </c>
       <c r="G121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8806</t>
+          <t>VLINE-8805</t>
         </is>
       </c>
       <c r="H121" s="1" t="inlineStr">
         <is>
-          <t>XRN018</t>
+          <t>XRN017</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="1" t="inlineStr">
         <is>
-          <t>S312</t>
+          <t>RL310</t>
         </is>
       </c>
       <c r="B122" s="1" t="inlineStr">
         <is>
-          <t>TJ096</t>
+          <t>TE2814</t>
         </is>
       </c>
       <c r="C122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8075</t>
+          <t>VLINE-8074</t>
         </is>
       </c>
       <c r="D122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8184</t>
+          <t>VLINE-8183</t>
         </is>
       </c>
       <c r="E122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8433</t>
+          <t>VLINE-8432</t>
         </is>
       </c>
       <c r="F122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8743</t>
+          <t>VLINE-8742</t>
         </is>
       </c>
       <c r="G122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8807</t>
+          <t>VLINE-8806</t>
         </is>
       </c>
       <c r="H122" s="1" t="inlineStr">
         <is>
-          <t>XRN020</t>
+          <t>XRN018</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="1" t="inlineStr">
         <is>
-          <t>S317</t>
+          <t>S312</t>
         </is>
       </c>
       <c r="B123" s="1" t="inlineStr">
         <is>
-          <t>TJ107</t>
+          <t>TJ096</t>
         </is>
       </c>
       <c r="C123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8076</t>
+          <t>VLINE-8075</t>
         </is>
       </c>
       <c r="D123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8185</t>
+          <t>VLINE-8184</t>
         </is>
       </c>
       <c r="E123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8434</t>
+          <t>VLINE-8433</t>
         </is>
       </c>
       <c r="F123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8744</t>
+          <t>VLINE-8743</t>
         </is>
       </c>
       <c r="G123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8808</t>
+          <t>VLINE-8807</t>
         </is>
       </c>
       <c r="H123" s="1" t="inlineStr">
         <is>
-          <t>XRN021</t>
+          <t>XRN020</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="1" t="inlineStr">
         <is>
-          <t>S3301</t>
+          <t>S317</t>
         </is>
       </c>
       <c r="B124" s="1" t="inlineStr">
         <is>
-          <t>TT03</t>
+          <t>TJ107</t>
         </is>
       </c>
       <c r="C124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8077</t>
+          <t>VLINE-8076</t>
         </is>
       </c>
       <c r="D124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8186</t>
+          <t>VLINE-8185</t>
         </is>
       </c>
       <c r="E124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8435</t>
+          <t>VLINE-8434</t>
         </is>
       </c>
       <c r="F124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8745</t>
+          <t>VLINE-8744</t>
         </is>
       </c>
       <c r="G124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8809</t>
+          <t>VLINE-8808</t>
         </is>
       </c>
       <c r="H124" s="1" t="inlineStr">
         <is>
-          <t>XRN023</t>
+          <t>XRN021</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="1" t="inlineStr">
         <is>
-          <t>S3302</t>
+          <t>S3301</t>
         </is>
       </c>
       <c r="B125" s="1" t="inlineStr">
         <is>
-          <t>TT04</t>
+          <t>TT03</t>
         </is>
       </c>
       <c r="C125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8080</t>
+          <t>VLINE-8077</t>
         </is>
       </c>
       <c r="D125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8187</t>
+          <t>VLINE-8186</t>
         </is>
       </c>
       <c r="E125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8438</t>
+          <t>VLINE-8435</t>
         </is>
       </c>
       <c r="F125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8746</t>
+          <t>VLINE-8745</t>
         </is>
       </c>
       <c r="G125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8810</t>
+          <t>VLINE-8809</t>
         </is>
       </c>
       <c r="H125" s="1" t="inlineStr">
         <is>
-          <t>XRN025</t>
+          <t>XRN023</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="1" t="inlineStr">
         <is>
-          <t>S3304</t>
+          <t>S3302</t>
         </is>
       </c>
       <c r="B126" s="1" t="inlineStr">
         <is>
-          <t>TT05</t>
+          <t>TT04</t>
         </is>
       </c>
       <c r="C126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8081</t>
+          <t>VLINE-8080</t>
         </is>
       </c>
       <c r="D126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8188</t>
+          <t>VLINE-8187</t>
         </is>
       </c>
       <c r="E126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8440</t>
+          <t>VLINE-8438</t>
         </is>
       </c>
       <c r="F126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8747</t>
+          <t>VLINE-8746</t>
         </is>
       </c>
       <c r="G126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8811</t>
+          <t>VLINE-8810</t>
         </is>
       </c>
       <c r="H126" s="1" t="inlineStr">
         <is>
-          <t>XRN026</t>
+          <t>XRN025</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
         <is>
-          <t>S3305</t>
+          <t>S3304</t>
         </is>
       </c>
       <c r="B127" s="1" t="inlineStr">
         <is>
-          <t>TT07</t>
+          <t>TT05</t>
         </is>
       </c>
       <c r="C127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8084</t>
+          <t>VLINE-8081</t>
         </is>
       </c>
       <c r="D127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8189</t>
+          <t>VLINE-8188</t>
         </is>
       </c>
       <c r="E127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8441</t>
+          <t>VLINE-8440</t>
         </is>
       </c>
       <c r="F127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8748</t>
+          <t>VLINE-8747</t>
         </is>
       </c>
       <c r="G127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8812</t>
+          <t>VLINE-8811</t>
         </is>
       </c>
       <c r="H127" s="1" t="inlineStr">
         <is>
-          <t>XRN027</t>
+          <t>XRN026</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
         <is>
-          <t>S3306</t>
+          <t>S3305</t>
         </is>
       </c>
       <c r="B128" s="1" t="inlineStr">
         <is>
-          <t>TT08</t>
+          <t>TT07</t>
         </is>
       </c>
       <c r="C128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8088</t>
+          <t>VLINE-8084</t>
         </is>
       </c>
       <c r="D128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8291</t>
+          <t>VLINE-8189</t>
         </is>
       </c>
       <c r="E128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8442</t>
+          <t>VLINE-8441</t>
         </is>
       </c>
       <c r="F128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8749</t>
+          <t>VLINE-8748</t>
         </is>
       </c>
       <c r="G128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8813</t>
+          <t>VLINE-8812</t>
         </is>
       </c>
       <c r="H128" s="1" t="inlineStr">
         <is>
-          <t>Y163</t>
+          <t>XRN027</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
         <is>
-          <t>S3307</t>
+          <t>S3306</t>
         </is>
       </c>
       <c r="B129" s="1" t="inlineStr">
         <is>
-          <t>TT103</t>
+          <t>TT08</t>
         </is>
       </c>
       <c r="C129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8089</t>
+          <t>VLINE-8088</t>
         </is>
       </c>
       <c r="D129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8293</t>
+          <t>VLINE-8291</t>
         </is>
       </c>
       <c r="E129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8443</t>
+          <t>VLINE-8442</t>
         </is>
       </c>
       <c r="F129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8750</t>
+          <t>VLINE-8749</t>
         </is>
       </c>
       <c r="G129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8814</t>
+          <t>VLINE-8813</t>
+        </is>
+      </c>
+      <c r="H129" s="1" t="inlineStr">
+        <is>
+          <t>Y163</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="1" t="inlineStr">
         <is>
-          <t>S3309</t>
+          <t>S3307</t>
         </is>
       </c>
       <c r="B130" s="1" t="inlineStr">
         <is>
-          <t>TT106</t>
+          <t>TT103</t>
         </is>
       </c>
       <c r="C130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8104</t>
+          <t>VLINE-8089</t>
         </is>
       </c>
       <c r="D130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8303</t>
+          <t>VLINE-8293</t>
         </is>
       </c>
       <c r="E130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8444</t>
+          <t>VLINE-8443</t>
         </is>
       </c>
       <c r="F130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8751</t>
+          <t>VLINE-8750</t>
         </is>
       </c>
       <c r="G130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8816</t>
+          <t>VLINE-8814</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="1" t="inlineStr">
         <is>
-          <t>S3310</t>
+          <t>S3309</t>
         </is>
       </c>
       <c r="B131" s="1" t="inlineStr">
         <is>
-          <t>TT107</t>
+          <t>TT106</t>
         </is>
       </c>
       <c r="C131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8107</t>
+          <t>VLINE-8104</t>
         </is>
       </c>
       <c r="D131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8304</t>
+          <t>VLINE-8303</t>
         </is>
       </c>
       <c r="E131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8446</t>
+          <t>VLINE-8444</t>
         </is>
       </c>
       <c r="F131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8752</t>
+          <t>VLINE-8751</t>
         </is>
       </c>
       <c r="G131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8817</t>
+          <t>VLINE-8816</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="1" t="inlineStr">
         <is>
-          <t>S7001</t>
+          <t>S3310</t>
         </is>
       </c>
       <c r="B132" s="1" t="inlineStr">
         <is>
-          <t>TT108</t>
+          <t>TT107</t>
         </is>
       </c>
       <c r="C132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8110</t>
+          <t>VLINE-8107</t>
         </is>
       </c>
       <c r="D132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8306</t>
+          <t>VLINE-8304</t>
         </is>
       </c>
       <c r="E132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8447</t>
+          <t>VLINE-8446</t>
         </is>
       </c>
       <c r="F132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8753</t>
+          <t>VLINE-8752</t>
         </is>
       </c>
       <c r="G132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8818</t>
+          <t>VLINE-8817</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="1" t="inlineStr">
         <is>
-          <t>S7002</t>
+          <t>S7001</t>
         </is>
       </c>
       <c r="B133" s="1" t="inlineStr">
         <is>
-          <t>TT110</t>
+          <t>TT108</t>
         </is>
       </c>
       <c r="C133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8111</t>
+          <t>VLINE-8110</t>
         </is>
       </c>
       <c r="D133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8311</t>
+          <t>VLINE-8306</t>
         </is>
       </c>
       <c r="E133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8449</t>
+          <t>VLINE-8447</t>
         </is>
       </c>
       <c r="F133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8754</t>
+          <t>VLINE-8753</t>
         </is>
       </c>
       <c r="G133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8819</t>
+          <t>VLINE-8818</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="1" t="inlineStr">
         <is>
-          <t>S7003</t>
+          <t>S7002</t>
         </is>
       </c>
       <c r="B134" s="1" t="inlineStr">
         <is>
-          <t>TT113</t>
+          <t>TT110</t>
         </is>
       </c>
       <c r="C134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8113</t>
+          <t>VLINE-8111</t>
         </is>
       </c>
       <c r="D134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8313</t>
+          <t>VLINE-8311</t>
         </is>
       </c>
       <c r="E134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8450</t>
+          <t>VLINE-8449</t>
         </is>
       </c>
       <c r="F134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8755</t>
+          <t>VLINE-8754</t>
         </is>
       </c>
       <c r="G134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8822</t>
+          <t>VLINE-8819</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="1" t="inlineStr">
         <is>
-          <t>S7004</t>
+          <t>S7003</t>
         </is>
       </c>
       <c r="B135" s="1" t="inlineStr">
         <is>
-          <t>TT114</t>
+          <t>TT113</t>
         </is>
       </c>
       <c r="C135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8114</t>
+          <t>VLINE-8113</t>
         </is>
       </c>
       <c r="D135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8314</t>
+          <t>VLINE-8313</t>
         </is>
       </c>
       <c r="E135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8451</t>
+          <t>VLINE-8450</t>
         </is>
       </c>
       <c r="F135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8756</t>
+          <t>VLINE-8755</t>
         </is>
       </c>
       <c r="G135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8860</t>
+          <t>VLINE-8822</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="1" t="inlineStr">
         <is>
-          <t>S7005</t>
+          <t>S7004</t>
         </is>
       </c>
       <c r="B136" s="1" t="inlineStr">
         <is>
-          <t>TT115</t>
+          <t>TT114</t>
         </is>
       </c>
       <c r="C136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8115</t>
+          <t>VLINE-8114</t>
         </is>
       </c>
       <c r="D136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8316</t>
+          <t>VLINE-8314</t>
         </is>
       </c>
       <c r="E136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8452</t>
+          <t>VLINE-8451</t>
         </is>
       </c>
       <c r="F136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8757</t>
+          <t>VLINE-8756</t>
         </is>
       </c>
       <c r="G136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8861</t>
+          <t>VLINE-8860</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="1" t="inlineStr">
         <is>
-          <t>S7006</t>
+          <t>S7005</t>
         </is>
       </c>
       <c r="B137" s="1" t="inlineStr">
         <is>
-          <t>TT116</t>
+          <t>TT115</t>
         </is>
       </c>
       <c r="C137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8119</t>
+          <t>VLINE-8115</t>
         </is>
       </c>
       <c r="D137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8318</t>
+          <t>VLINE-8316</t>
         </is>
       </c>
       <c r="E137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8453</t>
+          <t>VLINE-8452</t>
         </is>
       </c>
       <c r="F137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8758</t>
+          <t>VLINE-8757</t>
         </is>
       </c>
       <c r="G137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8862</t>
+          <t>VLINE-8861</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="1" t="inlineStr">
         <is>
-          <t>S7007</t>
+          <t>S7006</t>
         </is>
       </c>
       <c r="B138" s="1" t="inlineStr">
         <is>
-          <t>TT117</t>
+          <t>TT116</t>
         </is>
       </c>
       <c r="C138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8120</t>
+          <t>VLINE-8119</t>
         </is>
       </c>
       <c r="D138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8321</t>
+          <t>VLINE-8318</t>
         </is>
       </c>
       <c r="E138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8454</t>
+          <t>VLINE-8453</t>
         </is>
       </c>
       <c r="F138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8759</t>
+          <t>VLINE-8758</t>
         </is>
       </c>
       <c r="G138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8863</t>
+          <t>VLINE-8862</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="1" t="inlineStr">
         <is>
-          <t>S7008</t>
+          <t>S7007</t>
         </is>
       </c>
       <c r="B139" s="1" t="inlineStr">
         <is>
-          <t>TT122</t>
+          <t>TT117</t>
         </is>
       </c>
       <c r="C139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8121</t>
+          <t>VLINE-8120</t>
         </is>
       </c>
       <c r="D139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8323</t>
+          <t>VLINE-8321</t>
         </is>
       </c>
       <c r="E139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8455</t>
+          <t>VLINE-8454</t>
         </is>
       </c>
       <c r="F139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8760</t>
+          <t>VLINE-8759</t>
         </is>
       </c>
       <c r="G139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8864</t>
+          <t>VLINE-8863</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="1" t="inlineStr">
         <is>
-          <t>S7012</t>
+          <t>S7008</t>
         </is>
       </c>
       <c r="B140" s="1" t="inlineStr">
         <is>
-          <t>TT127</t>
+          <t>TT122</t>
         </is>
       </c>
       <c r="C140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8123</t>
+          <t>VLINE-8121</t>
         </is>
       </c>
       <c r="D140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8324</t>
+          <t>VLINE-8323</t>
         </is>
       </c>
       <c r="E140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8456</t>
+          <t>VLINE-8455</t>
         </is>
       </c>
       <c r="F140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8761</t>
+          <t>VLINE-8760</t>
         </is>
       </c>
       <c r="G140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8865</t>
+          <t>VLINE-8864</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="1" t="inlineStr">
         <is>
-          <t>S7013</t>
+          <t>S7012</t>
         </is>
       </c>
       <c r="B141" s="1" t="inlineStr">
         <is>
-          <t>TT128</t>
+          <t>TT127</t>
         </is>
       </c>
       <c r="C141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8124</t>
+          <t>VLINE-8123</t>
         </is>
       </c>
       <c r="D141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8325</t>
+          <t>VLINE-8324</t>
         </is>
       </c>
       <c r="E141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8457</t>
+          <t>VLINE-8456</t>
         </is>
       </c>
       <c r="F141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8762</t>
+          <t>VLINE-8761</t>
         </is>
       </c>
       <c r="G141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8866</t>
+          <t>VLINE-8865</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="1" t="inlineStr">
         <is>
-          <t>S7014</t>
+          <t>S7013</t>
         </is>
       </c>
       <c r="B142" s="1" t="inlineStr">
         <is>
-          <t>TT130</t>
+          <t>TT128</t>
         </is>
       </c>
       <c r="C142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8126</t>
+          <t>VLINE-8124</t>
         </is>
       </c>
       <c r="D142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8328</t>
+          <t>VLINE-8325</t>
         </is>
       </c>
       <c r="E142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8460</t>
+          <t>VLINE-8457</t>
         </is>
       </c>
       <c r="F142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8763</t>
+          <t>VLINE-8762</t>
         </is>
       </c>
       <c r="G142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8867</t>
+          <t>VLINE-8866</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="1" t="inlineStr">
         <is>
-          <t>S7015</t>
+          <t>S7014</t>
         </is>
       </c>
       <c r="B143" s="1" t="inlineStr">
         <is>
-          <t>TT131</t>
+          <t>TT130</t>
         </is>
       </c>
       <c r="C143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8127</t>
+          <t>VLINE-8126</t>
         </is>
       </c>
       <c r="D143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8329</t>
+          <t>VLINE-8328</t>
         </is>
       </c>
       <c r="E143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8461</t>
+          <t>VLINE-8460</t>
         </is>
       </c>
       <c r="F143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8765</t>
+          <t>VLINE-8763</t>
         </is>
       </c>
       <c r="G143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8868</t>
+          <t>VLINE-8867</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="1" t="inlineStr">
         <is>
-          <t>S7017</t>
+          <t>S7015</t>
         </is>
       </c>
       <c r="B144" s="1" t="inlineStr">
         <is>
-          <t>TT202</t>
+          <t>TT131</t>
         </is>
       </c>
       <c r="C144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8128</t>
+          <t>VLINE-8127</t>
         </is>
       </c>
       <c r="D144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8332</t>
+          <t>VLINE-8329</t>
         </is>
       </c>
       <c r="E144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8464</t>
+          <t>VLINE-8461</t>
         </is>
       </c>
       <c r="F144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8766</t>
+          <t>VLINE-8765</t>
         </is>
       </c>
       <c r="G144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8869</t>
+          <t>VLINE-8868</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="1" t="inlineStr">
         <is>
-          <t>S7018</t>
+          <t>S7017</t>
         </is>
       </c>
       <c r="B145" s="1" t="inlineStr">
         <is>
-          <t>TT206</t>
+          <t>TT202</t>
         </is>
       </c>
       <c r="C145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8129</t>
+          <t>VLINE-8128</t>
         </is>
       </c>
       <c r="D145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8336</t>
+          <t>VLINE-8332</t>
         </is>
       </c>
       <c r="E145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8465</t>
+          <t>VLINE-8464</t>
         </is>
       </c>
       <c r="F145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8767</t>
+          <t>VLINE-8766</t>
         </is>
       </c>
       <c r="G145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8890</t>
+          <t>VLINE-8869</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="1" t="inlineStr">
         <is>
-          <t>S7020</t>
+          <t>S7018</t>
         </is>
       </c>
       <c r="B146" s="1" t="inlineStr">
         <is>
-          <t>VL352</t>
+          <t>TT206</t>
         </is>
       </c>
       <c r="C146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8131</t>
+          <t>VLINE-8129</t>
         </is>
       </c>
       <c r="D146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8337</t>
+          <t>VLINE-8336</t>
         </is>
       </c>
       <c r="E146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8468</t>
+          <t>VLINE-8465</t>
         </is>
       </c>
       <c r="F146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8768</t>
+          <t>VLINE-8767</t>
         </is>
       </c>
       <c r="G146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8891</t>
+          <t>VLINE-8890</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="1" t="inlineStr">
         <is>
-          <t>S7022</t>
+          <t>S7020</t>
         </is>
       </c>
       <c r="B147" s="1" t="inlineStr">
         <is>
-          <t>VL353</t>
+          <t>VL352</t>
         </is>
       </c>
       <c r="C147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8132</t>
+          <t>VLINE-8131</t>
         </is>
       </c>
       <c r="D147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8338</t>
+          <t>VLINE-8337</t>
         </is>
       </c>
       <c r="E147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8469</t>
+          <t>VLINE-8468</t>
         </is>
       </c>
       <c r="F147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8769</t>
+          <t>VLINE-8768</t>
         </is>
       </c>
       <c r="G147" s="1" t="inlineStr">
         <is>
-          <t>WH001</t>
+          <t>VLINE-8891</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="1" t="inlineStr">
         <is>
-          <t>SCT001</t>
+          <t>S7022</t>
         </is>
       </c>
       <c r="B148" s="1" t="inlineStr">
         <is>
-          <t>VL357</t>
+          <t>VL353</t>
         </is>
       </c>
       <c r="C148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8133</t>
+          <t>VLINE-8132</t>
         </is>
       </c>
       <c r="D148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8339</t>
+          <t>VLINE-8338</t>
         </is>
       </c>
       <c r="E148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8605</t>
+          <t>VLINE-8469</t>
         </is>
       </c>
       <c r="F148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8770</t>
+          <t>VLINE-8769</t>
         </is>
       </c>
       <c r="G148" s="1" t="inlineStr">
         <is>
-          <t>WH003</t>
+          <t>WH001</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="1" t="inlineStr">
         <is>
-          <t>SCT002</t>
+          <t>SCT001</t>
         </is>
       </c>
       <c r="B149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8004</t>
+          <t>VL357</t>
         </is>
       </c>
       <c r="C149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8134</t>
+          <t>VLINE-8133</t>
         </is>
       </c>
       <c r="D149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8362</t>
+          <t>VLINE-8339</t>
         </is>
       </c>
       <c r="E149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8610</t>
+          <t>VLINE-8605</t>
         </is>
       </c>
       <c r="F149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8772</t>
+          <t>VLINE-8770</t>
         </is>
       </c>
       <c r="G149" s="1" t="inlineStr">
         <is>
-          <t>WL02</t>
+          <t>WH003</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="1" t="inlineStr">
         <is>
-          <t>SCT006</t>
+          <t>SCT002</t>
         </is>
       </c>
       <c r="B150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8007</t>
+          <t>VLINE-8004</t>
         </is>
       </c>
       <c r="C150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8136</t>
+          <t>VLINE-8134</t>
         </is>
       </c>
       <c r="D150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8363</t>
+          <t>VLINE-8362</t>
         </is>
       </c>
       <c r="E150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8612</t>
+          <t>VLINE-8610</t>
         </is>
       </c>
       <c r="F150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8773</t>
+          <t>VLINE-8772</t>
         </is>
       </c>
       <c r="G150" s="1" t="inlineStr">
         <is>
-          <t>X12-X14</t>
+          <t>WL02</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="1" t="inlineStr">
         <is>
-          <t>SCT007</t>
+          <t>SCT006</t>
         </is>
       </c>
       <c r="B151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8011</t>
+          <t>VLINE-8007</t>
         </is>
       </c>
       <c r="C151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8137</t>
+          <t>VLINE-8136</t>
         </is>
       </c>
       <c r="D151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8365</t>
+          <t>VLINE-8363</t>
         </is>
       </c>
       <c r="E151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8615</t>
+          <t>VLINE-8612</t>
         </is>
       </c>
       <c r="F151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8774</t>
+          <t>VLINE-8773</t>
         </is>
       </c>
       <c r="G151" s="1" t="inlineStr">
         <is>
-          <t>X31</t>
+          <t>X12-X14</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="1" t="inlineStr">
         <is>
-          <t>SCT009</t>
+          <t>SCT007</t>
         </is>
       </c>
       <c r="B152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8013</t>
+          <t>VLINE-8011</t>
         </is>
       </c>
       <c r="C152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8140</t>
+          <t>VLINE-8137</t>
         </is>
       </c>
       <c r="D152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8366</t>
+          <t>VLINE-8365</t>
         </is>
       </c>
       <c r="E152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8617</t>
+          <t>VLINE-8615</t>
         </is>
       </c>
       <c r="F152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8776</t>
+          <t>VLINE-8774</t>
         </is>
       </c>
       <c r="G152" s="1" t="inlineStr">
         <is>
-          <t>XP2000</t>
+          <t>X31</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="1" t="inlineStr">
         <is>
-          <t>SCT011</t>
+          <t>SCT009</t>
         </is>
       </c>
       <c r="B153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8019</t>
+          <t>VLINE-8013</t>
         </is>
       </c>
       <c r="C153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8141</t>
+          <t>VLINE-8140</t>
         </is>
       </c>
       <c r="D153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8368</t>
+          <t>VLINE-8366</t>
         </is>
       </c>
       <c r="E153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8620</t>
+          <t>VLINE-8617</t>
         </is>
       </c>
       <c r="F153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8778</t>
+          <t>VLINE-8776</t>
         </is>
       </c>
       <c r="G153" s="1" t="inlineStr">
         <is>
-          <t>XP2003</t>
+          <t>XP2000</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="1" t="inlineStr">
         <is>
-          <t>SCT013</t>
+          <t>SCT011</t>
         </is>
       </c>
       <c r="B154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8020</t>
+          <t>VLINE-8019</t>
         </is>
       </c>
       <c r="C154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8142</t>
+          <t>VLINE-8141</t>
         </is>
       </c>
       <c r="D154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8369</t>
+          <t>VLINE-8368</t>
         </is>
       </c>
       <c r="E154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8625</t>
+          <t>VLINE-8620</t>
         </is>
       </c>
       <c r="F154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8779</t>
+          <t>VLINE-8778</t>
         </is>
       </c>
       <c r="G154" s="1" t="inlineStr">
         <is>
-          <t>XP2004</t>
+          <t>XP2003</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="1" t="inlineStr">
         <is>
-          <t>SCT014</t>
+          <t>SCT013</t>
         </is>
       </c>
       <c r="B155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8023</t>
+          <t>VLINE-8020</t>
         </is>
       </c>
       <c r="C155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8144</t>
+          <t>VLINE-8142</t>
         </is>
       </c>
       <c r="D155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8403</t>
+          <t>VLINE-8369</t>
         </is>
       </c>
       <c r="E155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8630</t>
+          <t>VLINE-8625</t>
         </is>
       </c>
       <c r="F155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8780</t>
+          <t>VLINE-8779</t>
         </is>
       </c>
       <c r="G155" s="1" t="inlineStr">
         <is>
-          <t>XP2005</t>
+          <t>XP2004</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="1" t="inlineStr">
         <is>
-          <t>SCT015</t>
+          <t>SCT014</t>
         </is>
       </c>
       <c r="B156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8025</t>
+          <t>VLINE-8023</t>
         </is>
       </c>
       <c r="C156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8145</t>
+          <t>VLINE-8144</t>
         </is>
       </c>
       <c r="D156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8404</t>
+          <t>VLINE-8403</t>
         </is>
       </c>
       <c r="E156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8671</t>
+          <t>VLINE-8630</t>
         </is>
       </c>
       <c r="F156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8781</t>
+          <t>VLINE-8780</t>
         </is>
       </c>
       <c r="G156" s="1" t="inlineStr">
         <is>
-          <t>XP2007</t>
+          <t>XP2005</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="1" t="inlineStr">
         <is>
-          <t>SO2</t>
+          <t>SCT015</t>
         </is>
       </c>
       <c r="B157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8026</t>
+          <t>VLINE-8025</t>
         </is>
       </c>
       <c r="C157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8148</t>
+          <t>VLINE-8145</t>
         </is>
       </c>
       <c r="D157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8406</t>
+          <t>VLINE-8404</t>
         </is>
       </c>
       <c r="E157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8706</t>
+          <t>VLINE-8671</t>
         </is>
       </c>
       <c r="F157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8782</t>
+          <t>VLINE-8781</t>
         </is>
       </c>
       <c r="G157" s="1" t="inlineStr">
         <is>
-          <t>XP2008</t>
+          <t>XP2007</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="1" t="inlineStr">
         <is>
-          <t>SSR101</t>
+          <t>SO2</t>
         </is>
       </c>
       <c r="B158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8027</t>
+          <t>VLINE-8026</t>
         </is>
       </c>
       <c r="C158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8150</t>
+          <t>VLINE-8148</t>
         </is>
       </c>
       <c r="D158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8408</t>
+          <t>VLINE-8406</t>
         </is>
       </c>
       <c r="E158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8711</t>
+          <t>VLINE-8706</t>
         </is>
       </c>
       <c r="F158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8783</t>
+          <t>VLINE-8782</t>
         </is>
       </c>
       <c r="G158" s="1" t="inlineStr">
         <is>
-          <t>XP2010</t>
+          <t>XP2008</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="1" t="inlineStr">
         <is>
-          <t>SSR102</t>
+          <t>SSR101</t>
         </is>
       </c>
       <c r="B159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8028</t>
+          <t>VLINE-8027</t>
         </is>
       </c>
       <c r="C159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8151</t>
+          <t>VLINE-8150</t>
         </is>
       </c>
       <c r="D159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8410</t>
+          <t>VLINE-8408</t>
         </is>
       </c>
       <c r="E159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8714</t>
+          <t>VLINE-8711</t>
         </is>
       </c>
       <c r="F159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8784</t>
+          <t>VLINE-8783</t>
         </is>
       </c>
       <c r="G159" s="1" t="inlineStr">
         <is>
-          <t>XP2011</t>
+          <t>XP2010</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="1" t="inlineStr">
         <is>
-          <t>SSR103</t>
+          <t>SSR102</t>
         </is>
       </c>
       <c r="B160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8029</t>
+          <t>VLINE-8028</t>
         </is>
       </c>
       <c r="C160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8152</t>
+          <t>VLINE-8151</t>
         </is>
       </c>
       <c r="D160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8411</t>
+          <t>VLINE-8410</t>
         </is>
       </c>
       <c r="E160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8717</t>
+          <t>VLINE-8714</t>
         </is>
       </c>
       <c r="F160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8786</t>
+          <t>VLINE-8784</t>
         </is>
       </c>
       <c r="G160" s="1" t="inlineStr">
         <is>
-          <t>XP2012</t>
+          <t>XP2011</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="1" t="inlineStr">
         <is>
-          <t>SSR104</t>
+          <t>SSR103</t>
         </is>
       </c>
       <c r="B161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8030</t>
+          <t>VLINE-8029</t>
         </is>
       </c>
       <c r="C161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8153</t>
+          <t>VLINE-8152</t>
         </is>
       </c>
       <c r="D161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8413</t>
+          <t>VLINE-8411</t>
         </is>
       </c>
       <c r="E161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8720</t>
+          <t>VLINE-8717</t>
         </is>
       </c>
       <c r="F161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8787</t>
+          <t>VLINE-8786</t>
         </is>
       </c>
       <c r="G161" s="1" t="inlineStr">
         <is>
-          <t>XP2013</t>
+          <t>XP2012</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="1" t="inlineStr">
         <is>
-          <t>T363</t>
+          <t>SSR104</t>
         </is>
       </c>
       <c r="B162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8031</t>
+          <t>VLINE-8030</t>
         </is>
       </c>
       <c r="C162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8154</t>
+          <t>VLINE-8153</t>
         </is>
       </c>
       <c r="D162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8415</t>
+          <t>VLINE-8413</t>
         </is>
       </c>
       <c r="E162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8721</t>
+          <t>VLINE-8720</t>
         </is>
       </c>
       <c r="F162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8788</t>
+          <t>VLINE-8787</t>
         </is>
       </c>
       <c r="G162" s="1" t="inlineStr">
         <is>
-          <t>XP2014</t>
+          <t>XP2013</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="1" t="inlineStr">
         <is>
-          <t>T386</t>
+          <t>T363</t>
         </is>
       </c>
       <c r="B163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8032</t>
+          <t>VLINE-8031</t>
         </is>
       </c>
       <c r="C163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8155</t>
+          <t>VLINE-8154</t>
         </is>
       </c>
       <c r="D163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8417</t>
+          <t>VLINE-8415</t>
         </is>
       </c>
       <c r="E163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8723</t>
+          <t>VLINE-8721</t>
         </is>
       </c>
       <c r="F163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8790</t>
+          <t>VLINE-8788</t>
         </is>
       </c>
       <c r="G163" s="1" t="inlineStr">
         <is>
-          <t>XP2015</t>
+          <t>XP2014</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="1" t="inlineStr">
         <is>
-          <t>TDX101</t>
+          <t>T386</t>
         </is>
       </c>
       <c r="B164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8036</t>
+          <t>VLINE-8032</t>
         </is>
       </c>
       <c r="C164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8157</t>
+          <t>VLINE-8155</t>
         </is>
       </c>
       <c r="D164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8418</t>
+          <t>VLINE-8417</t>
         </is>
       </c>
       <c r="E164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8725</t>
+          <t>VLINE-8723</t>
         </is>
       </c>
       <c r="F164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8792</t>
+          <t>VLINE-8790</t>
         </is>
       </c>
       <c r="G164" s="1" t="inlineStr">
         <is>
-          <t>XP2016</t>
+          <t>XP2015</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="1" t="inlineStr">
         <is>
-          <t>TE2801</t>
+          <t>TDX101</t>
         </is>
       </c>
       <c r="B165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8038</t>
+          <t>VLINE-8036</t>
         </is>
       </c>
       <c r="C165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8158</t>
+          <t>VLINE-8157</t>
         </is>
       </c>
       <c r="D165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8419</t>
+          <t>VLINE-8418</t>
         </is>
       </c>
       <c r="E165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8726</t>
+          <t>VLINE-8725</t>
         </is>
       </c>
       <c r="F165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8793</t>
+          <t>VLINE-8792</t>
         </is>
       </c>
       <c r="G165" s="1" t="inlineStr">
         <is>
-          <t>XP2017</t>
+          <t>XP2016</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="1" t="inlineStr">
         <is>
-          <t>TE2802</t>
+          <t>TE2801</t>
         </is>
       </c>
       <c r="B166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8042</t>
+          <t>VLINE-8038</t>
         </is>
       </c>
       <c r="C166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8159</t>
+          <t>VLINE-8158</t>
         </is>
       </c>
       <c r="D166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8420</t>
+          <t>VLINE-8419</t>
         </is>
       </c>
       <c r="E166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8727</t>
+          <t>VLINE-8726</t>
         </is>
       </c>
       <c r="F166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8794</t>
+          <t>VLINE-8793</t>
         </is>
       </c>
       <c r="G166" s="1" t="inlineStr">
         <is>
-          <t>XP2019</t>
+          <t>XP2017</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="1" t="inlineStr">
         <is>
-          <t>TE2803</t>
+          <t>TE2802</t>
         </is>
       </c>
       <c r="B167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8051</t>
+          <t>VLINE-8042</t>
         </is>
       </c>
       <c r="C167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8160</t>
+          <t>VLINE-8159</t>
         </is>
       </c>
       <c r="D167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8421</t>
+          <t>VLINE-8420</t>
         </is>
       </c>
       <c r="E167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8729</t>
+          <t>VLINE-8727</t>
         </is>
       </c>
       <c r="F167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8795</t>
+          <t>VLINE-8794</t>
         </is>
       </c>
       <c r="G167" s="1" t="inlineStr">
         <is>
-          <t>XR552</t>
+          <t>XP2019</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="1" t="inlineStr">
         <is>
-          <t>TE2804</t>
+          <t>TE2803</t>
         </is>
       </c>
       <c r="B168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8052</t>
+          <t>VLINE-8051</t>
         </is>
       </c>
       <c r="C168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8161</t>
+          <t>VLINE-8160</t>
         </is>
       </c>
       <c r="D168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8422</t>
+          <t>VLINE-8421</t>
         </is>
       </c>
       <c r="E168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8730</t>
+          <t>VLINE-8729</t>
         </is>
       </c>
       <c r="F168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8796</t>
+          <t>VLINE-8795</t>
         </is>
       </c>
       <c r="G168" s="1" t="inlineStr">
         <is>
-          <t>XRN001</t>
+          <t>XR552</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="1" t="inlineStr">
         <is>
-          <t>TE2805</t>
+          <t>TE2804</t>
         </is>
       </c>
       <c r="B169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8053</t>
+          <t>VLINE-8052</t>
         </is>
       </c>
       <c r="C169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8162</t>
+          <t>VLINE-8161</t>
         </is>
       </c>
       <c r="D169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8424</t>
+          <t>VLINE-8422</t>
         </is>
       </c>
       <c r="E169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8731</t>
+          <t>VLINE-8730</t>
         </is>
       </c>
       <c r="F169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8797</t>
+          <t>VLINE-8796</t>
         </is>
       </c>
       <c r="G169" s="1" t="inlineStr">
         <is>
-          <t>XRN004</t>
+          <t>XRN001</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="1" t="inlineStr">
         <is>
-          <t>TE2806</t>
+          <t>TE2805</t>
         </is>
       </c>
       <c r="B170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8055</t>
+          <t>VLINE-8053</t>
         </is>
       </c>
       <c r="C170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8171</t>
+          <t>VLINE-8162</t>
         </is>
       </c>
       <c r="D170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8425</t>
+          <t>VLINE-8424</t>
         </is>
       </c>
       <c r="E170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8733</t>
+          <t>VLINE-8731</t>
         </is>
       </c>
       <c r="F170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8799</t>
+          <t>VLINE-8797</t>
         </is>
       </c>
       <c r="G170" s="1" t="inlineStr">
         <is>
-          <t>XRN005</t>
+          <t>XRN004</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update loco downloads 2026-04-05 19:50:15
</commit_message>
<xml_diff>
--- a/downloads/loco_numbers_only.xlsx
+++ b/downloads/loco_numbers_only.xlsx
@@ -2794,32 +2794,32 @@
       </c>
       <c r="C58" s="1" t="inlineStr">
         <is>
-          <t>MM-242M</t>
+          <t>MM-224M</t>
         </is>
       </c>
       <c r="D58" s="1" t="inlineStr">
         <is>
-          <t>MM-734M</t>
+          <t>MM-722M</t>
         </is>
       </c>
       <c r="E58" s="1" t="inlineStr">
         <is>
-          <t>MM-912M</t>
+          <t>MM-906M</t>
         </is>
       </c>
       <c r="F58" s="1" t="inlineStr">
         <is>
-          <t>MM-9945M</t>
+          <t>MM-9938M</t>
         </is>
       </c>
       <c r="G58" s="1" t="inlineStr">
         <is>
-          <t>NR38</t>
+          <t>NR31</t>
         </is>
       </c>
       <c r="H58" s="1" t="inlineStr">
         <is>
-          <t>NR115</t>
+          <t>NR110</t>
         </is>
       </c>
     </row>
@@ -2836,32 +2836,32 @@
       </c>
       <c r="C59" s="1" t="inlineStr">
         <is>
-          <t>MM-256M</t>
+          <t>MM-242M</t>
         </is>
       </c>
       <c r="D59" s="1" t="inlineStr">
         <is>
-          <t>MM-736M</t>
+          <t>MM-726M</t>
         </is>
       </c>
       <c r="E59" s="1" t="inlineStr">
         <is>
-          <t>MM-914M</t>
+          <t>MM-908M</t>
         </is>
       </c>
       <c r="F59" s="1" t="inlineStr">
         <is>
-          <t>MM-9946M</t>
+          <t>MM-9941M</t>
         </is>
       </c>
       <c r="G59" s="1" t="inlineStr">
         <is>
-          <t>NR39</t>
+          <t>NR34</t>
         </is>
       </c>
       <c r="H59" s="1" t="inlineStr">
         <is>
-          <t>NR118</t>
+          <t>NR111</t>
         </is>
       </c>
     </row>
@@ -2878,32 +2878,32 @@
       </c>
       <c r="C60" s="1" t="inlineStr">
         <is>
-          <t>MM-258M</t>
+          <t>MM-256M</t>
         </is>
       </c>
       <c r="D60" s="1" t="inlineStr">
         <is>
-          <t>MM-738M</t>
+          <t>MM-728M</t>
         </is>
       </c>
       <c r="E60" s="1" t="inlineStr">
         <is>
-          <t>MM-920M</t>
+          <t>MM-910M</t>
         </is>
       </c>
       <c r="F60" s="1" t="inlineStr">
         <is>
-          <t>MM-9949M</t>
+          <t>MM-9943M</t>
         </is>
       </c>
       <c r="G60" s="1" t="inlineStr">
         <is>
-          <t>NR40</t>
+          <t>NR36</t>
         </is>
       </c>
       <c r="H60" s="1" t="inlineStr">
         <is>
-          <t>NR119</t>
+          <t>NR112</t>
         </is>
       </c>
     </row>
@@ -2920,32 +2920,32 @@
       </c>
       <c r="C61" s="1" t="inlineStr">
         <is>
-          <t>MM-264M</t>
+          <t>MM-258M</t>
         </is>
       </c>
       <c r="D61" s="1" t="inlineStr">
         <is>
-          <t>MM-740M</t>
+          <t>MM-734M</t>
         </is>
       </c>
       <c r="E61" s="1" t="inlineStr">
         <is>
-          <t>MM-922M</t>
+          <t>MM-912M</t>
         </is>
       </c>
       <c r="F61" s="1" t="inlineStr">
         <is>
-          <t>MM-9950M</t>
+          <t>MM-9945M</t>
         </is>
       </c>
       <c r="G61" s="1" t="inlineStr">
         <is>
-          <t>NR43</t>
+          <t>NR37</t>
         </is>
       </c>
       <c r="H61" s="1" t="inlineStr">
         <is>
-          <t>NR120</t>
+          <t>NR113</t>
         </is>
       </c>
     </row>
@@ -2962,32 +2962,32 @@
       </c>
       <c r="C62" s="1" t="inlineStr">
         <is>
-          <t>MM-268M</t>
+          <t>MM-264M</t>
         </is>
       </c>
       <c r="D62" s="1" t="inlineStr">
         <is>
-          <t>MM-742M</t>
+          <t>MM-736M</t>
         </is>
       </c>
       <c r="E62" s="1" t="inlineStr">
         <is>
-          <t>MM-924M</t>
+          <t>MM-914M</t>
         </is>
       </c>
       <c r="F62" s="1" t="inlineStr">
         <is>
-          <t>MM-9951M</t>
+          <t>MM-9946M</t>
         </is>
       </c>
       <c r="G62" s="1" t="inlineStr">
         <is>
-          <t>NR44</t>
+          <t>NR38</t>
         </is>
       </c>
       <c r="H62" s="1" t="inlineStr">
         <is>
-          <t>NR122</t>
+          <t>NR115</t>
         </is>
       </c>
     </row>
@@ -3004,32 +3004,32 @@
       </c>
       <c r="C63" s="1" t="inlineStr">
         <is>
-          <t>MM-278M</t>
+          <t>MM-268M</t>
         </is>
       </c>
       <c r="D63" s="1" t="inlineStr">
         <is>
-          <t>MM-744M</t>
+          <t>MM-738M</t>
         </is>
       </c>
       <c r="E63" s="1" t="inlineStr">
         <is>
-          <t>MM-926M</t>
+          <t>MM-920M</t>
         </is>
       </c>
       <c r="F63" s="1" t="inlineStr">
         <is>
-          <t>MM-9952M</t>
+          <t>MM-9949M</t>
         </is>
       </c>
       <c r="G63" s="1" t="inlineStr">
         <is>
-          <t>NR45</t>
+          <t>NR39</t>
         </is>
       </c>
       <c r="H63" s="1" t="inlineStr">
         <is>
-          <t>P14</t>
+          <t>NR118</t>
         </is>
       </c>
     </row>
@@ -3046,32 +3046,32 @@
       </c>
       <c r="C64" s="1" t="inlineStr">
         <is>
-          <t>MM-282M</t>
+          <t>MM-278M</t>
         </is>
       </c>
       <c r="D64" s="1" t="inlineStr">
         <is>
-          <t>MM-752M</t>
+          <t>MM-740M</t>
         </is>
       </c>
       <c r="E64" s="1" t="inlineStr">
         <is>
-          <t>MM-934M</t>
+          <t>MM-922M</t>
         </is>
       </c>
       <c r="F64" s="1" t="inlineStr">
         <is>
-          <t>MM-9953M</t>
+          <t>MM-9950M</t>
         </is>
       </c>
       <c r="G64" s="1" t="inlineStr">
         <is>
-          <t>NR47</t>
+          <t>NR40</t>
         </is>
       </c>
       <c r="H64" s="1" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>NR119</t>
         </is>
       </c>
     </row>
@@ -3088,32 +3088,32 @@
       </c>
       <c r="C65" s="1" t="inlineStr">
         <is>
-          <t>MM-352M</t>
+          <t>MM-282M</t>
         </is>
       </c>
       <c r="D65" s="1" t="inlineStr">
         <is>
-          <t>MM-756M</t>
+          <t>MM-742M</t>
         </is>
       </c>
       <c r="E65" s="1" t="inlineStr">
         <is>
-          <t>MM-936M</t>
+          <t>MM-924M</t>
         </is>
       </c>
       <c r="F65" s="1" t="inlineStr">
         <is>
-          <t>MM-9954M</t>
+          <t>MM-9951M</t>
         </is>
       </c>
       <c r="G65" s="1" t="inlineStr">
         <is>
-          <t>NR48</t>
+          <t>NR43</t>
         </is>
       </c>
       <c r="H65" s="1" t="inlineStr">
         <is>
-          <t>P2501</t>
+          <t>NR120</t>
         </is>
       </c>
     </row>
@@ -3130,32 +3130,32 @@
       </c>
       <c r="C66" s="1" t="inlineStr">
         <is>
-          <t>MM-358M</t>
+          <t>MM-284M</t>
         </is>
       </c>
       <c r="D66" s="1" t="inlineStr">
         <is>
-          <t>MM-760M</t>
+          <t>MM-744M</t>
         </is>
       </c>
       <c r="E66" s="1" t="inlineStr">
         <is>
-          <t>MM-938M</t>
+          <t>MM-926M</t>
         </is>
       </c>
       <c r="F66" s="1" t="inlineStr">
         <is>
-          <t>MM-9955M</t>
+          <t>MM-9952M</t>
         </is>
       </c>
       <c r="G66" s="1" t="inlineStr">
         <is>
-          <t>NR51</t>
+          <t>NR44</t>
         </is>
       </c>
       <c r="H66" s="1" t="inlineStr">
         <is>
-          <t>P2502</t>
+          <t>NR122</t>
         </is>
       </c>
     </row>
@@ -3172,32 +3172,32 @@
       </c>
       <c r="C67" s="1" t="inlineStr">
         <is>
-          <t>MM-372M</t>
+          <t>MM-352M</t>
         </is>
       </c>
       <c r="D67" s="1" t="inlineStr">
         <is>
-          <t>MM-764M</t>
+          <t>MM-752M</t>
         </is>
       </c>
       <c r="E67" s="1" t="inlineStr">
         <is>
-          <t>MM-940M</t>
+          <t>MM-934M</t>
         </is>
       </c>
       <c r="F67" s="1" t="inlineStr">
         <is>
-          <t>MM-9957M</t>
+          <t>MM-9953M</t>
         </is>
       </c>
       <c r="G67" s="1" t="inlineStr">
         <is>
-          <t>NR52</t>
+          <t>NR45</t>
         </is>
       </c>
       <c r="H67" s="1" t="inlineStr">
         <is>
-          <t>P2503</t>
+          <t>P14</t>
         </is>
       </c>
     </row>
@@ -3214,32 +3214,32 @@
       </c>
       <c r="C68" s="1" t="inlineStr">
         <is>
-          <t>MM-378M</t>
+          <t>MM-358M</t>
         </is>
       </c>
       <c r="D68" s="1" t="inlineStr">
         <is>
-          <t>MM-768M</t>
+          <t>MM-756M</t>
         </is>
       </c>
       <c r="E68" s="1" t="inlineStr">
         <is>
-          <t>MM-944M</t>
+          <t>MM-936M</t>
         </is>
       </c>
       <c r="F68" s="1" t="inlineStr">
         <is>
-          <t>MM-9959M</t>
+          <t>MM-9954M</t>
         </is>
       </c>
       <c r="G68" s="1" t="inlineStr">
         <is>
-          <t>NR53</t>
+          <t>NR47</t>
         </is>
       </c>
       <c r="H68" s="1" t="inlineStr">
         <is>
-          <t>P2504</t>
+          <t>P16</t>
         </is>
       </c>
     </row>
@@ -3256,32 +3256,32 @@
       </c>
       <c r="C69" s="1" t="inlineStr">
         <is>
-          <t>MM-382M</t>
+          <t>MM-372M</t>
         </is>
       </c>
       <c r="D69" s="1" t="inlineStr">
         <is>
-          <t>MM-774M</t>
+          <t>MM-760M</t>
         </is>
       </c>
       <c r="E69" s="1" t="inlineStr">
         <is>
-          <t>MM-948M</t>
+          <t>MM-938M</t>
         </is>
       </c>
       <c r="F69" s="1" t="inlineStr">
         <is>
-          <t>MM-9960M</t>
+          <t>MM-9955M</t>
         </is>
       </c>
       <c r="G69" s="1" t="inlineStr">
         <is>
-          <t>NR54</t>
+          <t>NR48</t>
         </is>
       </c>
       <c r="H69" s="1" t="inlineStr">
         <is>
-          <t>P2505</t>
+          <t>P2501</t>
         </is>
       </c>
     </row>
@@ -3298,32 +3298,32 @@
       </c>
       <c r="C70" s="1" t="inlineStr">
         <is>
-          <t>MM-392M</t>
+          <t>MM-378M</t>
         </is>
       </c>
       <c r="D70" s="1" t="inlineStr">
         <is>
-          <t>MM-776M</t>
+          <t>MM-764M</t>
         </is>
       </c>
       <c r="E70" s="1" t="inlineStr">
         <is>
-          <t>MM-952M</t>
+          <t>MM-940M</t>
         </is>
       </c>
       <c r="F70" s="1" t="inlineStr">
         <is>
-          <t>MM-9961M</t>
+          <t>MM-9957M</t>
         </is>
       </c>
       <c r="G70" s="1" t="inlineStr">
         <is>
-          <t>NR57</t>
+          <t>NR51</t>
         </is>
       </c>
       <c r="H70" s="1" t="inlineStr">
         <is>
-          <t>P2506</t>
+          <t>P2502</t>
         </is>
       </c>
     </row>
@@ -3340,32 +3340,32 @@
       </c>
       <c r="C71" s="1" t="inlineStr">
         <is>
-          <t>MM-418M</t>
+          <t>MM-382M</t>
         </is>
       </c>
       <c r="D71" s="1" t="inlineStr">
         <is>
-          <t>MM-778M</t>
+          <t>MM-768M</t>
         </is>
       </c>
       <c r="E71" s="1" t="inlineStr">
         <is>
-          <t>MM-954M</t>
+          <t>MM-944M</t>
         </is>
       </c>
       <c r="F71" s="1" t="inlineStr">
         <is>
-          <t>MM-9962M</t>
+          <t>MM-9959M</t>
         </is>
       </c>
       <c r="G71" s="1" t="inlineStr">
         <is>
-          <t>NR59</t>
+          <t>NR52</t>
         </is>
       </c>
       <c r="H71" s="1" t="inlineStr">
         <is>
-          <t>P2507</t>
+          <t>P2503</t>
         </is>
       </c>
     </row>
@@ -3382,32 +3382,32 @@
       </c>
       <c r="C72" s="1" t="inlineStr">
         <is>
-          <t>MM-430M</t>
+          <t>MM-392M</t>
         </is>
       </c>
       <c r="D72" s="1" t="inlineStr">
         <is>
-          <t>MM-780M</t>
+          <t>MM-774M</t>
         </is>
       </c>
       <c r="E72" s="1" t="inlineStr">
         <is>
-          <t>MM-956M</t>
+          <t>MM-948M</t>
         </is>
       </c>
       <c r="F72" s="1" t="inlineStr">
         <is>
-          <t>MM-9963M</t>
+          <t>MM-9960M</t>
         </is>
       </c>
       <c r="G72" s="1" t="inlineStr">
         <is>
-          <t>NR61</t>
+          <t>NR53</t>
         </is>
       </c>
       <c r="H72" s="1" t="inlineStr">
         <is>
-          <t>P2508</t>
+          <t>P2504</t>
         </is>
       </c>
     </row>
@@ -3424,32 +3424,32 @@
       </c>
       <c r="C73" s="1" t="inlineStr">
         <is>
-          <t>MM-444M</t>
+          <t>MM-418M</t>
         </is>
       </c>
       <c r="D73" s="1" t="inlineStr">
         <is>
-          <t>MM-784M</t>
+          <t>MM-776M</t>
         </is>
       </c>
       <c r="E73" s="1" t="inlineStr">
         <is>
-          <t>MM-958M</t>
+          <t>MM-952M</t>
         </is>
       </c>
       <c r="F73" s="1" t="inlineStr">
         <is>
-          <t>MM-9964M</t>
+          <t>MM-9961M</t>
         </is>
       </c>
       <c r="G73" s="1" t="inlineStr">
         <is>
-          <t>NR62</t>
+          <t>NR54</t>
         </is>
       </c>
       <c r="H73" s="1" t="inlineStr">
         <is>
-          <t>P2509</t>
+          <t>P2505</t>
         </is>
       </c>
     </row>
@@ -3466,32 +3466,32 @@
       </c>
       <c r="C74" s="1" t="inlineStr">
         <is>
-          <t>MM-464M</t>
+          <t>MM-430M</t>
         </is>
       </c>
       <c r="D74" s="1" t="inlineStr">
         <is>
-          <t>MM-790M</t>
+          <t>MM-778M</t>
         </is>
       </c>
       <c r="E74" s="1" t="inlineStr">
         <is>
-          <t>MM-962M</t>
+          <t>MM-954M</t>
         </is>
       </c>
       <c r="F74" s="1" t="inlineStr">
         <is>
-          <t>MM-9965M</t>
+          <t>MM-9962M</t>
         </is>
       </c>
       <c r="G74" s="1" t="inlineStr">
         <is>
-          <t>NR64</t>
+          <t>NR57</t>
         </is>
       </c>
       <c r="H74" s="1" t="inlineStr">
         <is>
-          <t>P2510</t>
+          <t>P2506</t>
         </is>
       </c>
     </row>
@@ -3508,32 +3508,32 @@
       </c>
       <c r="C75" s="1" t="inlineStr">
         <is>
-          <t>MM-486M</t>
+          <t>MM-444M</t>
         </is>
       </c>
       <c r="D75" s="1" t="inlineStr">
         <is>
-          <t>MM-792M</t>
+          <t>MM-780M</t>
         </is>
       </c>
       <c r="E75" s="1" t="inlineStr">
         <is>
-          <t>MM-964M</t>
+          <t>MM-956M</t>
         </is>
       </c>
       <c r="F75" s="1" t="inlineStr">
         <is>
-          <t>MM-9966M</t>
+          <t>MM-9963M</t>
         </is>
       </c>
       <c r="G75" s="1" t="inlineStr">
         <is>
-          <t>NR65</t>
+          <t>NR59</t>
         </is>
       </c>
       <c r="H75" s="1" t="inlineStr">
         <is>
-          <t>P2511</t>
+          <t>P2507</t>
         </is>
       </c>
     </row>
@@ -3550,32 +3550,32 @@
       </c>
       <c r="C76" s="1" t="inlineStr">
         <is>
-          <t>MM-496M</t>
+          <t>MM-464M</t>
         </is>
       </c>
       <c r="D76" s="1" t="inlineStr">
         <is>
-          <t>MM-796M</t>
+          <t>MM-784M</t>
         </is>
       </c>
       <c r="E76" s="1" t="inlineStr">
         <is>
-          <t>MM-966M</t>
+          <t>MM-958M</t>
         </is>
       </c>
       <c r="F76" s="1" t="inlineStr">
         <is>
-          <t>MM-9967M</t>
+          <t>MM-9964M</t>
         </is>
       </c>
       <c r="G76" s="1" t="inlineStr">
         <is>
-          <t>NR66</t>
+          <t>NR61</t>
         </is>
       </c>
       <c r="H76" s="1" t="inlineStr">
         <is>
-          <t>P2513</t>
+          <t>P2508</t>
         </is>
       </c>
     </row>
@@ -3592,32 +3592,32 @@
       </c>
       <c r="C77" s="1" t="inlineStr">
         <is>
-          <t>MM-514M</t>
+          <t>MM-486M</t>
         </is>
       </c>
       <c r="D77" s="1" t="inlineStr">
         <is>
-          <t>MM-798M</t>
+          <t>MM-790M</t>
         </is>
       </c>
       <c r="E77" s="1" t="inlineStr">
         <is>
-          <t>MM-968M</t>
+          <t>MM-962M</t>
         </is>
       </c>
       <c r="F77" s="1" t="inlineStr">
         <is>
-          <t>MM-9969M</t>
+          <t>MM-9965M</t>
         </is>
       </c>
       <c r="G77" s="1" t="inlineStr">
         <is>
-          <t>NR67</t>
+          <t>NR62</t>
         </is>
       </c>
       <c r="H77" s="1" t="inlineStr">
         <is>
-          <t>P2514</t>
+          <t>P2509</t>
         </is>
       </c>
     </row>
@@ -3634,32 +3634,32 @@
       </c>
       <c r="C78" s="1" t="inlineStr">
         <is>
-          <t>MM-526M</t>
+          <t>MM-496M</t>
         </is>
       </c>
       <c r="D78" s="1" t="inlineStr">
         <is>
-          <t>MM-800M</t>
+          <t>MM-792M</t>
         </is>
       </c>
       <c r="E78" s="1" t="inlineStr">
         <is>
-          <t>MM-970M</t>
+          <t>MM-964M</t>
         </is>
       </c>
       <c r="F78" s="1" t="inlineStr">
         <is>
-          <t>MM-9970M</t>
+          <t>MM-9966M</t>
         </is>
       </c>
       <c r="G78" s="1" t="inlineStr">
         <is>
-          <t>NR68</t>
+          <t>NR64</t>
         </is>
       </c>
       <c r="H78" s="1" t="inlineStr">
         <is>
-          <t>P2515</t>
+          <t>P2510</t>
         </is>
       </c>
     </row>
@@ -3676,32 +3676,32 @@
       </c>
       <c r="C79" s="1" t="inlineStr">
         <is>
-          <t>MM-534M</t>
+          <t>MM-514M</t>
         </is>
       </c>
       <c r="D79" s="1" t="inlineStr">
         <is>
-          <t>MM-802M</t>
+          <t>MM-796M</t>
         </is>
       </c>
       <c r="E79" s="1" t="inlineStr">
         <is>
-          <t>MM-972M</t>
+          <t>MM-966M</t>
         </is>
       </c>
       <c r="F79" s="1" t="inlineStr">
         <is>
-          <t>MMY032</t>
+          <t>MM-9967M</t>
         </is>
       </c>
       <c r="G79" s="1" t="inlineStr">
         <is>
-          <t>NR69</t>
+          <t>NR65</t>
         </is>
       </c>
       <c r="H79" s="1" t="inlineStr">
         <is>
-          <t>P2516</t>
+          <t>P2511</t>
         </is>
       </c>
     </row>
@@ -3718,32 +3718,32 @@
       </c>
       <c r="C80" s="1" t="inlineStr">
         <is>
-          <t>MM-536M</t>
+          <t>MM-526M</t>
         </is>
       </c>
       <c r="D80" s="1" t="inlineStr">
         <is>
-          <t>MM-804M</t>
+          <t>MM-798M</t>
         </is>
       </c>
       <c r="E80" s="1" t="inlineStr">
         <is>
-          <t>MM-974M</t>
+          <t>MM-968M</t>
         </is>
       </c>
       <c r="F80" s="1" t="inlineStr">
         <is>
-          <t>MRL001</t>
+          <t>MM-9968M</t>
         </is>
       </c>
       <c r="G80" s="1" t="inlineStr">
         <is>
-          <t>NR71</t>
+          <t>NR66</t>
         </is>
       </c>
       <c r="H80" s="1" t="inlineStr">
         <is>
-          <t>PB1</t>
+          <t>P2513</t>
         </is>
       </c>
     </row>
@@ -3760,32 +3760,32 @@
       </c>
       <c r="C81" s="1" t="inlineStr">
         <is>
-          <t>MM-542M</t>
+          <t>MM-534M</t>
         </is>
       </c>
       <c r="D81" s="1" t="inlineStr">
         <is>
-          <t>MM-808M</t>
+          <t>MM-800M</t>
         </is>
       </c>
       <c r="E81" s="1" t="inlineStr">
         <is>
-          <t>MM-976M</t>
+          <t>MM-970M</t>
         </is>
       </c>
       <c r="F81" s="1" t="inlineStr">
         <is>
-          <t>MRL004</t>
+          <t>MM-9969M</t>
         </is>
       </c>
       <c r="G81" s="1" t="inlineStr">
         <is>
-          <t>NR72</t>
+          <t>NR67</t>
         </is>
       </c>
       <c r="H81" s="1" t="inlineStr">
         <is>
-          <t>PB2</t>
+          <t>P2514</t>
         </is>
       </c>
     </row>
@@ -3802,32 +3802,32 @@
       </c>
       <c r="C82" s="1" t="inlineStr">
         <is>
-          <t>MM-544M</t>
+          <t>MM-536M</t>
         </is>
       </c>
       <c r="D82" s="1" t="inlineStr">
         <is>
-          <t>MM-810M</t>
+          <t>MM-802M</t>
         </is>
       </c>
       <c r="E82" s="1" t="inlineStr">
         <is>
-          <t>MM-980M</t>
+          <t>MM-972M</t>
         </is>
       </c>
       <c r="F82" s="1" t="inlineStr">
         <is>
-          <t>MRL006</t>
+          <t>MM-9970M</t>
         </is>
       </c>
       <c r="G82" s="1" t="inlineStr">
         <is>
-          <t>NR75</t>
+          <t>NR68</t>
         </is>
       </c>
       <c r="H82" s="1" t="inlineStr">
         <is>
-          <t>PB4</t>
+          <t>P2515</t>
         </is>
       </c>
     </row>
@@ -3844,32 +3844,32 @@
       </c>
       <c r="C83" s="1" t="inlineStr">
         <is>
-          <t>MM-546M</t>
+          <t>MM-542M</t>
         </is>
       </c>
       <c r="D83" s="1" t="inlineStr">
         <is>
-          <t>MM-814M</t>
+          <t>MM-804M</t>
         </is>
       </c>
       <c r="E83" s="1" t="inlineStr">
         <is>
-          <t>MM-982M</t>
+          <t>MM-974M</t>
         </is>
       </c>
       <c r="F83" s="1" t="inlineStr">
         <is>
-          <t>N452</t>
+          <t>MMY032</t>
         </is>
       </c>
       <c r="G83" s="1" t="inlineStr">
         <is>
-          <t>NR77</t>
+          <t>NR69</t>
         </is>
       </c>
       <c r="H83" s="1" t="inlineStr">
         <is>
-          <t>PHC001</t>
+          <t>P2516</t>
         </is>
       </c>
     </row>
@@ -3886,32 +3886,32 @@
       </c>
       <c r="C84" s="1" t="inlineStr">
         <is>
-          <t>MM-551M</t>
+          <t>MM-544M</t>
         </is>
       </c>
       <c r="D84" s="1" t="inlineStr">
         <is>
-          <t>MM-816M</t>
+          <t>MM-808M</t>
         </is>
       </c>
       <c r="E84" s="1" t="inlineStr">
         <is>
-          <t>MM-984M</t>
+          <t>MM-976M</t>
         </is>
       </c>
       <c r="F84" s="1" t="inlineStr">
         <is>
-          <t>N453</t>
+          <t>MRL001</t>
         </is>
       </c>
       <c r="G84" s="1" t="inlineStr">
         <is>
-          <t>NR78</t>
+          <t>NR71</t>
         </is>
       </c>
       <c r="H84" s="1" t="inlineStr">
         <is>
-          <t>PHC002</t>
+          <t>PB1</t>
         </is>
       </c>
     </row>
@@ -3928,32 +3928,32 @@
       </c>
       <c r="C85" s="1" t="inlineStr">
         <is>
-          <t>MM-552M</t>
+          <t>MM-546M</t>
         </is>
       </c>
       <c r="D85" s="1" t="inlineStr">
         <is>
-          <t>MM-818M</t>
+          <t>MM-810M</t>
         </is>
       </c>
       <c r="E85" s="1" t="inlineStr">
         <is>
-          <t>MM-986M</t>
+          <t>MM-980M</t>
         </is>
       </c>
       <c r="F85" s="1" t="inlineStr">
         <is>
-          <t>N457</t>
+          <t>MRL004</t>
         </is>
       </c>
       <c r="G85" s="1" t="inlineStr">
         <is>
-          <t>NR81</t>
+          <t>NR72</t>
         </is>
       </c>
       <c r="H85" s="1" t="inlineStr">
         <is>
-          <t>Q4001</t>
+          <t>PB2</t>
         </is>
       </c>
     </row>
@@ -3970,32 +3970,32 @@
       </c>
       <c r="C86" s="1" t="inlineStr">
         <is>
-          <t>MM-580M</t>
+          <t>MM-550M</t>
         </is>
       </c>
       <c r="D86" s="1" t="inlineStr">
         <is>
-          <t>MM-820M</t>
+          <t>MM-814M</t>
         </is>
       </c>
       <c r="E86" s="1" t="inlineStr">
         <is>
-          <t>MM-9902M</t>
+          <t>MM-982M</t>
         </is>
       </c>
       <c r="F86" s="1" t="inlineStr">
         <is>
-          <t>N458</t>
+          <t>MRL006</t>
         </is>
       </c>
       <c r="G86" s="1" t="inlineStr">
         <is>
-          <t>NR82</t>
+          <t>NR75</t>
         </is>
       </c>
       <c r="H86" s="1" t="inlineStr">
         <is>
-          <t>Q4003</t>
+          <t>PB4</t>
         </is>
       </c>
     </row>
@@ -4012,32 +4012,32 @@
       </c>
       <c r="C87" s="1" t="inlineStr">
         <is>
-          <t>MM-588M</t>
+          <t>MM-551M</t>
         </is>
       </c>
       <c r="D87" s="1" t="inlineStr">
         <is>
-          <t>MM-824M</t>
+          <t>MM-816M</t>
         </is>
       </c>
       <c r="E87" s="1" t="inlineStr">
         <is>
-          <t>MM-9903M</t>
+          <t>MM-984M</t>
         </is>
       </c>
       <c r="F87" s="1" t="inlineStr">
         <is>
-          <t>N461</t>
+          <t>N452</t>
         </is>
       </c>
       <c r="G87" s="1" t="inlineStr">
         <is>
-          <t>NR83</t>
+          <t>NR77</t>
         </is>
       </c>
       <c r="H87" s="1" t="inlineStr">
         <is>
-          <t>Q4004</t>
+          <t>PHC001</t>
         </is>
       </c>
     </row>
@@ -4054,32 +4054,32 @@
       </c>
       <c r="C88" s="1" t="inlineStr">
         <is>
-          <t>MM-602M</t>
+          <t>MM-552M</t>
         </is>
       </c>
       <c r="D88" s="1" t="inlineStr">
         <is>
-          <t>MM-826M</t>
+          <t>MM-818M</t>
         </is>
       </c>
       <c r="E88" s="1" t="inlineStr">
         <is>
-          <t>MM-9904M</t>
+          <t>MM-986M</t>
         </is>
       </c>
       <c r="F88" s="1" t="inlineStr">
         <is>
-          <t>N465</t>
+          <t>N453</t>
         </is>
       </c>
       <c r="G88" s="1" t="inlineStr">
         <is>
-          <t>NR84</t>
+          <t>NR78</t>
         </is>
       </c>
       <c r="H88" s="1" t="inlineStr">
         <is>
-          <t>Q4005</t>
+          <t>PHC002</t>
         </is>
       </c>
     </row>
@@ -4096,32 +4096,32 @@
       </c>
       <c r="C89" s="1" t="inlineStr">
         <is>
-          <t>MM-608M</t>
+          <t>MM-580M</t>
         </is>
       </c>
       <c r="D89" s="1" t="inlineStr">
         <is>
-          <t>MM-828M</t>
+          <t>MM-820M</t>
         </is>
       </c>
       <c r="E89" s="1" t="inlineStr">
         <is>
-          <t>MM-9906M</t>
+          <t>MM-9902M</t>
         </is>
       </c>
       <c r="F89" s="1" t="inlineStr">
         <is>
-          <t>N466</t>
+          <t>N457</t>
         </is>
       </c>
       <c r="G89" s="1" t="inlineStr">
         <is>
-          <t>NR85</t>
+          <t>NR81</t>
         </is>
       </c>
       <c r="H89" s="1" t="inlineStr">
         <is>
-          <t>Q4006</t>
+          <t>Q4001</t>
         </is>
       </c>
     </row>
@@ -4138,32 +4138,32 @@
       </c>
       <c r="C90" s="1" t="inlineStr">
         <is>
-          <t>MM-616M</t>
+          <t>MM-588M</t>
         </is>
       </c>
       <c r="D90" s="1" t="inlineStr">
         <is>
-          <t>MM-830M</t>
+          <t>MM-824M</t>
         </is>
       </c>
       <c r="E90" s="1" t="inlineStr">
         <is>
-          <t>MM-9907M</t>
+          <t>MM-9903M</t>
         </is>
       </c>
       <c r="F90" s="1" t="inlineStr">
         <is>
-          <t>N467</t>
+          <t>N458</t>
         </is>
       </c>
       <c r="G90" s="1" t="inlineStr">
         <is>
-          <t>NR86</t>
+          <t>NR82</t>
         </is>
       </c>
       <c r="H90" s="1" t="inlineStr">
         <is>
-          <t>Q4007</t>
+          <t>Q4003</t>
         </is>
       </c>
     </row>
@@ -4180,32 +4180,32 @@
       </c>
       <c r="C91" s="1" t="inlineStr">
         <is>
-          <t>MM-624M</t>
+          <t>MM-602M</t>
         </is>
       </c>
       <c r="D91" s="1" t="inlineStr">
         <is>
-          <t>MM-832M</t>
+          <t>MM-826M</t>
         </is>
       </c>
       <c r="E91" s="1" t="inlineStr">
         <is>
-          <t>MM-9908M</t>
+          <t>MM-9904M</t>
         </is>
       </c>
       <c r="F91" s="1" t="inlineStr">
         <is>
-          <t>N469</t>
+          <t>N461</t>
         </is>
       </c>
       <c r="G91" s="1" t="inlineStr">
         <is>
-          <t>NR87</t>
+          <t>NR83</t>
         </is>
       </c>
       <c r="H91" s="1" t="inlineStr">
         <is>
-          <t>Q4009</t>
+          <t>Q4004</t>
         </is>
       </c>
     </row>
@@ -4222,32 +4222,32 @@
       </c>
       <c r="C92" s="1" t="inlineStr">
         <is>
-          <t>MM-632M</t>
+          <t>MM-608M</t>
         </is>
       </c>
       <c r="D92" s="1" t="inlineStr">
         <is>
-          <t>MM-834M</t>
+          <t>MM-828M</t>
         </is>
       </c>
       <c r="E92" s="1" t="inlineStr">
         <is>
-          <t>MM-9909M</t>
+          <t>MM-9906M</t>
         </is>
       </c>
       <c r="F92" s="1" t="inlineStr">
         <is>
-          <t>N473</t>
+          <t>N465</t>
         </is>
       </c>
       <c r="G92" s="1" t="inlineStr">
         <is>
-          <t>NR88</t>
+          <t>NR84</t>
         </is>
       </c>
       <c r="H92" s="1" t="inlineStr">
         <is>
-          <t>Q4011</t>
+          <t>Q4005</t>
         </is>
       </c>
     </row>
@@ -4264,32 +4264,32 @@
       </c>
       <c r="C93" s="1" t="inlineStr">
         <is>
-          <t>MM-636M</t>
+          <t>MM-616M</t>
         </is>
       </c>
       <c r="D93" s="1" t="inlineStr">
         <is>
-          <t>MM-838M</t>
+          <t>MM-830M</t>
         </is>
       </c>
       <c r="E93" s="1" t="inlineStr">
         <is>
-          <t>MM-9912M</t>
+          <t>MM-9907M</t>
         </is>
       </c>
       <c r="F93" s="1" t="inlineStr">
         <is>
-          <t>NR1</t>
+          <t>N466</t>
         </is>
       </c>
       <c r="G93" s="1" t="inlineStr">
         <is>
-          <t>NR89</t>
+          <t>NR85</t>
         </is>
       </c>
       <c r="H93" s="1" t="inlineStr">
         <is>
-          <t>Q4012</t>
+          <t>Q4006</t>
         </is>
       </c>
     </row>
@@ -4306,32 +4306,32 @@
       </c>
       <c r="C94" s="1" t="inlineStr">
         <is>
-          <t>MM-640M</t>
+          <t>MM-624M</t>
         </is>
       </c>
       <c r="D94" s="1" t="inlineStr">
         <is>
-          <t>MM-840M</t>
+          <t>MM-832M</t>
         </is>
       </c>
       <c r="E94" s="1" t="inlineStr">
         <is>
-          <t>MM-9913M</t>
+          <t>MM-9908M</t>
         </is>
       </c>
       <c r="F94" s="1" t="inlineStr">
         <is>
-          <t>NR2</t>
+          <t>N467</t>
         </is>
       </c>
       <c r="G94" s="1" t="inlineStr">
         <is>
-          <t>NR90</t>
+          <t>NR86</t>
         </is>
       </c>
       <c r="H94" s="1" t="inlineStr">
         <is>
-          <t>Q4013</t>
+          <t>Q4007</t>
         </is>
       </c>
     </row>
@@ -4348,32 +4348,32 @@
       </c>
       <c r="C95" s="1" t="inlineStr">
         <is>
-          <t>MM-654M</t>
+          <t>MM-632M</t>
         </is>
       </c>
       <c r="D95" s="1" t="inlineStr">
         <is>
-          <t>MM-842M</t>
+          <t>MM-834M</t>
         </is>
       </c>
       <c r="E95" s="1" t="inlineStr">
         <is>
-          <t>MM-9914M</t>
+          <t>MM-9909M</t>
         </is>
       </c>
       <c r="F95" s="1" t="inlineStr">
         <is>
-          <t>NR4</t>
+          <t>N469</t>
         </is>
       </c>
       <c r="G95" s="1" t="inlineStr">
         <is>
-          <t>NR91</t>
+          <t>NR87</t>
         </is>
       </c>
       <c r="H95" s="1" t="inlineStr">
         <is>
-          <t>Q4014</t>
+          <t>Q4009</t>
         </is>
       </c>
     </row>
@@ -4390,32 +4390,32 @@
       </c>
       <c r="C96" s="1" t="inlineStr">
         <is>
-          <t>MM-656M</t>
+          <t>MM-636M</t>
         </is>
       </c>
       <c r="D96" s="1" t="inlineStr">
         <is>
-          <t>MM-844M</t>
+          <t>MM-838M</t>
         </is>
       </c>
       <c r="E96" s="1" t="inlineStr">
         <is>
-          <t>MM-9915M</t>
+          <t>MM-9912M</t>
         </is>
       </c>
       <c r="F96" s="1" t="inlineStr">
         <is>
-          <t>NR5</t>
+          <t>N473</t>
         </is>
       </c>
       <c r="G96" s="1" t="inlineStr">
         <is>
-          <t>NR92</t>
+          <t>NR88</t>
         </is>
       </c>
       <c r="H96" s="1" t="inlineStr">
         <is>
-          <t>Q4015</t>
+          <t>Q4011</t>
         </is>
       </c>
     </row>
@@ -4432,32 +4432,32 @@
       </c>
       <c r="C97" s="1" t="inlineStr">
         <is>
-          <t>MM-660M</t>
+          <t>MM-640M</t>
         </is>
       </c>
       <c r="D97" s="1" t="inlineStr">
         <is>
-          <t>MM-852M</t>
+          <t>MM-840M</t>
         </is>
       </c>
       <c r="E97" s="1" t="inlineStr">
         <is>
-          <t>MM-9917M</t>
+          <t>MM-9913M</t>
         </is>
       </c>
       <c r="F97" s="1" t="inlineStr">
         <is>
-          <t>NR7</t>
+          <t>NR1</t>
         </is>
       </c>
       <c r="G97" s="1" t="inlineStr">
         <is>
-          <t>NR93</t>
+          <t>NR89</t>
         </is>
       </c>
       <c r="H97" s="1" t="inlineStr">
         <is>
-          <t>Q4016</t>
+          <t>Q4012</t>
         </is>
       </c>
     </row>
@@ -4474,32 +4474,32 @@
       </c>
       <c r="C98" s="1" t="inlineStr">
         <is>
-          <t>MM-661M</t>
+          <t>MM-654M</t>
         </is>
       </c>
       <c r="D98" s="1" t="inlineStr">
         <is>
-          <t>MM-858M</t>
+          <t>MM-842M</t>
         </is>
       </c>
       <c r="E98" s="1" t="inlineStr">
         <is>
-          <t>MM-9918M</t>
+          <t>MM-9914M</t>
         </is>
       </c>
       <c r="F98" s="1" t="inlineStr">
         <is>
-          <t>NR8</t>
+          <t>NR2</t>
         </is>
       </c>
       <c r="G98" s="1" t="inlineStr">
         <is>
-          <t>NR94</t>
+          <t>NR90</t>
         </is>
       </c>
       <c r="H98" s="1" t="inlineStr">
         <is>
-          <t>Q4017</t>
+          <t>Q4013</t>
         </is>
       </c>
     </row>
@@ -4516,32 +4516,32 @@
       </c>
       <c r="C99" s="1" t="inlineStr">
         <is>
-          <t>MM-662M</t>
+          <t>MM-656M</t>
         </is>
       </c>
       <c r="D99" s="1" t="inlineStr">
         <is>
-          <t>MM-860M</t>
+          <t>MM-844M</t>
         </is>
       </c>
       <c r="E99" s="1" t="inlineStr">
         <is>
-          <t>MM-9919M</t>
+          <t>MM-9915M</t>
         </is>
       </c>
       <c r="F99" s="1" t="inlineStr">
         <is>
-          <t>NR9</t>
+          <t>NR4</t>
         </is>
       </c>
       <c r="G99" s="1" t="inlineStr">
         <is>
-          <t>NR95</t>
+          <t>NR91</t>
         </is>
       </c>
       <c r="H99" s="1" t="inlineStr">
         <is>
-          <t>Q4019</t>
+          <t>Q4014</t>
         </is>
       </c>
     </row>
@@ -4558,32 +4558,32 @@
       </c>
       <c r="C100" s="1" t="inlineStr">
         <is>
-          <t>MM-664M</t>
+          <t>MM-660M</t>
         </is>
       </c>
       <c r="D100" s="1" t="inlineStr">
         <is>
-          <t>MM-862M</t>
+          <t>MM-852M</t>
         </is>
       </c>
       <c r="E100" s="1" t="inlineStr">
         <is>
-          <t>MM-9920M</t>
+          <t>MM-9917M</t>
         </is>
       </c>
       <c r="F100" s="1" t="inlineStr">
         <is>
-          <t>NR12</t>
+          <t>NR5</t>
         </is>
       </c>
       <c r="G100" s="1" t="inlineStr">
         <is>
-          <t>NR96</t>
+          <t>NR92</t>
         </is>
       </c>
       <c r="H100" s="1" t="inlineStr">
         <is>
-          <t>QBX003</t>
+          <t>Q4015</t>
         </is>
       </c>
     </row>
@@ -4600,32 +4600,32 @@
       </c>
       <c r="C101" s="1" t="inlineStr">
         <is>
-          <t>MM-666M</t>
+          <t>MM-661M</t>
         </is>
       </c>
       <c r="D101" s="1" t="inlineStr">
         <is>
-          <t>MM-868M</t>
+          <t>MM-858M</t>
         </is>
       </c>
       <c r="E101" s="1" t="inlineStr">
         <is>
-          <t>MM-9922M</t>
+          <t>MM-9918M</t>
         </is>
       </c>
       <c r="F101" s="1" t="inlineStr">
         <is>
-          <t>NR15</t>
+          <t>NR7</t>
         </is>
       </c>
       <c r="G101" s="1" t="inlineStr">
         <is>
-          <t>NR97</t>
+          <t>NR93</t>
         </is>
       </c>
       <c r="H101" s="1" t="inlineStr">
         <is>
-          <t>QBX004</t>
+          <t>Q4016</t>
         </is>
       </c>
     </row>
@@ -4642,32 +4642,32 @@
       </c>
       <c r="C102" s="1" t="inlineStr">
         <is>
-          <t>MM-668M</t>
+          <t>MM-662M</t>
         </is>
       </c>
       <c r="D102" s="1" t="inlineStr">
         <is>
-          <t>MM-870M</t>
+          <t>MM-860M</t>
         </is>
       </c>
       <c r="E102" s="1" t="inlineStr">
         <is>
-          <t>MM-9923M</t>
+          <t>MM-9919M</t>
         </is>
       </c>
       <c r="F102" s="1" t="inlineStr">
         <is>
-          <t>NR16</t>
+          <t>NR8</t>
         </is>
       </c>
       <c r="G102" s="1" t="inlineStr">
         <is>
-          <t>NR98</t>
+          <t>NR94</t>
         </is>
       </c>
       <c r="H102" s="1" t="inlineStr">
         <is>
-          <t>QBX005</t>
+          <t>Q4017</t>
         </is>
       </c>
     </row>
@@ -4684,32 +4684,32 @@
       </c>
       <c r="C103" s="1" t="inlineStr">
         <is>
-          <t>MM-673M</t>
+          <t>MM-664M</t>
         </is>
       </c>
       <c r="D103" s="1" t="inlineStr">
         <is>
-          <t>MM-872M</t>
+          <t>MM-862M</t>
         </is>
       </c>
       <c r="E103" s="1" t="inlineStr">
         <is>
-          <t>MM-9924M</t>
+          <t>MM-9920M</t>
         </is>
       </c>
       <c r="F103" s="1" t="inlineStr">
         <is>
-          <t>NR18</t>
+          <t>NR9</t>
         </is>
       </c>
       <c r="G103" s="1" t="inlineStr">
         <is>
-          <t>NR99</t>
+          <t>NR95</t>
         </is>
       </c>
       <c r="H103" s="1" t="inlineStr">
         <is>
-          <t>QBX006</t>
+          <t>Q4019</t>
         </is>
       </c>
     </row>
@@ -4726,32 +4726,32 @@
       </c>
       <c r="C104" s="1" t="inlineStr">
         <is>
-          <t>MM-674M</t>
+          <t>MM-666M</t>
         </is>
       </c>
       <c r="D104" s="1" t="inlineStr">
         <is>
-          <t>MM-874M</t>
+          <t>MM-868M</t>
         </is>
       </c>
       <c r="E104" s="1" t="inlineStr">
         <is>
-          <t>MM-9926M</t>
+          <t>MM-9922M</t>
         </is>
       </c>
       <c r="F104" s="1" t="inlineStr">
         <is>
-          <t>NR19</t>
+          <t>NR12</t>
         </is>
       </c>
       <c r="G104" s="1" t="inlineStr">
         <is>
-          <t>NR101</t>
+          <t>NR96</t>
         </is>
       </c>
       <c r="H104" s="1" t="inlineStr">
         <is>
-          <t>QE001</t>
+          <t>QBX003</t>
         </is>
       </c>
     </row>
@@ -4768,32 +4768,32 @@
       </c>
       <c r="C105" s="1" t="inlineStr">
         <is>
-          <t>MM-676M</t>
+          <t>MM-668M</t>
         </is>
       </c>
       <c r="D105" s="1" t="inlineStr">
         <is>
-          <t>MM-876M</t>
+          <t>MM-870M</t>
         </is>
       </c>
       <c r="E105" s="1" t="inlineStr">
         <is>
-          <t>MM-9928M</t>
+          <t>MM-9923M</t>
         </is>
       </c>
       <c r="F105" s="1" t="inlineStr">
         <is>
-          <t>NR21</t>
+          <t>NR15</t>
         </is>
       </c>
       <c r="G105" s="1" t="inlineStr">
         <is>
-          <t>NR102</t>
+          <t>NR97</t>
         </is>
       </c>
       <c r="H105" s="1" t="inlineStr">
         <is>
-          <t>QE002</t>
+          <t>QBX004</t>
         </is>
       </c>
     </row>
@@ -4810,32 +4810,32 @@
       </c>
       <c r="C106" s="1" t="inlineStr">
         <is>
-          <t>MM-680M</t>
+          <t>MM-673M</t>
         </is>
       </c>
       <c r="D106" s="1" t="inlineStr">
         <is>
-          <t>MM-882M</t>
+          <t>MM-872M</t>
         </is>
       </c>
       <c r="E106" s="1" t="inlineStr">
         <is>
-          <t>MM-9929M</t>
+          <t>MM-9924M</t>
         </is>
       </c>
       <c r="F106" s="1" t="inlineStr">
         <is>
-          <t>NR25</t>
+          <t>NR16</t>
         </is>
       </c>
       <c r="G106" s="1" t="inlineStr">
         <is>
-          <t>NR103</t>
+          <t>NR98</t>
         </is>
       </c>
       <c r="H106" s="1" t="inlineStr">
         <is>
-          <t>QE003</t>
+          <t>QBX005</t>
         </is>
       </c>
     </row>
@@ -4852,32 +4852,32 @@
       </c>
       <c r="C107" s="1" t="inlineStr">
         <is>
-          <t>MM-706M</t>
+          <t>MM-674M</t>
         </is>
       </c>
       <c r="D107" s="1" t="inlineStr">
         <is>
-          <t>MM-894M</t>
+          <t>MM-874M</t>
         </is>
       </c>
       <c r="E107" s="1" t="inlineStr">
         <is>
-          <t>MM-9932M</t>
+          <t>MM-9926M</t>
         </is>
       </c>
       <c r="F107" s="1" t="inlineStr">
         <is>
-          <t>NR27</t>
+          <t>NR18</t>
         </is>
       </c>
       <c r="G107" s="1" t="inlineStr">
         <is>
-          <t>NR105</t>
+          <t>NR99</t>
         </is>
       </c>
       <c r="H107" s="1" t="inlineStr">
         <is>
-          <t>QE004</t>
+          <t>QBX006</t>
         </is>
       </c>
     </row>
@@ -4894,32 +4894,32 @@
       </c>
       <c r="C108" s="1" t="inlineStr">
         <is>
-          <t>MM-708M</t>
+          <t>MM-676M</t>
         </is>
       </c>
       <c r="D108" s="1" t="inlineStr">
         <is>
-          <t>MM-896M</t>
+          <t>MM-876M</t>
         </is>
       </c>
       <c r="E108" s="1" t="inlineStr">
         <is>
-          <t>MM-9933M</t>
+          <t>MM-9928M</t>
         </is>
       </c>
       <c r="F108" s="1" t="inlineStr">
         <is>
-          <t>NR28</t>
+          <t>NR19</t>
         </is>
       </c>
       <c r="G108" s="1" t="inlineStr">
         <is>
-          <t>NR108</t>
+          <t>NR101</t>
         </is>
       </c>
       <c r="H108" s="1" t="inlineStr">
         <is>
-          <t>QE006</t>
+          <t>QE001</t>
         </is>
       </c>
     </row>
@@ -4936,32 +4936,32 @@
       </c>
       <c r="C109" s="1" t="inlineStr">
         <is>
-          <t>MM-710M</t>
+          <t>MM-680M</t>
         </is>
       </c>
       <c r="D109" s="1" t="inlineStr">
         <is>
-          <t>MM-902M</t>
+          <t>MM-882M</t>
         </is>
       </c>
       <c r="E109" s="1" t="inlineStr">
         <is>
-          <t>MM-9934M</t>
+          <t>MM-9929M</t>
         </is>
       </c>
       <c r="F109" s="1" t="inlineStr">
         <is>
-          <t>NR30</t>
+          <t>NR21</t>
         </is>
       </c>
       <c r="G109" s="1" t="inlineStr">
         <is>
-          <t>NR109</t>
+          <t>NR102</t>
         </is>
       </c>
       <c r="H109" s="1" t="inlineStr">
         <is>
-          <t>QL001</t>
+          <t>QE002</t>
         </is>
       </c>
     </row>
@@ -4978,32 +4978,32 @@
       </c>
       <c r="C110" s="1" t="inlineStr">
         <is>
-          <t>MM-716M</t>
+          <t>MM-706M</t>
         </is>
       </c>
       <c r="D110" s="1" t="inlineStr">
         <is>
-          <t>MM-904M</t>
+          <t>MM-894M</t>
         </is>
       </c>
       <c r="E110" s="1" t="inlineStr">
         <is>
-          <t>MM-9936M</t>
+          <t>MM-9932M</t>
         </is>
       </c>
       <c r="F110" s="1" t="inlineStr">
         <is>
-          <t>NR31</t>
+          <t>NR25</t>
         </is>
       </c>
       <c r="G110" s="1" t="inlineStr">
         <is>
-          <t>NR110</t>
+          <t>NR103</t>
         </is>
       </c>
       <c r="H110" s="1" t="inlineStr">
         <is>
-          <t>QL002</t>
+          <t>QE003</t>
         </is>
       </c>
     </row>
@@ -5015,37 +5015,37 @@
       </c>
       <c r="B111" s="1" t="inlineStr">
         <is>
-          <t>MM-218M</t>
+          <t>MM-216M</t>
         </is>
       </c>
       <c r="C111" s="1" t="inlineStr">
         <is>
-          <t>MM-722M</t>
+          <t>MM-708M</t>
         </is>
       </c>
       <c r="D111" s="1" t="inlineStr">
         <is>
-          <t>MM-906M</t>
+          <t>MM-896M</t>
         </is>
       </c>
       <c r="E111" s="1" t="inlineStr">
         <is>
-          <t>MM-9938M</t>
+          <t>MM-9933M</t>
         </is>
       </c>
       <c r="F111" s="1" t="inlineStr">
         <is>
-          <t>NR34</t>
+          <t>NR27</t>
         </is>
       </c>
       <c r="G111" s="1" t="inlineStr">
         <is>
-          <t>NR111</t>
+          <t>NR105</t>
         </is>
       </c>
       <c r="H111" s="1" t="inlineStr">
         <is>
-          <t>QL004</t>
+          <t>QE004</t>
         </is>
       </c>
     </row>
@@ -5057,37 +5057,37 @@
       </c>
       <c r="B112" s="1" t="inlineStr">
         <is>
-          <t>MM-222M</t>
+          <t>MM-218M</t>
         </is>
       </c>
       <c r="C112" s="1" t="inlineStr">
         <is>
-          <t>MM-726M</t>
+          <t>MM-710M</t>
         </is>
       </c>
       <c r="D112" s="1" t="inlineStr">
         <is>
-          <t>MM-908M</t>
+          <t>MM-902M</t>
         </is>
       </c>
       <c r="E112" s="1" t="inlineStr">
         <is>
-          <t>MM-9941M</t>
+          <t>MM-9934M</t>
         </is>
       </c>
       <c r="F112" s="1" t="inlineStr">
         <is>
-          <t>NR36</t>
+          <t>NR28</t>
         </is>
       </c>
       <c r="G112" s="1" t="inlineStr">
         <is>
-          <t>NR112</t>
+          <t>NR108</t>
         </is>
       </c>
       <c r="H112" s="1" t="inlineStr">
         <is>
-          <t>QL007</t>
+          <t>QE006</t>
         </is>
       </c>
     </row>
@@ -5099,2234 +5099,2254 @@
       </c>
       <c r="B113" s="1" t="inlineStr">
         <is>
-          <t>MM-224M</t>
+          <t>MM-222M</t>
         </is>
       </c>
       <c r="C113" s="1" t="inlineStr">
         <is>
-          <t>MM-728M</t>
+          <t>MM-716M</t>
         </is>
       </c>
       <c r="D113" s="1" t="inlineStr">
         <is>
-          <t>MM-910M</t>
+          <t>MM-904M</t>
         </is>
       </c>
       <c r="E113" s="1" t="inlineStr">
         <is>
-          <t>MM-9943M</t>
+          <t>MM-9936M</t>
         </is>
       </c>
       <c r="F113" s="1" t="inlineStr">
         <is>
-          <t>NR37</t>
+          <t>NR30</t>
         </is>
       </c>
       <c r="G113" s="1" t="inlineStr">
         <is>
-          <t>NR113</t>
+          <t>NR109</t>
         </is>
       </c>
       <c r="H113" s="1" t="inlineStr">
         <is>
-          <t>QL008</t>
+          <t>QL001</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
         <is>
-          <t>QL010</t>
+          <t>QL002</t>
         </is>
       </c>
       <c r="B115" s="1" t="inlineStr">
         <is>
-          <t>SSR103</t>
+          <t>SCT015</t>
         </is>
       </c>
       <c r="C115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8029</t>
+          <t>VLINE-8025</t>
         </is>
       </c>
       <c r="D115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8152</t>
+          <t>VLINE-8145</t>
         </is>
       </c>
       <c r="E115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8411</t>
+          <t>VLINE-8404</t>
         </is>
       </c>
       <c r="F115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8717</t>
+          <t>VLINE-8671</t>
         </is>
       </c>
       <c r="G115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8786</t>
+          <t>VLINE-8781</t>
         </is>
       </c>
       <c r="H115" s="1" t="inlineStr">
         <is>
-          <t>XP2012</t>
+          <t>XP2007</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
         <is>
-          <t>QL011</t>
+          <t>QL004</t>
         </is>
       </c>
       <c r="B116" s="1" t="inlineStr">
         <is>
-          <t>SSR104</t>
+          <t>SO2</t>
         </is>
       </c>
       <c r="C116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8030</t>
+          <t>VLINE-8026</t>
         </is>
       </c>
       <c r="D116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8153</t>
+          <t>VLINE-8148</t>
         </is>
       </c>
       <c r="E116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8413</t>
+          <t>VLINE-8406</t>
         </is>
       </c>
       <c r="F116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8720</t>
+          <t>VLINE-8706</t>
         </is>
       </c>
       <c r="G116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8787</t>
+          <t>VLINE-8782</t>
         </is>
       </c>
       <c r="H116" s="1" t="inlineStr">
         <is>
-          <t>XP2013</t>
+          <t>XP2008</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="1" t="inlineStr">
         <is>
-          <t>QL014</t>
+          <t>QL007</t>
         </is>
       </c>
       <c r="B117" s="1" t="inlineStr">
         <is>
-          <t>T363</t>
+          <t>SSR101</t>
         </is>
       </c>
       <c r="C117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8031</t>
+          <t>VLINE-8027</t>
         </is>
       </c>
       <c r="D117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8154</t>
+          <t>VLINE-8150</t>
         </is>
       </c>
       <c r="E117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8415</t>
+          <t>VLINE-8408</t>
         </is>
       </c>
       <c r="F117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8721</t>
+          <t>VLINE-8711</t>
         </is>
       </c>
       <c r="G117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8788</t>
+          <t>VLINE-8783</t>
         </is>
       </c>
       <c r="H117" s="1" t="inlineStr">
         <is>
-          <t>XP2014</t>
+          <t>XP2010</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
         <is>
-          <t>QL018</t>
+          <t>QL008</t>
         </is>
       </c>
       <c r="B118" s="1" t="inlineStr">
         <is>
-          <t>T386</t>
+          <t>SSR102</t>
         </is>
       </c>
       <c r="C118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8032</t>
+          <t>VLINE-8028</t>
         </is>
       </c>
       <c r="D118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8155</t>
+          <t>VLINE-8151</t>
         </is>
       </c>
       <c r="E118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8417</t>
+          <t>VLINE-8410</t>
         </is>
       </c>
       <c r="F118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8723</t>
+          <t>VLINE-8714</t>
         </is>
       </c>
       <c r="G118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8790</t>
+          <t>VLINE-8784</t>
         </is>
       </c>
       <c r="H118" s="1" t="inlineStr">
         <is>
-          <t>XP2015</t>
+          <t>XP2011</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
         <is>
-          <t>QR1744</t>
+          <t>QL010</t>
         </is>
       </c>
       <c r="B119" s="1" t="inlineStr">
         <is>
-          <t>TDX101</t>
+          <t>SSR103</t>
         </is>
       </c>
       <c r="C119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8036</t>
+          <t>VLINE-8029</t>
         </is>
       </c>
       <c r="D119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8157</t>
+          <t>VLINE-8152</t>
         </is>
       </c>
       <c r="E119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8418</t>
+          <t>VLINE-8411</t>
         </is>
       </c>
       <c r="F119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8725</t>
+          <t>VLINE-8717</t>
         </is>
       </c>
       <c r="G119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8792</t>
+          <t>VLINE-8786</t>
         </is>
       </c>
       <c r="H119" s="1" t="inlineStr">
         <is>
-          <t>XP2016</t>
+          <t>XP2012</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="1" t="inlineStr">
         <is>
-          <t>QR1771</t>
+          <t>QL011</t>
         </is>
       </c>
       <c r="B120" s="1" t="inlineStr">
         <is>
-          <t>TE2801</t>
+          <t>SSR104</t>
         </is>
       </c>
       <c r="C120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8038</t>
+          <t>VLINE-8030</t>
         </is>
       </c>
       <c r="D120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8158</t>
+          <t>VLINE-8153</t>
         </is>
       </c>
       <c r="E120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8419</t>
+          <t>VLINE-8413</t>
         </is>
       </c>
       <c r="F120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8726</t>
+          <t>VLINE-8720</t>
         </is>
       </c>
       <c r="G120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8793</t>
+          <t>VLINE-8787</t>
         </is>
       </c>
       <c r="H120" s="1" t="inlineStr">
         <is>
-          <t>XP2017</t>
+          <t>XP2013</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="1" t="inlineStr">
         <is>
-          <t>QR5404</t>
+          <t>QL014</t>
         </is>
       </c>
       <c r="B121" s="1" t="inlineStr">
         <is>
-          <t>TE2802</t>
+          <t>T363</t>
         </is>
       </c>
       <c r="C121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8042</t>
+          <t>VLINE-8031</t>
         </is>
       </c>
       <c r="D121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8159</t>
+          <t>VLINE-8154</t>
         </is>
       </c>
       <c r="E121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8420</t>
+          <t>VLINE-8415</t>
         </is>
       </c>
       <c r="F121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8727</t>
+          <t>VLINE-8721</t>
         </is>
       </c>
       <c r="G121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8794</t>
+          <t>VLINE-8788</t>
         </is>
       </c>
       <c r="H121" s="1" t="inlineStr">
         <is>
-          <t>XP2019</t>
+          <t>XP2014</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="1" t="inlineStr">
         <is>
-          <t>R711</t>
+          <t>QL018</t>
         </is>
       </c>
       <c r="B122" s="1" t="inlineStr">
         <is>
-          <t>TE2803</t>
+          <t>T386</t>
         </is>
       </c>
       <c r="C122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8051</t>
+          <t>VLINE-8032</t>
         </is>
       </c>
       <c r="D122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8160</t>
+          <t>VLINE-8155</t>
         </is>
       </c>
       <c r="E122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8421</t>
+          <t>VLINE-8417</t>
         </is>
       </c>
       <c r="F122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8729</t>
+          <t>VLINE-8723</t>
         </is>
       </c>
       <c r="G122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8795</t>
+          <t>VLINE-8790</t>
         </is>
       </c>
       <c r="H122" s="1" t="inlineStr">
         <is>
-          <t>XR552</t>
+          <t>XP2015</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="1" t="inlineStr">
         <is>
-          <t>R766</t>
+          <t>QR1744</t>
         </is>
       </c>
       <c r="B123" s="1" t="inlineStr">
         <is>
-          <t>TE2804</t>
+          <t>TDX101</t>
         </is>
       </c>
       <c r="C123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8052</t>
+          <t>VLINE-8036</t>
         </is>
       </c>
       <c r="D123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8161</t>
+          <t>VLINE-8157</t>
         </is>
       </c>
       <c r="E123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8422</t>
+          <t>VLINE-8418</t>
         </is>
       </c>
       <c r="F123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8730</t>
+          <t>VLINE-8725</t>
         </is>
       </c>
       <c r="G123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8796</t>
+          <t>VLINE-8792</t>
         </is>
       </c>
       <c r="H123" s="1" t="inlineStr">
         <is>
-          <t>XRN001</t>
+          <t>XP2016</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="1" t="inlineStr">
         <is>
-          <t>RB2353</t>
+          <t>QR1771</t>
         </is>
       </c>
       <c r="B124" s="1" t="inlineStr">
         <is>
-          <t>TE2805</t>
+          <t>TE2801</t>
         </is>
       </c>
       <c r="C124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8053</t>
+          <t>VLINE-8038</t>
         </is>
       </c>
       <c r="D124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8162</t>
+          <t>VLINE-8158</t>
         </is>
       </c>
       <c r="E124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8424</t>
+          <t>VLINE-8419</t>
         </is>
       </c>
       <c r="F124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8731</t>
+          <t>VLINE-8726</t>
         </is>
       </c>
       <c r="G124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8797</t>
+          <t>VLINE-8793</t>
         </is>
       </c>
       <c r="H124" s="1" t="inlineStr">
         <is>
-          <t>XRN004</t>
+          <t>XP2017</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="1" t="inlineStr">
         <is>
-          <t>RCTST4</t>
+          <t>QR5404</t>
         </is>
       </c>
       <c r="B125" s="1" t="inlineStr">
         <is>
-          <t>TE2806</t>
+          <t>TE2802</t>
         </is>
       </c>
       <c r="C125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8055</t>
+          <t>VLINE-8042</t>
         </is>
       </c>
       <c r="D125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8171</t>
+          <t>VLINE-8159</t>
         </is>
       </c>
       <c r="E125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8425</t>
+          <t>VLINE-8420</t>
         </is>
       </c>
       <c r="F125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8733</t>
+          <t>VLINE-8727</t>
         </is>
       </c>
       <c r="G125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8799</t>
+          <t>VLINE-8794</t>
         </is>
       </c>
       <c r="H125" s="1" t="inlineStr">
         <is>
-          <t>XRN005</t>
+          <t>XP2019</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="1" t="inlineStr">
         <is>
-          <t>RL301</t>
+          <t>R711</t>
         </is>
       </c>
       <c r="B126" s="1" t="inlineStr">
         <is>
-          <t>TE2807</t>
+          <t>TE2803</t>
         </is>
       </c>
       <c r="C126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8056</t>
+          <t>VLINE-8051</t>
         </is>
       </c>
       <c r="D126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8172</t>
+          <t>VLINE-8160</t>
         </is>
       </c>
       <c r="E126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8426</t>
+          <t>VLINE-8421</t>
         </is>
       </c>
       <c r="F126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8735</t>
+          <t>VLINE-8729</t>
         </is>
       </c>
       <c r="G126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8800</t>
+          <t>VLINE-8795</t>
         </is>
       </c>
       <c r="H126" s="1" t="inlineStr">
         <is>
-          <t>XRN006</t>
+          <t>XR552</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
         <is>
-          <t>RL302</t>
+          <t>R766</t>
         </is>
       </c>
       <c r="B127" s="1" t="inlineStr">
         <is>
-          <t>TE2808</t>
+          <t>TE2804</t>
         </is>
       </c>
       <c r="C127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8057</t>
+          <t>VLINE-8052</t>
         </is>
       </c>
       <c r="D127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8176</t>
+          <t>VLINE-8161</t>
         </is>
       </c>
       <c r="E127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8427</t>
+          <t>VLINE-8422</t>
         </is>
       </c>
       <c r="F127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8736</t>
+          <t>VLINE-8730</t>
         </is>
       </c>
       <c r="G127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8801</t>
+          <t>VLINE-8796</t>
         </is>
       </c>
       <c r="H127" s="1" t="inlineStr">
         <is>
-          <t>XRN007</t>
+          <t>XRN001</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
         <is>
-          <t>RL304</t>
+          <t>RB2353</t>
         </is>
       </c>
       <c r="B128" s="1" t="inlineStr">
         <is>
-          <t>TE2809</t>
+          <t>TE2805</t>
         </is>
       </c>
       <c r="C128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8058</t>
+          <t>VLINE-8053</t>
         </is>
       </c>
       <c r="D128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8179</t>
+          <t>VLINE-8162</t>
         </is>
       </c>
       <c r="E128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8428</t>
+          <t>VLINE-8424</t>
         </is>
       </c>
       <c r="F128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8737</t>
+          <t>VLINE-8731</t>
         </is>
       </c>
       <c r="G128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8802</t>
+          <t>VLINE-8797</t>
         </is>
       </c>
       <c r="H128" s="1" t="inlineStr">
         <is>
-          <t>XRN009</t>
+          <t>XRN004</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
         <is>
-          <t>RL305</t>
+          <t>RCTST4</t>
         </is>
       </c>
       <c r="B129" s="1" t="inlineStr">
         <is>
-          <t>TE2810</t>
+          <t>TE2806</t>
         </is>
       </c>
       <c r="C129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8059</t>
+          <t>VLINE-8055</t>
         </is>
       </c>
       <c r="D129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8180</t>
+          <t>VLINE-8171</t>
         </is>
       </c>
       <c r="E129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8429</t>
+          <t>VLINE-8425</t>
         </is>
       </c>
       <c r="F129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8739</t>
+          <t>VLINE-8733</t>
         </is>
       </c>
       <c r="G129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8803</t>
+          <t>VLINE-8799</t>
         </is>
       </c>
       <c r="H129" s="1" t="inlineStr">
         <is>
-          <t>XRN011</t>
+          <t>XRN005</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="1" t="inlineStr">
         <is>
-          <t>RL307</t>
+          <t>RL301</t>
         </is>
       </c>
       <c r="B130" s="1" t="inlineStr">
         <is>
-          <t>TE2812</t>
+          <t>TE2807</t>
         </is>
       </c>
       <c r="C130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8061</t>
+          <t>VLINE-8056</t>
         </is>
       </c>
       <c r="D130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8181</t>
+          <t>VLINE-8172</t>
         </is>
       </c>
       <c r="E130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8430</t>
+          <t>VLINE-8426</t>
         </is>
       </c>
       <c r="F130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8740</t>
+          <t>VLINE-8735</t>
         </is>
       </c>
       <c r="G130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8804</t>
+          <t>VLINE-8800</t>
         </is>
       </c>
       <c r="H130" s="1" t="inlineStr">
         <is>
-          <t>XRN014</t>
+          <t>XRN006</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="1" t="inlineStr">
         <is>
-          <t>RL309</t>
+          <t>RL302</t>
         </is>
       </c>
       <c r="B131" s="1" t="inlineStr">
         <is>
-          <t>TE2813</t>
+          <t>TE2808</t>
         </is>
       </c>
       <c r="C131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8072</t>
+          <t>VLINE-8057</t>
         </is>
       </c>
       <c r="D131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8182</t>
+          <t>VLINE-8176</t>
         </is>
       </c>
       <c r="E131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8431</t>
+          <t>VLINE-8427</t>
         </is>
       </c>
       <c r="F131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8741</t>
+          <t>VLINE-8736</t>
         </is>
       </c>
       <c r="G131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8805</t>
+          <t>VLINE-8801</t>
         </is>
       </c>
       <c r="H131" s="1" t="inlineStr">
         <is>
-          <t>XRN017</t>
+          <t>XRN007</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="1" t="inlineStr">
         <is>
-          <t>RL310</t>
+          <t>RL304</t>
         </is>
       </c>
       <c r="B132" s="1" t="inlineStr">
         <is>
-          <t>TE2814</t>
+          <t>TE2809</t>
         </is>
       </c>
       <c r="C132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8074</t>
+          <t>VLINE-8058</t>
         </is>
       </c>
       <c r="D132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8183</t>
+          <t>VLINE-8179</t>
         </is>
       </c>
       <c r="E132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8432</t>
+          <t>VLINE-8428</t>
         </is>
       </c>
       <c r="F132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8742</t>
+          <t>VLINE-8737</t>
         </is>
       </c>
       <c r="G132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8806</t>
+          <t>VLINE-8802</t>
         </is>
       </c>
       <c r="H132" s="1" t="inlineStr">
         <is>
-          <t>XRN018</t>
+          <t>XRN009</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="1" t="inlineStr">
         <is>
-          <t>S312</t>
+          <t>RL305</t>
         </is>
       </c>
       <c r="B133" s="1" t="inlineStr">
         <is>
-          <t>TJ096</t>
+          <t>TE2810</t>
         </is>
       </c>
       <c r="C133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8075</t>
+          <t>VLINE-8059</t>
         </is>
       </c>
       <c r="D133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8184</t>
+          <t>VLINE-8180</t>
         </is>
       </c>
       <c r="E133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8433</t>
+          <t>VLINE-8429</t>
         </is>
       </c>
       <c r="F133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8743</t>
+          <t>VLINE-8739</t>
         </is>
       </c>
       <c r="G133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8807</t>
+          <t>VLINE-8803</t>
         </is>
       </c>
       <c r="H133" s="1" t="inlineStr">
         <is>
-          <t>XRN020</t>
+          <t>XRN011</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="1" t="inlineStr">
         <is>
-          <t>S317</t>
+          <t>RL307</t>
         </is>
       </c>
       <c r="B134" s="1" t="inlineStr">
         <is>
-          <t>TJ107</t>
+          <t>TE2812</t>
         </is>
       </c>
       <c r="C134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8076</t>
+          <t>VLINE-8061</t>
         </is>
       </c>
       <c r="D134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8185</t>
+          <t>VLINE-8181</t>
         </is>
       </c>
       <c r="E134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8434</t>
+          <t>VLINE-8430</t>
         </is>
       </c>
       <c r="F134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8744</t>
+          <t>VLINE-8740</t>
         </is>
       </c>
       <c r="G134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8808</t>
+          <t>VLINE-8804</t>
         </is>
       </c>
       <c r="H134" s="1" t="inlineStr">
         <is>
-          <t>XRN021</t>
+          <t>XRN014</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="1" t="inlineStr">
         <is>
-          <t>S3301</t>
+          <t>RL309</t>
         </is>
       </c>
       <c r="B135" s="1" t="inlineStr">
         <is>
-          <t>TT03</t>
+          <t>TE2813</t>
         </is>
       </c>
       <c r="C135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8077</t>
+          <t>VLINE-8072</t>
         </is>
       </c>
       <c r="D135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8186</t>
+          <t>VLINE-8182</t>
         </is>
       </c>
       <c r="E135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8435</t>
+          <t>VLINE-8431</t>
         </is>
       </c>
       <c r="F135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8745</t>
+          <t>VLINE-8741</t>
         </is>
       </c>
       <c r="G135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8809</t>
+          <t>VLINE-8805</t>
         </is>
       </c>
       <c r="H135" s="1" t="inlineStr">
         <is>
-          <t>XRN023</t>
+          <t>XRN017</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="1" t="inlineStr">
         <is>
-          <t>S3302</t>
+          <t>RL310</t>
         </is>
       </c>
       <c r="B136" s="1" t="inlineStr">
         <is>
-          <t>TT04</t>
+          <t>TE2814</t>
         </is>
       </c>
       <c r="C136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8080</t>
+          <t>VLINE-8074</t>
         </is>
       </c>
       <c r="D136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8187</t>
+          <t>VLINE-8183</t>
         </is>
       </c>
       <c r="E136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8438</t>
+          <t>VLINE-8432</t>
         </is>
       </c>
       <c r="F136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8746</t>
+          <t>VLINE-8742</t>
         </is>
       </c>
       <c r="G136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8810</t>
+          <t>VLINE-8806</t>
         </is>
       </c>
       <c r="H136" s="1" t="inlineStr">
         <is>
-          <t>XRN025</t>
+          <t>XRN018</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="1" t="inlineStr">
         <is>
-          <t>S3304</t>
+          <t>S312</t>
         </is>
       </c>
       <c r="B137" s="1" t="inlineStr">
         <is>
-          <t>TT05</t>
+          <t>TJ096</t>
         </is>
       </c>
       <c r="C137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8081</t>
+          <t>VLINE-8075</t>
         </is>
       </c>
       <c r="D137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8188</t>
+          <t>VLINE-8184</t>
         </is>
       </c>
       <c r="E137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8440</t>
+          <t>VLINE-8433</t>
         </is>
       </c>
       <c r="F137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8747</t>
+          <t>VLINE-8743</t>
         </is>
       </c>
       <c r="G137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8811</t>
+          <t>VLINE-8807</t>
         </is>
       </c>
       <c r="H137" s="1" t="inlineStr">
         <is>
-          <t>XRN026</t>
+          <t>XRN020</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="1" t="inlineStr">
         <is>
-          <t>S3305</t>
+          <t>S317</t>
         </is>
       </c>
       <c r="B138" s="1" t="inlineStr">
         <is>
-          <t>TT07</t>
+          <t>TJ107</t>
         </is>
       </c>
       <c r="C138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8084</t>
+          <t>VLINE-8076</t>
         </is>
       </c>
       <c r="D138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8189</t>
+          <t>VLINE-8185</t>
         </is>
       </c>
       <c r="E138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8441</t>
+          <t>VLINE-8434</t>
         </is>
       </c>
       <c r="F138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8748</t>
+          <t>VLINE-8744</t>
         </is>
       </c>
       <c r="G138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8812</t>
+          <t>VLINE-8808</t>
         </is>
       </c>
       <c r="H138" s="1" t="inlineStr">
         <is>
-          <t>XRN027</t>
+          <t>XRN021</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="1" t="inlineStr">
         <is>
-          <t>S3306</t>
+          <t>S3301</t>
         </is>
       </c>
       <c r="B139" s="1" t="inlineStr">
         <is>
-          <t>TT08</t>
+          <t>TT03</t>
         </is>
       </c>
       <c r="C139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8088</t>
+          <t>VLINE-8077</t>
         </is>
       </c>
       <c r="D139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8291</t>
+          <t>VLINE-8186</t>
         </is>
       </c>
       <c r="E139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8442</t>
+          <t>VLINE-8435</t>
         </is>
       </c>
       <c r="F139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8749</t>
+          <t>VLINE-8745</t>
         </is>
       </c>
       <c r="G139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8813</t>
+          <t>VLINE-8809</t>
         </is>
       </c>
       <c r="H139" s="1" t="inlineStr">
         <is>
-          <t>Y163</t>
+          <t>XRN023</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="1" t="inlineStr">
         <is>
-          <t>S3307</t>
+          <t>S3302</t>
         </is>
       </c>
       <c r="B140" s="1" t="inlineStr">
         <is>
-          <t>TT103</t>
+          <t>TT04</t>
         </is>
       </c>
       <c r="C140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8089</t>
+          <t>VLINE-8080</t>
         </is>
       </c>
       <c r="D140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8293</t>
+          <t>VLINE-8187</t>
         </is>
       </c>
       <c r="E140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8443</t>
+          <t>VLINE-8438</t>
         </is>
       </c>
       <c r="F140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8750</t>
+          <t>VLINE-8746</t>
         </is>
       </c>
       <c r="G140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8814</t>
+          <t>VLINE-8810</t>
+        </is>
+      </c>
+      <c r="H140" s="1" t="inlineStr">
+        <is>
+          <t>XRN025</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="1" t="inlineStr">
         <is>
-          <t>S3309</t>
+          <t>S3304</t>
         </is>
       </c>
       <c r="B141" s="1" t="inlineStr">
         <is>
-          <t>TT106</t>
+          <t>TT05</t>
         </is>
       </c>
       <c r="C141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8104</t>
+          <t>VLINE-8081</t>
         </is>
       </c>
       <c r="D141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8303</t>
+          <t>VLINE-8188</t>
         </is>
       </c>
       <c r="E141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8444</t>
+          <t>VLINE-8440</t>
         </is>
       </c>
       <c r="F141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8751</t>
+          <t>VLINE-8747</t>
         </is>
       </c>
       <c r="G141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8816</t>
+          <t>VLINE-8811</t>
+        </is>
+      </c>
+      <c r="H141" s="1" t="inlineStr">
+        <is>
+          <t>XRN026</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="1" t="inlineStr">
         <is>
-          <t>S3310</t>
+          <t>S3305</t>
         </is>
       </c>
       <c r="B142" s="1" t="inlineStr">
         <is>
-          <t>TT107</t>
+          <t>TT07</t>
         </is>
       </c>
       <c r="C142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8107</t>
+          <t>VLINE-8084</t>
         </is>
       </c>
       <c r="D142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8304</t>
+          <t>VLINE-8189</t>
         </is>
       </c>
       <c r="E142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8446</t>
+          <t>VLINE-8441</t>
         </is>
       </c>
       <c r="F142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8752</t>
+          <t>VLINE-8748</t>
         </is>
       </c>
       <c r="G142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8817</t>
+          <t>VLINE-8812</t>
+        </is>
+      </c>
+      <c r="H142" s="1" t="inlineStr">
+        <is>
+          <t>XRN027</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="1" t="inlineStr">
         <is>
-          <t>S7001</t>
+          <t>S3306</t>
         </is>
       </c>
       <c r="B143" s="1" t="inlineStr">
         <is>
-          <t>TT108</t>
+          <t>TT08</t>
         </is>
       </c>
       <c r="C143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8110</t>
+          <t>VLINE-8088</t>
         </is>
       </c>
       <c r="D143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8306</t>
+          <t>VLINE-8291</t>
         </is>
       </c>
       <c r="E143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8447</t>
+          <t>VLINE-8442</t>
         </is>
       </c>
       <c r="F143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8753</t>
+          <t>VLINE-8749</t>
         </is>
       </c>
       <c r="G143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8818</t>
+          <t>VLINE-8813</t>
+        </is>
+      </c>
+      <c r="H143" s="1" t="inlineStr">
+        <is>
+          <t>Y163</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="1" t="inlineStr">
         <is>
-          <t>S7002</t>
+          <t>S3307</t>
         </is>
       </c>
       <c r="B144" s="1" t="inlineStr">
         <is>
-          <t>TT110</t>
+          <t>TT103</t>
         </is>
       </c>
       <c r="C144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8111</t>
+          <t>VLINE-8089</t>
         </is>
       </c>
       <c r="D144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8311</t>
+          <t>VLINE-8293</t>
         </is>
       </c>
       <c r="E144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8449</t>
+          <t>VLINE-8443</t>
         </is>
       </c>
       <c r="F144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8754</t>
+          <t>VLINE-8750</t>
         </is>
       </c>
       <c r="G144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8819</t>
+          <t>VLINE-8814</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="1" t="inlineStr">
         <is>
-          <t>S7003</t>
+          <t>S3309</t>
         </is>
       </c>
       <c r="B145" s="1" t="inlineStr">
         <is>
-          <t>TT113</t>
+          <t>TT106</t>
         </is>
       </c>
       <c r="C145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8113</t>
+          <t>VLINE-8104</t>
         </is>
       </c>
       <c r="D145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8313</t>
+          <t>VLINE-8303</t>
         </is>
       </c>
       <c r="E145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8450</t>
+          <t>VLINE-8444</t>
         </is>
       </c>
       <c r="F145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8755</t>
+          <t>VLINE-8751</t>
         </is>
       </c>
       <c r="G145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8822</t>
+          <t>VLINE-8816</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="1" t="inlineStr">
         <is>
-          <t>S7004</t>
+          <t>S3310</t>
         </is>
       </c>
       <c r="B146" s="1" t="inlineStr">
         <is>
-          <t>TT114</t>
+          <t>TT107</t>
         </is>
       </c>
       <c r="C146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8114</t>
+          <t>VLINE-8107</t>
         </is>
       </c>
       <c r="D146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8314</t>
+          <t>VLINE-8304</t>
         </is>
       </c>
       <c r="E146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8451</t>
+          <t>VLINE-8446</t>
         </is>
       </c>
       <c r="F146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8756</t>
+          <t>VLINE-8752</t>
         </is>
       </c>
       <c r="G146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8860</t>
+          <t>VLINE-8817</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="1" t="inlineStr">
         <is>
-          <t>S7005</t>
+          <t>S7001</t>
         </is>
       </c>
       <c r="B147" s="1" t="inlineStr">
         <is>
-          <t>TT115</t>
+          <t>TT108</t>
         </is>
       </c>
       <c r="C147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8115</t>
+          <t>VLINE-8110</t>
         </is>
       </c>
       <c r="D147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8316</t>
+          <t>VLINE-8306</t>
         </is>
       </c>
       <c r="E147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8452</t>
+          <t>VLINE-8447</t>
         </is>
       </c>
       <c r="F147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8757</t>
+          <t>VLINE-8753</t>
         </is>
       </c>
       <c r="G147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8861</t>
+          <t>VLINE-8818</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="1" t="inlineStr">
         <is>
-          <t>S7006</t>
+          <t>S7002</t>
         </is>
       </c>
       <c r="B148" s="1" t="inlineStr">
         <is>
-          <t>TT116</t>
+          <t>TT110</t>
         </is>
       </c>
       <c r="C148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8119</t>
+          <t>VLINE-8111</t>
         </is>
       </c>
       <c r="D148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8318</t>
+          <t>VLINE-8311</t>
         </is>
       </c>
       <c r="E148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8453</t>
+          <t>VLINE-8449</t>
         </is>
       </c>
       <c r="F148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8758</t>
+          <t>VLINE-8754</t>
         </is>
       </c>
       <c r="G148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8862</t>
+          <t>VLINE-8819</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="1" t="inlineStr">
         <is>
-          <t>S7007</t>
+          <t>S7003</t>
         </is>
       </c>
       <c r="B149" s="1" t="inlineStr">
         <is>
-          <t>TT117</t>
+          <t>TT113</t>
         </is>
       </c>
       <c r="C149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8120</t>
+          <t>VLINE-8113</t>
         </is>
       </c>
       <c r="D149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8321</t>
+          <t>VLINE-8313</t>
         </is>
       </c>
       <c r="E149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8454</t>
+          <t>VLINE-8450</t>
         </is>
       </c>
       <c r="F149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8759</t>
+          <t>VLINE-8755</t>
         </is>
       </c>
       <c r="G149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8863</t>
+          <t>VLINE-8822</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="1" t="inlineStr">
         <is>
-          <t>S7008</t>
+          <t>S7004</t>
         </is>
       </c>
       <c r="B150" s="1" t="inlineStr">
         <is>
-          <t>TT122</t>
+          <t>TT114</t>
         </is>
       </c>
       <c r="C150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8121</t>
+          <t>VLINE-8114</t>
         </is>
       </c>
       <c r="D150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8323</t>
+          <t>VLINE-8314</t>
         </is>
       </c>
       <c r="E150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8455</t>
+          <t>VLINE-8451</t>
         </is>
       </c>
       <c r="F150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8760</t>
+          <t>VLINE-8756</t>
         </is>
       </c>
       <c r="G150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8864</t>
+          <t>VLINE-8860</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="1" t="inlineStr">
         <is>
-          <t>S7012</t>
+          <t>S7005</t>
         </is>
       </c>
       <c r="B151" s="1" t="inlineStr">
         <is>
-          <t>TT127</t>
+          <t>TT115</t>
         </is>
       </c>
       <c r="C151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8123</t>
+          <t>VLINE-8115</t>
         </is>
       </c>
       <c r="D151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8324</t>
+          <t>VLINE-8316</t>
         </is>
       </c>
       <c r="E151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8456</t>
+          <t>VLINE-8452</t>
         </is>
       </c>
       <c r="F151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8761</t>
+          <t>VLINE-8757</t>
         </is>
       </c>
       <c r="G151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8865</t>
+          <t>VLINE-8861</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="1" t="inlineStr">
         <is>
-          <t>S7013</t>
+          <t>S7006</t>
         </is>
       </c>
       <c r="B152" s="1" t="inlineStr">
         <is>
-          <t>TT128</t>
+          <t>TT116</t>
         </is>
       </c>
       <c r="C152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8124</t>
+          <t>VLINE-8119</t>
         </is>
       </c>
       <c r="D152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8325</t>
+          <t>VLINE-8318</t>
         </is>
       </c>
       <c r="E152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8457</t>
+          <t>VLINE-8453</t>
         </is>
       </c>
       <c r="F152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8762</t>
+          <t>VLINE-8758</t>
         </is>
       </c>
       <c r="G152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8866</t>
+          <t>VLINE-8862</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="1" t="inlineStr">
         <is>
-          <t>S7014</t>
+          <t>S7007</t>
         </is>
       </c>
       <c r="B153" s="1" t="inlineStr">
         <is>
-          <t>TT130</t>
+          <t>TT117</t>
         </is>
       </c>
       <c r="C153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8126</t>
+          <t>VLINE-8120</t>
         </is>
       </c>
       <c r="D153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8328</t>
+          <t>VLINE-8321</t>
         </is>
       </c>
       <c r="E153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8460</t>
+          <t>VLINE-8454</t>
         </is>
       </c>
       <c r="F153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8763</t>
+          <t>VLINE-8759</t>
         </is>
       </c>
       <c r="G153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8867</t>
+          <t>VLINE-8863</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="1" t="inlineStr">
         <is>
-          <t>S7015</t>
+          <t>S7008</t>
         </is>
       </c>
       <c r="B154" s="1" t="inlineStr">
         <is>
-          <t>TT131</t>
+          <t>TT122</t>
         </is>
       </c>
       <c r="C154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8127</t>
+          <t>VLINE-8121</t>
         </is>
       </c>
       <c r="D154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8329</t>
+          <t>VLINE-8323</t>
         </is>
       </c>
       <c r="E154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8461</t>
+          <t>VLINE-8455</t>
         </is>
       </c>
       <c r="F154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8765</t>
+          <t>VLINE-8760</t>
         </is>
       </c>
       <c r="G154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8868</t>
+          <t>VLINE-8864</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="1" t="inlineStr">
         <is>
-          <t>S7017</t>
+          <t>S7012</t>
         </is>
       </c>
       <c r="B155" s="1" t="inlineStr">
         <is>
-          <t>TT202</t>
+          <t>TT127</t>
         </is>
       </c>
       <c r="C155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8128</t>
+          <t>VLINE-8123</t>
         </is>
       </c>
       <c r="D155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8332</t>
+          <t>VLINE-8324</t>
         </is>
       </c>
       <c r="E155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8464</t>
+          <t>VLINE-8456</t>
         </is>
       </c>
       <c r="F155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8766</t>
+          <t>VLINE-8761</t>
         </is>
       </c>
       <c r="G155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8869</t>
+          <t>VLINE-8865</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="1" t="inlineStr">
         <is>
-          <t>S7018</t>
+          <t>S7013</t>
         </is>
       </c>
       <c r="B156" s="1" t="inlineStr">
         <is>
-          <t>TT206</t>
+          <t>TT128</t>
         </is>
       </c>
       <c r="C156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8129</t>
+          <t>VLINE-8124</t>
         </is>
       </c>
       <c r="D156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8336</t>
+          <t>VLINE-8325</t>
         </is>
       </c>
       <c r="E156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8465</t>
+          <t>VLINE-8457</t>
         </is>
       </c>
       <c r="F156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8767</t>
+          <t>VLINE-8762</t>
         </is>
       </c>
       <c r="G156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8890</t>
+          <t>VLINE-8866</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="1" t="inlineStr">
         <is>
-          <t>S7020</t>
+          <t>S7014</t>
         </is>
       </c>
       <c r="B157" s="1" t="inlineStr">
         <is>
-          <t>VL352</t>
+          <t>TT130</t>
         </is>
       </c>
       <c r="C157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8131</t>
+          <t>VLINE-8126</t>
         </is>
       </c>
       <c r="D157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8337</t>
+          <t>VLINE-8328</t>
         </is>
       </c>
       <c r="E157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8468</t>
+          <t>VLINE-8460</t>
         </is>
       </c>
       <c r="F157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8768</t>
+          <t>VLINE-8763</t>
         </is>
       </c>
       <c r="G157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8891</t>
+          <t>VLINE-8867</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="1" t="inlineStr">
         <is>
-          <t>S7022</t>
+          <t>S7015</t>
         </is>
       </c>
       <c r="B158" s="1" t="inlineStr">
         <is>
-          <t>VL353</t>
+          <t>TT131</t>
         </is>
       </c>
       <c r="C158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8132</t>
+          <t>VLINE-8127</t>
         </is>
       </c>
       <c r="D158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8338</t>
+          <t>VLINE-8329</t>
         </is>
       </c>
       <c r="E158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8469</t>
+          <t>VLINE-8461</t>
         </is>
       </c>
       <c r="F158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8769</t>
+          <t>VLINE-8765</t>
         </is>
       </c>
       <c r="G158" s="1" t="inlineStr">
         <is>
-          <t>WH001</t>
+          <t>VLINE-8868</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="1" t="inlineStr">
         <is>
-          <t>SCT001</t>
+          <t>S7017</t>
         </is>
       </c>
       <c r="B159" s="1" t="inlineStr">
         <is>
-          <t>VL357</t>
+          <t>TT202</t>
         </is>
       </c>
       <c r="C159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8133</t>
+          <t>VLINE-8128</t>
         </is>
       </c>
       <c r="D159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8339</t>
+          <t>VLINE-8332</t>
         </is>
       </c>
       <c r="E159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8605</t>
+          <t>VLINE-8464</t>
         </is>
       </c>
       <c r="F159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8770</t>
+          <t>VLINE-8766</t>
         </is>
       </c>
       <c r="G159" s="1" t="inlineStr">
         <is>
-          <t>WH003</t>
+          <t>VLINE-8869</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="1" t="inlineStr">
         <is>
-          <t>SCT002</t>
+          <t>S7018</t>
         </is>
       </c>
       <c r="B160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8004</t>
+          <t>TT206</t>
         </is>
       </c>
       <c r="C160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8134</t>
+          <t>VLINE-8129</t>
         </is>
       </c>
       <c r="D160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8362</t>
+          <t>VLINE-8336</t>
         </is>
       </c>
       <c r="E160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8610</t>
+          <t>VLINE-8465</t>
         </is>
       </c>
       <c r="F160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8772</t>
+          <t>VLINE-8767</t>
         </is>
       </c>
       <c r="G160" s="1" t="inlineStr">
         <is>
-          <t>WL02</t>
+          <t>VLINE-8890</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="1" t="inlineStr">
         <is>
-          <t>SCT006</t>
+          <t>S7020</t>
         </is>
       </c>
       <c r="B161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8007</t>
+          <t>VL352</t>
         </is>
       </c>
       <c r="C161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8136</t>
+          <t>VLINE-8131</t>
         </is>
       </c>
       <c r="D161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8363</t>
+          <t>VLINE-8337</t>
         </is>
       </c>
       <c r="E161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8612</t>
+          <t>VLINE-8468</t>
         </is>
       </c>
       <c r="F161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8773</t>
+          <t>VLINE-8768</t>
         </is>
       </c>
       <c r="G161" s="1" t="inlineStr">
         <is>
-          <t>X12-X14</t>
+          <t>VLINE-8891</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="1" t="inlineStr">
         <is>
-          <t>SCT007</t>
+          <t>S7022</t>
         </is>
       </c>
       <c r="B162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8011</t>
+          <t>VL353</t>
         </is>
       </c>
       <c r="C162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8137</t>
+          <t>VLINE-8132</t>
         </is>
       </c>
       <c r="D162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8365</t>
+          <t>VLINE-8338</t>
         </is>
       </c>
       <c r="E162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8615</t>
+          <t>VLINE-8469</t>
         </is>
       </c>
       <c r="F162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8774</t>
+          <t>VLINE-8769</t>
         </is>
       </c>
       <c r="G162" s="1" t="inlineStr">
         <is>
-          <t>X31</t>
+          <t>WH001</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="1" t="inlineStr">
         <is>
-          <t>SCT009</t>
+          <t>SCT001</t>
         </is>
       </c>
       <c r="B163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8013</t>
+          <t>VL357</t>
         </is>
       </c>
       <c r="C163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8140</t>
+          <t>VLINE-8133</t>
         </is>
       </c>
       <c r="D163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8366</t>
+          <t>VLINE-8339</t>
         </is>
       </c>
       <c r="E163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8617</t>
+          <t>VLINE-8605</t>
         </is>
       </c>
       <c r="F163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8776</t>
+          <t>VLINE-8770</t>
         </is>
       </c>
       <c r="G163" s="1" t="inlineStr">
         <is>
-          <t>XP2000</t>
+          <t>WH003</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="1" t="inlineStr">
         <is>
-          <t>SCT011</t>
+          <t>SCT002</t>
         </is>
       </c>
       <c r="B164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8019</t>
+          <t>VLINE-8004</t>
         </is>
       </c>
       <c r="C164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8141</t>
+          <t>VLINE-8134</t>
         </is>
       </c>
       <c r="D164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8368</t>
+          <t>VLINE-8362</t>
         </is>
       </c>
       <c r="E164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8620</t>
+          <t>VLINE-8610</t>
         </is>
       </c>
       <c r="F164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8778</t>
+          <t>VLINE-8772</t>
         </is>
       </c>
       <c r="G164" s="1" t="inlineStr">
         <is>
-          <t>XP2003</t>
+          <t>WL02</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="1" t="inlineStr">
         <is>
-          <t>SCT013</t>
+          <t>SCT006</t>
         </is>
       </c>
       <c r="B165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8020</t>
+          <t>VLINE-8007</t>
         </is>
       </c>
       <c r="C165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8142</t>
+          <t>VLINE-8136</t>
         </is>
       </c>
       <c r="D165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8369</t>
+          <t>VLINE-8363</t>
         </is>
       </c>
       <c r="E165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8625</t>
+          <t>VLINE-8612</t>
         </is>
       </c>
       <c r="F165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8779</t>
+          <t>VLINE-8773</t>
         </is>
       </c>
       <c r="G165" s="1" t="inlineStr">
         <is>
-          <t>XP2004</t>
+          <t>X12-X14</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="1" t="inlineStr">
         <is>
-          <t>SCT014</t>
+          <t>SCT007</t>
         </is>
       </c>
       <c r="B166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8023</t>
+          <t>VLINE-8011</t>
         </is>
       </c>
       <c r="C166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8144</t>
+          <t>VLINE-8137</t>
         </is>
       </c>
       <c r="D166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8403</t>
+          <t>VLINE-8365</t>
         </is>
       </c>
       <c r="E166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8630</t>
+          <t>VLINE-8615</t>
         </is>
       </c>
       <c r="F166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8780</t>
+          <t>VLINE-8774</t>
         </is>
       </c>
       <c r="G166" s="1" t="inlineStr">
         <is>
-          <t>XP2005</t>
+          <t>X31</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="1" t="inlineStr">
         <is>
-          <t>SCT015</t>
+          <t>SCT009</t>
         </is>
       </c>
       <c r="B167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8025</t>
+          <t>VLINE-8013</t>
         </is>
       </c>
       <c r="C167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8145</t>
+          <t>VLINE-8140</t>
         </is>
       </c>
       <c r="D167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8404</t>
+          <t>VLINE-8366</t>
         </is>
       </c>
       <c r="E167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8671</t>
+          <t>VLINE-8617</t>
         </is>
       </c>
       <c r="F167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8781</t>
+          <t>VLINE-8776</t>
         </is>
       </c>
       <c r="G167" s="1" t="inlineStr">
         <is>
-          <t>XP2007</t>
+          <t>XP2000</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="1" t="inlineStr">
         <is>
-          <t>SO2</t>
+          <t>SCT011</t>
         </is>
       </c>
       <c r="B168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8026</t>
+          <t>VLINE-8019</t>
         </is>
       </c>
       <c r="C168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8148</t>
+          <t>VLINE-8141</t>
         </is>
       </c>
       <c r="D168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8406</t>
+          <t>VLINE-8368</t>
         </is>
       </c>
       <c r="E168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8706</t>
+          <t>VLINE-8620</t>
         </is>
       </c>
       <c r="F168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8782</t>
+          <t>VLINE-8778</t>
         </is>
       </c>
       <c r="G168" s="1" t="inlineStr">
         <is>
-          <t>XP2008</t>
+          <t>XP2003</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="1" t="inlineStr">
         <is>
-          <t>SSR101</t>
+          <t>SCT013</t>
         </is>
       </c>
       <c r="B169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8027</t>
+          <t>VLINE-8020</t>
         </is>
       </c>
       <c r="C169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8150</t>
+          <t>VLINE-8142</t>
         </is>
       </c>
       <c r="D169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8408</t>
+          <t>VLINE-8369</t>
         </is>
       </c>
       <c r="E169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8711</t>
+          <t>VLINE-8625</t>
         </is>
       </c>
       <c r="F169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8783</t>
+          <t>VLINE-8779</t>
         </is>
       </c>
       <c r="G169" s="1" t="inlineStr">
         <is>
-          <t>XP2010</t>
+          <t>XP2004</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="1" t="inlineStr">
         <is>
-          <t>SSR102</t>
+          <t>SCT014</t>
         </is>
       </c>
       <c r="B170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8028</t>
+          <t>VLINE-8023</t>
         </is>
       </c>
       <c r="C170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8151</t>
+          <t>VLINE-8144</t>
         </is>
       </c>
       <c r="D170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8410</t>
+          <t>VLINE-8403</t>
         </is>
       </c>
       <c r="E170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8714</t>
+          <t>VLINE-8630</t>
         </is>
       </c>
       <c r="F170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8784</t>
+          <t>VLINE-8780</t>
         </is>
       </c>
       <c r="G170" s="1" t="inlineStr">
         <is>
-          <t>XP2011</t>
+          <t>XP2005</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update loco downloads 2026-04-06 12:42:10
</commit_message>
<xml_diff>
--- a/downloads/loco_numbers_only.xlsx
+++ b/downloads/loco_numbers_only.xlsx
@@ -5141,37 +5141,37 @@
       </c>
       <c r="B115" s="1" t="inlineStr">
         <is>
-          <t>P2513</t>
+          <t>P2511</t>
         </is>
       </c>
       <c r="C115" s="1" t="inlineStr">
         <is>
-          <t>RL307</t>
+          <t>RL306</t>
         </is>
       </c>
       <c r="D115" s="1" t="inlineStr">
         <is>
-          <t>TE2808</t>
+          <t>TE2807</t>
         </is>
       </c>
       <c r="E115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8052</t>
+          <t>VLINE-8051</t>
         </is>
       </c>
       <c r="F115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8161</t>
+          <t>VLINE-8160</t>
         </is>
       </c>
       <c r="G115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8422</t>
+          <t>VLINE-8421</t>
         </is>
       </c>
       <c r="H115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8730</t>
+          <t>VLINE-8729</t>
         </is>
       </c>
     </row>
@@ -5183,37 +5183,37 @@
       </c>
       <c r="B116" s="1" t="inlineStr">
         <is>
-          <t>P2514</t>
+          <t>P2513</t>
         </is>
       </c>
       <c r="C116" s="1" t="inlineStr">
         <is>
-          <t>RL309</t>
+          <t>RL307</t>
         </is>
       </c>
       <c r="D116" s="1" t="inlineStr">
         <is>
-          <t>TE2809</t>
+          <t>TE2808</t>
         </is>
       </c>
       <c r="E116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8053</t>
+          <t>VLINE-8052</t>
         </is>
       </c>
       <c r="F116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8162</t>
+          <t>VLINE-8161</t>
         </is>
       </c>
       <c r="G116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8424</t>
+          <t>VLINE-8422</t>
         </is>
       </c>
       <c r="H116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8731</t>
+          <t>VLINE-8730</t>
         </is>
       </c>
     </row>
@@ -5225,37 +5225,37 @@
       </c>
       <c r="B117" s="1" t="inlineStr">
         <is>
-          <t>P2515</t>
+          <t>P2514</t>
         </is>
       </c>
       <c r="C117" s="1" t="inlineStr">
         <is>
-          <t>RL310</t>
+          <t>RL309</t>
         </is>
       </c>
       <c r="D117" s="1" t="inlineStr">
         <is>
-          <t>TE2810</t>
+          <t>TE2809</t>
         </is>
       </c>
       <c r="E117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8055</t>
+          <t>VLINE-8053</t>
         </is>
       </c>
       <c r="F117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8171</t>
+          <t>VLINE-8162</t>
         </is>
       </c>
       <c r="G117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8425</t>
+          <t>VLINE-8424</t>
         </is>
       </c>
       <c r="H117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8733</t>
+          <t>VLINE-8731</t>
         </is>
       </c>
     </row>
@@ -5267,37 +5267,37 @@
       </c>
       <c r="B118" s="1" t="inlineStr">
         <is>
-          <t>P2516</t>
+          <t>P2515</t>
         </is>
       </c>
       <c r="C118" s="1" t="inlineStr">
         <is>
-          <t>S312</t>
+          <t>RL310</t>
         </is>
       </c>
       <c r="D118" s="1" t="inlineStr">
         <is>
-          <t>TE2812</t>
+          <t>TE2810</t>
         </is>
       </c>
       <c r="E118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8056</t>
+          <t>VLINE-8055</t>
         </is>
       </c>
       <c r="F118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8172</t>
+          <t>VLINE-8171</t>
         </is>
       </c>
       <c r="G118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8426</t>
+          <t>VLINE-8425</t>
         </is>
       </c>
       <c r="H118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8735</t>
+          <t>VLINE-8733</t>
         </is>
       </c>
     </row>
@@ -5309,37 +5309,37 @@
       </c>
       <c r="B119" s="1" t="inlineStr">
         <is>
-          <t>PB1</t>
+          <t>P2516</t>
         </is>
       </c>
       <c r="C119" s="1" t="inlineStr">
         <is>
-          <t>S317</t>
+          <t>S312</t>
         </is>
       </c>
       <c r="D119" s="1" t="inlineStr">
         <is>
-          <t>TE2813</t>
+          <t>TE2812</t>
         </is>
       </c>
       <c r="E119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8057</t>
+          <t>VLINE-8056</t>
         </is>
       </c>
       <c r="F119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8176</t>
+          <t>VLINE-8172</t>
         </is>
       </c>
       <c r="G119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8427</t>
+          <t>VLINE-8426</t>
         </is>
       </c>
       <c r="H119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8736</t>
+          <t>VLINE-8735</t>
         </is>
       </c>
     </row>
@@ -5351,37 +5351,37 @@
       </c>
       <c r="B120" s="1" t="inlineStr">
         <is>
-          <t>PB2</t>
+          <t>PB1</t>
         </is>
       </c>
       <c r="C120" s="1" t="inlineStr">
         <is>
-          <t>S3301</t>
+          <t>S317</t>
         </is>
       </c>
       <c r="D120" s="1" t="inlineStr">
         <is>
-          <t>TE2814</t>
+          <t>TE2813</t>
         </is>
       </c>
       <c r="E120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8058</t>
+          <t>VLINE-8057</t>
         </is>
       </c>
       <c r="F120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8179</t>
+          <t>VLINE-8176</t>
         </is>
       </c>
       <c r="G120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8428</t>
+          <t>VLINE-8427</t>
         </is>
       </c>
       <c r="H120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8737</t>
+          <t>VLINE-8736</t>
         </is>
       </c>
     </row>
@@ -5393,37 +5393,37 @@
       </c>
       <c r="B121" s="1" t="inlineStr">
         <is>
-          <t>PB4</t>
+          <t>PB2</t>
         </is>
       </c>
       <c r="C121" s="1" t="inlineStr">
         <is>
-          <t>S3302</t>
+          <t>S3301</t>
         </is>
       </c>
       <c r="D121" s="1" t="inlineStr">
         <is>
-          <t>TJ096</t>
+          <t>TE2814</t>
         </is>
       </c>
       <c r="E121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8059</t>
+          <t>VLINE-8058</t>
         </is>
       </c>
       <c r="F121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8180</t>
+          <t>VLINE-8179</t>
         </is>
       </c>
       <c r="G121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8429</t>
+          <t>VLINE-8428</t>
         </is>
       </c>
       <c r="H121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8739</t>
+          <t>VLINE-8737</t>
         </is>
       </c>
     </row>
@@ -5435,37 +5435,37 @@
       </c>
       <c r="B122" s="1" t="inlineStr">
         <is>
-          <t>PHC001</t>
+          <t>PB4</t>
         </is>
       </c>
       <c r="C122" s="1" t="inlineStr">
         <is>
-          <t>S3304</t>
+          <t>S3302</t>
         </is>
       </c>
       <c r="D122" s="1" t="inlineStr">
         <is>
-          <t>TJ107</t>
+          <t>TJ096</t>
         </is>
       </c>
       <c r="E122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8061</t>
+          <t>VLINE-8059</t>
         </is>
       </c>
       <c r="F122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8181</t>
+          <t>VLINE-8180</t>
         </is>
       </c>
       <c r="G122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8430</t>
+          <t>VLINE-8429</t>
         </is>
       </c>
       <c r="H122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8740</t>
+          <t>VLINE-8739</t>
         </is>
       </c>
     </row>
@@ -5477,37 +5477,37 @@
       </c>
       <c r="B123" s="1" t="inlineStr">
         <is>
-          <t>PHC002</t>
+          <t>PHC001</t>
         </is>
       </c>
       <c r="C123" s="1" t="inlineStr">
         <is>
-          <t>S3305</t>
+          <t>S3304</t>
         </is>
       </c>
       <c r="D123" s="1" t="inlineStr">
         <is>
-          <t>TT03</t>
+          <t>TJ107</t>
         </is>
       </c>
       <c r="E123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8072</t>
+          <t>VLINE-8061</t>
         </is>
       </c>
       <c r="F123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8182</t>
+          <t>VLINE-8181</t>
         </is>
       </c>
       <c r="G123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8431</t>
+          <t>VLINE-8430</t>
         </is>
       </c>
       <c r="H123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8741</t>
+          <t>VLINE-8740</t>
         </is>
       </c>
     </row>
@@ -5519,37 +5519,37 @@
       </c>
       <c r="B124" s="1" t="inlineStr">
         <is>
-          <t>Q4001</t>
+          <t>PHC002</t>
         </is>
       </c>
       <c r="C124" s="1" t="inlineStr">
         <is>
-          <t>S3306</t>
+          <t>S3305</t>
         </is>
       </c>
       <c r="D124" s="1" t="inlineStr">
         <is>
-          <t>TT04</t>
+          <t>TT03</t>
         </is>
       </c>
       <c r="E124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8074</t>
+          <t>VLINE-8072</t>
         </is>
       </c>
       <c r="F124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8183</t>
+          <t>VLINE-8182</t>
         </is>
       </c>
       <c r="G124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8432</t>
+          <t>VLINE-8431</t>
         </is>
       </c>
       <c r="H124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8742</t>
+          <t>VLINE-8741</t>
         </is>
       </c>
     </row>
@@ -5561,37 +5561,37 @@
       </c>
       <c r="B125" s="1" t="inlineStr">
         <is>
-          <t>Q4003</t>
+          <t>Q4001</t>
         </is>
       </c>
       <c r="C125" s="1" t="inlineStr">
         <is>
-          <t>S3307</t>
+          <t>S3306</t>
         </is>
       </c>
       <c r="D125" s="1" t="inlineStr">
         <is>
-          <t>TT05</t>
+          <t>TT04</t>
         </is>
       </c>
       <c r="E125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8075</t>
+          <t>VLINE-8074</t>
         </is>
       </c>
       <c r="F125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8184</t>
+          <t>VLINE-8183</t>
         </is>
       </c>
       <c r="G125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8433</t>
+          <t>VLINE-8432</t>
         </is>
       </c>
       <c r="H125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8743</t>
+          <t>VLINE-8742</t>
         </is>
       </c>
     </row>
@@ -5603,37 +5603,37 @@
       </c>
       <c r="B126" s="1" t="inlineStr">
         <is>
-          <t>Q4004</t>
+          <t>Q4003</t>
         </is>
       </c>
       <c r="C126" s="1" t="inlineStr">
         <is>
-          <t>S3309</t>
+          <t>S3307</t>
         </is>
       </c>
       <c r="D126" s="1" t="inlineStr">
         <is>
-          <t>TT07</t>
+          <t>TT05</t>
         </is>
       </c>
       <c r="E126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8076</t>
+          <t>VLINE-8075</t>
         </is>
       </c>
       <c r="F126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8185</t>
+          <t>VLINE-8184</t>
         </is>
       </c>
       <c r="G126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8434</t>
+          <t>VLINE-8433</t>
         </is>
       </c>
       <c r="H126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8744</t>
+          <t>VLINE-8743</t>
         </is>
       </c>
     </row>
@@ -5645,37 +5645,37 @@
       </c>
       <c r="B127" s="1" t="inlineStr">
         <is>
-          <t>Q4005</t>
+          <t>Q4004</t>
         </is>
       </c>
       <c r="C127" s="1" t="inlineStr">
         <is>
-          <t>S3310</t>
+          <t>S3309</t>
         </is>
       </c>
       <c r="D127" s="1" t="inlineStr">
         <is>
-          <t>TT08</t>
+          <t>TT07</t>
         </is>
       </c>
       <c r="E127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8077</t>
+          <t>VLINE-8076</t>
         </is>
       </c>
       <c r="F127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8186</t>
+          <t>VLINE-8185</t>
         </is>
       </c>
       <c r="G127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8435</t>
+          <t>VLINE-8434</t>
         </is>
       </c>
       <c r="H127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8745</t>
+          <t>VLINE-8744</t>
         </is>
       </c>
     </row>
@@ -5687,37 +5687,37 @@
       </c>
       <c r="B128" s="1" t="inlineStr">
         <is>
-          <t>Q4006</t>
+          <t>Q4005</t>
         </is>
       </c>
       <c r="C128" s="1" t="inlineStr">
         <is>
-          <t>S7001</t>
+          <t>S3310</t>
         </is>
       </c>
       <c r="D128" s="1" t="inlineStr">
         <is>
-          <t>TT103</t>
+          <t>TT08</t>
         </is>
       </c>
       <c r="E128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8080</t>
+          <t>VLINE-8077</t>
         </is>
       </c>
       <c r="F128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8187</t>
+          <t>VLINE-8186</t>
         </is>
       </c>
       <c r="G128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8438</t>
+          <t>VLINE-8435</t>
         </is>
       </c>
       <c r="H128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8746</t>
+          <t>VLINE-8745</t>
         </is>
       </c>
     </row>
@@ -5729,37 +5729,37 @@
       </c>
       <c r="B129" s="1" t="inlineStr">
         <is>
-          <t>Q4007</t>
+          <t>Q4006</t>
         </is>
       </c>
       <c r="C129" s="1" t="inlineStr">
         <is>
-          <t>S7002</t>
+          <t>S7001</t>
         </is>
       </c>
       <c r="D129" s="1" t="inlineStr">
         <is>
-          <t>TT106</t>
+          <t>TT103</t>
         </is>
       </c>
       <c r="E129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8081</t>
+          <t>VLINE-8080</t>
         </is>
       </c>
       <c r="F129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8188</t>
+          <t>VLINE-8187</t>
         </is>
       </c>
       <c r="G129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8440</t>
+          <t>VLINE-8438</t>
         </is>
       </c>
       <c r="H129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8747</t>
+          <t>VLINE-8746</t>
         </is>
       </c>
     </row>
@@ -5771,37 +5771,37 @@
       </c>
       <c r="B130" s="1" t="inlineStr">
         <is>
-          <t>Q4009</t>
+          <t>Q4007</t>
         </is>
       </c>
       <c r="C130" s="1" t="inlineStr">
         <is>
-          <t>S7003</t>
+          <t>S7002</t>
         </is>
       </c>
       <c r="D130" s="1" t="inlineStr">
         <is>
-          <t>TT107</t>
+          <t>TT106</t>
         </is>
       </c>
       <c r="E130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8084</t>
+          <t>VLINE-8081</t>
         </is>
       </c>
       <c r="F130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8189</t>
+          <t>VLINE-8188</t>
         </is>
       </c>
       <c r="G130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8441</t>
+          <t>VLINE-8440</t>
         </is>
       </c>
       <c r="H130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8748</t>
+          <t>VLINE-8747</t>
         </is>
       </c>
     </row>
@@ -5813,37 +5813,37 @@
       </c>
       <c r="B131" s="1" t="inlineStr">
         <is>
-          <t>Q4011</t>
+          <t>Q4009</t>
         </is>
       </c>
       <c r="C131" s="1" t="inlineStr">
         <is>
-          <t>S7004</t>
+          <t>S7003</t>
         </is>
       </c>
       <c r="D131" s="1" t="inlineStr">
         <is>
-          <t>TT108</t>
+          <t>TT107</t>
         </is>
       </c>
       <c r="E131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8088</t>
+          <t>VLINE-8084</t>
         </is>
       </c>
       <c r="F131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8291</t>
+          <t>VLINE-8189</t>
         </is>
       </c>
       <c r="G131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8442</t>
+          <t>VLINE-8441</t>
         </is>
       </c>
       <c r="H131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8749</t>
+          <t>VLINE-8748</t>
         </is>
       </c>
     </row>
@@ -5855,37 +5855,37 @@
       </c>
       <c r="B132" s="1" t="inlineStr">
         <is>
-          <t>Q4012</t>
+          <t>Q4011</t>
         </is>
       </c>
       <c r="C132" s="1" t="inlineStr">
         <is>
-          <t>S7005</t>
+          <t>S7004</t>
         </is>
       </c>
       <c r="D132" s="1" t="inlineStr">
         <is>
-          <t>TT110</t>
+          <t>TT108</t>
         </is>
       </c>
       <c r="E132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8089</t>
+          <t>VLINE-8088</t>
         </is>
       </c>
       <c r="F132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8293</t>
+          <t>VLINE-8291</t>
         </is>
       </c>
       <c r="G132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8443</t>
+          <t>VLINE-8442</t>
         </is>
       </c>
       <c r="H132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8750</t>
+          <t>VLINE-8749</t>
         </is>
       </c>
     </row>
@@ -5897,37 +5897,37 @@
       </c>
       <c r="B133" s="1" t="inlineStr">
         <is>
-          <t>Q4013</t>
+          <t>Q4012</t>
         </is>
       </c>
       <c r="C133" s="1" t="inlineStr">
         <is>
-          <t>S7006</t>
+          <t>S7005</t>
         </is>
       </c>
       <c r="D133" s="1" t="inlineStr">
         <is>
-          <t>TT113</t>
+          <t>TT110</t>
         </is>
       </c>
       <c r="E133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8104</t>
+          <t>VLINE-8089</t>
         </is>
       </c>
       <c r="F133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8303</t>
+          <t>VLINE-8293</t>
         </is>
       </c>
       <c r="G133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8444</t>
+          <t>VLINE-8443</t>
         </is>
       </c>
       <c r="H133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8751</t>
+          <t>VLINE-8750</t>
         </is>
       </c>
     </row>
@@ -5939,37 +5939,37 @@
       </c>
       <c r="B134" s="1" t="inlineStr">
         <is>
-          <t>Q4014</t>
+          <t>Q4013</t>
         </is>
       </c>
       <c r="C134" s="1" t="inlineStr">
         <is>
-          <t>S7007</t>
+          <t>S7006</t>
         </is>
       </c>
       <c r="D134" s="1" t="inlineStr">
         <is>
-          <t>TT114</t>
+          <t>TT113</t>
         </is>
       </c>
       <c r="E134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8107</t>
+          <t>VLINE-8104</t>
         </is>
       </c>
       <c r="F134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8304</t>
+          <t>VLINE-8303</t>
         </is>
       </c>
       <c r="G134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8446</t>
+          <t>VLINE-8444</t>
         </is>
       </c>
       <c r="H134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8752</t>
+          <t>VLINE-8751</t>
         </is>
       </c>
     </row>
@@ -5981,37 +5981,37 @@
       </c>
       <c r="B135" s="1" t="inlineStr">
         <is>
-          <t>Q4015</t>
+          <t>Q4014</t>
         </is>
       </c>
       <c r="C135" s="1" t="inlineStr">
         <is>
-          <t>S7008</t>
+          <t>S7007</t>
         </is>
       </c>
       <c r="D135" s="1" t="inlineStr">
         <is>
-          <t>TT115</t>
+          <t>TT114</t>
         </is>
       </c>
       <c r="E135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8110</t>
+          <t>VLINE-8107</t>
         </is>
       </c>
       <c r="F135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8306</t>
+          <t>VLINE-8304</t>
         </is>
       </c>
       <c r="G135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8447</t>
+          <t>VLINE-8446</t>
         </is>
       </c>
       <c r="H135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8753</t>
+          <t>VLINE-8752</t>
         </is>
       </c>
     </row>
@@ -6023,37 +6023,37 @@
       </c>
       <c r="B136" s="1" t="inlineStr">
         <is>
-          <t>Q4016</t>
+          <t>Q4015</t>
         </is>
       </c>
       <c r="C136" s="1" t="inlineStr">
         <is>
-          <t>S7009</t>
+          <t>S7008</t>
         </is>
       </c>
       <c r="D136" s="1" t="inlineStr">
         <is>
-          <t>TT116</t>
+          <t>TT115</t>
         </is>
       </c>
       <c r="E136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8111</t>
+          <t>VLINE-8110</t>
         </is>
       </c>
       <c r="F136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8311</t>
+          <t>VLINE-8306</t>
         </is>
       </c>
       <c r="G136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8449</t>
+          <t>VLINE-8447</t>
         </is>
       </c>
       <c r="H136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8754</t>
+          <t>VLINE-8753</t>
         </is>
       </c>
     </row>
@@ -6065,37 +6065,37 @@
       </c>
       <c r="B137" s="1" t="inlineStr">
         <is>
-          <t>Q4017</t>
+          <t>Q4016</t>
         </is>
       </c>
       <c r="C137" s="1" t="inlineStr">
         <is>
-          <t>S7012</t>
+          <t>S7009</t>
         </is>
       </c>
       <c r="D137" s="1" t="inlineStr">
         <is>
-          <t>TT117</t>
+          <t>TT116</t>
         </is>
       </c>
       <c r="E137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8113</t>
+          <t>VLINE-8111</t>
         </is>
       </c>
       <c r="F137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8313</t>
+          <t>VLINE-8311</t>
         </is>
       </c>
       <c r="G137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8450</t>
+          <t>VLINE-8449</t>
         </is>
       </c>
       <c r="H137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8755</t>
+          <t>VLINE-8754</t>
         </is>
       </c>
     </row>
@@ -6107,37 +6107,37 @@
       </c>
       <c r="B138" s="1" t="inlineStr">
         <is>
-          <t>Q4019</t>
+          <t>Q4017</t>
         </is>
       </c>
       <c r="C138" s="1" t="inlineStr">
         <is>
-          <t>S7013</t>
+          <t>S7012</t>
         </is>
       </c>
       <c r="D138" s="1" t="inlineStr">
         <is>
-          <t>TT122</t>
+          <t>TT117</t>
         </is>
       </c>
       <c r="E138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8114</t>
+          <t>VLINE-8113</t>
         </is>
       </c>
       <c r="F138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8314</t>
+          <t>VLINE-8313</t>
         </is>
       </c>
       <c r="G138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8451</t>
+          <t>VLINE-8450</t>
         </is>
       </c>
       <c r="H138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8756</t>
+          <t>VLINE-8755</t>
         </is>
       </c>
     </row>
@@ -6149,37 +6149,37 @@
       </c>
       <c r="B139" s="1" t="inlineStr">
         <is>
-          <t>QBX003</t>
+          <t>Q4019</t>
         </is>
       </c>
       <c r="C139" s="1" t="inlineStr">
         <is>
-          <t>S7014</t>
+          <t>S7013</t>
         </is>
       </c>
       <c r="D139" s="1" t="inlineStr">
         <is>
-          <t>TT127</t>
+          <t>TT122</t>
         </is>
       </c>
       <c r="E139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8115</t>
+          <t>VLINE-8114</t>
         </is>
       </c>
       <c r="F139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8316</t>
+          <t>VLINE-8314</t>
         </is>
       </c>
       <c r="G139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8452</t>
+          <t>VLINE-8451</t>
         </is>
       </c>
       <c r="H139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8757</t>
+          <t>VLINE-8756</t>
         </is>
       </c>
     </row>
@@ -6191,37 +6191,37 @@
       </c>
       <c r="B140" s="1" t="inlineStr">
         <is>
-          <t>QBX004</t>
+          <t>QBX003</t>
         </is>
       </c>
       <c r="C140" s="1" t="inlineStr">
         <is>
-          <t>S7015</t>
+          <t>S7014</t>
         </is>
       </c>
       <c r="D140" s="1" t="inlineStr">
         <is>
-          <t>TT128</t>
+          <t>TT127</t>
         </is>
       </c>
       <c r="E140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8119</t>
+          <t>VLINE-8115</t>
         </is>
       </c>
       <c r="F140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8318</t>
+          <t>VLINE-8316</t>
         </is>
       </c>
       <c r="G140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8453</t>
+          <t>VLINE-8452</t>
         </is>
       </c>
       <c r="H140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8758</t>
+          <t>VLINE-8757</t>
         </is>
       </c>
     </row>
@@ -6233,37 +6233,37 @@
       </c>
       <c r="B141" s="1" t="inlineStr">
         <is>
-          <t>QBX005</t>
+          <t>QBX004</t>
         </is>
       </c>
       <c r="C141" s="1" t="inlineStr">
         <is>
-          <t>S7017</t>
+          <t>S7015</t>
         </is>
       </c>
       <c r="D141" s="1" t="inlineStr">
         <is>
-          <t>TT130</t>
+          <t>TT128</t>
         </is>
       </c>
       <c r="E141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8120</t>
+          <t>VLINE-8119</t>
         </is>
       </c>
       <c r="F141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8321</t>
+          <t>VLINE-8318</t>
         </is>
       </c>
       <c r="G141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8454</t>
+          <t>VLINE-8453</t>
         </is>
       </c>
       <c r="H141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8759</t>
+          <t>VLINE-8758</t>
         </is>
       </c>
     </row>
@@ -6275,37 +6275,37 @@
       </c>
       <c r="B142" s="1" t="inlineStr">
         <is>
-          <t>QBX006</t>
+          <t>QBX005</t>
         </is>
       </c>
       <c r="C142" s="1" t="inlineStr">
         <is>
-          <t>S7018</t>
+          <t>S7017</t>
         </is>
       </c>
       <c r="D142" s="1" t="inlineStr">
         <is>
-          <t>TT131</t>
+          <t>TT130</t>
         </is>
       </c>
       <c r="E142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8121</t>
+          <t>VLINE-8120</t>
         </is>
       </c>
       <c r="F142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8323</t>
+          <t>VLINE-8321</t>
         </is>
       </c>
       <c r="G142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8455</t>
+          <t>VLINE-8454</t>
         </is>
       </c>
       <c r="H142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8760</t>
+          <t>VLINE-8759</t>
         </is>
       </c>
     </row>
@@ -6317,37 +6317,37 @@
       </c>
       <c r="B143" s="1" t="inlineStr">
         <is>
-          <t>QE001</t>
+          <t>QBX006</t>
         </is>
       </c>
       <c r="C143" s="1" t="inlineStr">
         <is>
-          <t>S7020</t>
+          <t>S7018</t>
         </is>
       </c>
       <c r="D143" s="1" t="inlineStr">
         <is>
-          <t>TT202</t>
+          <t>TT131</t>
         </is>
       </c>
       <c r="E143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8123</t>
+          <t>VLINE-8121</t>
         </is>
       </c>
       <c r="F143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8324</t>
+          <t>VLINE-8323</t>
         </is>
       </c>
       <c r="G143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8456</t>
+          <t>VLINE-8455</t>
         </is>
       </c>
       <c r="H143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8761</t>
+          <t>VLINE-8760</t>
         </is>
       </c>
     </row>
@@ -6359,37 +6359,37 @@
       </c>
       <c r="B144" s="1" t="inlineStr">
         <is>
-          <t>QE002</t>
+          <t>QE001</t>
         </is>
       </c>
       <c r="C144" s="1" t="inlineStr">
         <is>
-          <t>S7022</t>
+          <t>S7020</t>
         </is>
       </c>
       <c r="D144" s="1" t="inlineStr">
         <is>
-          <t>TT206</t>
+          <t>TT202</t>
         </is>
       </c>
       <c r="E144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8124</t>
+          <t>VLINE-8123</t>
         </is>
       </c>
       <c r="F144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8325</t>
+          <t>VLINE-8324</t>
         </is>
       </c>
       <c r="G144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8457</t>
+          <t>VLINE-8456</t>
         </is>
       </c>
       <c r="H144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8762</t>
+          <t>VLINE-8761</t>
         </is>
       </c>
     </row>
@@ -6401,37 +6401,37 @@
       </c>
       <c r="B145" s="1" t="inlineStr">
         <is>
-          <t>QE003</t>
+          <t>QE002</t>
         </is>
       </c>
       <c r="C145" s="1" t="inlineStr">
         <is>
-          <t>SCT001</t>
+          <t>S7022</t>
         </is>
       </c>
       <c r="D145" s="1" t="inlineStr">
         <is>
-          <t>VL352</t>
+          <t>TT206</t>
         </is>
       </c>
       <c r="E145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8126</t>
+          <t>VLINE-8124</t>
         </is>
       </c>
       <c r="F145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8328</t>
+          <t>VLINE-8325</t>
         </is>
       </c>
       <c r="G145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8460</t>
+          <t>VLINE-8457</t>
         </is>
       </c>
       <c r="H145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8763</t>
+          <t>VLINE-8762</t>
         </is>
       </c>
     </row>
@@ -6443,37 +6443,37 @@
       </c>
       <c r="B146" s="1" t="inlineStr">
         <is>
-          <t>QE004</t>
+          <t>QE003</t>
         </is>
       </c>
       <c r="C146" s="1" t="inlineStr">
         <is>
-          <t>SCT002</t>
+          <t>SCT001</t>
         </is>
       </c>
       <c r="D146" s="1" t="inlineStr">
         <is>
-          <t>VL353</t>
+          <t>VL352</t>
         </is>
       </c>
       <c r="E146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8127</t>
+          <t>VLINE-8126</t>
         </is>
       </c>
       <c r="F146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8329</t>
+          <t>VLINE-8328</t>
         </is>
       </c>
       <c r="G146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8461</t>
+          <t>VLINE-8460</t>
         </is>
       </c>
       <c r="H146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8764</t>
+          <t>VLINE-8763</t>
         </is>
       </c>
     </row>
@@ -6485,37 +6485,37 @@
       </c>
       <c r="B147" s="1" t="inlineStr">
         <is>
-          <t>QE006</t>
+          <t>QE004</t>
         </is>
       </c>
       <c r="C147" s="1" t="inlineStr">
         <is>
-          <t>SCT006</t>
+          <t>SCT002</t>
         </is>
       </c>
       <c r="D147" s="1" t="inlineStr">
         <is>
-          <t>VL357</t>
+          <t>VL353</t>
         </is>
       </c>
       <c r="E147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8128</t>
+          <t>VLINE-8127</t>
         </is>
       </c>
       <c r="F147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8332</t>
+          <t>VLINE-8329</t>
         </is>
       </c>
       <c r="G147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8464</t>
+          <t>VLINE-8461</t>
         </is>
       </c>
       <c r="H147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8765</t>
+          <t>VLINE-8764</t>
         </is>
       </c>
     </row>
@@ -6527,37 +6527,37 @@
       </c>
       <c r="B148" s="1" t="inlineStr">
         <is>
-          <t>QL001</t>
+          <t>QE006</t>
         </is>
       </c>
       <c r="C148" s="1" t="inlineStr">
         <is>
-          <t>SCT007</t>
+          <t>SCT006</t>
         </is>
       </c>
       <c r="D148" s="1" t="inlineStr">
         <is>
-          <t>VL359</t>
+          <t>VL357</t>
         </is>
       </c>
       <c r="E148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8129</t>
+          <t>VLINE-8128</t>
         </is>
       </c>
       <c r="F148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8336</t>
+          <t>VLINE-8332</t>
         </is>
       </c>
       <c r="G148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8465</t>
+          <t>VLINE-8464</t>
         </is>
       </c>
       <c r="H148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8766</t>
+          <t>VLINE-8765</t>
         </is>
       </c>
     </row>
@@ -6569,37 +6569,37 @@
       </c>
       <c r="B149" s="1" t="inlineStr">
         <is>
-          <t>QL002</t>
+          <t>QL001</t>
         </is>
       </c>
       <c r="C149" s="1" t="inlineStr">
         <is>
-          <t>SCT009</t>
+          <t>SCT007</t>
         </is>
       </c>
       <c r="D149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8004</t>
+          <t>VL359</t>
         </is>
       </c>
       <c r="E149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8131</t>
+          <t>VLINE-8129</t>
         </is>
       </c>
       <c r="F149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8337</t>
+          <t>VLINE-8336</t>
         </is>
       </c>
       <c r="G149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8468</t>
+          <t>VLINE-8465</t>
         </is>
       </c>
       <c r="H149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8767</t>
+          <t>VLINE-8766</t>
         </is>
       </c>
     </row>
@@ -6611,37 +6611,37 @@
       </c>
       <c r="B150" s="1" t="inlineStr">
         <is>
-          <t>QL004</t>
+          <t>QL002</t>
         </is>
       </c>
       <c r="C150" s="1" t="inlineStr">
         <is>
-          <t>SCT011</t>
+          <t>SCT009</t>
         </is>
       </c>
       <c r="D150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8007</t>
+          <t>VLINE-8004</t>
         </is>
       </c>
       <c r="E150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8132</t>
+          <t>VLINE-8131</t>
         </is>
       </c>
       <c r="F150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8338</t>
+          <t>VLINE-8337</t>
         </is>
       </c>
       <c r="G150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8469</t>
+          <t>VLINE-8468</t>
         </is>
       </c>
       <c r="H150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8768</t>
+          <t>VLINE-8767</t>
         </is>
       </c>
     </row>
@@ -6653,37 +6653,37 @@
       </c>
       <c r="B151" s="1" t="inlineStr">
         <is>
-          <t>QL007</t>
+          <t>QL004</t>
         </is>
       </c>
       <c r="C151" s="1" t="inlineStr">
         <is>
-          <t>SCT013</t>
+          <t>SCT011</t>
         </is>
       </c>
       <c r="D151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8011</t>
+          <t>VLINE-8007</t>
         </is>
       </c>
       <c r="E151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8133</t>
+          <t>VLINE-8132</t>
         </is>
       </c>
       <c r="F151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8339</t>
+          <t>VLINE-8338</t>
         </is>
       </c>
       <c r="G151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8605</t>
+          <t>VLINE-8469</t>
         </is>
       </c>
       <c r="H151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8769</t>
+          <t>VLINE-8768</t>
         </is>
       </c>
     </row>
@@ -6695,37 +6695,37 @@
       </c>
       <c r="B152" s="1" t="inlineStr">
         <is>
-          <t>QL008</t>
+          <t>QL007</t>
         </is>
       </c>
       <c r="C152" s="1" t="inlineStr">
         <is>
-          <t>SCT014</t>
+          <t>SCT013</t>
         </is>
       </c>
       <c r="D152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8013</t>
+          <t>VLINE-8011</t>
         </is>
       </c>
       <c r="E152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8134</t>
+          <t>VLINE-8133</t>
         </is>
       </c>
       <c r="F152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8362</t>
+          <t>VLINE-8339</t>
         </is>
       </c>
       <c r="G152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8610</t>
+          <t>VLINE-8605</t>
         </is>
       </c>
       <c r="H152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8770</t>
+          <t>VLINE-8769</t>
         </is>
       </c>
     </row>
@@ -6737,37 +6737,37 @@
       </c>
       <c r="B153" s="1" t="inlineStr">
         <is>
-          <t>QL010</t>
+          <t>QL008</t>
         </is>
       </c>
       <c r="C153" s="1" t="inlineStr">
         <is>
-          <t>SCT015</t>
+          <t>SCT014</t>
         </is>
       </c>
       <c r="D153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8019</t>
+          <t>VLINE-8013</t>
         </is>
       </c>
       <c r="E153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8136</t>
+          <t>VLINE-8134</t>
         </is>
       </c>
       <c r="F153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8363</t>
+          <t>VLINE-8362</t>
         </is>
       </c>
       <c r="G153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8612</t>
+          <t>VLINE-8610</t>
         </is>
       </c>
       <c r="H153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8772</t>
+          <t>VLINE-8770</t>
         </is>
       </c>
     </row>
@@ -6779,37 +6779,37 @@
       </c>
       <c r="B154" s="1" t="inlineStr">
         <is>
-          <t>QL011</t>
+          <t>QL010</t>
         </is>
       </c>
       <c r="C154" s="1" t="inlineStr">
         <is>
-          <t>SO2</t>
+          <t>SCT015</t>
         </is>
       </c>
       <c r="D154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8020</t>
+          <t>VLINE-8019</t>
         </is>
       </c>
       <c r="E154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8137</t>
+          <t>VLINE-8136</t>
         </is>
       </c>
       <c r="F154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8365</t>
+          <t>VLINE-8363</t>
         </is>
       </c>
       <c r="G154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8615</t>
+          <t>VLINE-8612</t>
         </is>
       </c>
       <c r="H154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8773</t>
+          <t>VLINE-8772</t>
         </is>
       </c>
     </row>
@@ -6821,37 +6821,37 @@
       </c>
       <c r="B155" s="1" t="inlineStr">
         <is>
-          <t>QL012</t>
+          <t>QL011</t>
         </is>
       </c>
       <c r="C155" s="1" t="inlineStr">
         <is>
-          <t>SO3</t>
+          <t>SO2</t>
         </is>
       </c>
       <c r="D155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8023</t>
+          <t>VLINE-8020</t>
         </is>
       </c>
       <c r="E155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8140</t>
+          <t>VLINE-8137</t>
         </is>
       </c>
       <c r="F155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8366</t>
+          <t>VLINE-8365</t>
         </is>
       </c>
       <c r="G155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8617</t>
+          <t>VLINE-8615</t>
         </is>
       </c>
       <c r="H155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8774</t>
+          <t>VLINE-8773</t>
         </is>
       </c>
     </row>
@@ -6863,1137 +6863,1152 @@
       </c>
       <c r="B156" s="1" t="inlineStr">
         <is>
-          <t>QL014</t>
+          <t>QL012</t>
         </is>
       </c>
       <c r="C156" s="1" t="inlineStr">
         <is>
-          <t>SSR101</t>
+          <t>SO3</t>
         </is>
       </c>
       <c r="D156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8025</t>
+          <t>VLINE-8023</t>
         </is>
       </c>
       <c r="E156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8141</t>
+          <t>VLINE-8140</t>
         </is>
       </c>
       <c r="F156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8368</t>
+          <t>VLINE-8366</t>
         </is>
       </c>
       <c r="G156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8620</t>
+          <t>VLINE-8617</t>
         </is>
       </c>
       <c r="H156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8776</t>
+          <t>VLINE-8774</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="1" t="inlineStr">
         <is>
-          <t>NR122</t>
+          <t>NR121</t>
         </is>
       </c>
       <c r="B157" s="1" t="inlineStr">
         <is>
-          <t>QL017</t>
+          <t>QL014</t>
         </is>
       </c>
       <c r="C157" s="1" t="inlineStr">
         <is>
-          <t>SSR102</t>
+          <t>SSR101</t>
         </is>
       </c>
       <c r="D157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8026</t>
+          <t>VLINE-8025</t>
         </is>
       </c>
       <c r="E157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8142</t>
+          <t>VLINE-8141</t>
         </is>
       </c>
       <c r="F157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8369</t>
+          <t>VLINE-8368</t>
         </is>
       </c>
       <c r="G157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8625</t>
+          <t>VLINE-8620</t>
         </is>
       </c>
       <c r="H157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8778</t>
+          <t>VLINE-8776</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="1" t="inlineStr">
         <is>
-          <t>P14</t>
+          <t>NR122</t>
         </is>
       </c>
       <c r="B158" s="1" t="inlineStr">
         <is>
-          <t>QL018</t>
+          <t>QL017</t>
         </is>
       </c>
       <c r="C158" s="1" t="inlineStr">
         <is>
-          <t>SSR103</t>
+          <t>SSR102</t>
         </is>
       </c>
       <c r="D158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8027</t>
+          <t>VLINE-8026</t>
         </is>
       </c>
       <c r="E158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8144</t>
+          <t>VLINE-8142</t>
         </is>
       </c>
       <c r="F158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8403</t>
+          <t>VLINE-8369</t>
         </is>
       </c>
       <c r="G158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8630</t>
+          <t>VLINE-8625</t>
         </is>
       </c>
       <c r="H158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8779</t>
+          <t>VLINE-8778</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="1" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P14</t>
         </is>
       </c>
       <c r="B159" s="1" t="inlineStr">
         <is>
-          <t>QR1744</t>
+          <t>QL018</t>
         </is>
       </c>
       <c r="C159" s="1" t="inlineStr">
         <is>
-          <t>SSR104</t>
+          <t>SSR103</t>
         </is>
       </c>
       <c r="D159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8028</t>
+          <t>VLINE-8027</t>
         </is>
       </c>
       <c r="E159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8145</t>
+          <t>VLINE-8144</t>
         </is>
       </c>
       <c r="F159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8404</t>
+          <t>VLINE-8403</t>
         </is>
       </c>
       <c r="G159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8671</t>
+          <t>VLINE-8630</t>
         </is>
       </c>
       <c r="H159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8780</t>
+          <t>VLINE-8779</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="1" t="inlineStr">
         <is>
-          <t>P2501</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="B160" s="1" t="inlineStr">
         <is>
-          <t>QR1771</t>
+          <t>QR1744</t>
         </is>
       </c>
       <c r="C160" s="1" t="inlineStr">
         <is>
-          <t>T363</t>
+          <t>SSR104</t>
         </is>
       </c>
       <c r="D160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8029</t>
+          <t>VLINE-8028</t>
         </is>
       </c>
       <c r="E160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8148</t>
+          <t>VLINE-8145</t>
         </is>
       </c>
       <c r="F160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8406</t>
+          <t>VLINE-8404</t>
         </is>
       </c>
       <c r="G160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8706</t>
+          <t>VLINE-8671</t>
         </is>
       </c>
       <c r="H160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8781</t>
+          <t>VLINE-8780</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="1" t="inlineStr">
         <is>
-          <t>P2502</t>
+          <t>P2501</t>
         </is>
       </c>
       <c r="B161" s="1" t="inlineStr">
         <is>
-          <t>QR5404</t>
+          <t>QR1771</t>
         </is>
       </c>
       <c r="C161" s="1" t="inlineStr">
         <is>
-          <t>T381</t>
+          <t>T363</t>
         </is>
       </c>
       <c r="D161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8030</t>
+          <t>VLINE-8029</t>
         </is>
       </c>
       <c r="E161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8150</t>
+          <t>VLINE-8148</t>
         </is>
       </c>
       <c r="F161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8408</t>
+          <t>VLINE-8406</t>
         </is>
       </c>
       <c r="G161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8711</t>
+          <t>VLINE-8706</t>
         </is>
       </c>
       <c r="H161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8782</t>
+          <t>VLINE-8781</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="1" t="inlineStr">
         <is>
-          <t>P2503</t>
+          <t>P2502</t>
         </is>
       </c>
       <c r="B162" s="1" t="inlineStr">
         <is>
-          <t>R711</t>
+          <t>QR5404</t>
         </is>
       </c>
       <c r="C162" s="1" t="inlineStr">
         <is>
-          <t>T386</t>
+          <t>T381</t>
         </is>
       </c>
       <c r="D162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8031</t>
+          <t>VLINE-8030</t>
         </is>
       </c>
       <c r="E162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8151</t>
+          <t>VLINE-8150</t>
         </is>
       </c>
       <c r="F162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8410</t>
+          <t>VLINE-8408</t>
         </is>
       </c>
       <c r="G162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8714</t>
+          <t>VLINE-8711</t>
         </is>
       </c>
       <c r="H162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8783</t>
+          <t>VLINE-8782</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="1" t="inlineStr">
         <is>
-          <t>P2504</t>
+          <t>P2503</t>
         </is>
       </c>
       <c r="B163" s="1" t="inlineStr">
         <is>
-          <t>R766</t>
+          <t>R711</t>
         </is>
       </c>
       <c r="C163" s="1" t="inlineStr">
         <is>
-          <t>TDX101</t>
+          <t>T386</t>
         </is>
       </c>
       <c r="D163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8032</t>
+          <t>VLINE-8031</t>
         </is>
       </c>
       <c r="E163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8152</t>
+          <t>VLINE-8151</t>
         </is>
       </c>
       <c r="F163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8411</t>
+          <t>VLINE-8410</t>
         </is>
       </c>
       <c r="G163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8717</t>
+          <t>VLINE-8714</t>
         </is>
       </c>
       <c r="H163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8784</t>
+          <t>VLINE-8783</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="1" t="inlineStr">
         <is>
-          <t>P2505</t>
+          <t>P2504</t>
         </is>
       </c>
       <c r="B164" s="1" t="inlineStr">
         <is>
-          <t>RB2353</t>
+          <t>R766</t>
         </is>
       </c>
       <c r="C164" s="1" t="inlineStr">
         <is>
-          <t>TE2801</t>
+          <t>TDX101</t>
         </is>
       </c>
       <c r="D164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8036</t>
+          <t>VLINE-8032</t>
         </is>
       </c>
       <c r="E164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8153</t>
+          <t>VLINE-8152</t>
         </is>
       </c>
       <c r="F164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8413</t>
+          <t>VLINE-8411</t>
         </is>
       </c>
       <c r="G164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8720</t>
+          <t>VLINE-8717</t>
         </is>
       </c>
       <c r="H164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8786</t>
+          <t>VLINE-8784</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="1" t="inlineStr">
         <is>
-          <t>P2506</t>
+          <t>P2505</t>
         </is>
       </c>
       <c r="B165" s="1" t="inlineStr">
         <is>
-          <t>RCTST4</t>
+          <t>RB2353</t>
         </is>
       </c>
       <c r="C165" s="1" t="inlineStr">
         <is>
-          <t>TE2802</t>
+          <t>TE2801</t>
         </is>
       </c>
       <c r="D165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8038</t>
+          <t>VLINE-8036</t>
         </is>
       </c>
       <c r="E165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8154</t>
+          <t>VLINE-8153</t>
         </is>
       </c>
       <c r="F165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8415</t>
+          <t>VLINE-8413</t>
         </is>
       </c>
       <c r="G165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8721</t>
+          <t>VLINE-8720</t>
         </is>
       </c>
       <c r="H165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8787</t>
+          <t>VLINE-8786</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="1" t="inlineStr">
         <is>
-          <t>P2507</t>
+          <t>P2506</t>
         </is>
       </c>
       <c r="B166" s="1" t="inlineStr">
         <is>
-          <t>RL301</t>
+          <t>RCTST4</t>
         </is>
       </c>
       <c r="C166" s="1" t="inlineStr">
         <is>
-          <t>TE2803</t>
+          <t>TE2802</t>
         </is>
       </c>
       <c r="D166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8039</t>
+          <t>VLINE-8038</t>
         </is>
       </c>
       <c r="E166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8155</t>
+          <t>VLINE-8154</t>
         </is>
       </c>
       <c r="F166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8417</t>
+          <t>VLINE-8415</t>
         </is>
       </c>
       <c r="G166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8723</t>
+          <t>VLINE-8721</t>
         </is>
       </c>
       <c r="H166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8788</t>
+          <t>VLINE-8787</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="1" t="inlineStr">
         <is>
-          <t>P2508</t>
+          <t>P2507</t>
         </is>
       </c>
       <c r="B167" s="1" t="inlineStr">
         <is>
-          <t>RL302</t>
+          <t>RL301</t>
         </is>
       </c>
       <c r="C167" s="1" t="inlineStr">
         <is>
-          <t>TE2804</t>
+          <t>TE2803</t>
         </is>
       </c>
       <c r="D167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8042</t>
+          <t>VLINE-8039</t>
         </is>
       </c>
       <c r="E167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8157</t>
+          <t>VLINE-8155</t>
         </is>
       </c>
       <c r="F167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8418</t>
+          <t>VLINE-8417</t>
         </is>
       </c>
       <c r="G167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8725</t>
+          <t>VLINE-8723</t>
         </is>
       </c>
       <c r="H167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8790</t>
+          <t>VLINE-8788</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="1" t="inlineStr">
         <is>
-          <t>P2509</t>
+          <t>P2508</t>
         </is>
       </c>
       <c r="B168" s="1" t="inlineStr">
         <is>
-          <t>RL304</t>
+          <t>RL302</t>
         </is>
       </c>
       <c r="C168" s="1" t="inlineStr">
         <is>
-          <t>TE2805</t>
+          <t>TE2804</t>
         </is>
       </c>
       <c r="D168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8049</t>
+          <t>VLINE-8042</t>
         </is>
       </c>
       <c r="E168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8158</t>
+          <t>VLINE-8157</t>
         </is>
       </c>
       <c r="F168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8419</t>
+          <t>VLINE-8418</t>
         </is>
       </c>
       <c r="G168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8726</t>
+          <t>VLINE-8725</t>
         </is>
       </c>
       <c r="H168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8792</t>
+          <t>VLINE-8790</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="1" t="inlineStr">
         <is>
-          <t>P2510</t>
+          <t>P2509</t>
         </is>
       </c>
       <c r="B169" s="1" t="inlineStr">
         <is>
-          <t>RL305</t>
+          <t>RL304</t>
         </is>
       </c>
       <c r="C169" s="1" t="inlineStr">
         <is>
-          <t>TE2806</t>
+          <t>TE2805</t>
         </is>
       </c>
       <c r="D169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8050</t>
+          <t>VLINE-8049</t>
         </is>
       </c>
       <c r="E169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8159</t>
+          <t>VLINE-8158</t>
         </is>
       </c>
       <c r="F169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8420</t>
+          <t>VLINE-8419</t>
         </is>
       </c>
       <c r="G169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8727</t>
+          <t>VLINE-8726</t>
         </is>
       </c>
       <c r="H169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8793</t>
+          <t>VLINE-8792</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="1" t="inlineStr">
         <is>
-          <t>P2511</t>
+          <t>P2510</t>
         </is>
       </c>
       <c r="B170" s="1" t="inlineStr">
         <is>
-          <t>RL306</t>
+          <t>RL305</t>
         </is>
       </c>
       <c r="C170" s="1" t="inlineStr">
         <is>
-          <t>TE2807</t>
+          <t>TE2806</t>
         </is>
       </c>
       <c r="D170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8051</t>
+          <t>VLINE-8050</t>
         </is>
       </c>
       <c r="E170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8160</t>
+          <t>VLINE-8159</t>
         </is>
       </c>
       <c r="F170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8421</t>
+          <t>VLINE-8420</t>
         </is>
       </c>
       <c r="G170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8729</t>
+          <t>VLINE-8727</t>
         </is>
       </c>
       <c r="H170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8794</t>
+          <t>VLINE-8793</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8795</t>
+          <t>VLINE-8794</t>
         </is>
       </c>
       <c r="B172" s="1" t="inlineStr">
         <is>
-          <t>XP2016</t>
+          <t>XP2013</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8796</t>
+          <t>VLINE-8795</t>
         </is>
       </c>
       <c r="B173" s="1" t="inlineStr">
         <is>
-          <t>XP2017</t>
+          <t>XP2014</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8797</t>
+          <t>VLINE-8796</t>
         </is>
       </c>
       <c r="B174" s="1" t="inlineStr">
         <is>
-          <t>XP2019</t>
+          <t>XP2015</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8799</t>
+          <t>VLINE-8797</t>
         </is>
       </c>
       <c r="B175" s="1" t="inlineStr">
         <is>
-          <t>XR550</t>
+          <t>XP2016</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8800</t>
+          <t>VLINE-8799</t>
         </is>
       </c>
       <c r="B176" s="1" t="inlineStr">
         <is>
-          <t>XR552</t>
+          <t>XP2017</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8801</t>
+          <t>VLINE-8800</t>
         </is>
       </c>
       <c r="B177" s="1" t="inlineStr">
         <is>
-          <t>XR559</t>
+          <t>XP2019</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8802</t>
+          <t>VLINE-8801</t>
         </is>
       </c>
       <c r="B178" s="1" t="inlineStr">
         <is>
-          <t>XRN001</t>
+          <t>XR550</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8803</t>
+          <t>VLINE-8802</t>
         </is>
       </c>
       <c r="B179" s="1" t="inlineStr">
         <is>
-          <t>XRN004</t>
+          <t>XR552</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8804</t>
+          <t>VLINE-8803</t>
         </is>
       </c>
       <c r="B180" s="1" t="inlineStr">
         <is>
-          <t>XRN005</t>
+          <t>XR559</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8805</t>
+          <t>VLINE-8804</t>
         </is>
       </c>
       <c r="B181" s="1" t="inlineStr">
         <is>
-          <t>XRN006</t>
+          <t>XRN001</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8806</t>
+          <t>VLINE-8805</t>
         </is>
       </c>
       <c r="B182" s="1" t="inlineStr">
         <is>
-          <t>XRN007</t>
+          <t>XRN004</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8807</t>
+          <t>VLINE-8806</t>
         </is>
       </c>
       <c r="B183" s="1" t="inlineStr">
         <is>
-          <t>XRN009</t>
+          <t>XRN005</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8808</t>
+          <t>VLINE-8807</t>
         </is>
       </c>
       <c r="B184" s="1" t="inlineStr">
         <is>
-          <t>XRN011</t>
+          <t>XRN006</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8809</t>
+          <t>VLINE-8808</t>
         </is>
       </c>
       <c r="B185" s="1" t="inlineStr">
         <is>
-          <t>XRN014</t>
+          <t>XRN007</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8810</t>
+          <t>VLINE-8809</t>
         </is>
       </c>
       <c r="B186" s="1" t="inlineStr">
         <is>
-          <t>XRN017</t>
+          <t>XRN009</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8811</t>
+          <t>VLINE-8810</t>
         </is>
       </c>
       <c r="B187" s="1" t="inlineStr">
         <is>
-          <t>XRN018</t>
+          <t>XRN011</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8812</t>
+          <t>VLINE-8811</t>
         </is>
       </c>
       <c r="B188" s="1" t="inlineStr">
         <is>
-          <t>XRN020</t>
+          <t>XRN014</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8813</t>
+          <t>VLINE-8812</t>
         </is>
       </c>
       <c r="B189" s="1" t="inlineStr">
         <is>
-          <t>XRN021</t>
+          <t>XRN017</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8814</t>
+          <t>VLINE-8813</t>
         </is>
       </c>
       <c r="B190" s="1" t="inlineStr">
         <is>
-          <t>XRN023</t>
+          <t>XRN018</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8816</t>
+          <t>VLINE-8814</t>
         </is>
       </c>
       <c r="B191" s="1" t="inlineStr">
         <is>
-          <t>XRN025</t>
+          <t>XRN020</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8817</t>
+          <t>VLINE-8815</t>
         </is>
       </c>
       <c r="B192" s="1" t="inlineStr">
         <is>
-          <t>XRN026</t>
+          <t>XRN021</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8818</t>
+          <t>VLINE-8816</t>
         </is>
       </c>
       <c r="B193" s="1" t="inlineStr">
         <is>
-          <t>XRN027</t>
+          <t>XRN023</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8819</t>
+          <t>VLINE-8817</t>
         </is>
       </c>
       <c r="B194" s="1" t="inlineStr">
         <is>
-          <t>XRN029</t>
+          <t>XRN025</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8822</t>
+          <t>VLINE-8818</t>
         </is>
       </c>
       <c r="B195" s="1" t="inlineStr">
         <is>
-          <t>Y163</t>
+          <t>XRN026</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8860</t>
+          <t>VLINE-8819</t>
+        </is>
+      </c>
+      <c r="B196" s="1" t="inlineStr">
+        <is>
+          <t>XRN027</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8861</t>
+          <t>VLINE-8820</t>
+        </is>
+      </c>
+      <c r="B197" s="1" t="inlineStr">
+        <is>
+          <t>XRN029</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8862</t>
+          <t>VLINE-8822</t>
+        </is>
+      </c>
+      <c r="B198" s="1" t="inlineStr">
+        <is>
+          <t>Y163</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8863</t>
+          <t>VLINE-8860</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8864</t>
+          <t>VLINE-8861</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8865</t>
+          <t>VLINE-8862</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8866</t>
+          <t>VLINE-8863</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8867</t>
+          <t>VLINE-8864</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8868</t>
+          <t>VLINE-8865</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8869</t>
+          <t>VLINE-8866</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8890</t>
+          <t>VLINE-8867</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8891</t>
+          <t>VLINE-8868</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8893</t>
+          <t>VLINE-8869</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8895</t>
+          <t>VLINE-8890</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="1" t="inlineStr">
         <is>
-          <t>WH001</t>
+          <t>VLINE-8891</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="1" t="inlineStr">
         <is>
-          <t>WH003</t>
+          <t>VLINE-8893</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="1" t="inlineStr">
         <is>
-          <t>WL02</t>
+          <t>VLINE-8895</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" s="1" t="inlineStr">
         <is>
-          <t>X12-X14</t>
+          <t>WH001</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" s="1" t="inlineStr">
         <is>
-          <t>X31</t>
+          <t>WH003</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" s="1" t="inlineStr">
         <is>
-          <t>XP2000</t>
+          <t>WL02</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="1" t="inlineStr">
         <is>
-          <t>XP2001</t>
+          <t>X12-X14</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="1" t="inlineStr">
         <is>
-          <t>XP2003</t>
+          <t>X31</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="1" t="inlineStr">
         <is>
-          <t>XP2004</t>
+          <t>XP2000</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="1" t="inlineStr">
         <is>
-          <t>XP2005</t>
+          <t>XP2001</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" s="1" t="inlineStr">
         <is>
-          <t>XP2007</t>
+          <t>XP2003</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="1" t="inlineStr">
         <is>
-          <t>XP2008</t>
+          <t>XP2004</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="1" t="inlineStr">
         <is>
-          <t>XP2010</t>
+          <t>XP2005</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="1" t="inlineStr">
         <is>
-          <t>XP2011</t>
+          <t>XP2007</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" s="1" t="inlineStr">
         <is>
-          <t>XP2012</t>
+          <t>XP2008</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="1" t="inlineStr">
         <is>
-          <t>XP2013</t>
+          <t>XP2010</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" s="1" t="inlineStr">
         <is>
-          <t>XP2014</t>
+          <t>XP2011</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" s="1" t="inlineStr">
         <is>
-          <t>XP2015</t>
+          <t>XP2012</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update loco downloads 2026-04-06 14:59:29
</commit_message>
<xml_diff>
--- a/downloads/loco_numbers_only.xlsx
+++ b/downloads/loco_numbers_only.xlsx
@@ -2819,7 +2819,7 @@
       </c>
       <c r="H58" s="1" t="inlineStr">
         <is>
-          <t>N454</t>
+          <t>N453</t>
         </is>
       </c>
     </row>
@@ -2861,7 +2861,7 @@
       </c>
       <c r="H59" s="1" t="inlineStr">
         <is>
-          <t>N457</t>
+          <t>N454</t>
         </is>
       </c>
     </row>
@@ -2903,7 +2903,7 @@
       </c>
       <c r="H60" s="1" t="inlineStr">
         <is>
-          <t>N458</t>
+          <t>N457</t>
         </is>
       </c>
     </row>
@@ -2945,7 +2945,7 @@
       </c>
       <c r="H61" s="1" t="inlineStr">
         <is>
-          <t>N460</t>
+          <t>N458</t>
         </is>
       </c>
     </row>
@@ -2987,7 +2987,7 @@
       </c>
       <c r="H62" s="1" t="inlineStr">
         <is>
-          <t>N461</t>
+          <t>N460</t>
         </is>
       </c>
     </row>
@@ -3029,7 +3029,7 @@
       </c>
       <c r="H63" s="1" t="inlineStr">
         <is>
-          <t>N465</t>
+          <t>N461</t>
         </is>
       </c>
     </row>
@@ -3071,7 +3071,7 @@
       </c>
       <c r="H64" s="1" t="inlineStr">
         <is>
-          <t>N466</t>
+          <t>N465</t>
         </is>
       </c>
     </row>
@@ -3113,7 +3113,7 @@
       </c>
       <c r="H65" s="1" t="inlineStr">
         <is>
-          <t>N467</t>
+          <t>N466</t>
         </is>
       </c>
     </row>
@@ -3155,7 +3155,7 @@
       </c>
       <c r="H66" s="1" t="inlineStr">
         <is>
-          <t>N469</t>
+          <t>N467</t>
         </is>
       </c>
     </row>
@@ -3197,7 +3197,7 @@
       </c>
       <c r="H67" s="1" t="inlineStr">
         <is>
-          <t>N473</t>
+          <t>N469</t>
         </is>
       </c>
     </row>
@@ -3239,7 +3239,7 @@
       </c>
       <c r="H68" s="1" t="inlineStr">
         <is>
-          <t>NR1</t>
+          <t>N473</t>
         </is>
       </c>
     </row>
@@ -3281,7 +3281,7 @@
       </c>
       <c r="H69" s="1" t="inlineStr">
         <is>
-          <t>NR2</t>
+          <t>NR1</t>
         </is>
       </c>
     </row>
@@ -3323,7 +3323,7 @@
       </c>
       <c r="H70" s="1" t="inlineStr">
         <is>
-          <t>NR4</t>
+          <t>NR2</t>
         </is>
       </c>
     </row>
@@ -3365,7 +3365,7 @@
       </c>
       <c r="H71" s="1" t="inlineStr">
         <is>
-          <t>NR5</t>
+          <t>NR4</t>
         </is>
       </c>
     </row>
@@ -3407,7 +3407,7 @@
       </c>
       <c r="H72" s="1" t="inlineStr">
         <is>
-          <t>NR7</t>
+          <t>NR5</t>
         </is>
       </c>
     </row>
@@ -3444,12 +3444,12 @@
       </c>
       <c r="G73" s="1" t="inlineStr">
         <is>
-          <t>MM-9926M</t>
+          <t>MM-9925M</t>
         </is>
       </c>
       <c r="H73" s="1" t="inlineStr">
         <is>
-          <t>NR8</t>
+          <t>NR7</t>
         </is>
       </c>
     </row>
@@ -3486,12 +3486,12 @@
       </c>
       <c r="G74" s="1" t="inlineStr">
         <is>
-          <t>MM-9928M</t>
+          <t>MM-9926M</t>
         </is>
       </c>
       <c r="H74" s="1" t="inlineStr">
         <is>
-          <t>NR9</t>
+          <t>NR8</t>
         </is>
       </c>
     </row>
@@ -3528,12 +3528,12 @@
       </c>
       <c r="G75" s="1" t="inlineStr">
         <is>
-          <t>MM-9929M</t>
+          <t>MM-9928M</t>
         </is>
       </c>
       <c r="H75" s="1" t="inlineStr">
         <is>
-          <t>NR10</t>
+          <t>NR9</t>
         </is>
       </c>
     </row>
@@ -3570,12 +3570,12 @@
       </c>
       <c r="G76" s="1" t="inlineStr">
         <is>
-          <t>MM-9932M</t>
+          <t>MM-9929M</t>
         </is>
       </c>
       <c r="H76" s="1" t="inlineStr">
         <is>
-          <t>NR12</t>
+          <t>NR10</t>
         </is>
       </c>
     </row>
@@ -3612,12 +3612,12 @@
       </c>
       <c r="G77" s="1" t="inlineStr">
         <is>
-          <t>MM-9933M</t>
+          <t>MM-9932M</t>
         </is>
       </c>
       <c r="H77" s="1" t="inlineStr">
         <is>
-          <t>NR13</t>
+          <t>NR12</t>
         </is>
       </c>
     </row>
@@ -3654,12 +3654,12 @@
       </c>
       <c r="G78" s="1" t="inlineStr">
         <is>
-          <t>MM-9934M</t>
+          <t>MM-9933M</t>
         </is>
       </c>
       <c r="H78" s="1" t="inlineStr">
         <is>
-          <t>NR15</t>
+          <t>NR13</t>
         </is>
       </c>
     </row>
@@ -3696,12 +3696,12 @@
       </c>
       <c r="G79" s="1" t="inlineStr">
         <is>
-          <t>MM-9936M</t>
+          <t>MM-9934M</t>
         </is>
       </c>
       <c r="H79" s="1" t="inlineStr">
         <is>
-          <t>NR16</t>
+          <t>NR15</t>
         </is>
       </c>
     </row>
@@ -3738,12 +3738,12 @@
       </c>
       <c r="G80" s="1" t="inlineStr">
         <is>
-          <t>MM-9938M</t>
+          <t>MM-9936M</t>
         </is>
       </c>
       <c r="H80" s="1" t="inlineStr">
         <is>
-          <t>NR18</t>
+          <t>NR16</t>
         </is>
       </c>
     </row>
@@ -3780,12 +3780,12 @@
       </c>
       <c r="G81" s="1" t="inlineStr">
         <is>
-          <t>MM-9941M</t>
+          <t>MM-9938M</t>
         </is>
       </c>
       <c r="H81" s="1" t="inlineStr">
         <is>
-          <t>NR19</t>
+          <t>NR18</t>
         </is>
       </c>
     </row>
@@ -3822,12 +3822,12 @@
       </c>
       <c r="G82" s="1" t="inlineStr">
         <is>
-          <t>MM-9943M</t>
+          <t>MM-9941M</t>
         </is>
       </c>
       <c r="H82" s="1" t="inlineStr">
         <is>
-          <t>NR20</t>
+          <t>NR19</t>
         </is>
       </c>
     </row>
@@ -3864,12 +3864,12 @@
       </c>
       <c r="G83" s="1" t="inlineStr">
         <is>
-          <t>MM-9945M</t>
+          <t>MM-9943M</t>
         </is>
       </c>
       <c r="H83" s="1" t="inlineStr">
         <is>
-          <t>NR21</t>
+          <t>NR20</t>
         </is>
       </c>
     </row>
@@ -3906,12 +3906,12 @@
       </c>
       <c r="G84" s="1" t="inlineStr">
         <is>
-          <t>MM-9946M</t>
+          <t>MM-9945M</t>
         </is>
       </c>
       <c r="H84" s="1" t="inlineStr">
         <is>
-          <t>NR25</t>
+          <t>NR21</t>
         </is>
       </c>
     </row>
@@ -3948,12 +3948,12 @@
       </c>
       <c r="G85" s="1" t="inlineStr">
         <is>
-          <t>MM-9949M</t>
+          <t>MM-9946M</t>
         </is>
       </c>
       <c r="H85" s="1" t="inlineStr">
         <is>
-          <t>NR27</t>
+          <t>NR25</t>
         </is>
       </c>
     </row>
@@ -3990,12 +3990,12 @@
       </c>
       <c r="G86" s="1" t="inlineStr">
         <is>
-          <t>MM-9950M</t>
+          <t>MM-9949M</t>
         </is>
       </c>
       <c r="H86" s="1" t="inlineStr">
         <is>
-          <t>NR28</t>
+          <t>NR27</t>
         </is>
       </c>
     </row>
@@ -4032,12 +4032,12 @@
       </c>
       <c r="G87" s="1" t="inlineStr">
         <is>
-          <t>MM-9951M</t>
+          <t>MM-9950M</t>
         </is>
       </c>
       <c r="H87" s="1" t="inlineStr">
         <is>
-          <t>NR29</t>
+          <t>NR28</t>
         </is>
       </c>
     </row>
@@ -4074,12 +4074,12 @@
       </c>
       <c r="G88" s="1" t="inlineStr">
         <is>
-          <t>MM-9952M</t>
+          <t>MM-9951M</t>
         </is>
       </c>
       <c r="H88" s="1" t="inlineStr">
         <is>
-          <t>NR30</t>
+          <t>NR29</t>
         </is>
       </c>
     </row>
@@ -4116,12 +4116,12 @@
       </c>
       <c r="G89" s="1" t="inlineStr">
         <is>
-          <t>MM-9953M</t>
+          <t>MM-9952M</t>
         </is>
       </c>
       <c r="H89" s="1" t="inlineStr">
         <is>
-          <t>NR31</t>
+          <t>NR30</t>
         </is>
       </c>
     </row>
@@ -4158,12 +4158,12 @@
       </c>
       <c r="G90" s="1" t="inlineStr">
         <is>
-          <t>MM-9954M</t>
+          <t>MM-9953M</t>
         </is>
       </c>
       <c r="H90" s="1" t="inlineStr">
         <is>
-          <t>NR34</t>
+          <t>NR31</t>
         </is>
       </c>
     </row>
@@ -4200,12 +4200,12 @@
       </c>
       <c r="G91" s="1" t="inlineStr">
         <is>
-          <t>MM-9955M</t>
+          <t>MM-9954M</t>
         </is>
       </c>
       <c r="H91" s="1" t="inlineStr">
         <is>
-          <t>NR36</t>
+          <t>NR34</t>
         </is>
       </c>
     </row>
@@ -4242,12 +4242,12 @@
       </c>
       <c r="G92" s="1" t="inlineStr">
         <is>
-          <t>MM-9957M</t>
+          <t>MM-9955M</t>
         </is>
       </c>
       <c r="H92" s="1" t="inlineStr">
         <is>
-          <t>NR37</t>
+          <t>NR36</t>
         </is>
       </c>
     </row>
@@ -4284,12 +4284,12 @@
       </c>
       <c r="G93" s="1" t="inlineStr">
         <is>
-          <t>MM-9958M</t>
+          <t>MM-9957M</t>
         </is>
       </c>
       <c r="H93" s="1" t="inlineStr">
         <is>
-          <t>NR38</t>
+          <t>NR37</t>
         </is>
       </c>
     </row>
@@ -4326,12 +4326,12 @@
       </c>
       <c r="G94" s="1" t="inlineStr">
         <is>
-          <t>MM-9959M</t>
+          <t>MM-9958M</t>
         </is>
       </c>
       <c r="H94" s="1" t="inlineStr">
         <is>
-          <t>NR39</t>
+          <t>NR38</t>
         </is>
       </c>
     </row>
@@ -4368,12 +4368,12 @@
       </c>
       <c r="G95" s="1" t="inlineStr">
         <is>
-          <t>MM-9960M</t>
+          <t>MM-9959M</t>
         </is>
       </c>
       <c r="H95" s="1" t="inlineStr">
         <is>
-          <t>NR40</t>
+          <t>NR39</t>
         </is>
       </c>
     </row>
@@ -4410,12 +4410,12 @@
       </c>
       <c r="G96" s="1" t="inlineStr">
         <is>
-          <t>MM-9961M</t>
+          <t>MM-9960M</t>
         </is>
       </c>
       <c r="H96" s="1" t="inlineStr">
         <is>
-          <t>NR43</t>
+          <t>NR40</t>
         </is>
       </c>
     </row>
@@ -4452,12 +4452,12 @@
       </c>
       <c r="G97" s="1" t="inlineStr">
         <is>
-          <t>MM-9962M</t>
+          <t>MM-9961M</t>
         </is>
       </c>
       <c r="H97" s="1" t="inlineStr">
         <is>
-          <t>NR44</t>
+          <t>NR43</t>
         </is>
       </c>
     </row>
@@ -4494,12 +4494,12 @@
       </c>
       <c r="G98" s="1" t="inlineStr">
         <is>
-          <t>MM-9963M</t>
+          <t>MM-9962M</t>
         </is>
       </c>
       <c r="H98" s="1" t="inlineStr">
         <is>
-          <t>NR45</t>
+          <t>NR44</t>
         </is>
       </c>
     </row>
@@ -4536,12 +4536,12 @@
       </c>
       <c r="G99" s="1" t="inlineStr">
         <is>
-          <t>MM-9964M</t>
+          <t>MM-9963M</t>
         </is>
       </c>
       <c r="H99" s="1" t="inlineStr">
         <is>
-          <t>NR46</t>
+          <t>NR45</t>
         </is>
       </c>
     </row>
@@ -4578,12 +4578,12 @@
       </c>
       <c r="G100" s="1" t="inlineStr">
         <is>
-          <t>MM-9965M</t>
+          <t>MM-9964M</t>
         </is>
       </c>
       <c r="H100" s="1" t="inlineStr">
         <is>
-          <t>NR47</t>
+          <t>NR46</t>
         </is>
       </c>
     </row>
@@ -4620,12 +4620,12 @@
       </c>
       <c r="G101" s="1" t="inlineStr">
         <is>
-          <t>MM-9966M</t>
+          <t>MM-9965M</t>
         </is>
       </c>
       <c r="H101" s="1" t="inlineStr">
         <is>
-          <t>NR48</t>
+          <t>NR47</t>
         </is>
       </c>
     </row>
@@ -4662,12 +4662,12 @@
       </c>
       <c r="G102" s="1" t="inlineStr">
         <is>
-          <t>MM-9967M</t>
+          <t>MM-9966M</t>
         </is>
       </c>
       <c r="H102" s="1" t="inlineStr">
         <is>
-          <t>NR51</t>
+          <t>NR48</t>
         </is>
       </c>
     </row>
@@ -4704,12 +4704,12 @@
       </c>
       <c r="G103" s="1" t="inlineStr">
         <is>
-          <t>MM-9968M</t>
+          <t>MM-9967M</t>
         </is>
       </c>
       <c r="H103" s="1" t="inlineStr">
         <is>
-          <t>NR52</t>
+          <t>NR51</t>
         </is>
       </c>
     </row>
@@ -4746,12 +4746,12 @@
       </c>
       <c r="G104" s="1" t="inlineStr">
         <is>
-          <t>MM-9969M</t>
+          <t>MM-9968M</t>
         </is>
       </c>
       <c r="H104" s="1" t="inlineStr">
         <is>
-          <t>NR53</t>
+          <t>NR52</t>
         </is>
       </c>
     </row>
@@ -4788,12 +4788,12 @@
       </c>
       <c r="G105" s="1" t="inlineStr">
         <is>
-          <t>MM-9970M</t>
+          <t>MM-9969M</t>
         </is>
       </c>
       <c r="H105" s="1" t="inlineStr">
         <is>
-          <t>NR54</t>
+          <t>NR53</t>
         </is>
       </c>
     </row>
@@ -4830,12 +4830,12 @@
       </c>
       <c r="G106" s="1" t="inlineStr">
         <is>
-          <t>MMY032</t>
+          <t>MM-9970M</t>
         </is>
       </c>
       <c r="H106" s="1" t="inlineStr">
         <is>
-          <t>NR57</t>
+          <t>NR54</t>
         </is>
       </c>
     </row>
@@ -4872,12 +4872,12 @@
       </c>
       <c r="G107" s="1" t="inlineStr">
         <is>
-          <t>MRL001</t>
+          <t>MMY032</t>
         </is>
       </c>
       <c r="H107" s="1" t="inlineStr">
         <is>
-          <t>NR58</t>
+          <t>NR57</t>
         </is>
       </c>
     </row>
@@ -4914,12 +4914,12 @@
       </c>
       <c r="G108" s="1" t="inlineStr">
         <is>
-          <t>MRL004</t>
+          <t>MRL001</t>
         </is>
       </c>
       <c r="H108" s="1" t="inlineStr">
         <is>
-          <t>NR59</t>
+          <t>NR58</t>
         </is>
       </c>
     </row>
@@ -4956,12 +4956,12 @@
       </c>
       <c r="G109" s="1" t="inlineStr">
         <is>
-          <t>MRL005</t>
+          <t>MRL004</t>
         </is>
       </c>
       <c r="H109" s="1" t="inlineStr">
         <is>
-          <t>NR61</t>
+          <t>NR59</t>
         </is>
       </c>
     </row>
@@ -4998,12 +4998,12 @@
       </c>
       <c r="G110" s="1" t="inlineStr">
         <is>
-          <t>MRL006</t>
+          <t>MRL005</t>
         </is>
       </c>
       <c r="H110" s="1" t="inlineStr">
         <is>
-          <t>NR62</t>
+          <t>NR61</t>
         </is>
       </c>
     </row>
@@ -5040,12 +5040,12 @@
       </c>
       <c r="G111" s="1" t="inlineStr">
         <is>
-          <t>MTPV2</t>
+          <t>MRL006</t>
         </is>
       </c>
       <c r="H111" s="1" t="inlineStr">
         <is>
-          <t>NR64</t>
+          <t>NR62</t>
         </is>
       </c>
     </row>
@@ -5082,12 +5082,12 @@
       </c>
       <c r="G112" s="1" t="inlineStr">
         <is>
-          <t>N452</t>
+          <t>MTPV2</t>
         </is>
       </c>
       <c r="H112" s="1" t="inlineStr">
         <is>
-          <t>NR65</t>
+          <t>NR64</t>
         </is>
       </c>
     </row>
@@ -5124,2896 +5124,2911 @@
       </c>
       <c r="G113" s="1" t="inlineStr">
         <is>
-          <t>N453</t>
+          <t>N452</t>
         </is>
       </c>
       <c r="H113" s="1" t="inlineStr">
         <is>
-          <t>NR66</t>
+          <t>NR65</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
         <is>
-          <t>NR67</t>
+          <t>NR66</t>
         </is>
       </c>
       <c r="B115" s="1" t="inlineStr">
         <is>
-          <t>P2510</t>
+          <t>P2509</t>
         </is>
       </c>
       <c r="C115" s="1" t="inlineStr">
         <is>
-          <t>RL305</t>
+          <t>RL304</t>
         </is>
       </c>
       <c r="D115" s="1" t="inlineStr">
         <is>
-          <t>TE2806</t>
+          <t>TE2805</t>
         </is>
       </c>
       <c r="E115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8050</t>
+          <t>VLINE-8049</t>
         </is>
       </c>
       <c r="F115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8159</t>
+          <t>VLINE-8158</t>
         </is>
       </c>
       <c r="G115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8420</t>
+          <t>VLINE-8418</t>
         </is>
       </c>
       <c r="H115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8727</t>
+          <t>VLINE-8725</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
         <is>
-          <t>NR68</t>
+          <t>NR67</t>
         </is>
       </c>
       <c r="B116" s="1" t="inlineStr">
         <is>
-          <t>P2511</t>
+          <t>P2510</t>
         </is>
       </c>
       <c r="C116" s="1" t="inlineStr">
         <is>
-          <t>RL306</t>
+          <t>RL305</t>
         </is>
       </c>
       <c r="D116" s="1" t="inlineStr">
         <is>
-          <t>TE2807</t>
+          <t>TE2806</t>
         </is>
       </c>
       <c r="E116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8051</t>
+          <t>VLINE-8050</t>
         </is>
       </c>
       <c r="F116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8160</t>
+          <t>VLINE-8159</t>
         </is>
       </c>
       <c r="G116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8421</t>
+          <t>VLINE-8419</t>
         </is>
       </c>
       <c r="H116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8729</t>
+          <t>VLINE-8726</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="1" t="inlineStr">
         <is>
-          <t>NR69</t>
+          <t>NR68</t>
         </is>
       </c>
       <c r="B117" s="1" t="inlineStr">
         <is>
-          <t>P2513</t>
+          <t>P2511</t>
         </is>
       </c>
       <c r="C117" s="1" t="inlineStr">
         <is>
-          <t>RL307</t>
+          <t>RL306</t>
         </is>
       </c>
       <c r="D117" s="1" t="inlineStr">
         <is>
-          <t>TE2808</t>
+          <t>TE2807</t>
         </is>
       </c>
       <c r="E117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8052</t>
+          <t>VLINE-8051</t>
         </is>
       </c>
       <c r="F117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8161</t>
+          <t>VLINE-8160</t>
         </is>
       </c>
       <c r="G117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8422</t>
+          <t>VLINE-8420</t>
         </is>
       </c>
       <c r="H117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8730</t>
+          <t>VLINE-8727</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
         <is>
-          <t>NR71</t>
+          <t>NR69</t>
         </is>
       </c>
       <c r="B118" s="1" t="inlineStr">
         <is>
-          <t>P2514</t>
+          <t>P2513</t>
         </is>
       </c>
       <c r="C118" s="1" t="inlineStr">
         <is>
-          <t>RL309</t>
+          <t>RL307</t>
         </is>
       </c>
       <c r="D118" s="1" t="inlineStr">
         <is>
-          <t>TE2809</t>
+          <t>TE2808</t>
         </is>
       </c>
       <c r="E118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8053</t>
+          <t>VLINE-8052</t>
         </is>
       </c>
       <c r="F118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8162</t>
+          <t>VLINE-8161</t>
         </is>
       </c>
       <c r="G118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8424</t>
+          <t>VLINE-8421</t>
         </is>
       </c>
       <c r="H118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8731</t>
+          <t>VLINE-8729</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
         <is>
-          <t>NR72</t>
+          <t>NR71</t>
         </is>
       </c>
       <c r="B119" s="1" t="inlineStr">
         <is>
-          <t>P2515</t>
+          <t>P2514</t>
         </is>
       </c>
       <c r="C119" s="1" t="inlineStr">
         <is>
-          <t>RL310</t>
+          <t>RL309</t>
         </is>
       </c>
       <c r="D119" s="1" t="inlineStr">
         <is>
-          <t>TE2810</t>
+          <t>TE2809</t>
         </is>
       </c>
       <c r="E119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8055</t>
+          <t>VLINE-8053</t>
         </is>
       </c>
       <c r="F119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8171</t>
+          <t>VLINE-8162</t>
         </is>
       </c>
       <c r="G119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8425</t>
+          <t>VLINE-8422</t>
         </is>
       </c>
       <c r="H119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8733</t>
+          <t>VLINE-8730</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="1" t="inlineStr">
         <is>
-          <t>NR75</t>
+          <t>NR72</t>
         </is>
       </c>
       <c r="B120" s="1" t="inlineStr">
         <is>
-          <t>P2516</t>
+          <t>P2515</t>
         </is>
       </c>
       <c r="C120" s="1" t="inlineStr">
         <is>
-          <t>S312</t>
+          <t>RL310</t>
         </is>
       </c>
       <c r="D120" s="1" t="inlineStr">
         <is>
-          <t>TE2812</t>
+          <t>TE2810</t>
         </is>
       </c>
       <c r="E120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8056</t>
+          <t>VLINE-8055</t>
         </is>
       </c>
       <c r="F120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8172</t>
+          <t>VLINE-8165</t>
         </is>
       </c>
       <c r="G120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8426</t>
+          <t>VLINE-8424</t>
         </is>
       </c>
       <c r="H120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8735</t>
+          <t>VLINE-8731</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="1" t="inlineStr">
         <is>
-          <t>NR77</t>
+          <t>NR75</t>
         </is>
       </c>
       <c r="B121" s="1" t="inlineStr">
         <is>
-          <t>PB1</t>
+          <t>P2516</t>
         </is>
       </c>
       <c r="C121" s="1" t="inlineStr">
         <is>
-          <t>S317</t>
+          <t>S312</t>
         </is>
       </c>
       <c r="D121" s="1" t="inlineStr">
         <is>
-          <t>TE2813</t>
+          <t>TE2812</t>
         </is>
       </c>
       <c r="E121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8057</t>
+          <t>VLINE-8056</t>
         </is>
       </c>
       <c r="F121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8176</t>
+          <t>VLINE-8171</t>
         </is>
       </c>
       <c r="G121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8427</t>
+          <t>VLINE-8425</t>
         </is>
       </c>
       <c r="H121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8736</t>
+          <t>VLINE-8733</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="1" t="inlineStr">
         <is>
-          <t>NR78</t>
+          <t>NR77</t>
         </is>
       </c>
       <c r="B122" s="1" t="inlineStr">
         <is>
-          <t>PB2</t>
+          <t>PB1</t>
         </is>
       </c>
       <c r="C122" s="1" t="inlineStr">
         <is>
-          <t>S3301</t>
+          <t>S317</t>
         </is>
       </c>
       <c r="D122" s="1" t="inlineStr">
         <is>
-          <t>TE2814</t>
+          <t>TE2813</t>
         </is>
       </c>
       <c r="E122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8058</t>
+          <t>VLINE-8057</t>
         </is>
       </c>
       <c r="F122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8179</t>
+          <t>VLINE-8172</t>
         </is>
       </c>
       <c r="G122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8428</t>
+          <t>VLINE-8426</t>
         </is>
       </c>
       <c r="H122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8737</t>
+          <t>VLINE-8735</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="1" t="inlineStr">
         <is>
-          <t>NR81</t>
+          <t>NR78</t>
         </is>
       </c>
       <c r="B123" s="1" t="inlineStr">
         <is>
-          <t>PB4</t>
+          <t>PB2</t>
         </is>
       </c>
       <c r="C123" s="1" t="inlineStr">
         <is>
-          <t>S3302</t>
+          <t>S3301</t>
         </is>
       </c>
       <c r="D123" s="1" t="inlineStr">
         <is>
-          <t>TJ096</t>
+          <t>TE2814</t>
         </is>
       </c>
       <c r="E123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8059</t>
+          <t>VLINE-8058</t>
         </is>
       </c>
       <c r="F123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8180</t>
+          <t>VLINE-8176</t>
         </is>
       </c>
       <c r="G123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8429</t>
+          <t>VLINE-8427</t>
         </is>
       </c>
       <c r="H123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8739</t>
+          <t>VLINE-8736</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="1" t="inlineStr">
         <is>
-          <t>NR82</t>
+          <t>NR81</t>
         </is>
       </c>
       <c r="B124" s="1" t="inlineStr">
         <is>
-          <t>PHC001</t>
+          <t>PB4</t>
         </is>
       </c>
       <c r="C124" s="1" t="inlineStr">
         <is>
-          <t>S3304</t>
+          <t>S3302</t>
         </is>
       </c>
       <c r="D124" s="1" t="inlineStr">
         <is>
-          <t>TJ107</t>
+          <t>TJ096</t>
         </is>
       </c>
       <c r="E124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8061</t>
+          <t>VLINE-8059</t>
         </is>
       </c>
       <c r="F124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8181</t>
+          <t>VLINE-8179</t>
         </is>
       </c>
       <c r="G124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8430</t>
+          <t>VLINE-8428</t>
         </is>
       </c>
       <c r="H124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8740</t>
+          <t>VLINE-8737</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="1" t="inlineStr">
         <is>
-          <t>NR83</t>
+          <t>NR82</t>
         </is>
       </c>
       <c r="B125" s="1" t="inlineStr">
         <is>
-          <t>PHC002</t>
+          <t>PHC001</t>
         </is>
       </c>
       <c r="C125" s="1" t="inlineStr">
         <is>
-          <t>S3305</t>
+          <t>S3304</t>
         </is>
       </c>
       <c r="D125" s="1" t="inlineStr">
         <is>
-          <t>TT03</t>
+          <t>TJ107</t>
         </is>
       </c>
       <c r="E125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8072</t>
+          <t>VLINE-8061</t>
         </is>
       </c>
       <c r="F125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8182</t>
+          <t>VLINE-8180</t>
         </is>
       </c>
       <c r="G125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8431</t>
+          <t>VLINE-8429</t>
         </is>
       </c>
       <c r="H125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8741</t>
+          <t>VLINE-8739</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="1" t="inlineStr">
         <is>
-          <t>NR84</t>
+          <t>NR83</t>
         </is>
       </c>
       <c r="B126" s="1" t="inlineStr">
         <is>
-          <t>Q4001</t>
+          <t>PHC002</t>
         </is>
       </c>
       <c r="C126" s="1" t="inlineStr">
         <is>
-          <t>S3306</t>
+          <t>S3305</t>
         </is>
       </c>
       <c r="D126" s="1" t="inlineStr">
         <is>
-          <t>TT04</t>
+          <t>TT03</t>
         </is>
       </c>
       <c r="E126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8074</t>
+          <t>VLINE-8072</t>
         </is>
       </c>
       <c r="F126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8183</t>
+          <t>VLINE-8181</t>
         </is>
       </c>
       <c r="G126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8432</t>
+          <t>VLINE-8430</t>
         </is>
       </c>
       <c r="H126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8742</t>
+          <t>VLINE-8740</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
         <is>
-          <t>NR85</t>
+          <t>NR84</t>
         </is>
       </c>
       <c r="B127" s="1" t="inlineStr">
         <is>
-          <t>Q4003</t>
+          <t>Q4001</t>
         </is>
       </c>
       <c r="C127" s="1" t="inlineStr">
         <is>
-          <t>S3307</t>
+          <t>S3306</t>
         </is>
       </c>
       <c r="D127" s="1" t="inlineStr">
         <is>
-          <t>TT05</t>
+          <t>TT04</t>
         </is>
       </c>
       <c r="E127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8075</t>
+          <t>VLINE-8074</t>
         </is>
       </c>
       <c r="F127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8184</t>
+          <t>VLINE-8182</t>
         </is>
       </c>
       <c r="G127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8433</t>
+          <t>VLINE-8431</t>
         </is>
       </c>
       <c r="H127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8743</t>
+          <t>VLINE-8741</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
         <is>
-          <t>NR86</t>
+          <t>NR85</t>
         </is>
       </c>
       <c r="B128" s="1" t="inlineStr">
         <is>
-          <t>Q4004</t>
+          <t>Q4003</t>
         </is>
       </c>
       <c r="C128" s="1" t="inlineStr">
         <is>
-          <t>S3309</t>
+          <t>S3307</t>
         </is>
       </c>
       <c r="D128" s="1" t="inlineStr">
         <is>
-          <t>TT07</t>
+          <t>TT05</t>
         </is>
       </c>
       <c r="E128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8076</t>
+          <t>VLINE-8075</t>
         </is>
       </c>
       <c r="F128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8185</t>
+          <t>VLINE-8183</t>
         </is>
       </c>
       <c r="G128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8434</t>
+          <t>VLINE-8432</t>
         </is>
       </c>
       <c r="H128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8744</t>
+          <t>VLINE-8742</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
         <is>
-          <t>NR87</t>
+          <t>NR86</t>
         </is>
       </c>
       <c r="B129" s="1" t="inlineStr">
         <is>
-          <t>Q4005</t>
+          <t>Q4004</t>
         </is>
       </c>
       <c r="C129" s="1" t="inlineStr">
         <is>
-          <t>S3310</t>
+          <t>S3309</t>
         </is>
       </c>
       <c r="D129" s="1" t="inlineStr">
         <is>
-          <t>TT08</t>
+          <t>TT07</t>
         </is>
       </c>
       <c r="E129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8077</t>
+          <t>VLINE-8076</t>
         </is>
       </c>
       <c r="F129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8186</t>
+          <t>VLINE-8184</t>
         </is>
       </c>
       <c r="G129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8435</t>
+          <t>VLINE-8433</t>
         </is>
       </c>
       <c r="H129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8745</t>
+          <t>VLINE-8743</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="1" t="inlineStr">
         <is>
-          <t>NR88</t>
+          <t>NR87</t>
         </is>
       </c>
       <c r="B130" s="1" t="inlineStr">
         <is>
-          <t>Q4006</t>
+          <t>Q4005</t>
         </is>
       </c>
       <c r="C130" s="1" t="inlineStr">
         <is>
-          <t>S7001</t>
+          <t>S3310</t>
         </is>
       </c>
       <c r="D130" s="1" t="inlineStr">
         <is>
-          <t>TT103</t>
+          <t>TT08</t>
         </is>
       </c>
       <c r="E130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8080</t>
+          <t>VLINE-8077</t>
         </is>
       </c>
       <c r="F130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8187</t>
+          <t>VLINE-8185</t>
         </is>
       </c>
       <c r="G130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8438</t>
+          <t>VLINE-8434</t>
         </is>
       </c>
       <c r="H130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8746</t>
+          <t>VLINE-8744</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="1" t="inlineStr">
         <is>
-          <t>NR89</t>
+          <t>NR88</t>
         </is>
       </c>
       <c r="B131" s="1" t="inlineStr">
         <is>
-          <t>Q4007</t>
+          <t>Q4006</t>
         </is>
       </c>
       <c r="C131" s="1" t="inlineStr">
         <is>
-          <t>S7002</t>
+          <t>S7001</t>
         </is>
       </c>
       <c r="D131" s="1" t="inlineStr">
         <is>
-          <t>TT106</t>
+          <t>TT103</t>
         </is>
       </c>
       <c r="E131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8081</t>
+          <t>VLINE-8080</t>
         </is>
       </c>
       <c r="F131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8188</t>
+          <t>VLINE-8186</t>
         </is>
       </c>
       <c r="G131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8440</t>
+          <t>VLINE-8435</t>
         </is>
       </c>
       <c r="H131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8747</t>
+          <t>VLINE-8745</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="1" t="inlineStr">
         <is>
-          <t>NR90</t>
+          <t>NR89</t>
         </is>
       </c>
       <c r="B132" s="1" t="inlineStr">
         <is>
-          <t>Q4009</t>
+          <t>Q4007</t>
         </is>
       </c>
       <c r="C132" s="1" t="inlineStr">
         <is>
-          <t>S7003</t>
+          <t>S7002</t>
         </is>
       </c>
       <c r="D132" s="1" t="inlineStr">
         <is>
-          <t>TT107</t>
+          <t>TT106</t>
         </is>
       </c>
       <c r="E132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8084</t>
+          <t>VLINE-8081</t>
         </is>
       </c>
       <c r="F132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8189</t>
+          <t>VLINE-8187</t>
         </is>
       </c>
       <c r="G132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8441</t>
+          <t>VLINE-8438</t>
         </is>
       </c>
       <c r="H132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8748</t>
+          <t>VLINE-8746</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="1" t="inlineStr">
         <is>
-          <t>NR91</t>
+          <t>NR90</t>
         </is>
       </c>
       <c r="B133" s="1" t="inlineStr">
         <is>
-          <t>Q4011</t>
+          <t>Q4009</t>
         </is>
       </c>
       <c r="C133" s="1" t="inlineStr">
         <is>
-          <t>S7004</t>
+          <t>S7003</t>
         </is>
       </c>
       <c r="D133" s="1" t="inlineStr">
         <is>
-          <t>TT108</t>
+          <t>TT107</t>
         </is>
       </c>
       <c r="E133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8088</t>
+          <t>VLINE-8084</t>
         </is>
       </c>
       <c r="F133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8291</t>
+          <t>VLINE-8188</t>
         </is>
       </c>
       <c r="G133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8442</t>
+          <t>VLINE-8440</t>
         </is>
       </c>
       <c r="H133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8749</t>
+          <t>VLINE-8747</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="1" t="inlineStr">
         <is>
-          <t>NR92</t>
+          <t>NR91</t>
         </is>
       </c>
       <c r="B134" s="1" t="inlineStr">
         <is>
-          <t>Q4012</t>
+          <t>Q4011</t>
         </is>
       </c>
       <c r="C134" s="1" t="inlineStr">
         <is>
-          <t>S7005</t>
+          <t>S7004</t>
         </is>
       </c>
       <c r="D134" s="1" t="inlineStr">
         <is>
-          <t>TT110</t>
+          <t>TT108</t>
         </is>
       </c>
       <c r="E134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8089</t>
+          <t>VLINE-8088</t>
         </is>
       </c>
       <c r="F134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8293</t>
+          <t>VLINE-8189</t>
         </is>
       </c>
       <c r="G134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8443</t>
+          <t>VLINE-8441</t>
         </is>
       </c>
       <c r="H134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8750</t>
+          <t>VLINE-8748</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="1" t="inlineStr">
         <is>
-          <t>NR93</t>
+          <t>NR92</t>
         </is>
       </c>
       <c r="B135" s="1" t="inlineStr">
         <is>
-          <t>Q4013</t>
+          <t>Q4012</t>
         </is>
       </c>
       <c r="C135" s="1" t="inlineStr">
         <is>
-          <t>S7006</t>
+          <t>S7005</t>
         </is>
       </c>
       <c r="D135" s="1" t="inlineStr">
         <is>
-          <t>TT113</t>
+          <t>TT110</t>
         </is>
       </c>
       <c r="E135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8104</t>
+          <t>VLINE-8089</t>
         </is>
       </c>
       <c r="F135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8303</t>
+          <t>VLINE-8291</t>
         </is>
       </c>
       <c r="G135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8444</t>
+          <t>VLINE-8442</t>
         </is>
       </c>
       <c r="H135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8751</t>
+          <t>VLINE-8749</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="1" t="inlineStr">
         <is>
-          <t>NR94</t>
+          <t>NR93</t>
         </is>
       </c>
       <c r="B136" s="1" t="inlineStr">
         <is>
-          <t>Q4014</t>
+          <t>Q4013</t>
         </is>
       </c>
       <c r="C136" s="1" t="inlineStr">
         <is>
-          <t>S7007</t>
+          <t>S7006</t>
         </is>
       </c>
       <c r="D136" s="1" t="inlineStr">
         <is>
-          <t>TT114</t>
+          <t>TT113</t>
         </is>
       </c>
       <c r="E136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8107</t>
+          <t>VLINE-8104</t>
         </is>
       </c>
       <c r="F136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8304</t>
+          <t>VLINE-8293</t>
         </is>
       </c>
       <c r="G136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8446</t>
+          <t>VLINE-8443</t>
         </is>
       </c>
       <c r="H136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8752</t>
+          <t>VLINE-8750</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="1" t="inlineStr">
         <is>
-          <t>NR95</t>
+          <t>NR94</t>
         </is>
       </c>
       <c r="B137" s="1" t="inlineStr">
         <is>
-          <t>Q4015</t>
+          <t>Q4014</t>
         </is>
       </c>
       <c r="C137" s="1" t="inlineStr">
         <is>
-          <t>S7008</t>
+          <t>S7007</t>
         </is>
       </c>
       <c r="D137" s="1" t="inlineStr">
         <is>
-          <t>TT115</t>
+          <t>TT114</t>
         </is>
       </c>
       <c r="E137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8110</t>
+          <t>VLINE-8107</t>
         </is>
       </c>
       <c r="F137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8306</t>
+          <t>VLINE-8303</t>
         </is>
       </c>
       <c r="G137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8447</t>
+          <t>VLINE-8444</t>
         </is>
       </c>
       <c r="H137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8753</t>
+          <t>VLINE-8751</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="1" t="inlineStr">
         <is>
-          <t>NR96</t>
+          <t>NR95</t>
         </is>
       </c>
       <c r="B138" s="1" t="inlineStr">
         <is>
-          <t>Q4016</t>
+          <t>Q4015</t>
         </is>
       </c>
       <c r="C138" s="1" t="inlineStr">
         <is>
-          <t>S7009</t>
+          <t>S7008</t>
         </is>
       </c>
       <c r="D138" s="1" t="inlineStr">
         <is>
-          <t>TT116</t>
+          <t>TT115</t>
         </is>
       </c>
       <c r="E138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8111</t>
+          <t>VLINE-8110</t>
         </is>
       </c>
       <c r="F138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8311</t>
+          <t>VLINE-8304</t>
         </is>
       </c>
       <c r="G138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8449</t>
+          <t>VLINE-8446</t>
         </is>
       </c>
       <c r="H138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8754</t>
+          <t>VLINE-8752</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="1" t="inlineStr">
         <is>
-          <t>NR97</t>
+          <t>NR96</t>
         </is>
       </c>
       <c r="B139" s="1" t="inlineStr">
         <is>
-          <t>Q4017</t>
+          <t>Q4016</t>
         </is>
       </c>
       <c r="C139" s="1" t="inlineStr">
         <is>
-          <t>S7012</t>
+          <t>S7009</t>
         </is>
       </c>
       <c r="D139" s="1" t="inlineStr">
         <is>
-          <t>TT117</t>
+          <t>TT116</t>
         </is>
       </c>
       <c r="E139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8113</t>
+          <t>VLINE-8111</t>
         </is>
       </c>
       <c r="F139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8313</t>
+          <t>VLINE-8306</t>
         </is>
       </c>
       <c r="G139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8450</t>
+          <t>VLINE-8447</t>
         </is>
       </c>
       <c r="H139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8755</t>
+          <t>VLINE-8753</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="1" t="inlineStr">
         <is>
-          <t>NR98</t>
+          <t>NR97</t>
         </is>
       </c>
       <c r="B140" s="1" t="inlineStr">
         <is>
-          <t>Q4019</t>
+          <t>Q4017</t>
         </is>
       </c>
       <c r="C140" s="1" t="inlineStr">
         <is>
-          <t>S7013</t>
+          <t>S7012</t>
         </is>
       </c>
       <c r="D140" s="1" t="inlineStr">
         <is>
-          <t>TT122</t>
+          <t>TT117</t>
         </is>
       </c>
       <c r="E140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8114</t>
+          <t>VLINE-8113</t>
         </is>
       </c>
       <c r="F140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8314</t>
+          <t>VLINE-8311</t>
         </is>
       </c>
       <c r="G140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8451</t>
+          <t>VLINE-8449</t>
         </is>
       </c>
       <c r="H140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8756</t>
+          <t>VLINE-8754</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="1" t="inlineStr">
         <is>
-          <t>NR99</t>
+          <t>NR98</t>
         </is>
       </c>
       <c r="B141" s="1" t="inlineStr">
         <is>
-          <t>QBX003</t>
+          <t>Q4019</t>
         </is>
       </c>
       <c r="C141" s="1" t="inlineStr">
         <is>
-          <t>S7014</t>
+          <t>S7013</t>
         </is>
       </c>
       <c r="D141" s="1" t="inlineStr">
         <is>
-          <t>TT127</t>
+          <t>TT122</t>
         </is>
       </c>
       <c r="E141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8115</t>
+          <t>VLINE-8114</t>
         </is>
       </c>
       <c r="F141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8316</t>
+          <t>VLINE-8313</t>
         </is>
       </c>
       <c r="G141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8452</t>
+          <t>VLINE-8450</t>
         </is>
       </c>
       <c r="H141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8757</t>
+          <t>VLINE-8755</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="1" t="inlineStr">
         <is>
-          <t>NR101</t>
+          <t>NR99</t>
         </is>
       </c>
       <c r="B142" s="1" t="inlineStr">
         <is>
-          <t>QBX004</t>
+          <t>QBX003</t>
         </is>
       </c>
       <c r="C142" s="1" t="inlineStr">
         <is>
-          <t>S7015</t>
+          <t>S7014</t>
         </is>
       </c>
       <c r="D142" s="1" t="inlineStr">
         <is>
-          <t>TT128</t>
+          <t>TT127</t>
         </is>
       </c>
       <c r="E142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8119</t>
+          <t>VLINE-8115</t>
         </is>
       </c>
       <c r="F142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8318</t>
+          <t>VLINE-8314</t>
         </is>
       </c>
       <c r="G142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8453</t>
+          <t>VLINE-8451</t>
         </is>
       </c>
       <c r="H142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8758</t>
+          <t>VLINE-8756</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="1" t="inlineStr">
         <is>
-          <t>NR102</t>
+          <t>NR101</t>
         </is>
       </c>
       <c r="B143" s="1" t="inlineStr">
         <is>
-          <t>QBX005</t>
+          <t>QBX004</t>
         </is>
       </c>
       <c r="C143" s="1" t="inlineStr">
         <is>
-          <t>S7017</t>
+          <t>S7015</t>
         </is>
       </c>
       <c r="D143" s="1" t="inlineStr">
         <is>
-          <t>TT130</t>
+          <t>TT128</t>
         </is>
       </c>
       <c r="E143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8120</t>
+          <t>VLINE-8119</t>
         </is>
       </c>
       <c r="F143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8321</t>
+          <t>VLINE-8316</t>
         </is>
       </c>
       <c r="G143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8454</t>
+          <t>VLINE-8452</t>
         </is>
       </c>
       <c r="H143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8759</t>
+          <t>VLINE-8757</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="1" t="inlineStr">
         <is>
-          <t>NR103</t>
+          <t>NR102</t>
         </is>
       </c>
       <c r="B144" s="1" t="inlineStr">
         <is>
-          <t>QBX006</t>
+          <t>QBX005</t>
         </is>
       </c>
       <c r="C144" s="1" t="inlineStr">
         <is>
-          <t>S7018</t>
+          <t>S7017</t>
         </is>
       </c>
       <c r="D144" s="1" t="inlineStr">
         <is>
-          <t>TT131</t>
+          <t>TT130</t>
         </is>
       </c>
       <c r="E144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8121</t>
+          <t>VLINE-8120</t>
         </is>
       </c>
       <c r="F144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8323</t>
+          <t>VLINE-8318</t>
         </is>
       </c>
       <c r="G144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8455</t>
+          <t>VLINE-8453</t>
         </is>
       </c>
       <c r="H144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8760</t>
+          <t>VLINE-8758</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="1" t="inlineStr">
         <is>
-          <t>NR105</t>
+          <t>NR103</t>
         </is>
       </c>
       <c r="B145" s="1" t="inlineStr">
         <is>
-          <t>QE001</t>
+          <t>QBX006</t>
         </is>
       </c>
       <c r="C145" s="1" t="inlineStr">
         <is>
-          <t>S7020</t>
+          <t>S7018</t>
         </is>
       </c>
       <c r="D145" s="1" t="inlineStr">
         <is>
-          <t>TT202</t>
+          <t>TT131</t>
         </is>
       </c>
       <c r="E145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8123</t>
+          <t>VLINE-8121</t>
         </is>
       </c>
       <c r="F145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8324</t>
+          <t>VLINE-8321</t>
         </is>
       </c>
       <c r="G145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8456</t>
+          <t>VLINE-8454</t>
         </is>
       </c>
       <c r="H145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8761</t>
+          <t>VLINE-8759</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="1" t="inlineStr">
         <is>
-          <t>NR106</t>
+          <t>NR105</t>
         </is>
       </c>
       <c r="B146" s="1" t="inlineStr">
         <is>
-          <t>QE002</t>
+          <t>QE001</t>
         </is>
       </c>
       <c r="C146" s="1" t="inlineStr">
         <is>
-          <t>S7022</t>
+          <t>S7020</t>
         </is>
       </c>
       <c r="D146" s="1" t="inlineStr">
         <is>
-          <t>TT206</t>
+          <t>TT202</t>
         </is>
       </c>
       <c r="E146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8124</t>
+          <t>VLINE-8123</t>
         </is>
       </c>
       <c r="F146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8325</t>
+          <t>VLINE-8323</t>
         </is>
       </c>
       <c r="G146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8457</t>
+          <t>VLINE-8455</t>
         </is>
       </c>
       <c r="H146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8762</t>
+          <t>VLINE-8760</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="1" t="inlineStr">
         <is>
-          <t>NR107</t>
+          <t>NR106</t>
         </is>
       </c>
       <c r="B147" s="1" t="inlineStr">
         <is>
-          <t>QE003</t>
+          <t>QE002</t>
         </is>
       </c>
       <c r="C147" s="1" t="inlineStr">
         <is>
-          <t>SCT001</t>
+          <t>S7022</t>
         </is>
       </c>
       <c r="D147" s="1" t="inlineStr">
         <is>
-          <t>VL352</t>
+          <t>TT206</t>
         </is>
       </c>
       <c r="E147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8126</t>
+          <t>VLINE-8124</t>
         </is>
       </c>
       <c r="F147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8328</t>
+          <t>VLINE-8324</t>
         </is>
       </c>
       <c r="G147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8460</t>
+          <t>VLINE-8456</t>
         </is>
       </c>
       <c r="H147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8763</t>
+          <t>VLINE-8761</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="1" t="inlineStr">
         <is>
-          <t>NR108</t>
+          <t>NR107</t>
         </is>
       </c>
       <c r="B148" s="1" t="inlineStr">
         <is>
-          <t>QE004</t>
+          <t>QE003</t>
         </is>
       </c>
       <c r="C148" s="1" t="inlineStr">
         <is>
-          <t>SCT002</t>
+          <t>SCT001</t>
         </is>
       </c>
       <c r="D148" s="1" t="inlineStr">
         <is>
-          <t>VL353</t>
+          <t>VL352</t>
         </is>
       </c>
       <c r="E148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8127</t>
+          <t>VLINE-8126</t>
         </is>
       </c>
       <c r="F148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8329</t>
+          <t>VLINE-8325</t>
         </is>
       </c>
       <c r="G148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8461</t>
+          <t>VLINE-8457</t>
         </is>
       </c>
       <c r="H148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8764</t>
+          <t>VLINE-8762</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="1" t="inlineStr">
         <is>
-          <t>NR109</t>
+          <t>NR108</t>
         </is>
       </c>
       <c r="B149" s="1" t="inlineStr">
         <is>
-          <t>QE006</t>
+          <t>QE004</t>
         </is>
       </c>
       <c r="C149" s="1" t="inlineStr">
         <is>
-          <t>SCT006</t>
+          <t>SCT002</t>
         </is>
       </c>
       <c r="D149" s="1" t="inlineStr">
         <is>
-          <t>VL357</t>
+          <t>VL353</t>
         </is>
       </c>
       <c r="E149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8128</t>
+          <t>VLINE-8127</t>
         </is>
       </c>
       <c r="F149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8332</t>
+          <t>VLINE-8328</t>
         </is>
       </c>
       <c r="G149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8464</t>
+          <t>VLINE-8460</t>
         </is>
       </c>
       <c r="H149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8765</t>
+          <t>VLINE-8763</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="1" t="inlineStr">
         <is>
-          <t>NR110</t>
+          <t>NR109</t>
         </is>
       </c>
       <c r="B150" s="1" t="inlineStr">
         <is>
-          <t>QL001</t>
+          <t>QE006</t>
         </is>
       </c>
       <c r="C150" s="1" t="inlineStr">
         <is>
-          <t>SCT007</t>
+          <t>SCT006</t>
         </is>
       </c>
       <c r="D150" s="1" t="inlineStr">
         <is>
-          <t>VL359</t>
+          <t>VL357</t>
         </is>
       </c>
       <c r="E150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8129</t>
+          <t>VLINE-8128</t>
         </is>
       </c>
       <c r="F150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8336</t>
+          <t>VLINE-8329</t>
         </is>
       </c>
       <c r="G150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8465</t>
+          <t>VLINE-8461</t>
         </is>
       </c>
       <c r="H150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8766</t>
+          <t>VLINE-8764</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="1" t="inlineStr">
         <is>
-          <t>NR111</t>
+          <t>NR110</t>
         </is>
       </c>
       <c r="B151" s="1" t="inlineStr">
         <is>
-          <t>QL002</t>
+          <t>QL001</t>
         </is>
       </c>
       <c r="C151" s="1" t="inlineStr">
         <is>
-          <t>SCT009</t>
+          <t>SCT007</t>
         </is>
       </c>
       <c r="D151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8004</t>
+          <t>VL359</t>
         </is>
       </c>
       <c r="E151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8131</t>
+          <t>VLINE-8129</t>
         </is>
       </c>
       <c r="F151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8337</t>
+          <t>VLINE-8332</t>
         </is>
       </c>
       <c r="G151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8468</t>
+          <t>VLINE-8464</t>
         </is>
       </c>
       <c r="H151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8767</t>
+          <t>VLINE-8765</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="1" t="inlineStr">
         <is>
-          <t>NR112</t>
+          <t>NR111</t>
         </is>
       </c>
       <c r="B152" s="1" t="inlineStr">
         <is>
-          <t>QL004</t>
+          <t>QL002</t>
         </is>
       </c>
       <c r="C152" s="1" t="inlineStr">
         <is>
-          <t>SCT011</t>
+          <t>SCT009</t>
         </is>
       </c>
       <c r="D152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8007</t>
+          <t>VLINE-8004</t>
         </is>
       </c>
       <c r="E152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8132</t>
+          <t>VLINE-8131</t>
         </is>
       </c>
       <c r="F152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8338</t>
+          <t>VLINE-8336</t>
         </is>
       </c>
       <c r="G152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8469</t>
+          <t>VLINE-8465</t>
         </is>
       </c>
       <c r="H152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8768</t>
+          <t>VLINE-8766</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="1" t="inlineStr">
         <is>
-          <t>NR113</t>
+          <t>NR112</t>
         </is>
       </c>
       <c r="B153" s="1" t="inlineStr">
         <is>
-          <t>QL007</t>
+          <t>QL004</t>
         </is>
       </c>
       <c r="C153" s="1" t="inlineStr">
         <is>
-          <t>SCT013</t>
+          <t>SCT011</t>
         </is>
       </c>
       <c r="D153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8011</t>
+          <t>VLINE-8007</t>
         </is>
       </c>
       <c r="E153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8133</t>
+          <t>VLINE-8132</t>
         </is>
       </c>
       <c r="F153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8339</t>
+          <t>VLINE-8337</t>
         </is>
       </c>
       <c r="G153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8605</t>
+          <t>VLINE-8468</t>
         </is>
       </c>
       <c r="H153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8769</t>
+          <t>VLINE-8767</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="1" t="inlineStr">
         <is>
-          <t>NR115</t>
+          <t>NR113</t>
         </is>
       </c>
       <c r="B154" s="1" t="inlineStr">
         <is>
-          <t>QL008</t>
+          <t>QL007</t>
         </is>
       </c>
       <c r="C154" s="1" t="inlineStr">
         <is>
-          <t>SCT014</t>
+          <t>SCT013</t>
         </is>
       </c>
       <c r="D154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8013</t>
+          <t>VLINE-8011</t>
         </is>
       </c>
       <c r="E154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8134</t>
+          <t>VLINE-8133</t>
         </is>
       </c>
       <c r="F154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8362</t>
+          <t>VLINE-8338</t>
         </is>
       </c>
       <c r="G154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8610</t>
+          <t>VLINE-8469</t>
         </is>
       </c>
       <c r="H154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8770</t>
+          <t>VLINE-8768</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="1" t="inlineStr">
         <is>
-          <t>NR118</t>
+          <t>NR115</t>
         </is>
       </c>
       <c r="B155" s="1" t="inlineStr">
         <is>
-          <t>QL010</t>
+          <t>QL008</t>
         </is>
       </c>
       <c r="C155" s="1" t="inlineStr">
         <is>
-          <t>SCT015</t>
+          <t>SCT014</t>
         </is>
       </c>
       <c r="D155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8019</t>
+          <t>VLINE-8013</t>
         </is>
       </c>
       <c r="E155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8136</t>
+          <t>VLINE-8134</t>
         </is>
       </c>
       <c r="F155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8363</t>
+          <t>VLINE-8339</t>
         </is>
       </c>
       <c r="G155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8612</t>
+          <t>VLINE-8605</t>
         </is>
       </c>
       <c r="H155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8772</t>
+          <t>VLINE-8769</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="1" t="inlineStr">
         <is>
-          <t>NR119</t>
+          <t>NR118</t>
         </is>
       </c>
       <c r="B156" s="1" t="inlineStr">
         <is>
-          <t>QL011</t>
+          <t>QL010</t>
         </is>
       </c>
       <c r="C156" s="1" t="inlineStr">
         <is>
-          <t>SO2</t>
+          <t>SCT015</t>
         </is>
       </c>
       <c r="D156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8020</t>
+          <t>VLINE-8019</t>
         </is>
       </c>
       <c r="E156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8137</t>
+          <t>VLINE-8136</t>
         </is>
       </c>
       <c r="F156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8365</t>
+          <t>VLINE-8362</t>
         </is>
       </c>
       <c r="G156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8615</t>
+          <t>VLINE-8610</t>
         </is>
       </c>
       <c r="H156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8773</t>
+          <t>VLINE-8770</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="1" t="inlineStr">
         <is>
-          <t>NR120</t>
+          <t>NR119</t>
         </is>
       </c>
       <c r="B157" s="1" t="inlineStr">
         <is>
-          <t>QL012</t>
+          <t>QL011</t>
         </is>
       </c>
       <c r="C157" s="1" t="inlineStr">
         <is>
-          <t>SO3</t>
+          <t>SO2</t>
         </is>
       </c>
       <c r="D157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8023</t>
+          <t>VLINE-8020</t>
         </is>
       </c>
       <c r="E157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8140</t>
+          <t>VLINE-8137</t>
         </is>
       </c>
       <c r="F157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8366</t>
+          <t>VLINE-8363</t>
         </is>
       </c>
       <c r="G157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8617</t>
+          <t>VLINE-8612</t>
         </is>
       </c>
       <c r="H157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8774</t>
+          <t>VLINE-8772</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="1" t="inlineStr">
         <is>
-          <t>NR121</t>
+          <t>NR120</t>
         </is>
       </c>
       <c r="B158" s="1" t="inlineStr">
         <is>
-          <t>QL014</t>
+          <t>QL012</t>
         </is>
       </c>
       <c r="C158" s="1" t="inlineStr">
         <is>
-          <t>SSR101</t>
+          <t>SO3</t>
         </is>
       </c>
       <c r="D158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8025</t>
+          <t>VLINE-8023</t>
         </is>
       </c>
       <c r="E158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8141</t>
+          <t>VLINE-8140</t>
         </is>
       </c>
       <c r="F158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8368</t>
+          <t>VLINE-8365</t>
         </is>
       </c>
       <c r="G158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8620</t>
+          <t>VLINE-8615</t>
         </is>
       </c>
       <c r="H158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8776</t>
+          <t>VLINE-8773</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="1" t="inlineStr">
         <is>
-          <t>NR122</t>
+          <t>NR121</t>
         </is>
       </c>
       <c r="B159" s="1" t="inlineStr">
         <is>
-          <t>QL017</t>
+          <t>QL014</t>
         </is>
       </c>
       <c r="C159" s="1" t="inlineStr">
         <is>
-          <t>SSR102</t>
+          <t>SSR101</t>
         </is>
       </c>
       <c r="D159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8026</t>
+          <t>VLINE-8025</t>
         </is>
       </c>
       <c r="E159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8142</t>
+          <t>VLINE-8141</t>
         </is>
       </c>
       <c r="F159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8369</t>
+          <t>VLINE-8366</t>
         </is>
       </c>
       <c r="G159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8625</t>
+          <t>VLINE-8617</t>
         </is>
       </c>
       <c r="H159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8778</t>
+          <t>VLINE-8774</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="1" t="inlineStr">
         <is>
-          <t>P14</t>
+          <t>NR122</t>
         </is>
       </c>
       <c r="B160" s="1" t="inlineStr">
         <is>
-          <t>QL018</t>
+          <t>QL017</t>
         </is>
       </c>
       <c r="C160" s="1" t="inlineStr">
         <is>
-          <t>SSR103</t>
+          <t>SSR102</t>
         </is>
       </c>
       <c r="D160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8027</t>
+          <t>VLINE-8026</t>
         </is>
       </c>
       <c r="E160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8144</t>
+          <t>VLINE-8142</t>
         </is>
       </c>
       <c r="F160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8403</t>
+          <t>VLINE-8368</t>
         </is>
       </c>
       <c r="G160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8630</t>
+          <t>VLINE-8620</t>
         </is>
       </c>
       <c r="H160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8779</t>
+          <t>VLINE-8776</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="1" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P14</t>
         </is>
       </c>
       <c r="B161" s="1" t="inlineStr">
         <is>
-          <t>QR1744</t>
+          <t>QL018</t>
         </is>
       </c>
       <c r="C161" s="1" t="inlineStr">
         <is>
-          <t>SSR104</t>
+          <t>SSR103</t>
         </is>
       </c>
       <c r="D161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8028</t>
+          <t>VLINE-8027</t>
         </is>
       </c>
       <c r="E161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8145</t>
+          <t>VLINE-8144</t>
         </is>
       </c>
       <c r="F161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8404</t>
+          <t>VLINE-8369</t>
         </is>
       </c>
       <c r="G161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8671</t>
+          <t>VLINE-8625</t>
         </is>
       </c>
       <c r="H161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8780</t>
+          <t>VLINE-8778</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="1" t="inlineStr">
         <is>
-          <t>P2501</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="B162" s="1" t="inlineStr">
         <is>
-          <t>QR1771</t>
+          <t>QR1744</t>
         </is>
       </c>
       <c r="C162" s="1" t="inlineStr">
         <is>
-          <t>T363</t>
+          <t>SSR104</t>
         </is>
       </c>
       <c r="D162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8029</t>
+          <t>VLINE-8028</t>
         </is>
       </c>
       <c r="E162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8148</t>
+          <t>VLINE-8145</t>
         </is>
       </c>
       <c r="F162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8406</t>
+          <t>VLINE-8403</t>
         </is>
       </c>
       <c r="G162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8706</t>
+          <t>VLINE-8630</t>
         </is>
       </c>
       <c r="H162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8781</t>
+          <t>VLINE-8779</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="1" t="inlineStr">
         <is>
-          <t>P2502</t>
+          <t>P2501</t>
         </is>
       </c>
       <c r="B163" s="1" t="inlineStr">
         <is>
-          <t>QR5404</t>
+          <t>QR1771</t>
         </is>
       </c>
       <c r="C163" s="1" t="inlineStr">
         <is>
-          <t>T381</t>
+          <t>T363</t>
         </is>
       </c>
       <c r="D163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8030</t>
+          <t>VLINE-8029</t>
         </is>
       </c>
       <c r="E163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8150</t>
+          <t>VLINE-8148</t>
         </is>
       </c>
       <c r="F163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8408</t>
+          <t>VLINE-8404</t>
         </is>
       </c>
       <c r="G163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8711</t>
+          <t>VLINE-8671</t>
         </is>
       </c>
       <c r="H163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8782</t>
+          <t>VLINE-8780</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="1" t="inlineStr">
         <is>
-          <t>P2503</t>
+          <t>P2502</t>
         </is>
       </c>
       <c r="B164" s="1" t="inlineStr">
         <is>
-          <t>R711</t>
+          <t>QR5404</t>
         </is>
       </c>
       <c r="C164" s="1" t="inlineStr">
         <is>
-          <t>T386</t>
+          <t>T381</t>
         </is>
       </c>
       <c r="D164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8031</t>
+          <t>VLINE-8030</t>
         </is>
       </c>
       <c r="E164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8151</t>
+          <t>VLINE-8150</t>
         </is>
       </c>
       <c r="F164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8410</t>
+          <t>VLINE-8406</t>
         </is>
       </c>
       <c r="G164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8714</t>
+          <t>VLINE-8706</t>
         </is>
       </c>
       <c r="H164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8783</t>
+          <t>VLINE-8781</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="1" t="inlineStr">
         <is>
-          <t>P2504</t>
+          <t>P2503</t>
         </is>
       </c>
       <c r="B165" s="1" t="inlineStr">
         <is>
-          <t>R766</t>
+          <t>R711</t>
         </is>
       </c>
       <c r="C165" s="1" t="inlineStr">
         <is>
-          <t>TDX101</t>
+          <t>T386</t>
         </is>
       </c>
       <c r="D165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8032</t>
+          <t>VLINE-8031</t>
         </is>
       </c>
       <c r="E165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8152</t>
+          <t>VLINE-8151</t>
         </is>
       </c>
       <c r="F165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8411</t>
+          <t>VLINE-8408</t>
         </is>
       </c>
       <c r="G165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8717</t>
+          <t>VLINE-8711</t>
         </is>
       </c>
       <c r="H165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8784</t>
+          <t>VLINE-8782</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="1" t="inlineStr">
         <is>
-          <t>P2505</t>
+          <t>P2504</t>
         </is>
       </c>
       <c r="B166" s="1" t="inlineStr">
         <is>
-          <t>RB2353</t>
+          <t>R766</t>
         </is>
       </c>
       <c r="C166" s="1" t="inlineStr">
         <is>
-          <t>TE2801</t>
+          <t>TDX101</t>
         </is>
       </c>
       <c r="D166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8036</t>
+          <t>VLINE-8032</t>
         </is>
       </c>
       <c r="E166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8153</t>
+          <t>VLINE-8152</t>
         </is>
       </c>
       <c r="F166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8413</t>
+          <t>VLINE-8410</t>
         </is>
       </c>
       <c r="G166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8720</t>
+          <t>VLINE-8714</t>
         </is>
       </c>
       <c r="H166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8786</t>
+          <t>VLINE-8783</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="1" t="inlineStr">
         <is>
-          <t>P2506</t>
+          <t>P2505</t>
         </is>
       </c>
       <c r="B167" s="1" t="inlineStr">
         <is>
-          <t>RCTST4</t>
+          <t>RB2353</t>
         </is>
       </c>
       <c r="C167" s="1" t="inlineStr">
         <is>
-          <t>TE2802</t>
+          <t>TE2801</t>
         </is>
       </c>
       <c r="D167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8038</t>
+          <t>VLINE-8036</t>
         </is>
       </c>
       <c r="E167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8154</t>
+          <t>VLINE-8153</t>
         </is>
       </c>
       <c r="F167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8415</t>
+          <t>VLINE-8411</t>
         </is>
       </c>
       <c r="G167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8721</t>
+          <t>VLINE-8717</t>
         </is>
       </c>
       <c r="H167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8787</t>
+          <t>VLINE-8784</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="1" t="inlineStr">
         <is>
-          <t>P2507</t>
+          <t>P2506</t>
         </is>
       </c>
       <c r="B168" s="1" t="inlineStr">
         <is>
-          <t>RL301</t>
+          <t>RCTST4</t>
         </is>
       </c>
       <c r="C168" s="1" t="inlineStr">
         <is>
-          <t>TE2803</t>
+          <t>TE2802</t>
         </is>
       </c>
       <c r="D168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8039</t>
+          <t>VLINE-8038</t>
         </is>
       </c>
       <c r="E168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8155</t>
+          <t>VLINE-8154</t>
         </is>
       </c>
       <c r="F168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8417</t>
+          <t>VLINE-8413</t>
         </is>
       </c>
       <c r="G168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8723</t>
+          <t>VLINE-8720</t>
         </is>
       </c>
       <c r="H168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8788</t>
+          <t>VLINE-8786</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="1" t="inlineStr">
         <is>
-          <t>P2508</t>
+          <t>P2507</t>
         </is>
       </c>
       <c r="B169" s="1" t="inlineStr">
         <is>
-          <t>RL302</t>
+          <t>RL301</t>
         </is>
       </c>
       <c r="C169" s="1" t="inlineStr">
         <is>
-          <t>TE2804</t>
+          <t>TE2803</t>
         </is>
       </c>
       <c r="D169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8042</t>
+          <t>VLINE-8039</t>
         </is>
       </c>
       <c r="E169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8157</t>
+          <t>VLINE-8155</t>
         </is>
       </c>
       <c r="F169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8418</t>
+          <t>VLINE-8415</t>
         </is>
       </c>
       <c r="G169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8725</t>
+          <t>VLINE-8721</t>
         </is>
       </c>
       <c r="H169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8790</t>
+          <t>VLINE-8787</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="1" t="inlineStr">
         <is>
-          <t>P2509</t>
+          <t>P2508</t>
         </is>
       </c>
       <c r="B170" s="1" t="inlineStr">
         <is>
-          <t>RL304</t>
+          <t>RL302</t>
         </is>
       </c>
       <c r="C170" s="1" t="inlineStr">
         <is>
-          <t>TE2805</t>
+          <t>TE2804</t>
         </is>
       </c>
       <c r="D170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8049</t>
+          <t>VLINE-8042</t>
         </is>
       </c>
       <c r="E170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8158</t>
+          <t>VLINE-8157</t>
         </is>
       </c>
       <c r="F170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8419</t>
+          <t>VLINE-8417</t>
         </is>
       </c>
       <c r="G170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8726</t>
+          <t>VLINE-8723</t>
         </is>
       </c>
       <c r="H170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8792</t>
+          <t>VLINE-8788</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8793</t>
+          <t>VLINE-8790</t>
         </is>
       </c>
       <c r="B172" s="1" t="inlineStr">
         <is>
-          <t>XP2012</t>
+          <t>XP2008</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8794</t>
+          <t>VLINE-8792</t>
         </is>
       </c>
       <c r="B173" s="1" t="inlineStr">
         <is>
-          <t>XP2013</t>
+          <t>XP2010</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8795</t>
+          <t>VLINE-8793</t>
         </is>
       </c>
       <c r="B174" s="1" t="inlineStr">
         <is>
-          <t>XP2014</t>
+          <t>XP2011</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8796</t>
+          <t>VLINE-8794</t>
         </is>
       </c>
       <c r="B175" s="1" t="inlineStr">
         <is>
-          <t>XP2015</t>
+          <t>XP2012</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8797</t>
+          <t>VLINE-8795</t>
         </is>
       </c>
       <c r="B176" s="1" t="inlineStr">
         <is>
-          <t>XP2016</t>
+          <t>XP2013</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8799</t>
+          <t>VLINE-8796</t>
         </is>
       </c>
       <c r="B177" s="1" t="inlineStr">
         <is>
-          <t>XP2017</t>
+          <t>XP2014</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8800</t>
+          <t>VLINE-8797</t>
         </is>
       </c>
       <c r="B178" s="1" t="inlineStr">
         <is>
-          <t>XP2019</t>
+          <t>XP2015</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8801</t>
+          <t>VLINE-8799</t>
         </is>
       </c>
       <c r="B179" s="1" t="inlineStr">
         <is>
-          <t>XR550</t>
+          <t>XP2016</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8802</t>
+          <t>VLINE-8800</t>
         </is>
       </c>
       <c r="B180" s="1" t="inlineStr">
         <is>
-          <t>XR552</t>
+          <t>XP2017</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8803</t>
+          <t>VLINE-8801</t>
         </is>
       </c>
       <c r="B181" s="1" t="inlineStr">
         <is>
-          <t>XR559</t>
+          <t>XP2019</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8804</t>
+          <t>VLINE-8802</t>
         </is>
       </c>
       <c r="B182" s="1" t="inlineStr">
         <is>
-          <t>XRN001</t>
+          <t>XR550</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8805</t>
+          <t>VLINE-8803</t>
         </is>
       </c>
       <c r="B183" s="1" t="inlineStr">
         <is>
-          <t>XRN004</t>
+          <t>XR552</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8806</t>
+          <t>VLINE-8804</t>
         </is>
       </c>
       <c r="B184" s="1" t="inlineStr">
         <is>
-          <t>XRN005</t>
+          <t>XR559</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8807</t>
+          <t>VLINE-8805</t>
         </is>
       </c>
       <c r="B185" s="1" t="inlineStr">
         <is>
-          <t>XRN006</t>
+          <t>XRN001</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8808</t>
+          <t>VLINE-8806</t>
         </is>
       </c>
       <c r="B186" s="1" t="inlineStr">
         <is>
-          <t>XRN007</t>
+          <t>XRN004</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8809</t>
+          <t>VLINE-8807</t>
         </is>
       </c>
       <c r="B187" s="1" t="inlineStr">
         <is>
-          <t>XRN009</t>
+          <t>XRN005</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8810</t>
+          <t>VLINE-8808</t>
         </is>
       </c>
       <c r="B188" s="1" t="inlineStr">
         <is>
-          <t>XRN011</t>
+          <t>XRN006</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8811</t>
+          <t>VLINE-8809</t>
         </is>
       </c>
       <c r="B189" s="1" t="inlineStr">
         <is>
-          <t>XRN014</t>
+          <t>XRN007</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8812</t>
+          <t>VLINE-8810</t>
         </is>
       </c>
       <c r="B190" s="1" t="inlineStr">
         <is>
-          <t>XRN017</t>
+          <t>XRN009</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8813</t>
+          <t>VLINE-8811</t>
         </is>
       </c>
       <c r="B191" s="1" t="inlineStr">
         <is>
-          <t>XRN018</t>
+          <t>XRN011</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8814</t>
+          <t>VLINE-8812</t>
         </is>
       </c>
       <c r="B192" s="1" t="inlineStr">
         <is>
-          <t>XRN020</t>
+          <t>XRN014</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8815</t>
+          <t>VLINE-8813</t>
         </is>
       </c>
       <c r="B193" s="1" t="inlineStr">
         <is>
-          <t>XRN021</t>
+          <t>XRN017</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8816</t>
+          <t>VLINE-8814</t>
         </is>
       </c>
       <c r="B194" s="1" t="inlineStr">
         <is>
-          <t>XRN023</t>
+          <t>XRN018</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8817</t>
+          <t>VLINE-8815</t>
         </is>
       </c>
       <c r="B195" s="1" t="inlineStr">
         <is>
-          <t>XRN025</t>
+          <t>XRN020</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8818</t>
+          <t>VLINE-8816</t>
         </is>
       </c>
       <c r="B196" s="1" t="inlineStr">
         <is>
-          <t>XRN026</t>
+          <t>XRN021</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8819</t>
+          <t>VLINE-8817</t>
         </is>
       </c>
       <c r="B197" s="1" t="inlineStr">
         <is>
-          <t>XRN027</t>
+          <t>XRN023</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8820</t>
+          <t>VLINE-8818</t>
         </is>
       </c>
       <c r="B198" s="1" t="inlineStr">
         <is>
-          <t>XRN029</t>
+          <t>XRN025</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8822</t>
+          <t>VLINE-8819</t>
         </is>
       </c>
       <c r="B199" s="1" t="inlineStr">
         <is>
-          <t>Y163</t>
+          <t>XRN026</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8860</t>
+          <t>VLINE-8820</t>
+        </is>
+      </c>
+      <c r="B200" s="1" t="inlineStr">
+        <is>
+          <t>XRN027</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8861</t>
+          <t>VLINE-8821</t>
+        </is>
+      </c>
+      <c r="B201" s="1" t="inlineStr">
+        <is>
+          <t>XRN029</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8862</t>
+          <t>VLINE-8822</t>
+        </is>
+      </c>
+      <c r="B202" s="1" t="inlineStr">
+        <is>
+          <t>Y163</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8863</t>
+          <t>VLINE-8860</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8864</t>
+          <t>VLINE-8861</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8865</t>
+          <t>VLINE-8862</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8866</t>
+          <t>VLINE-8863</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8867</t>
+          <t>VLINE-8864</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8868</t>
+          <t>VLINE-8865</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8869</t>
+          <t>VLINE-8866</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8890</t>
+          <t>VLINE-8867</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8891</t>
+          <t>VLINE-8868</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8893</t>
+          <t>VLINE-8869</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8895</t>
+          <t>VLINE-8890</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" s="1" t="inlineStr">
         <is>
-          <t>WH001</t>
+          <t>VLINE-8891</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" s="1" t="inlineStr">
         <is>
-          <t>WH003</t>
+          <t>VLINE-8893</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="1" t="inlineStr">
         <is>
-          <t>WL02</t>
+          <t>VLINE-8895</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="1" t="inlineStr">
         <is>
-          <t>X12-X14</t>
+          <t>WH001</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="1" t="inlineStr">
         <is>
-          <t>X31</t>
+          <t>WH003</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="1" t="inlineStr">
         <is>
-          <t>XP2000</t>
+          <t>WL02</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" s="1" t="inlineStr">
         <is>
-          <t>XP2001</t>
+          <t>X12-X14</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="1" t="inlineStr">
         <is>
-          <t>XP2003</t>
+          <t>X31</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="1" t="inlineStr">
         <is>
-          <t>XP2004</t>
+          <t>XP2000</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="1" t="inlineStr">
         <is>
-          <t>XP2005</t>
+          <t>XP2001</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" s="1" t="inlineStr">
         <is>
-          <t>XP2007</t>
+          <t>XP2003</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="1" t="inlineStr">
         <is>
-          <t>XP2008</t>
+          <t>XP2004</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" s="1" t="inlineStr">
         <is>
-          <t>XP2010</t>
+          <t>XP2005</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" s="1" t="inlineStr">
         <is>
-          <t>XP2011</t>
+          <t>XP2007</t>
         </is>
       </c>
     </row>

</xml_diff>